<commit_message>
Add Topics Queue sheet with 30 prioritized topics
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -7,14 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handles" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Post Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Post Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Handles'!$A$1:$Y$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Topics'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Post Log'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Topics Queue'!$A$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Handles'!$A$1:$Y$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Topics'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Post Log'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +39,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001e2d3d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,11 +80,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,6 +452,585 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Scheduled Date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Psychological Safety</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>First run</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Growth Mindset</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Education footer variant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Psychological Safety in Schools</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Education footer variant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Education footer variant</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>High-Performing Teams</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Leadership During Crisis</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E31"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -602,7 +1194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -645,7 +1237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Update handle database — Emotional Intelligence
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -525,10 +525,14 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -1031,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:Y18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1188,6 +1192,1255 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Daniel Goleman</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Psychologist &amp; Science Journalist</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Author of 'Emotional Intelligence'</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Popularised the concept of emotional intelligence in his 1995 bestseller</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>danielgoleman</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>@DanielGolemanEI</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dr. Marc Brackett</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Director, Yale Center for EI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Yale University</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Creator of the RULER framework, author of Permission to Feel</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>@marc.brackett</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>@marcbrackett</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Brené Brown</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Research Professor &amp; Author</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>University of Houston</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>World-renowned researcher on vulnerability, courage, and empathy</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>brenebrown</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>favikon.com</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>@brenebrown</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>@BreneBrown</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>@brenebrown</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dr. Susan David</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Psychologist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Creator of the concept of Emotional Agility, WSJ #1 bestseller</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>@susandavid_phd</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>@SusanDavid_PhD</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dr. Travis Bradberry</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Co-founder, TalentSmartEQ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Author of 'Emotional Intelligence 2.0'</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Co-author of the world's bestselling EQ book with 5M+ copies sold</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>@talentsmarteq</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Adam Grant</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Organizational Psychologist</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Wharton School, UPenn</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>#1 NYT bestselling author, host of Re:Thinking podcast</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AdamMGrant</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>@adamgrant</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>@adamgrant</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>@AdamMGrant</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dr. Tasha Eurich</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Organizational Psychologist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The Eurich Group</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Leading researcher on self-awareness, NYT bestselling author of Insight</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TashaEurich</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>@tashaeurich</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>@tashaeurich</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Justin Bariso</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Author &amp; EQ Consultant</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EQ Applied LLC</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Known as The EQ Guy, Inc.com columnist, author of EQ Applied</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>@JustinJBariso</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jamil Zaki</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Professor of Psychology</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Director of Stanford Social Neuroscience Lab, author of The War for Kindness</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>@zakijam</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Shawn Achor</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Positive Psychology Researcher</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GoodThink Inc.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NYT bestselling author of The Happiness Advantage, TED talk 25M+ views</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>shawnachor</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>@shawnachor</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>@shawnachor</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dr. Robin Stern</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Co-founder, Yale Center for EI</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yale University</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Co-developer of RULER, author of The Gaslight Effect</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>@RobinSStern</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Dr. Richard Boyatzis</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Distinguished University Professor</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Case Western Reserve University</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Pioneering researcher on emotional intelligence in leadership</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>@RBoyatzis</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Dr. Helen Riess</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Associate Professor of Psychiatry</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Founder of Empathetics, author of The Empathy Effect</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>@HelenRiessMD</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>JP Pawliw-Fry</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Leadership &amp; Performance Expert</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>IHHP</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NYT bestselling co-author of Performing Under Pressure</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Liz Fosslien</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Author &amp; Illustrator</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Author of 'No Hard Feelings'</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Bestselling author making the science of emotions at work accessible</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>@fosslien</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Erica Dhawan</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Keynote Speaker &amp; Author</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Author of 'Digital Body Language'</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Leading authority on Connectional Intelligence and digital body language</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>@ericadhawan</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>@ericadhawan</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Amy Edmondson</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Professor, Harvard Business School</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Harvard University</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Pioneered concept of psychological safety, #1 Thinkers50 ranked</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>@AmyCEdmondson</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1200,7 +2453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1228,6 +2481,26 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Slug</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>emotional-intelligence</t>
         </is>
       </c>
     </row>
@@ -1243,7 +2516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1292,6 +2565,302 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>69c2194747c72b7746515fe5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-03-28T16:12:00Z</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>69c2194947c72b774651600b</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-03-28T18:02:00Z</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>69c2195e47c72b774651606c</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-28T01:02:00Z</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>69c2196106e664e154fe5aa6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-03-28T14:30:00Z</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>69c2196247c72b77465160aa</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-03-28T14:30:00Z</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>69c2198347c72b77465161d0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-03-25T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>69c2197706e664e154fe5b63</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-03-28T21:30:00Z</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>69c2198447c72b77465161f8</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-03-28T06:12:00Z</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Servant Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -546,10 +546,14 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
@@ -1035,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:Y33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2441,6 +2445,1091 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ken Blanchard</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Author &amp; Leadership Expert</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The Ken Blanchard Companies</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Co-author of The One Minute Manager, champion of servant leadership</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>KenBlanchard</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ken.blanchard</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>@kenblanchard</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Simon Sinek</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Author &amp; Optimist</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>The Optimism Company</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Author of Leaders Eat Last and Start With Why, TED talk 60M+ views</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>simonsinek</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>@simonsinek</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>@simonsinek</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>@simonsinek</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>@SimonSinek</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>youtube.com</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>John Maxwell</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Leadership Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Maxwell Leadership</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>#1 NYT bestselling author of 70+ books on leadership</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>JohnCMaxwellOfficial</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>@johncmaxwell</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>@JohnCMaxwell</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>@thejohncmaxwell</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>The Table Group</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Author of Five Dysfunctions of a Team, creator of Working Genius</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>@patricklencioniofficial</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>@patricklencioni</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Stephen M.R. Covey</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Author &amp; Trust Expert</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CoveyLink / FranklinCovey</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Author of The Speed of Trust and Trust &amp; Inspire</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>@stephenmrcovey</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>@StephenMRCovey</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Marshall Goldsmith</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Marshall Goldsmith Inc.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Only two-time #1 Leadership Thinker (Thinkers50), author of What Got You Here</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Marshall.Goldsmith.Library</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>@marshall_goldsmith</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>@CoachGoldsmith</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Liz Wiseman</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Author &amp; Researcher</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The Wiseman Group</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Author of Multipliers, #1 leadership thinker Thinkers50 2019</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>liz.wiseman.author</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>@bylizwiseman</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>@LizWiseman</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cheryl Bachelder</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Former CEO of Popeyes</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Author of Dare to Serve</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Turned Popeyes around using servant leadership principles</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>@CABachelder</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mark Miller</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Author &amp; Former VP</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Chick-fil-A / Lead Every Day</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Spent 40+ years at Chick-fil-A, bestselling author of The Heart of Leadership</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>James Hunter</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>J.D. Hunter Associates</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Author of The Servant, sold over 6 million copies</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Art Barter</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Servant Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Turned Datron from $10M to $200M company using servant leadership</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Matt Tenney</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Author</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Inspire Greatness</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Author of Serve to Be Great, TED talk 1M+ views</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Howard Behar</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Former President</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Starbucks</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Led Starbucks from 28 to 15,000+ stores, author of It's Not About the Coffee</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Larry Spears</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CEO, Spears Center</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Spears Center for Servant Leadership</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Former CEO of Greenleaf Center, defined 10 servant leadership characteristics</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Ben Lichtenwalner</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Modern Servant Leader</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Founded ModernServantLeader.com, leading voice on modern servant leadership</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2453,7 +3542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2501,6 +3590,26 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>emotional-intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>servant-leadership</t>
         </is>
       </c>
     </row>
@@ -2516,7 +3625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2861,6 +3970,302 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>69c21cb606e664e154fe69a2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-03-28T18:02:00Z</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>69c21cb906e664e154fe69d5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-03-28T20:02:00Z</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>69c21cb947c72b77465170ad</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-03-28T03:02:00Z</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>69c21cbb06e664e154fe69fb</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-28T16:12:00Z</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>69c21cd306e664e154fe6a29</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-03-28T16:12:00Z</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>69c21cd447c72b77465170fc</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-26T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>69c21cd547c72b7746517123</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-28T23:02:00Z</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Servant Leadership</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>69c21cd606e664e154fe6a4f</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-28T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Trust in Teams
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -567,10 +567,14 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1039,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y33"/>
+  <dimension ref="A1:Y42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3530,6 +3534,489 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rachel Botsman</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Author &amp; Trust Fellow</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Oxford University</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>First Trust Fellow at Oxford, author of 'Who Can You Trust?' on trust in the digital age.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>@rachelbotsman</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>@rachelbotsman</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Assumed from IG</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>@rachelbotsman</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Frances Frei</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Professor of TOM</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Created the trust triangle framework of authenticity, logic, and empathy.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>@francesxfrei</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>@FrancesFrei</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>David Horsager</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CEO, Trust Edge Leadership Institute</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Trust Edge Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Invented the Enterprise Trust Index and developed the 8-Pillar Framework.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>DavidHorsager</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>@davidhorsager</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>@DavidHorsager</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>HorsagerLeadership</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Charles Feltman</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Insight Coaching</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Author of 'The Thin Book of Trust', defining trust through sincerity, reliability, competence, and care.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Charles.Feltman</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Dennis Reina</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Trust Building Consultant</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Reina Trust Building</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Pioneer in workplace trust research, co-author of 'Trust &amp; Betrayal in the Workplace'.</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>@DrDennisReina</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Henry Cloud</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Psychologist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Cloud-Townsend</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Clinical psychologist and bestselling author of 'Trust', exploring when to give and withhold trust.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>@drhenrycloudofficial</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>@DrHenryCloud</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Paul Zak</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Neuroeconomist</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Claremont Graduate University</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Discovered the neuroscience behind trust, showing how oxytocin drives team connection.</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>@pauljzak</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Keith Ferrazzi</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Executive Team Coach</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Ferrazzi Greenlight</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Author of 'Leading Without Authority', teaching co-elevation as the path to team trust.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>keithferrazzi</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>@keithferrazzi</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>@ferrazzi</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Erin Meyer</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Professor, INSEAD</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>INSEAD</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Author of 'The Culture Map', revealing how trust is built differently across cultures.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>@erinmeyerspeaks</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>@ErinMeyerINSEAD</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3542,7 +4029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3610,6 +4097,26 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>servant-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>trust-in-teams</t>
         </is>
       </c>
     </row>
@@ -3625,7 +4132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4266,6 +4773,302 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>69c2217806e664e154fe8495</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-28T20:02:00Z</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>69c221aa06e664e154fe8754</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-28T21:30:00Z</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>69c221ab06e664e154fe877a</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-28T05:02:00Z</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>69c2218d47c72b7746518bc7</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-03-28T18:02:00Z</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>69c221ba47c72b7746518e10</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-03-26T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>69c221ac47c72b7746518cf8</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-03-29T01:02:00Z</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>69c2218e06e664e154fe8606</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-28T18:02:00Z</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Trust in Teams</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>69c221bb06e664e154fe88b8</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-28T10:02:00Z</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Change Management
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -588,10 +588,14 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1043,7 +1047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4017,6 +4021,1345 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>John Kotter</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Professor Emeritus</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Creator of 8-Step Change Model, author of Leading Change</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>@kotter_inc</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Instagram search</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>@JohnPKotter</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Peter F. Gallagher</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>#1 CM Thought Leader</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Leadership of Change</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>#1 Thinkers360 Change Management 2020-2025, 15x author</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>@peter_f_gallagher</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Daryl Conner</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Founder &amp; Chairman</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Conner Advisory</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Author of Managing at the Speed of Change, 50+ years studying change</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>@changethinking</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr"/>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Rosabeth Moss Kanter</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Author of The Change Masters, pioneer in organisational change</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>@RosabethKanter</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr"/>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Paul Gibbons</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Author &amp; Change Scientist</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Phronesis Media</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Author of The Science of Organizational Change and The Future of Change Management (2024)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>@PaulGGibbons</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>X search</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Hilary Scarlett</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Scarlett &amp; Grey</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Author of Neuroscience for Organizational Change (3rd ed 2025)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>@Hilary_Scarlett</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>April Rinne</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Futurist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Author of Flux: 8 Superpowers for Thriving in Constant Change, Forbes 50 Female Futurists</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>@aprilrinne</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>@aprilrinne</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Lena Ross</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Agile Change Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Author of Change Management: The Essentials, creator of #changehacks</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>changehacks</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>@changeessentials</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>@LenaEmelyRoss</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Jason Little</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Lean Change Management</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Author of Lean Change Management and Change Agility, created iterative Lean Change framework</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Theresa Moulton</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Editor-in-Chief</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Change Management Review</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Founded leading global media platform for CM professionals, hosts 120+ podcast episodes</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr"/>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Jenelle McMaster</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Regional Deputy CEO Oceania</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Host of Change Happens - Australia #1 management podcast, 20+ years transformational change</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Isolde Kanikani</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>VP Global Board</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ACMP</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>VP of Association of Change Management Professionals, author of 4 books on change leadership</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tricia Kennedy</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Kennedy Consulting Services</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Co-author of Change Myths and The Future of Change Management, human-centred change specialist</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Esther Derby</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Author &amp; Change Expert</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>esther derby associates</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Author of 7 Rules for Positive Productive Change, 4 decades in organisational change</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>@estherderby</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>Mentioned on website</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Tim Creasey</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Chief Innovation Officer</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Prosci</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Architect of world's largest CM body of knowledge, co-author Best Practices in Change Management</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>@timcreasey</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Elsbeth Johnson</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Senior Lecturer</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>MIT Sloan School of Management</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Author of Step Up Step Back, researches strategic change without leader dependency</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>@elsbeth_johnson</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Dr. Jen Frahm</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Agile Change Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Author of Conversations of Change and Change. Leader, Melbourne-based transformation expert</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>@jenfrahm</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Search results</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr"/>
+      <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4029,7 +5372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4117,6 +5460,26 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>trust-in-teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>change-management</t>
         </is>
       </c>
     </row>
@@ -4132,7 +5495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5069,6 +6432,302 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>69c22a9e47c72b774651bdda</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-03-28T21:30:00Z</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>69c22aa006e664e154feb8c8</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-28T23:02:00Z</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>69c22aa247c72b774651be00</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-28T20:02:00Z</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>69c22ab806e664e154feb8f9</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-28T20:02:00Z</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>69c22ab947c72b774651be2a</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-28T07:02:00Z</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>69c22ab947c72b774651be5d</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-29T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>69c22aba06e664e154feb932</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-28T11:30:00Z</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Change Management</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>69c22ac506e664e154feb9be</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-27T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mark Growth Mindset as DONE
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -609,10 +609,14 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
@@ -4042,13 +4046,11 @@
           <t>Creator of the 8-Step Change Process, author of Leading Change</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>kotter_inc</t>
@@ -4064,13 +4066,11 @@
           <t>Instagram search</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>JohnPKotter</t>
@@ -4086,27 +4086,21 @@
           <t>X search</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4129,13 +4123,11 @@
           <t>#1 Change Management Thought Leader on Thinkers360, 20 books</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>peter_f_gallagher</t>
@@ -4151,41 +4143,31 @@
           <t>Instagram search</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
       <c r="X44" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4208,27 +4190,21 @@
           <t>45+ years in change execution, author of Managing at the Speed of Change</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>changethinking</t>
@@ -4244,27 +4220,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4302,20 +4272,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>chipheath</t>
@@ -4331,27 +4297,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr"/>
-      <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4389,48 +4349,36 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4453,27 +4401,21 @@
           <t>Author of The Science of Organizational Change, top 10 change book of all time</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>paulggibbons</t>
@@ -4489,27 +4431,21 @@
           <t>LinkedIn/X</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4547,20 +4483,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>rickmaurer2</t>
@@ -4576,27 +4508,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
       <c r="X49" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4619,27 +4545,21 @@
           <t>Author of 7 Rules for Positive, Productive Change, agile change pioneer</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>estherderby</t>
@@ -4655,20 +4575,16 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr"/>
-      <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr">
         <is>
           <t>estherderby</t>
@@ -4721,20 +4637,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>drjenfrahm</t>
@@ -4750,27 +4662,21 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr"/>
-      <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
       <c r="X51" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4793,55 +4699,41 @@
           <t>Author of Change Management: The Essentials, blends neuroscience and design thinking</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr"/>
-      <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4879,20 +4771,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>april_callis</t>
@@ -4908,27 +4796,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr"/>
-      <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4951,55 +4833,41 @@
           <t>25+ years in change consulting, hosts leading change management podcast</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
       <c r="X54" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5022,55 +4890,41 @@
           <t>Pioneer of Conscious Change Leadership, co-author of Beyond Change Management</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5093,55 +4947,41 @@
           <t>Original creator of Organisation Transformation field, co-author of The Change Leader's Roadmap</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr"/>
       <c r="X56" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5164,27 +5004,21 @@
           <t>Built the Managed Change Model over 4 decades, certified 700+ practitioners</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
           <t>jennlamarsh</t>
@@ -5200,27 +5034,21 @@
           <t>X search</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr"/>
-      <c r="T57" t="inlineStr"/>
       <c r="U57" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5243,55 +5071,41 @@
           <t>Global authority on people side of change, champion of the ADKAR model</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr"/>
-      <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V58" t="inlineStr"/>
-      <c r="W58" t="inlineStr"/>
       <c r="X58" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5314,27 +5128,21 @@
           <t>30+ years in large-scale change, author of Change Management Training</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
           <t>elainebiech</t>
@@ -5350,27 +5158,21 @@
           <t>X search</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr"/>
-      <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y59" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>

</xml_diff>

<commit_message>
Update handle database — Resilience
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -630,10 +630,14 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1051,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y59"/>
+  <dimension ref="A1:Y76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5174,6 +5178,1833 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Dr. Karen Reivich</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Director of Training Programs</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Penn Positive Psychology Center</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Co-author of The Resilience Factor; trained 40,000+ Army Master Resilience Trainers</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>@reivich</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>@KarenReivich</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr"/>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dr. Lucy Hone</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>NZ Institute of Wellbeing &amp; Resilience</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TED talk 9M+ views; author of Resilient Grieving</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>DrLucyHone</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>@drlucyhone</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>@drlucyhone</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Dr. Taryn Marie Stejskal</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Founder &amp; CRO</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Resilience Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>WSJ bestselling author of The 5 Practices of Highly Resilient People</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>DrTarynMarie</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>@drtarynmarie</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>@drtarynmarie</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>@drtarynmarie</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>@dr.tarynmarie1729</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Anne Grady</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Resilience Expert &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Anne Grady Group</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Author of Mind Over Moment; two-time TEDx speaker</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>AnneGradyGroup</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>@annegradygroup</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>@annegradygroup</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>@AnneGradyGroup</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Kelly McGonigal</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Health Psychologist</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Author of The Upside of Stress; TED talk 30M+ views</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>kellymcgonigalauthor</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>@kellymariemcgonigal</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>@kellymcgonigal</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr"/>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Dr. Michael Ungar</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Canada Research Chair</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Dalhousie University</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>#1 ranked social work scholar; author of Change Your World</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>@michaelungar.phd</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>@MichaelUngarPhD</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Dr. Amit Sood</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Founder &amp; Executive Director</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Global Center for Resiliency &amp; Wellbeing</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Former Mayo Clinic Professor; 35+ clinical trials on resilience</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>@AmitSoodMD</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Graeme Cowan</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Founding Director</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>R U OK?</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Australia's leading team resilience speaker; author of Great Leaders Care</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>@graemecowan</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>@GraemeCowan</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr"/>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Angela Duckworth</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Professor of Psychology</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>University of Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Author of Grit; MacArthur Fellow; founder of Character Lab</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>angeladuckworthgrit</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>@angelalduckworth</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>@angeladuckw</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr"/>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Donna Jackson Nakazawa</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Science Journalist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Author of Childhood Disrupted on ACEs and resilience</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>donnajacksonnakazawaauthor</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>@donnajacksonnakazawa</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>@DonnaJackNak</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr"/>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Allison Graham</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Workplace Resilience Speaker</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Author of The Stress Illusion; featured on CTV, Global News</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>@allisondgraham</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>@allisondgraham</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>@AllisonDGraham</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Beth Benatti Kennedy</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Benatti Leadership Development</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Creator of Benatti Resiliency Model; author of ReThink Resilience</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>@coachbkennedy</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr"/>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Brad Hook</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Resilience Institute Global</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Author of Resilience Mastery; host of The Resilience Podcast</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>byBradleyHook</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>@bradleyhook</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Andrew Zolli</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Chief Impact Officer</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Planet</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Author of Resilience: Why Things Bounce Back</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>@andrew_zolli</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr"/>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Dr. Raphael Rose</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>UCLA Psychology</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>10+ years NASA resilience research; creator of SMART-OP</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Suniya Luthar</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Professor Emerita</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Columbia University</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Pioneering researcher on resilience in adversity</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>@suniya_luthar</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr"/>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Eduardo Briceño</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Author &amp; Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Growth.how</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Co-founded Mindset Works with Carol Dweck; author of The Performance Paradox</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>@ebriceno8</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>@ebriceno8</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr"/>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5186,7 +7017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5294,6 +7125,26 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>change-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>resilience</t>
         </is>
       </c>
     </row>
@@ -5309,7 +7160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6542,6 +8393,302 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>69c2333f47c72b774651e3d0</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-03-29T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>69c2335747c72b774651e406</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-29T20:30:00Z</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>69c2336106e664e154fedbda</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-29T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>69c2336447c72b774651e431</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-03-29T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>69c2336f06e664e154fedc49</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-29T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>69c2337506e664e154fedc6e</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-28T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>69c2334206e664e154fedb76</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-30T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>69c2336706e664e154fedc23</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-29T10:02:00Z</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Coaching Cultures
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -651,10 +651,14 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1055,7 +1059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y76"/>
+  <dimension ref="A1:Y93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5199,7 +5203,6 @@
           <t>Co-author of The Resilience Factor; trained 40,000+ Army Master Resilience Trainers</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5225,7 +5228,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5251,7 +5253,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5262,7 +5263,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5273,7 +5273,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W60" t="inlineStr"/>
       <c r="X60" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5336,7 +5335,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5347,7 +5345,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5373,7 +5370,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5384,7 +5380,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W61" t="inlineStr"/>
       <c r="X61" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5477,7 +5472,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5503,7 +5497,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W62" t="inlineStr"/>
       <c r="X62" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5596,7 +5589,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5607,7 +5599,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5618,7 +5609,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W63" t="inlineStr"/>
       <c r="X63" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5681,7 +5671,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5707,7 +5696,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5718,7 +5706,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5729,7 +5716,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W64" t="inlineStr"/>
       <c r="X64" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5762,7 +5748,6 @@
           <t>#1 ranked social work scholar; author of Change Your World</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5788,7 +5773,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5814,7 +5798,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5825,7 +5808,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5836,7 +5818,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5869,7 +5850,6 @@
           <t>Former Mayo Clinic Professor; 35+ clinical trials on resilience</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5880,7 +5860,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5891,7 +5870,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5917,7 +5895,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5928,7 +5905,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T66" t="inlineStr"/>
       <c r="U66" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5939,7 +5915,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W66" t="inlineStr"/>
       <c r="X66" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5972,7 +5947,6 @@
           <t>Australia's leading team resilience speaker; author of Great Leaders Care</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -5998,7 +5972,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6024,7 +5997,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6035,7 +6007,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr"/>
       <c r="U67" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6046,7 +6017,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6109,7 +6079,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6135,7 +6104,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6146,7 +6114,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6157,7 +6124,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6180,7 +6146,6 @@
           <t>Science Journalist &amp; Author</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>Author of Childhood Disrupted on ACEs and resilience</t>
@@ -6216,7 +6181,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6242,7 +6206,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6253,7 +6216,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6264,7 +6226,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6287,13 +6248,11 @@
           <t>Workplace Resilience Speaker</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>Author of The Stress Illusion; featured on CTV, Global News</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6349,7 +6308,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6360,7 +6318,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr"/>
       <c r="U70" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6371,7 +6328,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6404,7 +6360,6 @@
           <t>Creator of Benatti Resiliency Model; author of ReThink Resilience</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6415,7 +6370,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6426,7 +6380,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6452,7 +6405,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr"/>
       <c r="R71" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6463,7 +6415,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6474,7 +6425,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6522,7 +6472,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6533,7 +6482,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6559,7 +6507,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6570,7 +6517,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6581,7 +6527,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6614,7 +6559,6 @@
           <t>Author of Resilience: Why Things Bounce Back</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6625,7 +6569,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6636,7 +6579,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6662,7 +6604,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6673,7 +6614,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6684,7 +6624,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W73" t="inlineStr"/>
       <c r="X73" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6717,7 +6656,6 @@
           <t>10+ years NASA resilience research; creator of SMART-OP</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6728,7 +6666,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6739,7 +6676,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6750,7 +6686,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6761,7 +6696,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q74" t="inlineStr"/>
       <c r="R74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6772,7 +6706,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6783,7 +6716,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6816,7 +6748,6 @@
           <t>Pioneering researcher on resilience in adversity</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6827,7 +6758,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6838,7 +6768,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6864,7 +6793,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6875,7 +6803,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6886,7 +6813,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6919,7 +6845,6 @@
           <t>Co-founded Mindset Works with Carol Dweck; author of The Performance Paradox</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6960,7 +6885,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6971,7 +6895,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6982,7 +6905,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -6993,7 +6915,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -7004,6 +6925,1369 @@
           <t>web search</t>
         </is>
       </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Michael Bungay Stanier</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Author &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Box of Crayons</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Author of The Coaching Habit - best-selling coaching book of the century</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>boxofcrayons.biz</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>@mbs_works</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>@boxofcrayons</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>X.com</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr"/>
+      <c r="W77" t="inlineStr"/>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Peter Hawkins</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Emeritus Professor</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Henley Business School</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Author of Creating a Coaching Culture, pioneer of systemic team coaching</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr"/>
+      <c r="W78" t="inlineStr"/>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Jonathan Passmore</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Henley Business School / EZRA</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Created LEAD Framework for coaching cultures, 45+ books</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr"/>
+      <c r="W79" t="inlineStr"/>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Marcia Reynolds</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Covisioning LLC</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Past ICF Global President, author of Coach the Person Not the Problem</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>@dr_marcia_reynolds</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>@MarciaReynolds</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>X.com</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr"/>
+      <c r="W80" t="inlineStr"/>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Julie Starr</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Starr Coaching</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Author of The Coaching Manual and Brilliant Coaching</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr"/>
+      <c r="W81" t="inlineStr"/>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Myles Downey</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>The School of Coaching</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Author of Effective Coaching, creator of Enable automated coaching</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>@mylesdowneycoach</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>@mylesdowney</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>X.com</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr"/>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr"/>
+      <c r="W82" t="inlineStr"/>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Thomas G. Crane</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Crane Consulting</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Author of The Heart of Coaching, pioneer of transformational coaching culture</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr"/>
+      <c r="W83" t="inlineStr"/>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Gillian Jones</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Emerge Consultancy</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Co-author of How to Create a Coaching Culture and 50 Top Tools for Coaching</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr"/>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr"/>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Ro Gorell</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Change Optimised</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Co-author of How to Create a Coaching Culture</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr"/>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr"/>
+      <c r="W85" t="inlineStr"/>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Bill Eckstrom</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>EcSell Institute</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Co-author of The Coaching Effect, researched 100K+ coaching interactions</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>EcSell page</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>@ecsellinstitute</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>X.com</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr"/>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr"/>
+      <c r="W86" t="inlineStr"/>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Sarah Wirth</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>EcSell Institute</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Co-author of The Coaching Effect</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="inlineStr"/>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr"/>
+      <c r="W87" t="inlineStr"/>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>JP Nerbun</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TOC Culture Consulting</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Co-host of Coaching Culture Podcast, creator of Culture System</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>tocculture</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>@tocculture</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>@JpNerbun</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>X.com</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>@tocculture</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>@tocculture</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr"/>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Nate Sanderson</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TOC Culture Consulting</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Co-host of Coaching Culture Podcast</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>tocculture</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>@tocculture</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>@tocculture</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>@tocculture</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr"/>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Karen Morley</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Karen Morley &amp; Associates</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Author of Lead Like a Coach, Australian psychologist</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr"/>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr"/>
+      <c r="T90" t="inlineStr"/>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr"/>
+      <c r="W90" t="inlineStr"/>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Behnam Bakhshandeh</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Primeco Education</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Editor of Building an Organizational Coaching Culture</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="inlineStr"/>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr"/>
+      <c r="W91" t="inlineStr"/>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Elena Aguilar</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Bright Morning</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Author of 8 books including The Art of Coaching and Coaching for Equity</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>@brightmorningteam</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr"/>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr"/>
+      <c r="W92" t="inlineStr"/>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Diane Sweeney</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Diane Sweeney Consulting</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Creator of Student-Centered Coaching</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>sweeneydiane</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr"/>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr"/>
+      <c r="W93" t="inlineStr"/>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -7017,7 +8301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7145,6 +8429,26 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>resilience</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>17</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>coaching-cultures</t>
         </is>
       </c>
     </row>
@@ -7160,7 +8464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8689,6 +9993,302 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>69c23f9047c72b77465229be</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-31T19:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>69c23f9c06e664e154ff22f3</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-31T20:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>69c23fa647c72b77465229e5</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-03-31T17:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>69c23fa847c72b7746522a1f</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-03-31T17:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>69c23fb047c72b7746522a6c</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-30T22:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>69c23fb606e664e154ff235a</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-29T23:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>69c23fba47c72b7746522a92</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-04-01T00:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Coaching Cultures</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>69c23fbe06e664e154ff2381</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-31T10:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Strategic Planning
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -672,10 +672,14 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1059,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y93"/>
+  <dimension ref="A1:Y110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6977,13 +6981,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr">
         <is>
           <t>@boxofcrayons</t>
@@ -6999,27 +7001,21 @@
           <t>X.com</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S77" t="inlineStr"/>
-      <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V77" t="inlineStr"/>
-      <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7042,55 +7038,41 @@
           <t>Author of Creating a Coaching Culture, pioneer of systemic team coaching</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S78" t="inlineStr"/>
-      <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V78" t="inlineStr"/>
-      <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7113,55 +7095,41 @@
           <t>Created LEAD Framework for coaching cultures, 45+ books</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr"/>
-      <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S79" t="inlineStr"/>
-      <c r="T79" t="inlineStr"/>
       <c r="U79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V79" t="inlineStr"/>
-      <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7184,13 +7152,11 @@
           <t>Past ICF Global President, author of Coach the Person Not the Problem</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>@dr_marcia_reynolds</t>
@@ -7206,13 +7172,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr">
         <is>
           <t>@MarciaReynolds</t>
@@ -7228,27 +7192,21 @@
           <t>X.com</t>
         </is>
       </c>
-      <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S80" t="inlineStr"/>
-      <c r="T80" t="inlineStr"/>
       <c r="U80" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V80" t="inlineStr"/>
-      <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7271,55 +7229,41 @@
           <t>Author of The Coaching Manual and Brilliant Coaching</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S81" t="inlineStr"/>
-      <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V81" t="inlineStr"/>
-      <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7342,13 +7286,11 @@
           <t>Author of Effective Coaching, creator of Enable automated coaching</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>@mylesdowneycoach</t>
@@ -7364,13 +7306,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr">
         <is>
           <t>@mylesdowney</t>
@@ -7386,27 +7326,21 @@
           <t>X.com</t>
         </is>
       </c>
-      <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V82" t="inlineStr"/>
-      <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7429,55 +7363,41 @@
           <t>Author of The Heart of Coaching, pioneer of transformational coaching culture</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S83" t="inlineStr"/>
-      <c r="T83" t="inlineStr"/>
       <c r="U83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V83" t="inlineStr"/>
-      <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7500,55 +7420,41 @@
           <t>Co-author of How to Create a Coaching Culture and 50 Top Tools for Coaching</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S84" t="inlineStr"/>
-      <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V84" t="inlineStr"/>
-      <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7571,55 +7477,41 @@
           <t>Co-author of How to Create a Coaching Culture</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S85" t="inlineStr"/>
-      <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V85" t="inlineStr"/>
-      <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7642,7 +7534,6 @@
           <t>Co-author of The Coaching Effect, researched 100K+ coaching interactions</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -7653,20 +7544,16 @@
           <t>EcSell page</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr">
         <is>
           <t>@ecsellinstitute</t>
@@ -7682,27 +7569,21 @@
           <t>X.com</t>
         </is>
       </c>
-      <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S86" t="inlineStr"/>
-      <c r="T86" t="inlineStr"/>
       <c r="U86" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V86" t="inlineStr"/>
-      <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7725,55 +7606,41 @@
           <t>Co-author of The Coaching Effect</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S87" t="inlineStr"/>
-      <c r="T87" t="inlineStr"/>
       <c r="U87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V87" t="inlineStr"/>
-      <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7826,13 +7693,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr">
         <is>
           <t>@JpNerbun</t>
@@ -7878,13 +7743,11 @@
           <t>YouTube</t>
         </is>
       </c>
-      <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7937,20 +7800,16 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr"/>
       <c r="Q89" t="inlineStr">
         <is>
           <t>@tocculture</t>
@@ -7981,13 +7840,11 @@
           <t>YouTube</t>
         </is>
       </c>
-      <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8010,55 +7867,41 @@
           <t>Author of Lead Like a Coach, Australian psychologist</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
       <c r="R90" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S90" t="inlineStr"/>
-      <c r="T90" t="inlineStr"/>
       <c r="U90" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V90" t="inlineStr"/>
-      <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8081,55 +7924,41 @@
           <t>Editor of Building an Organizational Coaching Culture</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr"/>
-      <c r="T91" t="inlineStr"/>
       <c r="U91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V91" t="inlineStr"/>
-      <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8152,13 +7981,11 @@
           <t>Author of 8 books including The Art of Coaching and Coaching for Equity</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>@brightmorningteam</t>
@@ -8174,41 +8001,31 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
       <c r="R92" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S92" t="inlineStr"/>
-      <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V92" t="inlineStr"/>
-      <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8246,48 +8063,1451 @@
           <t>Facebook</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr"/>
-      <c r="Q93" t="inlineStr"/>
       <c r="R93" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S93" t="inlineStr"/>
-      <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V93" t="inlineStr"/>
-      <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Roger Martin</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Former Dean &amp; Strategy Professor</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Rotman School of Management</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Co-author of Playing to Win, #1 Thinkers50 management thinker</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>@RogerLMartin</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr"/>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr"/>
+      <c r="W94" t="inlineStr"/>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Rita McGrath</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Professor of Strategy</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Columbia Business School</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Author of The End of Competitive Advantage</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>linktree</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>linktree</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>@rgmcgrath</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr"/>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>linktree</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr"/>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Henry Mintzberg</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Professor Emeritus</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>McGill University</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Author of The Rise and Fall of Strategic Planning</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>idcrawl</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>@Mintzberg141</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr"/>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>mintzberg.org</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr"/>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Alex Osterwalder</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Strategyzer</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Creator of the Business Model Canvas</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>alexosterwalder.com</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>@alexosterwalder</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>@AlexOsterwalder</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr"/>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr"/>
+      <c r="T97" t="inlineStr"/>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>alexosterwalder.com</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr"/>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Renée Mauborgne</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Professor of Strategy</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>INSEAD</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Co-creator of Blue Ocean Strategy</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>blueoceanstrategy.com</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>@blueoceanstrtgy</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>@blueoceanstrtgy</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>blueoceanstrategy.com</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr"/>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr"/>
+      <c r="T98" t="inlineStr"/>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>blueoceanstrategy.com</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr"/>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Rich Horwath</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Strategic Thinking Institute</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Author of Strategic, #1 strategy keynote speaker</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>@richhorwathceo</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>@RichHorwath</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr"/>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr"/>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr"/>
+      <c r="W99" t="inlineStr"/>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Erica Olsen</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>COO &amp; Co-Founder</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>OnStrategy</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Author of Strategic Planning for Dummies</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>@OnStrategyHQ</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>twitter.com</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr"/>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr"/>
+      <c r="T100" t="inlineStr"/>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>onstrategyhq.com</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr"/>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Kaihan Krippendorff</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Outthinker</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Former McKinsey, Thinkers50 top-20, host of Chief Strategy Officer Podcast</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>kaihan.net</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>@kaihankrippendorff</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>@Kaihan</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr"/>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr"/>
+      <c r="T101" t="inlineStr"/>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>kaihan.net</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr"/>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Graham Kenny</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Strategic Factors</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Australia-based strategy specialist, prolific HBR author</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>@gkkenny</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr"/>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr"/>
+      <c r="T102" t="inlineStr"/>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr"/>
+      <c r="W102" t="inlineStr"/>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Ann Latham</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Uncommon Clarity</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>The Queen of Clarity, author of The Power of Clarity</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr"/>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr"/>
+      <c r="T103" t="inlineStr"/>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr"/>
+      <c r="W103" t="inlineStr"/>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Jeroen Kraaijenbrink</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Strategy Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Netherlands-based, Forbes contributor, author of five strategy books</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>@JKraaijenbrink</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr"/>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr"/>
+      <c r="T104" t="inlineStr"/>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr"/>
+      <c r="W104" t="inlineStr"/>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Stephen Bungay</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Strategy Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Author of The Art of Action on strategy-to-execution</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>@steve_bungay</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>twitter.com</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr"/>
+      <c r="T105" t="inlineStr"/>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr"/>
+      <c r="W105" t="inlineStr"/>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Fred Pelard</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Strategy Trainer &amp; Author</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Independent / HappyBunny.ai</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>INSEAD-trained, author of How to Be Strategic (Penguin)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>@fredpelard</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr"/>
+      <c r="T106" t="inlineStr"/>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr"/>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>John Bryson</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Professor Emeritus</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>University of Minnesota</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Definitive authority on public/nonprofit strategic planning (6 editions)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr"/>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr"/>
+      <c r="T107" t="inlineStr"/>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr"/>
+      <c r="W107" t="inlineStr"/>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Tendayi Viki</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Strategyzer</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Author of The Corporate Startup, innovation strategy specialist</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>@tendayiviki</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr"/>
+      <c r="T108" t="inlineStr"/>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr"/>
+      <c r="W108" t="inlineStr"/>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Lisa Kay Solomon</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Designer in Residence</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Stanford d.school</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Co-author of Moments of Impact on strategic conversations</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>@lisakaysolomon</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr"/>
+      <c r="T109" t="inlineStr"/>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Max McKeown</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Strategy Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Author of The Strategy Book, CMI Book of the Year winner</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>@mckeown_max_</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>@MaxMckeown</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr"/>
+      <c r="T110" t="inlineStr"/>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr"/>
+      <c r="W110" t="inlineStr"/>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -8301,7 +9521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8449,6 +9669,26 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>coaching-cultures</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>17</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>strategic-planning</t>
         </is>
       </c>
     </row>
@@ -8464,7 +9704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10289,6 +11529,302 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>69c254525f17bfad33bd59a1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-04-03T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>69c254545f17bfad33bd59c7</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-04-03T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>69c25456cbcf37d2ac46ca40</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-04-02T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>69c25457cbcf37d2ac46ca8c</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-04-02T22:02:00Z</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>69c2546d5f17bfad33bd5a7a</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-04-02T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>69c2546ecbcf37d2ac46cb10</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-03-30T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>69c2546fcbcf37d2ac46cb37</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-04-03T06:02:00Z</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Strategic Planning</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>69c25470cbcf37d2ac46cb5d</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-04-02T15:02:00Z</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Conflict Resolution
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -693,10 +693,14 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1063,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y110"/>
+  <dimension ref="A1:Y127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8115,27 +8119,21 @@
           <t>Co-author of Playing to Win, #1 Thinkers50 management thinker</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr">
         <is>
           <t>@RogerLMartin</t>
@@ -8151,27 +8149,21 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q94" t="inlineStr"/>
       <c r="R94" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S94" t="inlineStr"/>
-      <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V94" t="inlineStr"/>
-      <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8194,7 +8186,6 @@
           <t>Author of The End of Competitive Advantage</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8205,7 +8196,6 @@
           <t>linktree</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8216,13 +8206,11 @@
           <t>linktree</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr">
         <is>
           <t>@rgmcgrath</t>
@@ -8238,14 +8226,11 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q95" t="inlineStr"/>
       <c r="R95" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S95" t="inlineStr"/>
-      <c r="T95" t="inlineStr"/>
       <c r="U95" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8256,13 +8241,11 @@
           <t>linktree</t>
         </is>
       </c>
-      <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8285,7 +8268,6 @@
           <t>Author of The Rise and Fall of Strategic Planning</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8296,20 +8278,16 @@
           <t>idcrawl</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr">
         <is>
           <t>@Mintzberg141</t>
@@ -8325,14 +8303,11 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q96" t="inlineStr"/>
       <c r="R96" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S96" t="inlineStr"/>
-      <c r="T96" t="inlineStr"/>
       <c r="U96" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8343,13 +8318,11 @@
           <t>mintzberg.org</t>
         </is>
       </c>
-      <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8372,7 +8345,6 @@
           <t>Creator of the Business Model Canvas</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8398,13 +8370,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr">
         <is>
           <t>@AlexOsterwalder</t>
@@ -8420,14 +8390,11 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q97" t="inlineStr"/>
       <c r="R97" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S97" t="inlineStr"/>
-      <c r="T97" t="inlineStr"/>
       <c r="U97" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8438,13 +8405,11 @@
           <t>alexosterwalder.com</t>
         </is>
       </c>
-      <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8467,7 +8432,6 @@
           <t>Co-creator of Blue Ocean Strategy</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8493,13 +8457,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr">
         <is>
           <t>@blueoceanstrtgy</t>
@@ -8515,14 +8477,11 @@
           <t>blueoceanstrategy.com</t>
         </is>
       </c>
-      <c r="Q98" t="inlineStr"/>
       <c r="R98" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S98" t="inlineStr"/>
-      <c r="T98" t="inlineStr"/>
       <c r="U98" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8533,13 +8492,11 @@
           <t>blueoceanstrategy.com</t>
         </is>
       </c>
-      <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8562,13 +8519,11 @@
           <t>Author of Strategic, #1 strategy keynote speaker</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>@richhorwathceo</t>
@@ -8584,13 +8539,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr">
         <is>
           <t>@RichHorwath</t>
@@ -8606,27 +8559,21 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q99" t="inlineStr"/>
       <c r="R99" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S99" t="inlineStr"/>
-      <c r="T99" t="inlineStr"/>
       <c r="U99" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V99" t="inlineStr"/>
-      <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8649,27 +8596,21 @@
           <t>Author of Strategic Planning for Dummies</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr">
         <is>
           <t>@OnStrategyHQ</t>
@@ -8685,14 +8626,11 @@
           <t>twitter.com</t>
         </is>
       </c>
-      <c r="Q100" t="inlineStr"/>
       <c r="R100" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S100" t="inlineStr"/>
-      <c r="T100" t="inlineStr"/>
       <c r="U100" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8703,13 +8641,11 @@
           <t>onstrategyhq.com</t>
         </is>
       </c>
-      <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8732,7 +8668,6 @@
           <t>Former McKinsey, Thinkers50 top-20, host of Chief Strategy Officer Podcast</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8758,13 +8693,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr">
         <is>
           <t>@Kaihan</t>
@@ -8780,14 +8713,11 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q101" t="inlineStr"/>
       <c r="R101" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S101" t="inlineStr"/>
-      <c r="T101" t="inlineStr"/>
       <c r="U101" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -8798,13 +8728,11 @@
           <t>kaihan.net</t>
         </is>
       </c>
-      <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8827,27 +8755,21 @@
           <t>Australia-based strategy specialist, prolific HBR author</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr">
         <is>
           <t>@gkkenny</t>
@@ -8863,27 +8785,21 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q102" t="inlineStr"/>
       <c r="R102" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S102" t="inlineStr"/>
-      <c r="T102" t="inlineStr"/>
       <c r="U102" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V102" t="inlineStr"/>
-      <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8906,55 +8822,41 @@
           <t>The Queen of Clarity, author of The Power of Clarity</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr"/>
-      <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr"/>
-      <c r="Q103" t="inlineStr"/>
       <c r="R103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S103" t="inlineStr"/>
-      <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V103" t="inlineStr"/>
-      <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8977,27 +8879,21 @@
           <t>Netherlands-based, Forbes contributor, author of five strategy books</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M104" t="inlineStr"/>
       <c r="N104" t="inlineStr">
         <is>
           <t>@JKraaijenbrink</t>
@@ -9013,27 +8909,21 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q104" t="inlineStr"/>
       <c r="R104" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S104" t="inlineStr"/>
-      <c r="T104" t="inlineStr"/>
       <c r="U104" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V104" t="inlineStr"/>
-      <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9056,27 +8946,21 @@
           <t>Author of The Art of Action on strategy-to-execution</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr">
         <is>
           <t>@steve_bungay</t>
@@ -9092,27 +8976,21 @@
           <t>twitter.com</t>
         </is>
       </c>
-      <c r="Q105" t="inlineStr"/>
       <c r="R105" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S105" t="inlineStr"/>
-      <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V105" t="inlineStr"/>
-      <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -9135,13 +9013,11 @@
           <t>INSEAD-trained, author of How to Be Strategic (Penguin)</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
           <t>@fredpelard</t>
@@ -9157,41 +9033,31 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M106" t="inlineStr"/>
-      <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P106" t="inlineStr"/>
-      <c r="Q106" t="inlineStr"/>
       <c r="R106" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr"/>
-      <c r="T106" t="inlineStr"/>
       <c r="U106" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V106" t="inlineStr"/>
-      <c r="W106" t="inlineStr"/>
       <c r="X106" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -9214,55 +9080,41 @@
           <t>Definitive authority on public/nonprofit strategic planning (6 editions)</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr"/>
-      <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P107" t="inlineStr"/>
-      <c r="Q107" t="inlineStr"/>
       <c r="R107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S107" t="inlineStr"/>
-      <c r="T107" t="inlineStr"/>
       <c r="U107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V107" t="inlineStr"/>
-      <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9285,27 +9137,21 @@
           <t>Author of The Corporate Startup, innovation strategy specialist</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr"/>
       <c r="N108" t="inlineStr">
         <is>
           <t>@tendayiviki</t>
@@ -9321,27 +9167,21 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q108" t="inlineStr"/>
       <c r="R108" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S108" t="inlineStr"/>
-      <c r="T108" t="inlineStr"/>
       <c r="U108" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V108" t="inlineStr"/>
-      <c r="W108" t="inlineStr"/>
       <c r="X108" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9364,27 +9204,21 @@
           <t>Co-author of Moments of Impact on strategic conversations</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr">
         <is>
           <t>@lisakaysolomon</t>
@@ -9400,27 +9234,21 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q109" t="inlineStr"/>
       <c r="R109" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S109" t="inlineStr"/>
-      <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V109" t="inlineStr"/>
-      <c r="W109" t="inlineStr"/>
       <c r="X109" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9443,13 +9271,11 @@
           <t>Author of The Strategy Book, CMI Book of the Year winner</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
           <t>@mckeown_max_</t>
@@ -9465,13 +9291,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr">
         <is>
           <t>@MaxMckeown</t>
@@ -9487,27 +9311,1436 @@
           <t>x.com</t>
         </is>
       </c>
-      <c r="Q110" t="inlineStr"/>
       <c r="R110" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S110" t="inlineStr"/>
-      <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V110" t="inlineStr"/>
-      <c r="W110" t="inlineStr"/>
       <c r="X110" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Jefferson Fisher</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Trial Lawyer &amp; Communication Expert</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Fisher Firm</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Built 8M+ followers teaching conflict resolution through bite-sized communication scripts</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>jefferson_fisher</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>jefferson_fisher</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Inferred from IG</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr"/>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>justaskjefferson</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>TikTok profile</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>JeffersonFisher</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>Inferred</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr"/>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Sheila Heen</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Professor of Practice</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Harvard Law School</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Co-author of 'Difficult Conversations', foremost negotiation &amp; conflict resolution expert</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>sheilaheen</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr"/>
+      <c r="T112" t="inlineStr"/>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr"/>
+      <c r="W112" t="inlineStr"/>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Kwame Christian</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>American Negotiation Institute</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Host of 'Negotiate Anything' podcast with 16M+ downloads, Compassionate Curiosity Framework</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>kwamenegotiates</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr"/>
+      <c r="Q113" t="inlineStr"/>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr"/>
+      <c r="T113" t="inlineStr"/>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr"/>
+      <c r="W113" t="inlineStr"/>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Amanda Ripley</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Journalist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Good Conflict</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Author of 'High Conflict: Why We Get Trapped and How We Get Out'</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>ripleywriter</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ripleywriter</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>Inferred from IG</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>amandaripley</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr"/>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr"/>
+      <c r="T114" t="inlineStr"/>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr"/>
+      <c r="W114" t="inlineStr"/>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Bill Eddy</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CINO</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>High Conflict Institute</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Pioneer of High Conflict Personality Theory, creator of BIFF Response method</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr"/>
+      <c r="Q115" t="inlineStr"/>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr"/>
+      <c r="T115" t="inlineStr"/>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="inlineStr"/>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Jennifer Goldman-Wetzler</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Alignment Strategies Group</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Author of 'Optimal Outcomes', teaches conflict freedom at Columbia University</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>jgoldmanwetzler</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>jgoldmanwetzler</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>JGoldmanWetzler</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr"/>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr"/>
+      <c r="T116" t="inlineStr"/>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V116" t="inlineStr"/>
+      <c r="W116" t="inlineStr"/>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Liane Davey</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>3COze Inc.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>NYT Bestselling author of 'The Good Fight: Use Productive Conflict'</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>DrLianeDavey</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>lianedavey</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>LianeDavey</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr"/>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr"/>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Amy Gallo</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Contributing Editor</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Harvard Business Review</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Author of 'Getting Along' and 'HBR Guide to Dealing with Conflict'</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>amyegallo</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>amyegallo</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Nate Regier</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Next Element Consulting</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Author of 'Conflict Without Casualties' and 'Compassionate Accountability'</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>nate_regier</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Inferred</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>NextNate</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr"/>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>David Liddle</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>The TCM Group</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Creator of Resolution Framework, author of 'Managing Conflict', Thinkers50 Radar</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr"/>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr"/>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Kenneth Cloke</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Center for Dispute Resolution</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Pioneer mediator with 35+ years, author of 'Mediating Dangerously'</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="inlineStr"/>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr"/>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Dana Caspersen</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Conflict Engagement Specialist</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Author of 'Changing the Conversation: The 17 Principles of Conflict Resolution'</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>dcaspersen</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>danacaspersen</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr"/>
+      <c r="T122" t="inlineStr"/>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr"/>
+      <c r="W122" t="inlineStr"/>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Tammy Lenski</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Mediator &amp; Conflict Resolution Teacher</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Myriaccord</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Host of 'Disagree Better' podcast, author of 'The Conflict Pivot'</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>tammylenski</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr"/>
+      <c r="T123" t="inlineStr"/>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr"/>
+      <c r="W123" t="inlineStr"/>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Jeremy Pollack</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Pollack Peacebuilding Systems</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Stanford research fellow, author of 'The Conflict Resolution Playbook'</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="inlineStr"/>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr"/>
+      <c r="W124" t="inlineStr"/>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Cinnie Noble</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CINERGY Coaching</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Creator of CINERGY conflict coaching model, Member of the Order of Canada</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr"/>
+      <c r="T125" t="inlineStr"/>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr"/>
+      <c r="W125" t="inlineStr"/>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Lynne Maureen Hurdle</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Conflict Resolution Strategist</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>The Conflict Closer</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>TEDx speaker, 40+ years blending communication, conflict, and culture</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>theconflictcloser</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>conflictcloser</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr"/>
+      <c r="T126" t="inlineStr"/>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr"/>
+      <c r="W126" t="inlineStr"/>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Priya Parker</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Thrive Labs</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Author of 'The Art of Gathering' and 'The Art of Fighting', conflict facilitator</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>priyaparker</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>priyaparker</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr"/>
+      <c r="T127" t="inlineStr"/>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr"/>
+      <c r="W127" t="inlineStr"/>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -9521,7 +10754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9689,6 +10922,26 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>strategic-planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>conflict-resolution</t>
         </is>
       </c>
     </row>
@@ -9704,7 +10957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11825,6 +13078,302 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>69c25ae3deeb2e8a5502cecd</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-03-29T06:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>69c25afadeeb2e8a5502cf1b</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-03-29T07:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>69c25b10deeb2e8a5502cf47</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-03-28T19:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>69c25b125b8a7274b3b6c448</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-03-28T22:15:00.000Z</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>69c25b13deeb2e8a5502cf79</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-03-29T05:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>69c25b26deeb2e8a5502cfc4</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-03-31T23:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>69c25b28deeb2e8a5502cfeb</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-03-29T09:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>69c25b295b8a7274b3b6c4c8</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-03-29T03:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Organizational Culture, Adaptive Leadership, School Leadership (2026-03-25)
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -714,10 +714,14 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
@@ -731,10 +735,14 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
@@ -748,10 +756,14 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Education footer variant</t>
@@ -1067,7 +1079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y127"/>
+  <dimension ref="A1:Y178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9348,13 +9360,11 @@
           <t>Built 8M+ followers teaching conflict resolution through bite-sized communication scripts</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
           <t>jefferson_fisher</t>
@@ -9385,13 +9395,11 @@
           <t>Inferred from IG</t>
         </is>
       </c>
-      <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P111" t="inlineStr"/>
       <c r="Q111" t="inlineStr">
         <is>
           <t>justaskjefferson</t>
@@ -9422,13 +9430,11 @@
           <t>Inferred</t>
         </is>
       </c>
-      <c r="W111" t="inlineStr"/>
       <c r="X111" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9451,27 +9457,21 @@
           <t>Co-author of 'Difficult Conversations', foremost negotiation &amp; conflict resolution expert</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr"/>
       <c r="N112" t="inlineStr">
         <is>
           <t>sheilaheen</t>
@@ -9487,27 +9487,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q112" t="inlineStr"/>
       <c r="R112" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S112" t="inlineStr"/>
-      <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V112" t="inlineStr"/>
-      <c r="W112" t="inlineStr"/>
       <c r="X112" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9530,13 +9524,11 @@
           <t>Host of 'Negotiate Anything' podcast with 16M+ downloads, Compassionate Curiosity Framework</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
           <t>kwamenegotiates</t>
@@ -9552,41 +9544,31 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
       <c r="O113" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P113" t="inlineStr"/>
-      <c r="Q113" t="inlineStr"/>
       <c r="R113" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S113" t="inlineStr"/>
-      <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V113" t="inlineStr"/>
-      <c r="W113" t="inlineStr"/>
       <c r="X113" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9609,13 +9591,11 @@
           <t>Author of 'High Conflict: Why We Get Trapped and How We Get Out'</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
           <t>ripleywriter</t>
@@ -9661,27 +9641,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q114" t="inlineStr"/>
       <c r="R114" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S114" t="inlineStr"/>
-      <c r="T114" t="inlineStr"/>
       <c r="U114" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V114" t="inlineStr"/>
-      <c r="W114" t="inlineStr"/>
       <c r="X114" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9704,55 +9678,41 @@
           <t>Pioneer of High Conflict Personality Theory, creator of BIFF Response method</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr"/>
-      <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P115" t="inlineStr"/>
-      <c r="Q115" t="inlineStr"/>
       <c r="R115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S115" t="inlineStr"/>
-      <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V115" t="inlineStr"/>
-      <c r="W115" t="inlineStr"/>
       <c r="X115" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9805,13 +9765,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr"/>
       <c r="N116" t="inlineStr">
         <is>
           <t>JGoldmanWetzler</t>
@@ -9827,27 +9785,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q116" t="inlineStr"/>
       <c r="R116" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S116" t="inlineStr"/>
-      <c r="T116" t="inlineStr"/>
       <c r="U116" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V116" t="inlineStr"/>
-      <c r="W116" t="inlineStr"/>
       <c r="X116" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9900,13 +9852,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr"/>
       <c r="N117" t="inlineStr">
         <is>
           <t>LianeDavey</t>
@@ -9922,27 +9872,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q117" t="inlineStr"/>
       <c r="R117" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S117" t="inlineStr"/>
-      <c r="T117" t="inlineStr"/>
       <c r="U117" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V117" t="inlineStr"/>
-      <c r="W117" t="inlineStr"/>
       <c r="X117" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9965,13 +9909,11 @@
           <t>Author of 'Getting Along' and 'HBR Guide to Dealing with Conflict'</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr">
         <is>
           <t>amyegallo</t>
@@ -9987,13 +9929,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr"/>
       <c r="N118" t="inlineStr">
         <is>
           <t>amyegallo</t>
@@ -10009,27 +9949,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q118" t="inlineStr"/>
       <c r="R118" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S118" t="inlineStr"/>
-      <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V118" t="inlineStr"/>
-      <c r="W118" t="inlineStr"/>
       <c r="X118" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -10052,13 +9986,11 @@
           <t>Author of 'Conflict Without Casualties' and 'Compassionate Accountability'</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
           <t>nate_regier</t>
@@ -10074,13 +10006,11 @@
           <t>Inferred</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr"/>
       <c r="N119" t="inlineStr">
         <is>
           <t>NextNate</t>
@@ -10096,27 +10026,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q119" t="inlineStr"/>
       <c r="R119" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S119" t="inlineStr"/>
-      <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V119" t="inlineStr"/>
-      <c r="W119" t="inlineStr"/>
       <c r="X119" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -10139,55 +10063,41 @@
           <t>Creator of Resolution Framework, author of 'Managing Conflict', Thinkers50 Radar</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr"/>
-      <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P120" t="inlineStr"/>
-      <c r="Q120" t="inlineStr"/>
       <c r="R120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S120" t="inlineStr"/>
-      <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V120" t="inlineStr"/>
-      <c r="W120" t="inlineStr"/>
       <c r="X120" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -10210,55 +10120,41 @@
           <t>Pioneer mediator with 35+ years, author of 'Mediating Dangerously'</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="inlineStr"/>
       <c r="R121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S121" t="inlineStr"/>
-      <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr"/>
       <c r="X121" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -10281,13 +10177,11 @@
           <t>Author of 'Changing the Conversation: The 17 Principles of Conflict Resolution'</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>dcaspersen</t>
@@ -10303,13 +10197,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M122" t="inlineStr"/>
       <c r="N122" t="inlineStr">
         <is>
           <t>danacaspersen</t>
@@ -10325,27 +10217,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q122" t="inlineStr"/>
       <c r="R122" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S122" t="inlineStr"/>
-      <c r="T122" t="inlineStr"/>
       <c r="U122" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V122" t="inlineStr"/>
-      <c r="W122" t="inlineStr"/>
       <c r="X122" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -10368,27 +10254,21 @@
           <t>Host of 'Disagree Better' podcast, author of 'The Conflict Pivot'</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr">
         <is>
           <t>tammylenski</t>
@@ -10404,27 +10284,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q123" t="inlineStr"/>
       <c r="R123" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S123" t="inlineStr"/>
-      <c r="T123" t="inlineStr"/>
       <c r="U123" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V123" t="inlineStr"/>
-      <c r="W123" t="inlineStr"/>
       <c r="X123" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -10447,55 +10321,41 @@
           <t>Stanford research fellow, author of 'The Conflict Resolution Playbook'</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
       <c r="O124" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="P124" t="inlineStr"/>
-      <c r="Q124" t="inlineStr"/>
       <c r="R124" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S124" t="inlineStr"/>
-      <c r="T124" t="inlineStr"/>
       <c r="U124" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="V124" t="inlineStr"/>
-      <c r="W124" t="inlineStr"/>
       <c r="X124" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -10518,55 +10378,41 @@
           <t>Creator of CINERGY conflict coaching model, Member of the Order of Canada</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
       <c r="O125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr"/>
       <c r="R125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S125" t="inlineStr"/>
-      <c r="T125" t="inlineStr"/>
       <c r="U125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V125" t="inlineStr"/>
-      <c r="W125" t="inlineStr"/>
       <c r="X125" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -10619,41 +10465,31 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M126" t="inlineStr"/>
-      <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr"/>
       <c r="R126" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S126" t="inlineStr"/>
-      <c r="T126" t="inlineStr"/>
       <c r="U126" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V126" t="inlineStr"/>
-      <c r="W126" t="inlineStr"/>
       <c r="X126" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -10676,13 +10512,11 @@
           <t>Author of 'The Art of Gathering' and 'The Art of Fighting', conflict facilitator</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
           <t>priyaparker</t>
@@ -10698,13 +10532,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M127" t="inlineStr"/>
       <c r="N127" t="inlineStr">
         <is>
           <t>priyaparker</t>
@@ -10720,27 +10552,1067 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q127" t="inlineStr"/>
       <c r="R127" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S127" t="inlineStr"/>
-      <c r="T127" t="inlineStr"/>
       <c r="U127" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V127" t="inlineStr"/>
-      <c r="W127" t="inlineStr"/>
       <c r="X127" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Daniel Coyle</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>NYT Bestselling Author</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Author of 'The Culture Code'</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Chris Dyer</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>CEO &amp; Culture Consultant</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>PeopleG2</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Global Gurus #15 organizational culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Adrian Gostick</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>The Culture Works</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>NYT bestselling author of 'The Carrot Principle'</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Kim Scott</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Author &amp; CEO Coach</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Radical Candor</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Author of 'Radical Candor'</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Denise Lee Yohn</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Brand &amp; Culture Strategist</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Author of 'Fusion'</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Gustavo Razzetti</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Fearless Culture</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Workplace culture design consultant</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Mary Kelly</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>PhD, Leadership Expert</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Global Gurus #5 organizational culture 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Shane Green</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Culture Expert</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Author of 'Culture Hacker'</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Siobhan McHale</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Culture Transformation Expert</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Author of 'The Insider's Guide to Culture Change'</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Claire Hughes Johnson</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Former COO</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Author of 'Scaling People'</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Didier Elzinga</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Culture Amp</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Culture analytics platform pioneer</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Stan Slap</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Culture Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Author of 'Under the Hood'</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Jessica Miller-Merrell</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Workology</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>HR &amp; workplace culture digital creator</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Monte Wyatt</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Leadership &amp; Culture Expert</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Global Gurus #12 organizational culture 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Laura Whaley</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Content Creator</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Corporate culture TikTok creator</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Samantha Clarke</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Happiness Consultant</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Author of 'Love It or Leave It'</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>James Ferguson</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Culture Professional</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Global Gurus #20 organizational culture 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Ronald Heifetz</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Founder, Center for Public Leadership</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Harvard Kennedy School</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Creator of adaptive leadership framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Marty Linsky</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Cambridge Leadership Associates</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Co-author 'Leadership on the Line'</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Alexander Grashow</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Good Wolf Group</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Co-author 'The Practice of Adaptive Leadership'</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Sharon Daloz Parks</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Author &amp; Scholar</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Harvard</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Author of 'Leadership Can Be Taught'</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Dean Williams</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Harvard Kennedy School</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Author of 'Real Leadership'</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Eric Martin</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Adaptive Change Advisors</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Adaptive leadership practitioner</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Max Martina</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Cambridge Leadership Associates</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Global adaptive leadership consultant</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Jennifer Garvey Berger</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Author &amp; Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Cultivating Leadership</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Author 'Simple Habits for Complex Times'</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Bob Johansen</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Distinguished Fellow</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Institute for the Future</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Author of 'Leaders Make the Future'</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Glenda Eoyang</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Founding Executive Director</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Human Systems Dynamics Institute</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Adaptive action pioneer</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Ed O'Malley</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Kansas Leadership Center</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Author of 'For the Common Good'</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Julia Fabris McBride</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Kansas Leadership Center</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Co-author 'For the Common Good'</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Deborah Ancona</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>MIT Sloan School of Management</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Expert on distributed leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Robert Kegan</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Professor Emeritus</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Harvard Graduate School of Education</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Co-author 'Immunity to Change'</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Lisa Lahey</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Harvard Graduate School of Education</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Co-author 'Immunity to Change'</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Diana Wu David</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Director of Futures</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>ServiceNow</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Futurist and adaptive leadership thinker</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Keith Yamashita</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>SYPartners</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Advised CEOs of Apple, IBM, Starbucks</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Todd Whitaker</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Professor of Educational Leadership</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>University of Missouri</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Author of 60+ books on school leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Baruti Kafele</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Principal &amp; Education Speaker</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Principal Kafele Academy</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>YouTube AP &amp; New Principals Academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Jimmy Casas</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Author &amp; Education Speaker</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Author of 'Culturize'</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Joe Sanfelippo</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Fall Creek School District</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Social media for schools pioneer</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Danny Bauer</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Better Leaders Better Schools</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>#1 school leadership podcast</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Robyn Jackson</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Mindsteps Inc.</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Creator of the Buildership Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Sanée Bell</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Author of 'Be Excellent on Purpose'</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Jessica Cabeen</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr"/>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Author of 'Hacking Early Learning'</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Thomas Murray</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Director of Innovation</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Future Ready Schools</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Author of 'Personal &amp; Authentic'</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Hamish Brewer</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>The Relentless Principal</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr"/>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>TED speaker, transformed struggling schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Derek McCoy</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Principal &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr"/>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Award-winning education leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Joshua Stamper</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Aspire Podcast</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>School leadership podcast host</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Evan Robb</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr"/>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Author of 'The Principled Principal'</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Spike Cook</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>EdD, Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr"/>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Author of 'Connected Leadership'</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Rachael George</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Principal &amp; Education Leader</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Collaborative school leadership champion</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Jen Schwanke</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Author &amp; Principal</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Author of 'You're the Principal! Now What?'</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Weston Kieschnick</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Author &amp; ICLE Senior Fellow</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>ICLE</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Author of 'Bold School'</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -10754,7 +11626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10942,6 +11814,66 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>conflict-resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>organizational-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>17</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>adaptive-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>school-leadership</t>
         </is>
       </c>
     </row>
@@ -10957,7 +11889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -13374,6 +14306,822 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>69c318d872fa676e9bd0bbb1</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>69c318e3b2e701fae145665e</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>69c318f6b2e701fae14567da</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-04-04T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>69c318eeb2e701fae1456772</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>69c318fb72fa676e9bd0bd28</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>69c318feb2e701fae145682d</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>69c3190372fa676e9bd0bd5a</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Organizational Culture</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>69c3190772fa676e9bd0bd9a</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-04-04T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>69c3191c72fa676e9bd0bdfb</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>69c3192672fa676e9bd0be2d</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>69c3192772fa676e9bd0be52</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-04-05T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>69c3193272fa676e9bd0be8f</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>69c3193a72fa676e9bd0beda</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>69c3193e404909f7dd67c210</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>69c3194272fa676e9bd0bf16</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>69c31947404909f7dd67c25d</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-04-05T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>69c3195b72fa676e9bd0bfa9</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>69c31966404909f7dd67c400</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>69c31967404909f7dd67c425</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-04-06T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>69c31971404909f7dd67c455</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>69c31979404909f7dd67c481</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>69c3197d72fa676e9bd0c0f4</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>69c31981404909f7dd67c4b6</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>School Leadership</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>69c31986404909f7dd67c4db</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-04-06T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Executive Coaching, Team Culture, Psych Safety Schools
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -781,10 +781,14 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
@@ -798,10 +802,14 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
@@ -815,10 +823,14 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Education footer variant</t>
@@ -1079,7 +1091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y178"/>
+  <dimension ref="A1:Y223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10579,7 +10591,6 @@
           <t>NYT Bestselling Author</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>Author of 'The Culture Code'</t>
@@ -10663,7 +10674,6 @@
           <t>Brand &amp; Culture Strategist</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
           <t>Author of 'Fusion'</t>
@@ -10703,7 +10713,6 @@
           <t>PhD, Leadership Expert</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
           <t>Global Gurus #5 organizational culture 2026</t>
@@ -10721,7 +10730,6 @@
           <t>Culture Expert</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>Author of 'Culture Hacker'</t>
@@ -10739,7 +10747,6 @@
           <t>Culture Transformation Expert</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
           <t>Author of 'The Insider's Guide to Culture Change'</t>
@@ -10801,7 +10808,6 @@
           <t>Culture Consultant &amp; Author</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
           <t>Author of 'Under the Hood'</t>
@@ -10841,7 +10847,6 @@
           <t>Leadership &amp; Culture Expert</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>Global Gurus #12 organizational culture 2026</t>
@@ -10859,7 +10864,6 @@
           <t>Content Creator</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
           <t>Corporate culture TikTok creator</t>
@@ -10877,7 +10881,6 @@
           <t>Happiness Consultant</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
           <t>Author of 'Love It or Leave It'</t>
@@ -10895,7 +10898,6 @@
           <t>Culture Professional</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
           <t>Global Gurus #20 organizational culture 2026</t>
@@ -11331,7 +11333,6 @@
           <t>Author &amp; Education Speaker</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
           <t>Author of 'Culturize'</t>
@@ -11415,7 +11416,6 @@
           <t>Principal &amp; Author</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
           <t>Author of 'Be Excellent on Purpose'</t>
@@ -11433,7 +11433,6 @@
           <t>Principal &amp; Author</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
           <t>Author of 'Hacking Early Learning'</t>
@@ -11473,7 +11472,6 @@
           <t>The Relentless Principal</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
           <t>TED speaker, transformed struggling schools</t>
@@ -11491,7 +11489,6 @@
           <t>Principal &amp; Speaker</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
           <t>Award-winning education leader</t>
@@ -11531,7 +11528,6 @@
           <t>Principal &amp; Author</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
           <t>Author of 'The Principled Principal'</t>
@@ -11549,7 +11545,6 @@
           <t>EdD, Principal &amp; Author</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
           <t>Author of 'Connected Leadership'</t>
@@ -11567,7 +11562,6 @@
           <t>Principal &amp; Education Leader</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
           <t>Collaborative school leadership champion</t>
@@ -11585,7 +11579,6 @@
           <t>Author &amp; Principal</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
           <t>Author of 'You're the Principal! Now What?'</t>
@@ -11611,6 +11604,996 @@
       <c r="D178" t="inlineStr">
         <is>
           <t>Author of 'Bold School'</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Lolly Daskal</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Business Consultant</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Lead From Within</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Inc. Top-50 Leadership Expert, 1M+ X followers, author 'The Leadership Gap'</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Joshua Miller</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Master Certified Executive Coach</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Forbes Coaching Council</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>TEDx speaker, LinkedIn Top Voice, AI-ready leadership mindset</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Hortense Le Gentil</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Executive Leadership Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>30+ years, author 'The Unlocked Leader', Coaches50 2024 nominee</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Dr. Carol Parker Walsh</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Executive Leadership Coach &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Carol Parker Walsh Consulting</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>JD, PhD, PCC — women's executive leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Kelli Thompson</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Clarity &amp; Confidence Programs</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Fortune 500 clients, author 'Closing The Confidence Gap'</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Craig Groeschel</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Leadership Coach &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Life.Church</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>NYT bestselling author, 269K+ YouTube subscribers</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Alexandra Young</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>CEO &amp; Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>229K TikTok followers, co-host Brave &amp; Purposeful Leadership podcast</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Sue Reynolds</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>265K+ TikTok, ICF-certified, author 'Leadership Linguistics'</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Tom Cox</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Executive Leadership Business Coach</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Vertical Motion</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Author 'Executive Career Handbook', cross-border leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Cheryl Thompson</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Management Mentor &amp; Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Humorous take on leadership challenges, emotional stress guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Allison L. Barr</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Leadership Solutions Partner</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Center for Creative Leadership</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>MBA + Master's Psychology, 187K TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Nina Bowman</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Paravis Partners</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Harvard MBA, HBR contributor, C-level executive coaching</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Amy Jen Su</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Mariswood Group</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>HBR author, co-author 'Own the Room'</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Victoria Scott</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Executive &amp; Career Coach</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Victoria Scott Coaching LLC</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>20+ years IT leadership, PCC, imposter syndrome specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Maxine</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Business Coach &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Rising TikTok voice in executive leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Daniel Pink</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Behavioral Science Author</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>NYT bestselling author of 'Drive' and 'When', motivation science</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Julie Zhuo</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Former VP of Design</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Facebook (Meta)</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Author 'The Making of a Manager', scaling teams expert</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Josh Bersin</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Global HR Industry Analyst</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Leading voice on workplace trends, HR technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Laszlo Bock</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Former Head of People Operations</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Author 'Work Rules!', behavioral economics in HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Katelin Holloway</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Former VP of People</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Reddit</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>HR tech investor, progressive culture advocate</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Mel Robbins</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Behavioral Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Creator of 'The 5 Second Rule', millions of followers</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Chad Littlefield</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Corporate Connection Facilitator</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>We and Me</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>'Connection before content' philosophy, team building</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Leigh Elena Henderson</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>HR Executive &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>HR Besties</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Unfiltered workplace survival guides podcast co-host</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Ashley Herd</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Former Employment Attorney</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Manager Method</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Viral role-play videos teaching leadership &amp; HR compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Corporate Natalie</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Remote Work &amp; Culture Satirist</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Forbes 30 Under 30, Zoom culture humor</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>DeAndre Brown</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Gen Z Workplace Culture Advocate</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>'The Corporate Baddie', 9-to-5 boundaries advocate</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Erin McGoff</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Career Educator &amp; Filmmaker</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Author 'Secret Language of Work', toxic culture identification</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Arthur Carmazzi</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>#1 Organizational Culture Professional</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Global Gurus 2025</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>AI-powered Culture Evolution Process, O.C.E.A.N. framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Mark Collard</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Experiential Learning Designer</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>playmeo</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Most comprehensive database of team-building group games</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Suzi Kalsow</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Management Coach</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>'Coach it. Confront it. Lead it.' framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Carey Arensberg</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>4th Grade Teacher &amp; Trauma-Informed Practitioner</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Mobile County Schools</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>486K+ followers, Mobile County Teacher of the Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Gabe Dannenbring</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Middle School Science Teacher</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Ben Reifel School</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>1.6M TikTok, Netflix 'Surviving Paradise' star</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Jamie Gilbert</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>British Teacher, School Leader &amp; Children's Author</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>UK Schools</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>300K+ IG, 1M+ TikTok, ADHD/neurodiversity specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Doug Lemov</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Uncommon Schools</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Author 'Teach Like a Champion 3.0', classroom culture fundamentals</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Esther Wojcicki</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>40-Year Educator &amp; Author</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Palo Alto High School (retired)</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Author 'How to Raise Successful People', TRICK framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Catlin Tucker</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Education Expert &amp; International Speaker</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>24 years education, blended learning &amp; psych safety, 'The Balance' podcast</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Cassie Stephens</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Kindergarten Art Teacher &amp; Author</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>362K IG, author 'Art Teacherin 101', joyful classroom culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Zaretta Hammond</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Writer, Educator &amp; Literacy Advocate</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Ready for Rigor Framework creator, culturally responsive teaching</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Peyton Curley</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Elementary Teacher &amp; Children's Author</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>33K IG as @thesocialemotionalteacher, SEL children's books</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Ms. Bo</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>High School Counselor &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>140K+ TikTok as @thatschoolcounselor, school mental health</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Jennifer Gonzalez</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Teacher &amp; Educational Content Creator</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Cult of Pedagogy</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>One of most influential education websites/podcasts</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>CJ Reynolds</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Literature Teacher &amp; YouTube Educator</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>27K+ YouTube subscribers, culture of kindness</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Becky Jo Oglesby</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1st Grade Teacher &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>TikTok @capesintheclassroom, trauma-informed strategies</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Efthymia Kli</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Trauma &amp; Somatic Practitioner</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>156K IG @the.trauma.educator, neuroscience-based strategies</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Justin Minkel</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Elementary School Teacher</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Arkansas Schools</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Arkansas Teacher of the Year, high-need school advocacy</t>
         </is>
       </c>
     </row>
@@ -11626,7 +12609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11874,6 +12857,66 @@
       <c r="D12" t="inlineStr">
         <is>
           <t>school-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>executive-coaching</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>team-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Psychological Safety in Schools</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>psychological-safety-in-schools</t>
         </is>
       </c>
     </row>
@@ -11889,7 +12932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -14332,7 +15375,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14365,7 +15407,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14435,7 +15476,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14468,7 +15508,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14501,7 +15540,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14534,7 +15572,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14604,7 +15641,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14637,7 +15673,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14707,7 +15742,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14740,7 +15774,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14773,7 +15806,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14806,7 +15838,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14876,7 +15907,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14909,7 +15939,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -14979,7 +16008,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -15012,7 +16040,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -15045,7 +16072,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -15078,7 +16104,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -15119,6 +16144,894 @@
       <c r="G89" t="inlineStr">
         <is>
           <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>69c31ffa404909f7dd67f179</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-03-30T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>69c3200c086473f19ac3d135</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-03-30T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>69c32018404909f7dd67f1cc</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-04-08T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>69c32024404909f7dd67f222</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-03-30T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>69c3202c404909f7dd67f254</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-04-08T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>69c32036404909f7dd67f2a1</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-03-30T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>69c3203d404909f7dd67f2c7</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-03-30T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>69c32045086473f19ac3d23f</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-03-30T13:02:00Z</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>69c32195086473f19ac3d5fa</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-03-30T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>69c32197404909f7dd67f686</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-03-30T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>69c321a6404909f7dd67f77f</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2026-04-09T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>69c321a8086473f19ac3d704</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-03-30T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>69c321bd086473f19ac3d7b6</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-04-09T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>69c321bf404909f7dd67f857</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-03-30T20:30:00Z</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>69c321c0086473f19ac3d7dd</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2026-03-30T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Team Culture</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>69c321c1086473f19ac3d803</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>2026-03-30T14:01:00Z</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>69c32301086473f19ac3e00e</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>2026-03-30T22:02:00Z</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>69c32303404909f7dd67fffe</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2026-03-30T23:01:00Z</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>69c32321404909f7dd680106</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>2026-04-10T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>69c32323404909f7dd68014a</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>2026-03-30T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>69c32324086473f19ac3e198</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>2026-04-10T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>69c32326404909f7dd680196</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>2026-03-31T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>69c32327086473f19ac3e1e7</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>2026-03-30T22:02:00Z</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Psych Safety Schools</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>69c32328404909f7dd6801bc</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>2026-03-30T20:01:00Z</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update handle database — Women in Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -848,10 +848,14 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1091,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y223"/>
+  <dimension ref="A1:Y240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12597,6 +12601,1485 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Sally Helgesen</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Author &amp; Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>#1 Women's Leadership on Global Gurus, Thinkers50 Hall of Fame. Author of How Women Rise.</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>@sally_helgesen</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr"/>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr"/>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>@SallyHelgesen</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr"/>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr"/>
+      <c r="T224" t="inlineStr"/>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V224" t="inlineStr"/>
+      <c r="W224" t="inlineStr"/>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Shadé Zahrai</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Career Performance Specialist &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Neurofemina Institute</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>2M+ IG, 1.7M TikTok. Australian leadership creator empowering women through behavioural science.</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>@shadezahrai</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr"/>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr"/>
+      <c r="N225" t="inlineStr"/>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr"/>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>@shadezahrai</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>Shadé Zahrai</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V225" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="W225" t="inlineStr"/>
+      <c r="X225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Tiffany Dufu</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Tory Burch Foundation</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Author of Drop the Ball. Former President of The White House Project.</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>tiffanydufu</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>@tdufu</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr"/>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr"/>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>@tdufu</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>Twitter</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr"/>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr"/>
+      <c r="T226" t="inlineStr"/>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V226" t="inlineStr"/>
+      <c r="W226" t="inlineStr"/>
+      <c r="X226" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Deepa Purushothaman</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Author &amp; Leader in Practice</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Harvard Kennedy School</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>First Indian American woman partner at Deloitte. Author of The First, The Few, The Only.</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>@deepa.puru</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr"/>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr"/>
+      <c r="N227" t="inlineStr"/>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr"/>
+      <c r="Q227" t="inlineStr"/>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr"/>
+      <c r="T227" t="inlineStr"/>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V227" t="inlineStr"/>
+      <c r="W227" t="inlineStr"/>
+      <c r="X227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Ruchika Tulshyan Malhotra</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>CEO &amp; Author</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Candour</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Author of Inclusion on Purpose and Uncompete. Thinkers50 Radar. Writes for HBR.</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>@rtulshyan</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr"/>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr"/>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>@rtulshyan</t>
+        </is>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr"/>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr"/>
+      <c r="T228" t="inlineStr"/>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V228" t="inlineStr"/>
+      <c r="W228" t="inlineStr"/>
+      <c r="X228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Jennifer McCollum</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Catalyst</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Author of In Her Own Voice. 25 years of research on advancing women in leadership.</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>@jennifersmccollum</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr"/>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr"/>
+      <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P229" t="inlineStr"/>
+      <c r="Q229" t="inlineStr"/>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr"/>
+      <c r="T229" t="inlineStr"/>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V229" t="inlineStr"/>
+      <c r="W229" t="inlineStr"/>
+      <c r="X229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Kweilin Ellingrud</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>McKinsey Global Institute</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Co-author of The Broken Rung. Leads global D&amp;I at McKinsey.</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Kweilin.Ellingrud</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="inlineStr"/>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr"/>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>@kweiline</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr"/>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr"/>
+      <c r="T230" t="inlineStr"/>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V230" t="inlineStr"/>
+      <c r="W230" t="inlineStr"/>
+      <c r="X230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Siri Chilazi</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Senior Researcher</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Harvard Kennedy School WAPPP</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Co-author of Make Work Fair. Advises Fortune 500 on closing gender gaps.</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="inlineStr"/>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr"/>
+      <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="inlineStr"/>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr"/>
+      <c r="T231" t="inlineStr"/>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V231" t="inlineStr"/>
+      <c r="W231" t="inlineStr"/>
+      <c r="X231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Julia Boorstin</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Senior Media &amp; Tech Correspondent</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>CNBC</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Author of When Women Lead. Creator of CNBC Disruptor 50.</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>JuliaCNBC</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>@juliaboorstin</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr"/>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr"/>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>@JBoorstin</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr"/>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr"/>
+      <c r="T232" t="inlineStr"/>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V232" t="inlineStr"/>
+      <c r="W232" t="inlineStr"/>
+      <c r="X232" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Louise Thompson</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Leadership &amp; Career Coach</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>TikTok creator @leadwithlouise with 88K followers. Former NHS Communications Director.</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="inlineStr"/>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="inlineStr"/>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr"/>
+      <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr"/>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>@leadwithlouise</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr"/>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V233" t="inlineStr"/>
+      <c r="W233" t="inlineStr"/>
+      <c r="X233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Luvvie Ajayi Jones</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>4x NYT Bestselling Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Awe Luv Media</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Author of Professional Troublemaker. TED talk with 10M+ views.</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>luvvie</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>@luvvie</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>@luvvie</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Linktree</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>@Luvvie</t>
+        </is>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>@luvvie</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>Linktree</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr"/>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V234" t="inlineStr"/>
+      <c r="W234" t="inlineStr"/>
+      <c r="X234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Carla Harris</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Vice Chairman &amp; Senior Client Advisor</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Author of Lead to Win. Former Chair of National Women's Business Council.</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>CarlaAnnHarris</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>@carlaannharris</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr"/>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>@carlaannharris</t>
+        </is>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>@carlaannharris</t>
+        </is>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr"/>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V235" t="inlineStr"/>
+      <c r="W235" t="inlineStr"/>
+      <c r="X235" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Laura Liswood</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Secretary General</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Council of Women World Leaders</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Author of The Elephant and the Mouse. Former Goldman Sachs MD.</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr"/>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>@lauraliswood</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr"/>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>@LauraLiswood</t>
+        </is>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr"/>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S236" t="inlineStr"/>
+      <c r="T236" t="inlineStr"/>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V236" t="inlineStr"/>
+      <c r="W236" t="inlineStr"/>
+      <c r="X236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Dr. Michelle P. King</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Organizational Psychologist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Author of The Fix. Former Director of Inclusion at Netflix. 500+ global keynotes.</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="inlineStr"/>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr"/>
+      <c r="K237" t="inlineStr"/>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr"/>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>@_MichelleKing</t>
+        </is>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr"/>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S237" t="inlineStr"/>
+      <c r="T237" t="inlineStr"/>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V237" t="inlineStr"/>
+      <c r="W237" t="inlineStr"/>
+      <c r="X237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Selena Rezvani</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>WSJ Bestselling Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Quick Confidence</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Author of Quick Confidence. Forbes: premier expert on self-advocacy. 500K+ followers.</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>@selenarezvani</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr"/>
+      <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr"/>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>@selenarezvani</t>
+        </is>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr"/>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V238" t="inlineStr"/>
+      <c r="W238" t="inlineStr"/>
+      <c r="X238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Majo Molfino</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Author &amp; Women's Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Author of Break the Good Girl Myth. Host of HEROINE podcast (1M+ downloads).</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr"/>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>@majomolfino</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr"/>
+      <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr"/>
+      <c r="Q239" t="inlineStr"/>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr"/>
+      <c r="T239" t="inlineStr"/>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V239" t="inlineStr"/>
+      <c r="W239" t="inlineStr"/>
+      <c r="X239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Annemarie Cross</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Host, Women In Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Ambitious Entrepreneur Podcast Network</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Known as The Podcasting Queen. Australian brand strategist since 2008.</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr"/>
+      <c r="H240" t="inlineStr"/>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="inlineStr"/>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr"/>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>@AnnemarieCross</t>
+        </is>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr"/>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr"/>
+      <c r="T240" t="inlineStr"/>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V240" t="inlineStr"/>
+      <c r="W240" t="inlineStr"/>
+      <c r="X240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y240" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12609,7 +14092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -12917,6 +14400,26 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>psychological-safety-in-schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>17</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>women-in-leadership</t>
         </is>
       </c>
     </row>
@@ -12932,7 +14435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -17035,6 +18538,302 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>69c32721086473f19ac4037d</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>2026-03-31T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>69c32724404909f7dd6820f6</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>2026-03-31T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>69c32740404909f7dd6821ad</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>2026-04-11T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>69c32728404909f7dd68211c</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>2026-03-30T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>69c32742086473f19ac40464</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>2026-03-30T23:01:00Z</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>69c32743086473f19ac40489</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>2026-04-11T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>69c32744404909f7dd6821df</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2026-03-31T03:01:00Z</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>69c32745086473f19ac404ba</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>2026-03-30T21:02:00Z</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Remote Team Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -869,10 +869,14 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1095,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y240"/>
+  <dimension ref="A1:Y257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12622,13 +12626,11 @@
           <t>#1 Women's Leadership on Global Gurus, Thinkers50 Hall of Fame. Author of How Women Rise.</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
           <t>@sally_helgesen</t>
@@ -12644,13 +12646,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K224" t="inlineStr"/>
       <c r="L224" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M224" t="inlineStr"/>
       <c r="N224" t="inlineStr">
         <is>
           <t>@SallyHelgesen</t>
@@ -12666,27 +12666,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q224" t="inlineStr"/>
       <c r="R224" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S224" t="inlineStr"/>
-      <c r="T224" t="inlineStr"/>
       <c r="U224" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V224" t="inlineStr"/>
-      <c r="W224" t="inlineStr"/>
       <c r="X224" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -12709,13 +12703,11 @@
           <t>2M+ IG, 1.7M TikTok. Australian leadership creator empowering women through behavioural science.</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr">
         <is>
           <t>@shadezahrai</t>
@@ -12731,20 +12723,16 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K225" t="inlineStr"/>
       <c r="L225" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M225" t="inlineStr"/>
-      <c r="N225" t="inlineStr"/>
       <c r="O225" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P225" t="inlineStr"/>
       <c r="Q225" t="inlineStr">
         <is>
           <t>@shadezahrai</t>
@@ -12775,13 +12763,11 @@
           <t>YouTube</t>
         </is>
       </c>
-      <c r="W225" t="inlineStr"/>
       <c r="X225" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -12834,13 +12820,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K226" t="inlineStr"/>
       <c r="L226" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M226" t="inlineStr"/>
       <c r="N226" t="inlineStr">
         <is>
           <t>@tdufu</t>
@@ -12856,27 +12840,21 @@
           <t>Twitter</t>
         </is>
       </c>
-      <c r="Q226" t="inlineStr"/>
       <c r="R226" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S226" t="inlineStr"/>
-      <c r="T226" t="inlineStr"/>
       <c r="U226" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V226" t="inlineStr"/>
-      <c r="W226" t="inlineStr"/>
       <c r="X226" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -12899,13 +12877,11 @@
           <t>First Indian American woman partner at Deloitte. Author of The First, The Few, The Only.</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr">
         <is>
           <t>@deepa.puru</t>
@@ -12921,41 +12897,31 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K227" t="inlineStr"/>
       <c r="L227" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M227" t="inlineStr"/>
-      <c r="N227" t="inlineStr"/>
       <c r="O227" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P227" t="inlineStr"/>
-      <c r="Q227" t="inlineStr"/>
       <c r="R227" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S227" t="inlineStr"/>
-      <c r="T227" t="inlineStr"/>
       <c r="U227" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V227" t="inlineStr"/>
-      <c r="W227" t="inlineStr"/>
       <c r="X227" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -12978,13 +12944,11 @@
           <t>Author of Inclusion on Purpose and Uncompete. Thinkers50 Radar. Writes for HBR.</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr">
         <is>
           <t>@rtulshyan</t>
@@ -13000,13 +12964,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K228" t="inlineStr"/>
       <c r="L228" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M228" t="inlineStr"/>
       <c r="N228" t="inlineStr">
         <is>
           <t>@rtulshyan</t>
@@ -13022,27 +12984,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q228" t="inlineStr"/>
       <c r="R228" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S228" t="inlineStr"/>
-      <c r="T228" t="inlineStr"/>
       <c r="U228" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V228" t="inlineStr"/>
-      <c r="W228" t="inlineStr"/>
       <c r="X228" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -13065,13 +13021,11 @@
           <t>Author of In Her Own Voice. 25 years of research on advancing women in leadership.</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr">
         <is>
           <t>@jennifersmccollum</t>
@@ -13087,41 +13041,31 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K229" t="inlineStr"/>
       <c r="L229" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M229" t="inlineStr"/>
-      <c r="N229" t="inlineStr"/>
       <c r="O229" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P229" t="inlineStr"/>
-      <c r="Q229" t="inlineStr"/>
       <c r="R229" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S229" t="inlineStr"/>
-      <c r="T229" t="inlineStr"/>
       <c r="U229" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V229" t="inlineStr"/>
-      <c r="W229" t="inlineStr"/>
       <c r="X229" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -13159,20 +13103,16 @@
           <t>Facebook</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
       <c r="I230" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J230" t="inlineStr"/>
-      <c r="K230" t="inlineStr"/>
       <c r="L230" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M230" t="inlineStr"/>
       <c r="N230" t="inlineStr">
         <is>
           <t>@kweiline</t>
@@ -13188,27 +13128,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q230" t="inlineStr"/>
       <c r="R230" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S230" t="inlineStr"/>
-      <c r="T230" t="inlineStr"/>
       <c r="U230" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V230" t="inlineStr"/>
-      <c r="W230" t="inlineStr"/>
       <c r="X230" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -13231,55 +13165,41 @@
           <t>Co-author of Make Work Fair. Advises Fortune 500 on closing gender gaps.</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
       <c r="F231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr"/>
-      <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M231" t="inlineStr"/>
-      <c r="N231" t="inlineStr"/>
       <c r="O231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P231" t="inlineStr"/>
-      <c r="Q231" t="inlineStr"/>
       <c r="R231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S231" t="inlineStr"/>
-      <c r="T231" t="inlineStr"/>
       <c r="U231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V231" t="inlineStr"/>
-      <c r="W231" t="inlineStr"/>
       <c r="X231" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -13332,13 +13252,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K232" t="inlineStr"/>
       <c r="L232" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M232" t="inlineStr"/>
       <c r="N232" t="inlineStr">
         <is>
           <t>@JBoorstin</t>
@@ -13354,27 +13272,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q232" t="inlineStr"/>
       <c r="R232" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S232" t="inlineStr"/>
-      <c r="T232" t="inlineStr"/>
       <c r="U232" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V232" t="inlineStr"/>
-      <c r="W232" t="inlineStr"/>
       <c r="X232" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -13397,34 +13309,26 @@
           <t>TikTok creator @leadwithlouise with 88K followers. Former NHS Communications Director.</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G233" t="inlineStr"/>
-      <c r="H233" t="inlineStr"/>
       <c r="I233" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J233" t="inlineStr"/>
-      <c r="K233" t="inlineStr"/>
       <c r="L233" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M233" t="inlineStr"/>
-      <c r="N233" t="inlineStr"/>
       <c r="O233" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P233" t="inlineStr"/>
       <c r="Q233" t="inlineStr">
         <is>
           <t>@leadwithlouise</t>
@@ -13440,20 +13344,16 @@
           <t>TikTok</t>
         </is>
       </c>
-      <c r="T233" t="inlineStr"/>
       <c r="U233" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V233" t="inlineStr"/>
-      <c r="W233" t="inlineStr"/>
       <c r="X233" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -13551,20 +13451,16 @@
           <t>Linktree</t>
         </is>
       </c>
-      <c r="T234" t="inlineStr"/>
       <c r="U234" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V234" t="inlineStr"/>
-      <c r="W234" t="inlineStr"/>
       <c r="X234" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -13617,13 +13513,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K235" t="inlineStr"/>
       <c r="L235" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M235" t="inlineStr"/>
       <c r="N235" t="inlineStr">
         <is>
           <t>@carlaannharris</t>
@@ -13654,20 +13548,16 @@
           <t>TikTok</t>
         </is>
       </c>
-      <c r="T235" t="inlineStr"/>
       <c r="U235" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V235" t="inlineStr"/>
-      <c r="W235" t="inlineStr"/>
       <c r="X235" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -13690,13 +13580,11 @@
           <t>Author of The Elephant and the Mouse. Former Goldman Sachs MD.</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr">
         <is>
           <t>@lauraliswood</t>
@@ -13712,13 +13600,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K236" t="inlineStr"/>
       <c r="L236" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M236" t="inlineStr"/>
       <c r="N236" t="inlineStr">
         <is>
           <t>@LauraLiswood</t>
@@ -13734,27 +13620,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q236" t="inlineStr"/>
       <c r="R236" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S236" t="inlineStr"/>
-      <c r="T236" t="inlineStr"/>
       <c r="U236" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V236" t="inlineStr"/>
-      <c r="W236" t="inlineStr"/>
       <c r="X236" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -13777,27 +13657,21 @@
           <t>Author of The Fix. Former Director of Inclusion at Netflix. 500+ global keynotes.</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr"/>
-      <c r="H237" t="inlineStr"/>
       <c r="I237" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J237" t="inlineStr"/>
-      <c r="K237" t="inlineStr"/>
       <c r="L237" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M237" t="inlineStr"/>
       <c r="N237" t="inlineStr">
         <is>
           <t>@_MichelleKing</t>
@@ -13813,27 +13687,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q237" t="inlineStr"/>
       <c r="R237" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S237" t="inlineStr"/>
-      <c r="T237" t="inlineStr"/>
       <c r="U237" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V237" t="inlineStr"/>
-      <c r="W237" t="inlineStr"/>
       <c r="X237" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -13856,13 +13724,11 @@
           <t>Author of Quick Confidence. Forbes: premier expert on self-advocacy. 500K+ followers.</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr">
         <is>
           <t>@selenarezvani</t>
@@ -13878,20 +13744,16 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K238" t="inlineStr"/>
       <c r="L238" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M238" t="inlineStr"/>
-      <c r="N238" t="inlineStr"/>
       <c r="O238" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P238" t="inlineStr"/>
       <c r="Q238" t="inlineStr">
         <is>
           <t>@selenarezvani</t>
@@ -13907,20 +13769,16 @@
           <t>TikTok</t>
         </is>
       </c>
-      <c r="T238" t="inlineStr"/>
       <c r="U238" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V238" t="inlineStr"/>
-      <c r="W238" t="inlineStr"/>
       <c r="X238" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -13943,13 +13801,11 @@
           <t>Author of Break the Good Girl Myth. Host of HEROINE podcast (1M+ downloads).</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr">
         <is>
           <t>@majomolfino</t>
@@ -13965,41 +13821,31 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K239" t="inlineStr"/>
       <c r="L239" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M239" t="inlineStr"/>
-      <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P239" t="inlineStr"/>
-      <c r="Q239" t="inlineStr"/>
       <c r="R239" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S239" t="inlineStr"/>
-      <c r="T239" t="inlineStr"/>
       <c r="U239" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V239" t="inlineStr"/>
-      <c r="W239" t="inlineStr"/>
       <c r="X239" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -14022,27 +13868,21 @@
           <t>Known as The Podcasting Queen. Australian brand strategist since 2008.</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G240" t="inlineStr"/>
-      <c r="H240" t="inlineStr"/>
       <c r="I240" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J240" t="inlineStr"/>
-      <c r="K240" t="inlineStr"/>
       <c r="L240" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M240" t="inlineStr"/>
       <c r="N240" t="inlineStr">
         <is>
           <t>@AnnemarieCross</t>
@@ -14058,27 +13898,1388 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q240" t="inlineStr"/>
       <c r="R240" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S240" t="inlineStr"/>
-      <c r="T240" t="inlineStr"/>
       <c r="U240" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V240" t="inlineStr"/>
-      <c r="W240" t="inlineStr"/>
       <c r="X240" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Tsedal Neeley</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Author of 'Remote Work Revolution', virtual teams researcher</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr"/>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>tsedalneeley</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>tsedalneeley</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr"/>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>tsedal</t>
+        </is>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>Twitter</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr"/>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr"/>
+      <c r="T241" t="inlineStr"/>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V241" t="inlineStr"/>
+      <c r="W241" t="inlineStr"/>
+      <c r="X241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Nick Bloom</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Professor of Economics</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>World's foremost remote work researcher, WFH Research co-founder</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr"/>
+      <c r="H242" t="inlineStr"/>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="inlineStr"/>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr"/>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>I_Am_NickBloom</t>
+        </is>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q242" t="inlineStr"/>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr"/>
+      <c r="T242" t="inlineStr"/>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V242" t="inlineStr"/>
+      <c r="W242" t="inlineStr">
+        <is>
+          <t>nickbloom.bsky.social</t>
+        </is>
+      </c>
+      <c r="X242" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y242" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Darren Murph</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Head of Remote (Former)</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>GitLab</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Pioneered Head of Remote role, authored Remote Playbook</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>darren_murph</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr"/>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr"/>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>darrenmurph</t>
+        </is>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr"/>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr"/>
+      <c r="T243" t="inlineStr"/>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V243" t="inlineStr"/>
+      <c r="W243" t="inlineStr"/>
+      <c r="X243" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Liam Martin</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Time Doctor &amp; Running Remote</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Co-founded largest remote work conference and Time Doctor</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>liamremote</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>liamremote</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr"/>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>liamremote</t>
+        </is>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr"/>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr"/>
+      <c r="T244" t="inlineStr"/>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V244" t="inlineStr"/>
+      <c r="W244" t="inlineStr"/>
+      <c r="X244" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Kevin Eikenberry</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Remote Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Co-author 'The Long-Distance Leader', remote management expert</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>kevineikenberry</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr"/>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr"/>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>KevinEikenberry</t>
+        </is>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q245" t="inlineStr"/>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr"/>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>KevinEikenberryGroup</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V245" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="W245" t="inlineStr"/>
+      <c r="X245" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Wayne Turmel</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Remote Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Co-author 'The Long-Distance Leader', virtual communication specialist</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="inlineStr"/>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr"/>
+      <c r="K246" t="inlineStr"/>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr"/>
+      <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P246" t="inlineStr"/>
+      <c r="Q246" t="inlineStr"/>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr"/>
+      <c r="T246" t="inlineStr"/>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V246" t="inlineStr"/>
+      <c r="W246" t="inlineStr"/>
+      <c r="X246" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Sacha Connor</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Virtual Work Insider</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Trains enterprise leaders at Toyota, Sephora, Cisco on hybrid teams</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr"/>
+      <c r="H247" t="inlineStr"/>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr"/>
+      <c r="K247" t="inlineStr"/>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr"/>
+      <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr"/>
+      <c r="Q247" t="inlineStr"/>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr"/>
+      <c r="T247" t="inlineStr"/>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V247" t="inlineStr"/>
+      <c r="W247" t="inlineStr"/>
+      <c r="X247" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Laurel Farrer</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Distribute Consulting</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Remote Work Association founder, Top 100 Future of Work Leader</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr"/>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>laurel_farrer</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr"/>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr"/>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>laurel_farrer</t>
+        </is>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>Twitter</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr"/>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr"/>
+      <c r="T248" t="inlineStr"/>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V248" t="inlineStr"/>
+      <c r="W248" t="inlineStr"/>
+      <c r="X248" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Lisette Sutherland</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Collaboration Superpowers</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Author 'Work Together Anywhere', virtual collaboration podcast host</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr"/>
+      <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr"/>
+      <c r="K249" t="inlineStr"/>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr"/>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>lightling</t>
+        </is>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q249" t="inlineStr"/>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr"/>
+      <c r="T249" t="inlineStr"/>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V249" t="inlineStr"/>
+      <c r="W249" t="inlineStr"/>
+      <c r="X249" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Chase Warrington</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Head of Remote</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Doist</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Leads remote strategy across 35+ countries, About Abroad podcast host</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr"/>
+      <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr"/>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr"/>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>dcwarrington</t>
+        </is>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr"/>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr"/>
+      <c r="T250" t="inlineStr"/>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V250" t="inlineStr"/>
+      <c r="W250" t="inlineStr"/>
+      <c r="X250" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Ali Greene</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Co-Author</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Remote Works</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Former DuckDuckGo People Ops, co-wrote Remote Works playbook</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr"/>
+      <c r="H251" t="inlineStr"/>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr"/>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr"/>
+      <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr"/>
+      <c r="Q251" t="inlineStr"/>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr"/>
+      <c r="T251" t="inlineStr"/>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V251" t="inlineStr"/>
+      <c r="W251" t="inlineStr"/>
+      <c r="X251" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Tamara Sanderson</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Co-Author / Director</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Remote Works / Automattic</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Director at Automattic, worked across 70 countries distributed</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr"/>
+      <c r="H252" t="inlineStr"/>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr"/>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr"/>
+      <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr"/>
+      <c r="Q252" t="inlineStr"/>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr"/>
+      <c r="T252" t="inlineStr"/>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V252" t="inlineStr"/>
+      <c r="W252" t="inlineStr"/>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Rowena Hennigan</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>RoRemote</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>LinkedIn Top Voice, remote work educator, HBR/BBC/NYT featured</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr"/>
+      <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr"/>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr"/>
+      <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr"/>
+      <c r="Q253" t="inlineStr"/>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr"/>
+      <c r="T253" t="inlineStr"/>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V253" t="inlineStr"/>
+      <c r="W253" t="inlineStr"/>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Nadia Harris</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Remote Work Advocate</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Remote work lawyer, Global Remote Rights Award winner</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr"/>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>remoteworkadvocate</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr"/>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr"/>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>nadiaaharriss</t>
+        </is>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr"/>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr"/>
+      <c r="T254" t="inlineStr"/>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V254" t="inlineStr"/>
+      <c r="W254" t="inlineStr"/>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Mandy Fransz</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Remote Workers Worldwide</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Built 200K+ remote work community, LinkedIn Top Voice</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr"/>
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr"/>
+      <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr"/>
+      <c r="Q255" t="inlineStr"/>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr"/>
+      <c r="T255" t="inlineStr"/>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V255" t="inlineStr"/>
+      <c r="W255" t="inlineStr"/>
+      <c r="X255" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Debra Dinnocenzo</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>VirtualWorks!</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Virtual workplace pioneer since 1995, author Remote Leadership</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr"/>
+      <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr"/>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr"/>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>debradinnocenzo</t>
+        </is>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>Twitter</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr"/>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr"/>
+      <c r="T256" t="inlineStr"/>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V256" t="inlineStr"/>
+      <c r="W256" t="inlineStr"/>
+      <c r="X256" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Pilar Orti</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Virtual Not Distant</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>21st Century Work Life podcast host, office-optional culture expert</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr"/>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr"/>
+      <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr"/>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr"/>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>PilarOrti</t>
+        </is>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr"/>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr"/>
+      <c r="T257" t="inlineStr"/>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V257" t="inlineStr"/>
+      <c r="W257" t="inlineStr"/>
+      <c r="X257" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y257" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -14092,7 +15293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14420,6 +15621,26 @@
       <c r="D16" t="inlineStr">
         <is>
           <t>women-in-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>17</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>remote-team-leadership</t>
         </is>
       </c>
     </row>
@@ -14435,7 +15656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -18834,6 +20055,298 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>69c32ce2086473f19ac41eb1</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-03-31T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>69c32cf7404909f7dd683e0e</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>2026-03-31T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>pending_manual</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>69c32d3e404909f7dd68400a</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>2026-03-30T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>69c32d47086473f19ac420c5</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>2026-03-31T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>69c32d53404909f7dd6841c2</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2026-04-05T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>69c32d5d404909f7dd684232</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2026-03-31T04:02:00Z</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Remote Team Leadership</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>69c32d67086473f19ac422c0</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>2026-03-30T22:01:00Z</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Inclusive Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -890,10 +890,14 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1099,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y257"/>
+  <dimension ref="A1:Y274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13935,13 +13939,11 @@
           <t>Author of 'Remote Work Revolution', virtual teams researcher</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
           <t>tsedalneeley</t>
@@ -13967,7 +13969,6 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M241" t="inlineStr"/>
       <c r="N241" t="inlineStr">
         <is>
           <t>tsedal</t>
@@ -13983,27 +13984,21 @@
           <t>Twitter</t>
         </is>
       </c>
-      <c r="Q241" t="inlineStr"/>
       <c r="R241" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S241" t="inlineStr"/>
-      <c r="T241" t="inlineStr"/>
       <c r="U241" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V241" t="inlineStr"/>
-      <c r="W241" t="inlineStr"/>
       <c r="X241" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -14026,27 +14021,21 @@
           <t>World's foremost remote work researcher, WFH Research co-founder</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G242" t="inlineStr"/>
-      <c r="H242" t="inlineStr"/>
       <c r="I242" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J242" t="inlineStr"/>
-      <c r="K242" t="inlineStr"/>
       <c r="L242" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M242" t="inlineStr"/>
       <c r="N242" t="inlineStr">
         <is>
           <t>I_Am_NickBloom</t>
@@ -14062,20 +14051,16 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q242" t="inlineStr"/>
       <c r="R242" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S242" t="inlineStr"/>
-      <c r="T242" t="inlineStr"/>
       <c r="U242" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V242" t="inlineStr"/>
       <c r="W242" t="inlineStr">
         <is>
           <t>nickbloom.bsky.social</t>
@@ -14113,13 +14098,11 @@
           <t>Pioneered Head of Remote role, authored Remote Playbook</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr">
         <is>
           <t>darren_murph</t>
@@ -14135,13 +14118,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K243" t="inlineStr"/>
       <c r="L243" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M243" t="inlineStr"/>
       <c r="N243" t="inlineStr">
         <is>
           <t>darrenmurph</t>
@@ -14157,27 +14138,21 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q243" t="inlineStr"/>
       <c r="R243" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S243" t="inlineStr"/>
-      <c r="T243" t="inlineStr"/>
       <c r="U243" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V243" t="inlineStr"/>
-      <c r="W243" t="inlineStr"/>
       <c r="X243" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -14200,13 +14175,11 @@
           <t>Co-founded largest remote work conference and Time Doctor</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr">
         <is>
           <t>liamremote</t>
@@ -14232,7 +14205,6 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M244" t="inlineStr"/>
       <c r="N244" t="inlineStr">
         <is>
           <t>liamremote</t>
@@ -14248,27 +14220,21 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q244" t="inlineStr"/>
       <c r="R244" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S244" t="inlineStr"/>
-      <c r="T244" t="inlineStr"/>
       <c r="U244" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V244" t="inlineStr"/>
-      <c r="W244" t="inlineStr"/>
       <c r="X244" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -14291,13 +14257,11 @@
           <t>Co-author 'The Long-Distance Leader', remote management expert</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr">
         <is>
           <t>kevineikenberry</t>
@@ -14313,13 +14277,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K245" t="inlineStr"/>
       <c r="L245" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M245" t="inlineStr"/>
       <c r="N245" t="inlineStr">
         <is>
           <t>KevinEikenberry</t>
@@ -14335,13 +14297,11 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q245" t="inlineStr"/>
       <c r="R245" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S245" t="inlineStr"/>
       <c r="T245" t="inlineStr">
         <is>
           <t>KevinEikenberryGroup</t>
@@ -14357,13 +14317,11 @@
           <t>YouTube</t>
         </is>
       </c>
-      <c r="W245" t="inlineStr"/>
       <c r="X245" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -14386,55 +14344,41 @@
           <t>Co-author 'The Long-Distance Leader', virtual communication specialist</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G246" t="inlineStr"/>
-      <c r="H246" t="inlineStr"/>
       <c r="I246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr"/>
-      <c r="K246" t="inlineStr"/>
       <c r="L246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M246" t="inlineStr"/>
-      <c r="N246" t="inlineStr"/>
       <c r="O246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P246" t="inlineStr"/>
-      <c r="Q246" t="inlineStr"/>
       <c r="R246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S246" t="inlineStr"/>
-      <c r="T246" t="inlineStr"/>
       <c r="U246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V246" t="inlineStr"/>
-      <c r="W246" t="inlineStr"/>
       <c r="X246" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -14457,55 +14401,41 @@
           <t>Trains enterprise leaders at Toyota, Sephora, Cisco on hybrid teams</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr"/>
-      <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J247" t="inlineStr"/>
-      <c r="K247" t="inlineStr"/>
       <c r="L247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M247" t="inlineStr"/>
-      <c r="N247" t="inlineStr"/>
       <c r="O247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P247" t="inlineStr"/>
-      <c r="Q247" t="inlineStr"/>
       <c r="R247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S247" t="inlineStr"/>
-      <c r="T247" t="inlineStr"/>
       <c r="U247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V247" t="inlineStr"/>
-      <c r="W247" t="inlineStr"/>
       <c r="X247" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -14528,13 +14458,11 @@
           <t>Remote Work Association founder, Top 100 Future of Work Leader</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr">
         <is>
           <t>laurel_farrer</t>
@@ -14550,13 +14478,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K248" t="inlineStr"/>
       <c r="L248" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M248" t="inlineStr"/>
       <c r="N248" t="inlineStr">
         <is>
           <t>laurel_farrer</t>
@@ -14572,27 +14498,21 @@
           <t>Twitter</t>
         </is>
       </c>
-      <c r="Q248" t="inlineStr"/>
       <c r="R248" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S248" t="inlineStr"/>
-      <c r="T248" t="inlineStr"/>
       <c r="U248" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V248" t="inlineStr"/>
-      <c r="W248" t="inlineStr"/>
       <c r="X248" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -14615,27 +14535,21 @@
           <t>Author 'Work Together Anywhere', virtual collaboration podcast host</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr"/>
-      <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J249" t="inlineStr"/>
-      <c r="K249" t="inlineStr"/>
       <c r="L249" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M249" t="inlineStr"/>
       <c r="N249" t="inlineStr">
         <is>
           <t>lightling</t>
@@ -14651,27 +14565,21 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q249" t="inlineStr"/>
       <c r="R249" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S249" t="inlineStr"/>
-      <c r="T249" t="inlineStr"/>
       <c r="U249" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V249" t="inlineStr"/>
-      <c r="W249" t="inlineStr"/>
       <c r="X249" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -14694,27 +14602,21 @@
           <t>Leads remote strategy across 35+ countries, About Abroad podcast host</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G250" t="inlineStr"/>
-      <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J250" t="inlineStr"/>
-      <c r="K250" t="inlineStr"/>
       <c r="L250" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M250" t="inlineStr"/>
       <c r="N250" t="inlineStr">
         <is>
           <t>dcwarrington</t>
@@ -14730,27 +14632,21 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q250" t="inlineStr"/>
       <c r="R250" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S250" t="inlineStr"/>
-      <c r="T250" t="inlineStr"/>
       <c r="U250" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V250" t="inlineStr"/>
-      <c r="W250" t="inlineStr"/>
       <c r="X250" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -14773,55 +14669,41 @@
           <t>Former DuckDuckGo People Ops, co-wrote Remote Works playbook</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr"/>
-      <c r="H251" t="inlineStr"/>
       <c r="I251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J251" t="inlineStr"/>
-      <c r="K251" t="inlineStr"/>
       <c r="L251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M251" t="inlineStr"/>
-      <c r="N251" t="inlineStr"/>
       <c r="O251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P251" t="inlineStr"/>
-      <c r="Q251" t="inlineStr"/>
       <c r="R251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S251" t="inlineStr"/>
-      <c r="T251" t="inlineStr"/>
       <c r="U251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V251" t="inlineStr"/>
-      <c r="W251" t="inlineStr"/>
       <c r="X251" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -14844,55 +14726,41 @@
           <t>Director at Automattic, worked across 70 countries distributed</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr"/>
       <c r="F252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr"/>
-      <c r="H252" t="inlineStr"/>
       <c r="I252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr"/>
       <c r="L252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M252" t="inlineStr"/>
-      <c r="N252" t="inlineStr"/>
       <c r="O252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P252" t="inlineStr"/>
-      <c r="Q252" t="inlineStr"/>
       <c r="R252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S252" t="inlineStr"/>
-      <c r="T252" t="inlineStr"/>
       <c r="U252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V252" t="inlineStr"/>
-      <c r="W252" t="inlineStr"/>
       <c r="X252" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -14915,55 +14783,41 @@
           <t>LinkedIn Top Voice, remote work educator, HBR/BBC/NYT featured</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr"/>
-      <c r="H253" t="inlineStr"/>
       <c r="I253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J253" t="inlineStr"/>
-      <c r="K253" t="inlineStr"/>
       <c r="L253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M253" t="inlineStr"/>
-      <c r="N253" t="inlineStr"/>
       <c r="O253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P253" t="inlineStr"/>
-      <c r="Q253" t="inlineStr"/>
       <c r="R253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S253" t="inlineStr"/>
-      <c r="T253" t="inlineStr"/>
       <c r="U253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V253" t="inlineStr"/>
-      <c r="W253" t="inlineStr"/>
       <c r="X253" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -14986,13 +14840,11 @@
           <t>Remote work lawyer, Global Remote Rights Award winner</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr"/>
       <c r="H254" t="inlineStr">
         <is>
           <t>remoteworkadvocate</t>
@@ -15008,13 +14860,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K254" t="inlineStr"/>
       <c r="L254" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M254" t="inlineStr"/>
       <c r="N254" t="inlineStr">
         <is>
           <t>nadiaaharriss</t>
@@ -15030,27 +14880,21 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q254" t="inlineStr"/>
       <c r="R254" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S254" t="inlineStr"/>
-      <c r="T254" t="inlineStr"/>
       <c r="U254" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V254" t="inlineStr"/>
-      <c r="W254" t="inlineStr"/>
       <c r="X254" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -15073,55 +14917,41 @@
           <t>Built 200K+ remote work community, LinkedIn Top Voice</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
-      <c r="K255" t="inlineStr"/>
       <c r="L255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M255" t="inlineStr"/>
-      <c r="N255" t="inlineStr"/>
       <c r="O255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P255" t="inlineStr"/>
-      <c r="Q255" t="inlineStr"/>
       <c r="R255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S255" t="inlineStr"/>
-      <c r="T255" t="inlineStr"/>
       <c r="U255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V255" t="inlineStr"/>
-      <c r="W255" t="inlineStr"/>
       <c r="X255" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -15144,27 +14974,21 @@
           <t>Virtual workplace pioneer since 1995, author Remote Leadership</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr"/>
-      <c r="H256" t="inlineStr"/>
       <c r="I256" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
-      <c r="K256" t="inlineStr"/>
       <c r="L256" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M256" t="inlineStr"/>
       <c r="N256" t="inlineStr">
         <is>
           <t>debradinnocenzo</t>
@@ -15180,27 +15004,21 @@
           <t>Twitter</t>
         </is>
       </c>
-      <c r="Q256" t="inlineStr"/>
       <c r="R256" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S256" t="inlineStr"/>
-      <c r="T256" t="inlineStr"/>
       <c r="U256" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V256" t="inlineStr"/>
-      <c r="W256" t="inlineStr"/>
       <c r="X256" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -15223,27 +15041,21 @@
           <t>21st Century Work Life podcast host, office-optional culture expert</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G257" t="inlineStr"/>
-      <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J257" t="inlineStr"/>
-      <c r="K257" t="inlineStr"/>
       <c r="L257" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M257" t="inlineStr"/>
       <c r="N257" t="inlineStr">
         <is>
           <t>PilarOrti</t>
@@ -15259,27 +15071,1380 @@
           <t>Twitter/X</t>
         </is>
       </c>
-      <c r="Q257" t="inlineStr"/>
       <c r="R257" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S257" t="inlineStr"/>
-      <c r="T257" t="inlineStr"/>
       <c r="U257" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V257" t="inlineStr"/>
-      <c r="W257" t="inlineStr"/>
       <c r="X257" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Jennifer Brown</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Jennifer Brown Consulting</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Author of 'How to Be an Inclusive Leader'</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>@jenniferbrownspeaks</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>@jenniferbrownspeaks</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>@jenniferbrownspeaks</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>threads.com</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>@jennibrown</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr"/>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr"/>
+      <c r="T258" t="inlineStr"/>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V258" t="inlineStr"/>
+      <c r="W258" t="inlineStr"/>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Bernardo Ferdman</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Prof. Emeritus</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Alliant International University</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Co-editor of 'Inclusive Leadership' academic text</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr"/>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr"/>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="inlineStr"/>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr"/>
+      <c r="N259" t="inlineStr"/>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr"/>
+      <c r="Q259" t="inlineStr"/>
+      <c r="R259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S259" t="inlineStr"/>
+      <c r="T259" t="inlineStr"/>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V259" t="inlineStr"/>
+      <c r="W259" t="inlineStr"/>
+      <c r="X259" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Juliet Bourke</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Deloitte Australia</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Pioneered Six Signature Traits of Inclusive Leadership (HBR)</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr"/>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr"/>
+      <c r="H260" t="inlineStr"/>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr"/>
+      <c r="K260" t="inlineStr"/>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr"/>
+      <c r="N260" t="inlineStr"/>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr"/>
+      <c r="Q260" t="inlineStr"/>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr"/>
+      <c r="T260" t="inlineStr"/>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V260" t="inlineStr"/>
+      <c r="W260" t="inlineStr"/>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Dr. Stefanie K. Johnson</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>University of Colorado Boulder</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Author of 'Inclusify', Thinkers50 Radar</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>@DrStefJohnson</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>@drstefjohnson</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr"/>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr"/>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>@DrStefJohnson</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr"/>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr"/>
+      <c r="T261" t="inlineStr"/>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V261" t="inlineStr"/>
+      <c r="W261" t="inlineStr"/>
+      <c r="X261" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Síle Walsh</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Leadership Specialist</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Independent (Ireland)</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Award-winning author 'Inclusive Leadership: Navigating Organisational Complexity'</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr"/>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr"/>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr"/>
+      <c r="K262" t="inlineStr"/>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr"/>
+      <c r="N262" t="inlineStr"/>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr"/>
+      <c r="Q262" t="inlineStr"/>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr"/>
+      <c r="T262" t="inlineStr"/>
+      <c r="U262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V262" t="inlineStr"/>
+      <c r="W262" t="inlineStr"/>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Andrés Tapia</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Senior Client Partner</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Korn Ferry</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Author 'The 5 Disciplines of Inclusive Leaders' and 'The Inclusion Paradox'</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr"/>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr"/>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr"/>
+      <c r="K263" t="inlineStr"/>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr"/>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>@AndresTTapia</t>
+        </is>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>twitter.com</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr"/>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr"/>
+      <c r="T263" t="inlineStr"/>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr"/>
+      <c r="W263" t="inlineStr"/>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Ritu Bhasin</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>bhasin consulting inc.</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Creator of Three Selves Framework, author 'We've Got This'</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr"/>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>@ritu_bhasin</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr"/>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr"/>
+      <c r="N264" t="inlineStr"/>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr"/>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>@ritu_bhasin</t>
+        </is>
+      </c>
+      <c r="R264" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr"/>
+      <c r="U264" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V264" t="inlineStr"/>
+      <c r="W264" t="inlineStr"/>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Bernadette Smith</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Equality Institute</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Creator of ARC Method, author 'Inclusive 360'</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr"/>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr"/>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="inlineStr"/>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr"/>
+      <c r="N265" t="inlineStr"/>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr"/>
+      <c r="Q265" t="inlineStr"/>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr"/>
+      <c r="T265" t="inlineStr"/>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V265" t="inlineStr"/>
+      <c r="W265" t="inlineStr"/>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Tara Jaye Frank</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>The Waymakers Change Group</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Author 'The Waymakers' (Axiom Gold Medal), former Hallmark VP</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>@tarajayefrank</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>@tarajayefrank</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr"/>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr"/>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>@TaraJFrank</t>
+        </is>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr"/>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr"/>
+      <c r="T266" t="inlineStr"/>
+      <c r="U266" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V266" t="inlineStr"/>
+      <c r="W266" t="inlineStr"/>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Dr. Anthony Giannoumis</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Professor &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>OsloMet / Inclusive Creation</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Author 'Sins and Wins of Inclusive Leadership', UN award winner</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr"/>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr"/>
+      <c r="H267" t="inlineStr"/>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr"/>
+      <c r="N267" t="inlineStr"/>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr"/>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>@dranthonyg</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr"/>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr"/>
+      <c r="W267" t="inlineStr"/>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Eddie Pate</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Eddie Pate Consulting</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Co-author 'Daily Practices of Inclusive Leaders' (2024)</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr"/>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr"/>
+      <c r="H268" t="inlineStr"/>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr"/>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr"/>
+      <c r="N268" t="inlineStr"/>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr"/>
+      <c r="Q268" t="inlineStr"/>
+      <c r="R268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S268" t="inlineStr"/>
+      <c r="T268" t="inlineStr"/>
+      <c r="U268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V268" t="inlineStr"/>
+      <c r="W268" t="inlineStr"/>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Lily Zheng</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>DEI Strategist</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Author 'DEI Deconstructed', Forbes DEI Trailblazer</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr"/>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr"/>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>@lilyzheng308</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr"/>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr"/>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>@lilyzheng308</t>
+        </is>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>twitter.com</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr"/>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr"/>
+      <c r="T269" t="inlineStr"/>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V269" t="inlineStr"/>
+      <c r="W269" t="inlineStr"/>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Amri B. Johnson</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Inclusion Wins</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Author 'Reconstructing Inclusion', podcast host</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr"/>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr"/>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr"/>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr"/>
+      <c r="N270" t="inlineStr"/>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr"/>
+      <c r="Q270" t="inlineStr"/>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr"/>
+      <c r="T270" t="inlineStr"/>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr"/>
+      <c r="W270" t="inlineStr"/>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Minda Harts</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>NYU Wagner</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Author 'The Memo', LinkedIn #1 Top Voice Workplace Equity</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr"/>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>@mindaharts</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr"/>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr"/>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>@MindaHarts</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>twitter.com</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>@mindaharts1</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr"/>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V271" t="inlineStr"/>
+      <c r="W271" t="inlineStr"/>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Ernest Gundling</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Aperian Global</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Co-author 'Inclusive Leadership: Global Impact', UC Berkeley lecturer</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr"/>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
+      <c r="H272" t="inlineStr"/>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="inlineStr"/>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr"/>
+      <c r="N272" t="inlineStr"/>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr"/>
+      <c r="Q272" t="inlineStr"/>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr"/>
+      <c r="T272" t="inlineStr"/>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V272" t="inlineStr"/>
+      <c r="W272" t="inlineStr"/>
+      <c r="X272" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Jeanine Prime</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Former SVP Research</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Catalyst / Gartner</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Led cross-national inclusive leadership research</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr"/>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr"/>
+      <c r="H273" t="inlineStr"/>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="inlineStr"/>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr"/>
+      <c r="N273" t="inlineStr"/>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr"/>
+      <c r="Q273" t="inlineStr"/>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr"/>
+      <c r="T273" t="inlineStr"/>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V273" t="inlineStr"/>
+      <c r="W273" t="inlineStr"/>
+      <c r="X273" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Jonathan Stutz</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Global Diversity Partners</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Co-author 'Daily Practices of Inclusive Leaders' (2024)</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr"/>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr"/>
+      <c r="H274" t="inlineStr"/>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="inlineStr"/>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr"/>
+      <c r="N274" t="inlineStr"/>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr"/>
+      <c r="Q274" t="inlineStr"/>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr"/>
+      <c r="T274" t="inlineStr"/>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V274" t="inlineStr"/>
+      <c r="W274" t="inlineStr"/>
+      <c r="X274" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y274" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -15293,7 +16458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -15641,6 +16806,26 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>remote-team-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>inclusive-leadership</t>
         </is>
       </c>
     </row>
@@ -15656,7 +16841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G129"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -20155,7 +21340,6 @@
           <t>pending_manual</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>manual</t>
@@ -20342,6 +21526,302 @@
         </is>
       </c>
       <c r="G129" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>69c381c0d86d5be7603e0800</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2026-03-31T12:45:00Z</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>69c381c2d86d5be7603e0826</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>2026-03-31T13:30:00Z</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>69c3821150cd25c19e0e0df6</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-04-05T06:00:00Z</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>69c381d750cd25c19e0e0d30</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>2026-03-31T04:02:00Z</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>69c381e450cd25c19e0e0d56</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>2026-03-31T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>69c381fc50cd25c19e0e0d9f</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>2026-04-10T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>69c381fed86d5be7603e093f</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>2026-03-31T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Inclusive Leadership</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>69c38210d86d5be7603e09b2</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>2026-03-31T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
         <is>
           <t>addToQueue</t>
         </is>

</xml_diff>

<commit_message>
Update handle database — Decision Making
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -911,10 +911,14 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1103,7 +1107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y274"/>
+  <dimension ref="A1:Y291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15168,27 +15172,21 @@
           <t>website</t>
         </is>
       </c>
-      <c r="Q258" t="inlineStr"/>
       <c r="R258" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S258" t="inlineStr"/>
-      <c r="T258" t="inlineStr"/>
       <c r="U258" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V258" t="inlineStr"/>
-      <c r="W258" t="inlineStr"/>
       <c r="X258" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -15211,55 +15209,41 @@
           <t>Co-editor of 'Inclusive Leadership' academic text</t>
         </is>
       </c>
-      <c r="E259" t="inlineStr"/>
       <c r="F259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G259" t="inlineStr"/>
-      <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J259" t="inlineStr"/>
-      <c r="K259" t="inlineStr"/>
       <c r="L259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M259" t="inlineStr"/>
-      <c r="N259" t="inlineStr"/>
       <c r="O259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P259" t="inlineStr"/>
-      <c r="Q259" t="inlineStr"/>
       <c r="R259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S259" t="inlineStr"/>
-      <c r="T259" t="inlineStr"/>
       <c r="U259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V259" t="inlineStr"/>
-      <c r="W259" t="inlineStr"/>
       <c r="X259" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -15282,55 +15266,41 @@
           <t>Pioneered Six Signature Traits of Inclusive Leadership (HBR)</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
       <c r="I260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
-      <c r="K260" t="inlineStr"/>
       <c r="L260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M260" t="inlineStr"/>
-      <c r="N260" t="inlineStr"/>
       <c r="O260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P260" t="inlineStr"/>
-      <c r="Q260" t="inlineStr"/>
       <c r="R260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S260" t="inlineStr"/>
-      <c r="T260" t="inlineStr"/>
       <c r="U260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V260" t="inlineStr"/>
-      <c r="W260" t="inlineStr"/>
       <c r="X260" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -15383,13 +15353,11 @@
           <t>search</t>
         </is>
       </c>
-      <c r="K261" t="inlineStr"/>
       <c r="L261" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M261" t="inlineStr"/>
       <c r="N261" t="inlineStr">
         <is>
           <t>@DrStefJohnson</t>
@@ -15405,27 +15373,21 @@
           <t>search</t>
         </is>
       </c>
-      <c r="Q261" t="inlineStr"/>
       <c r="R261" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S261" t="inlineStr"/>
-      <c r="T261" t="inlineStr"/>
       <c r="U261" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V261" t="inlineStr"/>
-      <c r="W261" t="inlineStr"/>
       <c r="X261" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -15448,55 +15410,41 @@
           <t>Award-winning author 'Inclusive Leadership: Navigating Organisational Complexity'</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr"/>
       <c r="F262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr"/>
-      <c r="H262" t="inlineStr"/>
       <c r="I262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J262" t="inlineStr"/>
-      <c r="K262" t="inlineStr"/>
       <c r="L262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M262" t="inlineStr"/>
-      <c r="N262" t="inlineStr"/>
       <c r="O262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P262" t="inlineStr"/>
-      <c r="Q262" t="inlineStr"/>
       <c r="R262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S262" t="inlineStr"/>
-      <c r="T262" t="inlineStr"/>
       <c r="U262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V262" t="inlineStr"/>
-      <c r="W262" t="inlineStr"/>
       <c r="X262" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -15519,27 +15467,21 @@
           <t>Author 'The 5 Disciplines of Inclusive Leaders' and 'The Inclusion Paradox'</t>
         </is>
       </c>
-      <c r="E263" t="inlineStr"/>
       <c r="F263" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G263" t="inlineStr"/>
-      <c r="H263" t="inlineStr"/>
       <c r="I263" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
-      <c r="K263" t="inlineStr"/>
       <c r="L263" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M263" t="inlineStr"/>
       <c r="N263" t="inlineStr">
         <is>
           <t>@AndresTTapia</t>
@@ -15555,27 +15497,21 @@
           <t>twitter.com</t>
         </is>
       </c>
-      <c r="Q263" t="inlineStr"/>
       <c r="R263" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S263" t="inlineStr"/>
-      <c r="T263" t="inlineStr"/>
       <c r="U263" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V263" t="inlineStr"/>
-      <c r="W263" t="inlineStr"/>
       <c r="X263" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -15598,13 +15534,11 @@
           <t>Creator of Three Selves Framework, author 'We've Got This'</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr"/>
       <c r="F264" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G264" t="inlineStr"/>
       <c r="H264" t="inlineStr">
         <is>
           <t>@ritu_bhasin</t>
@@ -15620,20 +15554,16 @@
           <t>search</t>
         </is>
       </c>
-      <c r="K264" t="inlineStr"/>
       <c r="L264" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M264" t="inlineStr"/>
-      <c r="N264" t="inlineStr"/>
       <c r="O264" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P264" t="inlineStr"/>
       <c r="Q264" t="inlineStr">
         <is>
           <t>@ritu_bhasin</t>
@@ -15649,20 +15579,16 @@
           <t>search</t>
         </is>
       </c>
-      <c r="T264" t="inlineStr"/>
       <c r="U264" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V264" t="inlineStr"/>
-      <c r="W264" t="inlineStr"/>
       <c r="X264" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -15685,55 +15611,41 @@
           <t>Creator of ARC Method, author 'Inclusive 360'</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
-      <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J265" t="inlineStr"/>
-      <c r="K265" t="inlineStr"/>
       <c r="L265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M265" t="inlineStr"/>
-      <c r="N265" t="inlineStr"/>
       <c r="O265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P265" t="inlineStr"/>
-      <c r="Q265" t="inlineStr"/>
       <c r="R265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S265" t="inlineStr"/>
-      <c r="T265" t="inlineStr"/>
       <c r="U265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V265" t="inlineStr"/>
-      <c r="W265" t="inlineStr"/>
       <c r="X265" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -15786,13 +15698,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K266" t="inlineStr"/>
       <c r="L266" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M266" t="inlineStr"/>
       <c r="N266" t="inlineStr">
         <is>
           <t>@TaraJFrank</t>
@@ -15808,27 +15718,21 @@
           <t>search</t>
         </is>
       </c>
-      <c r="Q266" t="inlineStr"/>
       <c r="R266" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S266" t="inlineStr"/>
-      <c r="T266" t="inlineStr"/>
       <c r="U266" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V266" t="inlineStr"/>
-      <c r="W266" t="inlineStr"/>
       <c r="X266" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -15851,34 +15755,26 @@
           <t>Author 'Sins and Wins of Inclusive Leadership', UN award winner</t>
         </is>
       </c>
-      <c r="E267" t="inlineStr"/>
       <c r="F267" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G267" t="inlineStr"/>
-      <c r="H267" t="inlineStr"/>
       <c r="I267" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
-      <c r="K267" t="inlineStr"/>
       <c r="L267" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M267" t="inlineStr"/>
-      <c r="N267" t="inlineStr"/>
       <c r="O267" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P267" t="inlineStr"/>
       <c r="Q267" t="inlineStr">
         <is>
           <t>@dranthonyg</t>
@@ -15894,20 +15790,16 @@
           <t>tiktok.com</t>
         </is>
       </c>
-      <c r="T267" t="inlineStr"/>
       <c r="U267" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V267" t="inlineStr"/>
-      <c r="W267" t="inlineStr"/>
       <c r="X267" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -15930,55 +15822,41 @@
           <t>Co-author 'Daily Practices of Inclusive Leaders' (2024)</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr"/>
       <c r="F268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr"/>
-      <c r="H268" t="inlineStr"/>
       <c r="I268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J268" t="inlineStr"/>
-      <c r="K268" t="inlineStr"/>
       <c r="L268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M268" t="inlineStr"/>
-      <c r="N268" t="inlineStr"/>
       <c r="O268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P268" t="inlineStr"/>
-      <c r="Q268" t="inlineStr"/>
       <c r="R268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S268" t="inlineStr"/>
-      <c r="T268" t="inlineStr"/>
       <c r="U268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V268" t="inlineStr"/>
-      <c r="W268" t="inlineStr"/>
       <c r="X268" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -16001,13 +15879,11 @@
           <t>Author 'DEI Deconstructed', Forbes DEI Trailblazer</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr"/>
       <c r="F269" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G269" t="inlineStr"/>
       <c r="H269" t="inlineStr">
         <is>
           <t>@lilyzheng308</t>
@@ -16023,13 +15899,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K269" t="inlineStr"/>
       <c r="L269" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M269" t="inlineStr"/>
       <c r="N269" t="inlineStr">
         <is>
           <t>@lilyzheng308</t>
@@ -16045,27 +15919,21 @@
           <t>twitter.com</t>
         </is>
       </c>
-      <c r="Q269" t="inlineStr"/>
       <c r="R269" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S269" t="inlineStr"/>
-      <c r="T269" t="inlineStr"/>
       <c r="U269" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V269" t="inlineStr"/>
-      <c r="W269" t="inlineStr"/>
       <c r="X269" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -16088,55 +15956,41 @@
           <t>Author 'Reconstructing Inclusion', podcast host</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr"/>
       <c r="F270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr"/>
-      <c r="H270" t="inlineStr"/>
       <c r="I270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
-      <c r="K270" t="inlineStr"/>
       <c r="L270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M270" t="inlineStr"/>
-      <c r="N270" t="inlineStr"/>
       <c r="O270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P270" t="inlineStr"/>
-      <c r="Q270" t="inlineStr"/>
       <c r="R270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S270" t="inlineStr"/>
-      <c r="T270" t="inlineStr"/>
       <c r="U270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V270" t="inlineStr"/>
-      <c r="W270" t="inlineStr"/>
       <c r="X270" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -16159,13 +16013,11 @@
           <t>Author 'The Memo', LinkedIn #1 Top Voice Workplace Equity</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr"/>
       <c r="F271" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr"/>
       <c r="H271" t="inlineStr">
         <is>
           <t>@mindaharts</t>
@@ -16181,13 +16033,11 @@
           <t>instagram.com</t>
         </is>
       </c>
-      <c r="K271" t="inlineStr"/>
       <c r="L271" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M271" t="inlineStr"/>
       <c r="N271" t="inlineStr">
         <is>
           <t>@MindaHarts</t>
@@ -16218,20 +16068,16 @@
           <t>tiktok.com</t>
         </is>
       </c>
-      <c r="T271" t="inlineStr"/>
       <c r="U271" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V271" t="inlineStr"/>
-      <c r="W271" t="inlineStr"/>
       <c r="X271" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -16254,55 +16100,41 @@
           <t>Co-author 'Inclusive Leadership: Global Impact', UC Berkeley lecturer</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr"/>
       <c r="F272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
       <c r="I272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
-      <c r="K272" t="inlineStr"/>
       <c r="L272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M272" t="inlineStr"/>
-      <c r="N272" t="inlineStr"/>
       <c r="O272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P272" t="inlineStr"/>
-      <c r="Q272" t="inlineStr"/>
       <c r="R272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S272" t="inlineStr"/>
-      <c r="T272" t="inlineStr"/>
       <c r="U272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V272" t="inlineStr"/>
-      <c r="W272" t="inlineStr"/>
       <c r="X272" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -16325,55 +16157,41 @@
           <t>Led cross-national inclusive leadership research</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr"/>
       <c r="F273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G273" t="inlineStr"/>
-      <c r="H273" t="inlineStr"/>
       <c r="I273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr"/>
-      <c r="K273" t="inlineStr"/>
       <c r="L273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M273" t="inlineStr"/>
-      <c r="N273" t="inlineStr"/>
       <c r="O273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P273" t="inlineStr"/>
-      <c r="Q273" t="inlineStr"/>
       <c r="R273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S273" t="inlineStr"/>
-      <c r="T273" t="inlineStr"/>
       <c r="U273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V273" t="inlineStr"/>
-      <c r="W273" t="inlineStr"/>
       <c r="X273" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -16396,55 +16214,1432 @@
           <t>Co-author 'Daily Practices of Inclusive Leaders' (2024)</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr"/>
       <c r="F274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G274" t="inlineStr"/>
-      <c r="H274" t="inlineStr"/>
       <c r="I274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr"/>
-      <c r="K274" t="inlineStr"/>
       <c r="L274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M274" t="inlineStr"/>
-      <c r="N274" t="inlineStr"/>
       <c r="O274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P274" t="inlineStr"/>
-      <c r="Q274" t="inlineStr"/>
       <c r="R274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S274" t="inlineStr"/>
-      <c r="T274" t="inlineStr"/>
       <c r="U274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V274" t="inlineStr"/>
-      <c r="W274" t="inlineStr"/>
       <c r="X274" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Annie Duke</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Decision Strategist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Author of Thinking in Bets, How to Decide, and Quit — former poker champion turned decision science expert</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr"/>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>_annieduke</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr"/>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr"/>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>AnnieDuke</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr"/>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S275" t="inlineStr"/>
+      <c r="T275" t="inlineStr"/>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V275" t="inlineStr"/>
+      <c r="W275" t="inlineStr"/>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Gary Klein</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Cognitive Psychologist &amp; Researcher</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>ShadowBox LLC</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Pioneer of Naturalistic Decision Making — studied how experts make split-second decisions under pressure</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr"/>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="inlineStr"/>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr"/>
+      <c r="N276" t="inlineStr"/>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr"/>
+      <c r="Q276" t="inlineStr"/>
+      <c r="R276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S276" t="inlineStr"/>
+      <c r="T276" t="inlineStr"/>
+      <c r="U276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V276" t="inlineStr"/>
+      <c r="W276" t="inlineStr"/>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Shane Parrish</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Farnam Street</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Author of Clear Thinking and host of The Knowledge Project podcast — Wall Street's biggest influencer on decision making</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr"/>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr"/>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>farnamstreet</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr"/>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr"/>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>ShaneAParrish</t>
+        </is>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr"/>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S277" t="inlineStr"/>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>Farnam Street</t>
+        </is>
+      </c>
+      <c r="U277" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="W277" t="inlineStr"/>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Philip Tetlock</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Wharton School, University of Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Author of Superforecasting — proved certain people can predict the future far more accurately</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr"/>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr"/>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr"/>
+      <c r="K278" t="inlineStr"/>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr"/>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>PTetlock</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr"/>
+      <c r="R278" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr"/>
+      <c r="T278" t="inlineStr"/>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V278" t="inlineStr"/>
+      <c r="W278" t="inlineStr"/>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Cassie Kozyrkov</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Data Scientific (formerly Google Chief Decision Scientist)</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Founded Decision Intelligence and trained 20,000 Googlers to make better decisions using data and AI</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr"/>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>decisionleader</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr"/>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr"/>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>quaesita</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>IDCrawl search</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr"/>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr"/>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>Cassie Kozyrkov</t>
+        </is>
+      </c>
+      <c r="U279" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V279" t="inlineStr">
+        <is>
+          <t>YouTube channel 67K subs</t>
+        </is>
+      </c>
+      <c r="W279" t="inlineStr"/>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Sheena Iyengar</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Columbia Business School</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Pioneered the science of choice overload with her famous jam study — author of The Art of Choosing</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr"/>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr"/>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>sheenaiyengar</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr"/>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr"/>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>Sheena_Iyengar</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr"/>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr"/>
+      <c r="T280" t="inlineStr"/>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V280" t="inlineStr"/>
+      <c r="W280" t="inlineStr"/>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Gerd Gigerenzer</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Director Emeritus</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Max Planck Institute for Human Development</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>World's leading researcher on how simple heuristics outperform complex analysis — author of Gut Feelings</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr"/>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr"/>
+      <c r="H281" t="inlineStr"/>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="inlineStr"/>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr"/>
+      <c r="N281" t="inlineStr"/>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr"/>
+      <c r="Q281" t="inlineStr"/>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr"/>
+      <c r="T281" t="inlineStr"/>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V281" t="inlineStr"/>
+      <c r="W281" t="inlineStr"/>
+      <c r="X281" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Julia Galef</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Author &amp; Rationality Advocate</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Center for Applied Rationality (co-founder)</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Author of The Scout Mindset — teaches people to seek truth over confirmation</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr"/>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr"/>
+      <c r="H282" t="inlineStr"/>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="inlineStr"/>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr"/>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>juliagalef</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr"/>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr"/>
+      <c r="T282" t="inlineStr"/>
+      <c r="U282" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
+      <c r="X282" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Katy Milkman</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Wharton School, University of Pennsylvania</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Behavioral scientist, host of Choiceology podcast, author of How to Change — former president of SJDM</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr"/>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr"/>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="inlineStr"/>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr"/>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>katy_milkman</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr"/>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr"/>
+      <c r="T283" t="inlineStr"/>
+      <c r="U283" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V283" t="inlineStr"/>
+      <c r="W283" t="inlineStr"/>
+      <c r="X283" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Michael Mauboussin</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Head of Consilient Research</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Morgan Stanley Investment Management</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Author of Think Twice and More Than You Know — helps leaders separate skill from luck in decisions</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr"/>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr"/>
+      <c r="H284" t="inlineStr"/>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr"/>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr"/>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>mjmauboussin</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>X profile 154K followers</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr"/>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr"/>
+      <c r="T284" t="inlineStr"/>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V284" t="inlineStr"/>
+      <c r="W284" t="inlineStr"/>
+      <c r="X284" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Melina Palmer</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>The Brainy Business</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Host of The Brainy Business podcast with 1M+ downloads — applies behavioral economics to decision making</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>thebrainybiz</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>thebrainybiz</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr"/>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr"/>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>thebrainybiz</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr"/>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr"/>
+      <c r="T285" t="inlineStr"/>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V285" t="inlineStr"/>
+      <c r="W285" t="inlineStr"/>
+      <c r="X285" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Lorien Pratt</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Chief Scientist</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Quantellia</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>AI pioneer who invented transfer learning and co-created Decision Intelligence — author of The Decision Intelligence Handbook</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr"/>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr"/>
+      <c r="H286" t="inlineStr"/>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr"/>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr"/>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>LorienPratt</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr"/>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr"/>
+      <c r="T286" t="inlineStr"/>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V286" t="inlineStr"/>
+      <c r="W286" t="inlineStr"/>
+      <c r="X286" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Gleb Tsipursky</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Disaster Avoidance Experts</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Cognitive neuroscientist and author of Never Go With Your Gut — helps leaders avoid cognitive biases</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr"/>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>dr_gleb_tsipursky</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr"/>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr"/>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>gleb_tsipursky</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr"/>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr"/>
+      <c r="T287" t="inlineStr"/>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V287" t="inlineStr"/>
+      <c r="W287" t="inlineStr"/>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Phill Agnew</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Nudge Podcast / Buffer</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Host of UK's #1 marketing podcast on behavioral science — breaks down the psychology behind decisions</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr"/>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr"/>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr"/>
+      <c r="N288" t="inlineStr"/>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr"/>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>nudgepod</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>Nudge podcast website</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr"/>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V288" t="inlineStr"/>
+      <c r="W288" t="inlineStr"/>
+      <c r="X288" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Baruch Fischhoff</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Past president of the Society for Judgment and Decision Making — pioneer of risk communication and hindsight bias research</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr"/>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr"/>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr"/>
+      <c r="N289" t="inlineStr"/>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr"/>
+      <c r="Q289" t="inlineStr"/>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr"/>
+      <c r="T289" t="inlineStr"/>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V289" t="inlineStr"/>
+      <c r="W289" t="inlineStr"/>
+      <c r="X289" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Richard Thaler</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>University of Chicago Booth School of Business</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>2017 Nobel Prize winner in Economics — co-author of Nudge and author of Misbehaving</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr"/>
+      <c r="H290" t="inlineStr"/>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr"/>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr"/>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>R_Thaler</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>X profile 200K followers</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr"/>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr"/>
+      <c r="T290" t="inlineStr"/>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V290" t="inlineStr"/>
+      <c r="W290" t="inlineStr"/>
+      <c r="X290" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Cass Sunstein</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Harvard Law School</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Co-author of Nudge and founder of the Program on Behavioral Economics and Public Policy at Harvard</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr"/>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr"/>
+      <c r="H291" t="inlineStr"/>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr"/>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr"/>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>CassSunstein</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr"/>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr"/>
+      <c r="T291" t="inlineStr"/>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V291" t="inlineStr"/>
+      <c r="W291" t="inlineStr"/>
+      <c r="X291" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y291" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -16458,7 +17653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16826,6 +18021,26 @@
       <c r="D18" t="inlineStr">
         <is>
           <t>inclusive-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>17</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>decision-making</t>
         </is>
       </c>
     </row>
@@ -16841,7 +18056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -21827,6 +23042,302 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>69c39bf5b89dd76ae2acfb29</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2026-03-31T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>69c39c03ff77135659b67702</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2026-03-31T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>69c39c0bb89dd76ae2acfb5f</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-03-31T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>69c39c18b89dd76ae2acfb99</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>2026-03-31T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>69c39c2eb89dd76ae2acfdaf</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>2026-04-08T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>69c39c34b89dd76ae2acfe05</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>2026-04-08T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>69c39c1fff77135659b677a2</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>2026-03-31T21:15:00Z</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Decision Making</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>69c39c22ff77135659b677d8</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>2026-03-31T15:02:00Z</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Leadership Communication
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -932,10 +932,14 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1107,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y291"/>
+  <dimension ref="A1:Y308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16271,13 +16275,11 @@
           <t>Author of Thinking in Bets, How to Decide, and Quit — former poker champion turned decision science expert</t>
         </is>
       </c>
-      <c r="E275" t="inlineStr"/>
       <c r="F275" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G275" t="inlineStr"/>
       <c r="H275" t="inlineStr">
         <is>
           <t>_annieduke</t>
@@ -16293,13 +16295,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K275" t="inlineStr"/>
       <c r="L275" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M275" t="inlineStr"/>
       <c r="N275" t="inlineStr">
         <is>
           <t>AnnieDuke</t>
@@ -16315,27 +16315,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q275" t="inlineStr"/>
       <c r="R275" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S275" t="inlineStr"/>
-      <c r="T275" t="inlineStr"/>
       <c r="U275" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V275" t="inlineStr"/>
-      <c r="W275" t="inlineStr"/>
       <c r="X275" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -16358,55 +16352,41 @@
           <t>Pioneer of Naturalistic Decision Making — studied how experts make split-second decisions under pressure</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr"/>
       <c r="F276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
       <c r="I276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J276" t="inlineStr"/>
-      <c r="K276" t="inlineStr"/>
       <c r="L276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M276" t="inlineStr"/>
-      <c r="N276" t="inlineStr"/>
       <c r="O276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P276" t="inlineStr"/>
-      <c r="Q276" t="inlineStr"/>
       <c r="R276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S276" t="inlineStr"/>
-      <c r="T276" t="inlineStr"/>
       <c r="U276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V276" t="inlineStr"/>
-      <c r="W276" t="inlineStr"/>
       <c r="X276" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -16429,13 +16409,11 @@
           <t>Author of Clear Thinking and host of The Knowledge Project podcast — Wall Street's biggest influencer on decision making</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr"/>
       <c r="F277" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G277" t="inlineStr"/>
       <c r="H277" t="inlineStr">
         <is>
           <t>farnamstreet</t>
@@ -16451,13 +16429,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K277" t="inlineStr"/>
       <c r="L277" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M277" t="inlineStr"/>
       <c r="N277" t="inlineStr">
         <is>
           <t>ShaneAParrish</t>
@@ -16473,13 +16449,11 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q277" t="inlineStr"/>
       <c r="R277" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S277" t="inlineStr"/>
       <c r="T277" t="inlineStr">
         <is>
           <t>Farnam Street</t>
@@ -16495,13 +16469,11 @@
           <t>YouTube channel</t>
         </is>
       </c>
-      <c r="W277" t="inlineStr"/>
       <c r="X277" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -16524,27 +16496,21 @@
           <t>Author of Superforecasting — proved certain people can predict the future far more accurately</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr"/>
       <c r="F278" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G278" t="inlineStr"/>
-      <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
-      <c r="K278" t="inlineStr"/>
       <c r="L278" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M278" t="inlineStr"/>
       <c r="N278" t="inlineStr">
         <is>
           <t>PTetlock</t>
@@ -16560,27 +16526,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q278" t="inlineStr"/>
       <c r="R278" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S278" t="inlineStr"/>
-      <c r="T278" t="inlineStr"/>
       <c r="U278" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V278" t="inlineStr"/>
-      <c r="W278" t="inlineStr"/>
       <c r="X278" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -16603,13 +16563,11 @@
           <t>Founded Decision Intelligence and trained 20,000 Googlers to make better decisions using data and AI</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr"/>
       <c r="F279" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G279" t="inlineStr"/>
       <c r="H279" t="inlineStr">
         <is>
           <t>decisionleader</t>
@@ -16625,13 +16583,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K279" t="inlineStr"/>
       <c r="L279" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M279" t="inlineStr"/>
       <c r="N279" t="inlineStr">
         <is>
           <t>quaesita</t>
@@ -16647,13 +16603,11 @@
           <t>IDCrawl search</t>
         </is>
       </c>
-      <c r="Q279" t="inlineStr"/>
       <c r="R279" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S279" t="inlineStr"/>
       <c r="T279" t="inlineStr">
         <is>
           <t>Cassie Kozyrkov</t>
@@ -16669,13 +16623,11 @@
           <t>YouTube channel 67K subs</t>
         </is>
       </c>
-      <c r="W279" t="inlineStr"/>
       <c r="X279" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -16698,13 +16650,11 @@
           <t>Pioneered the science of choice overload with her famous jam study — author of The Art of Choosing</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr"/>
       <c r="F280" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G280" t="inlineStr"/>
       <c r="H280" t="inlineStr">
         <is>
           <t>sheenaiyengar</t>
@@ -16720,13 +16670,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K280" t="inlineStr"/>
       <c r="L280" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M280" t="inlineStr"/>
       <c r="N280" t="inlineStr">
         <is>
           <t>Sheena_Iyengar</t>
@@ -16742,27 +16690,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q280" t="inlineStr"/>
       <c r="R280" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S280" t="inlineStr"/>
-      <c r="T280" t="inlineStr"/>
       <c r="U280" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V280" t="inlineStr"/>
-      <c r="W280" t="inlineStr"/>
       <c r="X280" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -16785,55 +16727,41 @@
           <t>World's leading researcher on how simple heuristics outperform complex analysis — author of Gut Feelings</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr"/>
       <c r="F281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G281" t="inlineStr"/>
-      <c r="H281" t="inlineStr"/>
       <c r="I281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr"/>
-      <c r="K281" t="inlineStr"/>
       <c r="L281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M281" t="inlineStr"/>
-      <c r="N281" t="inlineStr"/>
       <c r="O281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P281" t="inlineStr"/>
-      <c r="Q281" t="inlineStr"/>
       <c r="R281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S281" t="inlineStr"/>
-      <c r="T281" t="inlineStr"/>
       <c r="U281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
       <c r="X281" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -16856,27 +16784,21 @@
           <t>Author of The Scout Mindset — teaches people to seek truth over confirmation</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr"/>
       <c r="F282" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G282" t="inlineStr"/>
-      <c r="H282" t="inlineStr"/>
       <c r="I282" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr"/>
-      <c r="K282" t="inlineStr"/>
       <c r="L282" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M282" t="inlineStr"/>
       <c r="N282" t="inlineStr">
         <is>
           <t>juliagalef</t>
@@ -16892,27 +16814,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q282" t="inlineStr"/>
       <c r="R282" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S282" t="inlineStr"/>
-      <c r="T282" t="inlineStr"/>
       <c r="U282" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V282" t="inlineStr"/>
-      <c r="W282" t="inlineStr"/>
       <c r="X282" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -16935,27 +16851,21 @@
           <t>Behavioral scientist, host of Choiceology podcast, author of How to Change — former president of SJDM</t>
         </is>
       </c>
-      <c r="E283" t="inlineStr"/>
       <c r="F283" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G283" t="inlineStr"/>
-      <c r="H283" t="inlineStr"/>
       <c r="I283" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J283" t="inlineStr"/>
-      <c r="K283" t="inlineStr"/>
       <c r="L283" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M283" t="inlineStr"/>
       <c r="N283" t="inlineStr">
         <is>
           <t>katy_milkman</t>
@@ -16971,27 +16881,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q283" t="inlineStr"/>
       <c r="R283" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S283" t="inlineStr"/>
-      <c r="T283" t="inlineStr"/>
       <c r="U283" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V283" t="inlineStr"/>
-      <c r="W283" t="inlineStr"/>
       <c r="X283" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -17014,27 +16918,21 @@
           <t>Author of Think Twice and More Than You Know — helps leaders separate skill from luck in decisions</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr"/>
       <c r="F284" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G284" t="inlineStr"/>
-      <c r="H284" t="inlineStr"/>
       <c r="I284" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
       <c r="L284" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M284" t="inlineStr"/>
       <c r="N284" t="inlineStr">
         <is>
           <t>mjmauboussin</t>
@@ -17050,27 +16948,21 @@
           <t>X profile 154K followers</t>
         </is>
       </c>
-      <c r="Q284" t="inlineStr"/>
       <c r="R284" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S284" t="inlineStr"/>
-      <c r="T284" t="inlineStr"/>
       <c r="U284" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V284" t="inlineStr"/>
-      <c r="W284" t="inlineStr"/>
       <c r="X284" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -17123,13 +17015,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K285" t="inlineStr"/>
       <c r="L285" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M285" t="inlineStr"/>
       <c r="N285" t="inlineStr">
         <is>
           <t>thebrainybiz</t>
@@ -17145,27 +17035,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q285" t="inlineStr"/>
       <c r="R285" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S285" t="inlineStr"/>
-      <c r="T285" t="inlineStr"/>
       <c r="U285" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V285" t="inlineStr"/>
-      <c r="W285" t="inlineStr"/>
       <c r="X285" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -17188,27 +17072,21 @@
           <t>AI pioneer who invented transfer learning and co-created Decision Intelligence — author of The Decision Intelligence Handbook</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr"/>
-      <c r="H286" t="inlineStr"/>
       <c r="I286" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr"/>
-      <c r="K286" t="inlineStr"/>
       <c r="L286" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M286" t="inlineStr"/>
       <c r="N286" t="inlineStr">
         <is>
           <t>LorienPratt</t>
@@ -17224,27 +17102,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q286" t="inlineStr"/>
       <c r="R286" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S286" t="inlineStr"/>
-      <c r="T286" t="inlineStr"/>
       <c r="U286" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V286" t="inlineStr"/>
-      <c r="W286" t="inlineStr"/>
       <c r="X286" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -17267,13 +17139,11 @@
           <t>Cognitive neuroscientist and author of Never Go With Your Gut — helps leaders avoid cognitive biases</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr"/>
       <c r="F287" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="G287" t="inlineStr"/>
       <c r="H287" t="inlineStr">
         <is>
           <t>dr_gleb_tsipursky</t>
@@ -17289,13 +17159,11 @@
           <t>Official website</t>
         </is>
       </c>
-      <c r="K287" t="inlineStr"/>
       <c r="L287" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M287" t="inlineStr"/>
       <c r="N287" t="inlineStr">
         <is>
           <t>gleb_tsipursky</t>
@@ -17311,27 +17179,21 @@
           <t>Official website</t>
         </is>
       </c>
-      <c r="Q287" t="inlineStr"/>
       <c r="R287" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S287" t="inlineStr"/>
-      <c r="T287" t="inlineStr"/>
       <c r="U287" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="V287" t="inlineStr"/>
-      <c r="W287" t="inlineStr"/>
       <c r="X287" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -17354,34 +17216,26 @@
           <t>Host of UK's #1 marketing podcast on behavioral science — breaks down the psychology behind decisions</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr"/>
       <c r="F288" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G288" t="inlineStr"/>
-      <c r="H288" t="inlineStr"/>
       <c r="I288" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
-      <c r="K288" t="inlineStr"/>
       <c r="L288" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M288" t="inlineStr"/>
-      <c r="N288" t="inlineStr"/>
       <c r="O288" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P288" t="inlineStr"/>
       <c r="Q288" t="inlineStr">
         <is>
           <t>nudgepod</t>
@@ -17397,20 +17251,16 @@
           <t>Nudge podcast website</t>
         </is>
       </c>
-      <c r="T288" t="inlineStr"/>
       <c r="U288" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V288" t="inlineStr"/>
-      <c r="W288" t="inlineStr"/>
       <c r="X288" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -17433,55 +17283,41 @@
           <t>Past president of the Society for Judgment and Decision Making — pioneer of risk communication and hindsight bias research</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G289" t="inlineStr"/>
-      <c r="H289" t="inlineStr"/>
       <c r="I289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J289" t="inlineStr"/>
-      <c r="K289" t="inlineStr"/>
       <c r="L289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M289" t="inlineStr"/>
-      <c r="N289" t="inlineStr"/>
       <c r="O289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P289" t="inlineStr"/>
-      <c r="Q289" t="inlineStr"/>
       <c r="R289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S289" t="inlineStr"/>
-      <c r="T289" t="inlineStr"/>
       <c r="U289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V289" t="inlineStr"/>
-      <c r="W289" t="inlineStr"/>
       <c r="X289" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -17504,27 +17340,21 @@
           <t>2017 Nobel Prize winner in Economics — co-author of Nudge and author of Misbehaving</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr"/>
       <c r="F290" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr"/>
-      <c r="H290" t="inlineStr"/>
       <c r="I290" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J290" t="inlineStr"/>
-      <c r="K290" t="inlineStr"/>
       <c r="L290" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M290" t="inlineStr"/>
       <c r="N290" t="inlineStr">
         <is>
           <t>R_Thaler</t>
@@ -17540,27 +17370,21 @@
           <t>X profile 200K followers</t>
         </is>
       </c>
-      <c r="Q290" t="inlineStr"/>
       <c r="R290" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S290" t="inlineStr"/>
-      <c r="T290" t="inlineStr"/>
       <c r="U290" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V290" t="inlineStr"/>
-      <c r="W290" t="inlineStr"/>
       <c r="X290" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -17583,27 +17407,21 @@
           <t>Co-author of Nudge and founder of the Program on Behavioral Economics and Public Policy at Harvard</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr"/>
       <c r="F291" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G291" t="inlineStr"/>
-      <c r="H291" t="inlineStr"/>
       <c r="I291" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J291" t="inlineStr"/>
-      <c r="K291" t="inlineStr"/>
       <c r="L291" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M291" t="inlineStr"/>
       <c r="N291" t="inlineStr">
         <is>
           <t>CassSunstein</t>
@@ -17619,27 +17437,1492 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q291" t="inlineStr"/>
       <c r="R291" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S291" t="inlineStr"/>
-      <c r="T291" t="inlineStr"/>
       <c r="U291" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V291" t="inlineStr"/>
-      <c r="W291" t="inlineStr"/>
       <c r="X291" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Matt Abrahams</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Lecturer, Stanford GSB</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Stanford Graduate School of Business</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Host of Think Fast Talk Smart podcast; author of Think Faster Talk Smarter</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr"/>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>@mattabrahams</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Instagram search</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr"/>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr"/>
+      <c r="N292" t="inlineStr"/>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr"/>
+      <c r="Q292" t="inlineStr"/>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr"/>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>Think Fast Talk Smart</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V292" t="inlineStr">
+        <is>
+          <t>YouTube search</t>
+        </is>
+      </c>
+      <c r="W292" t="inlineStr"/>
+      <c r="X292" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Nancy Duarte</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Duarte Inc.</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Pioneer of presentation design; author of Resonate and Slide:ology</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>@duarteinc</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Instagram search (company)</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr"/>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr"/>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>@nancyduarte</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr"/>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr"/>
+      <c r="T293" t="inlineStr"/>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V293" t="inlineStr"/>
+      <c r="W293" t="inlineStr"/>
+      <c r="X293" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Carmine Gallo</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Author &amp; Harvard Instructor</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Gallo Communications Group</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Author of Talk Like TED; communication advisor to Google, Intel, LinkedIn</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>@carminegallospeaker</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr"/>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr"/>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>@CarmineGallo14</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>@carminegallospeaker</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>TikTok search</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr"/>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V294" t="inlineStr"/>
+      <c r="W294" t="inlineStr"/>
+      <c r="X294" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Vanessa Van Edwards</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Science of People</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Behavioral researcher; author of Captivate; body language and charisma expert</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>@vvanedwards</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>@vvanedwards</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>@vvanedwards</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Cross-platform consistency</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>@vvanedwards</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>@vvanedwards</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>TikTok profile</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>Science of People</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V295" t="inlineStr">
+        <is>
+          <t>YouTube search</t>
+        </is>
+      </c>
+      <c r="W295" t="inlineStr"/>
+      <c r="X295" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Vinh Giang</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Communication Coach &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>STAGE</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Former magician; 6M+ IG followers; communication teacher based in Australia</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr"/>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>@askvinh</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr"/>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr"/>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>@AskVinh</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>@askvinh</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>TikTok profile</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>Vinh Giang</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V296" t="inlineStr">
+        <is>
+          <t>YouTube search</t>
+        </is>
+      </c>
+      <c r="W296" t="inlineStr"/>
+      <c r="X296" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Dianna Booher</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Booher Research Institute</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Author of 50 books incl. Communicate Like a Leader; Hall of Fame speaker</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>DiannaBooher</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>@diannabooher</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr"/>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr"/>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>@DiannaBooher</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr"/>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr"/>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>DiannaBooher</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V297" t="inlineStr">
+        <is>
+          <t>YouTube search</t>
+        </is>
+      </c>
+      <c r="W297" t="inlineStr"/>
+      <c r="X297" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Alex Lyon</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Professor of Communication</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>SUNY Brockport</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Creator of 500K+ subscriber YouTube channel Communication Coach Alex Lyon</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr"/>
+      <c r="H298" t="inlineStr"/>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="inlineStr"/>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr"/>
+      <c r="N298" t="inlineStr"/>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr"/>
+      <c r="Q298" t="inlineStr"/>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr"/>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>Communication Coach Alex Lyon</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="W298" t="inlineStr"/>
+      <c r="X298" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Conor Neill</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Senior Lecturer</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>IESE Business School</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>21 years teaching leadership communication at IESE; 230K YouTube subs</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr"/>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>@cuchullainn</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr"/>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr"/>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>@conorneill</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr"/>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr"/>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>Conor Neill</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V299" t="inlineStr">
+        <is>
+          <t>YouTube channel 230K</t>
+        </is>
+      </c>
+      <c r="W299" t="inlineStr"/>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Joel Schwartzberg</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Author &amp; Communication Coach</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Self / Local Wisdom</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Author of Get to the Point! and The Language of Leadership</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>@thejoeltruth</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr"/>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr"/>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>@TheJoelTruth</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr"/>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr"/>
+      <c r="T300" t="inlineStr"/>
+      <c r="U300" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V300" t="inlineStr"/>
+      <c r="W300" t="inlineStr"/>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Melody Wilding</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Author &amp; Executive Coach</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Author of Managing Up; Forbes and HBR contributor; coaches at Google, JP Morgan</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>@melodywilding</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr"/>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr"/>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>@MelodyWilding</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr"/>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr"/>
+      <c r="T301" t="inlineStr"/>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V301" t="inlineStr"/>
+      <c r="W301" t="inlineStr"/>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Laura Camacho</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Executive Communication Coach</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Speak Up with Laura</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Host of Speak Up podcast (#3 worldwide for communication); PhD</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr"/>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>@speakupwithlaura</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr"/>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr"/>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>@lauramcamacho</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr"/>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr"/>
+      <c r="T302" t="inlineStr"/>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V302" t="inlineStr"/>
+      <c r="W302" t="inlineStr"/>
+      <c r="X302" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Briar Goldberg</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Director of Speaker Coaching</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>TED</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Coached hundreds of TED speakers plus CEOs of Facebook, Ford, Levi's</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr"/>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr"/>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="inlineStr"/>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr"/>
+      <c r="N303" t="inlineStr"/>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr"/>
+      <c r="Q303" t="inlineStr"/>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S303" t="inlineStr"/>
+      <c r="T303" t="inlineStr"/>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V303" t="inlineStr"/>
+      <c r="W303" t="inlineStr"/>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Lucille Ossai</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Rethinking Business Communications</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Ranked #7 globally by Global Gurus; only African in top 30 communication</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr"/>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="inlineStr"/>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr"/>
+      <c r="N304" t="inlineStr"/>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr"/>
+      <c r="Q304" t="inlineStr"/>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S304" t="inlineStr"/>
+      <c r="T304" t="inlineStr"/>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V304" t="inlineStr"/>
+      <c r="W304" t="inlineStr"/>
+      <c r="X304" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Krister Ungerböck</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Author &amp; Leadership Language Expert</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Author of 22 Talk SHIFTs; former CEO who grew company 3000%</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr"/>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr"/>
+      <c r="K305" t="inlineStr"/>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr"/>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>@meetkrister</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>Twitter/X profile</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr"/>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S305" t="inlineStr"/>
+      <c r="T305" t="inlineStr"/>
+      <c r="U305" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V305" t="inlineStr"/>
+      <c r="W305" t="inlineStr"/>
+      <c r="X305" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Roberta Ndlela</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Communication Coach &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Host of Speaking and Communicating Podcast; South African; cross-cultural leadership</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr"/>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr"/>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>@coachandspeaker</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Instagram search</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr"/>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr"/>
+      <c r="N306" t="inlineStr"/>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr"/>
+      <c r="Q306" t="inlineStr"/>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S306" t="inlineStr"/>
+      <c r="T306" t="inlineStr"/>
+      <c r="U306" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V306" t="inlineStr"/>
+      <c r="W306" t="inlineStr"/>
+      <c r="X306" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Linjuan Rita Men</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>University of Florida</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Leading researcher on leadership communication and internal comms</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr"/>
+      <c r="H307" t="inlineStr"/>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="inlineStr"/>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr"/>
+      <c r="N307" t="inlineStr"/>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr"/>
+      <c r="Q307" t="inlineStr"/>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S307" t="inlineStr"/>
+      <c r="T307" t="inlineStr"/>
+      <c r="U307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V307" t="inlineStr"/>
+      <c r="W307" t="inlineStr"/>
+      <c r="X307" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Julien C. Mirivel</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Professor of Applied Communication</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>University of Arkansas at Little Rock</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Author of The Art of Positive Communication</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr"/>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr"/>
+      <c r="K308" t="inlineStr"/>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr"/>
+      <c r="N308" t="inlineStr"/>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr"/>
+      <c r="Q308" t="inlineStr"/>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S308" t="inlineStr"/>
+      <c r="T308" t="inlineStr"/>
+      <c r="U308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V308" t="inlineStr"/>
+      <c r="W308" t="inlineStr"/>
+      <c r="X308" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y308" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -17653,7 +18936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -18041,6 +19324,26 @@
       <c r="D19" t="inlineStr">
         <is>
           <t>decision-making</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>17</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>leadership-communication</t>
         </is>
       </c>
     </row>
@@ -18056,7 +19359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -23338,6 +24641,302 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>69c3a09db89dd76ae2ad1773</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>2026-04-01T06:02:00Z</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>69c3a09fff77135659b694e4</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>2026-04-01T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>69c3a0a1b89dd76ae2ad17cd</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>2026-03-31T21:15:00Z</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>69c3a0b5ff77135659b69591</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>2026-04-01T05:01:00Z</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>69c3a0c6b89dd76ae2ad1894</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>2026-04-12T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>69c3a0c7b89dd76ae2ad18ba</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>2026-04-12T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>69c3a0b6b89dd76ae2ad182a</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>2026-04-01T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Leadership Communication</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>69c3a0b7ff77135659b695c3</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>2026-04-01T03:02:00Z</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Burnout Prevention
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -953,10 +953,14 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1111,7 +1115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y308"/>
+  <dimension ref="A1:Y325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17474,13 +17478,11 @@
           <t>Host of Think Fast Talk Smart podcast; author of Think Faster Talk Smarter</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr"/>
       <c r="F292" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G292" t="inlineStr"/>
       <c r="H292" t="inlineStr">
         <is>
           <t>@mattabrahams</t>
@@ -17496,27 +17498,21 @@
           <t>Instagram search</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr"/>
       <c r="L292" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M292" t="inlineStr"/>
-      <c r="N292" t="inlineStr"/>
       <c r="O292" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P292" t="inlineStr"/>
-      <c r="Q292" t="inlineStr"/>
       <c r="R292" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S292" t="inlineStr"/>
       <c r="T292" t="inlineStr">
         <is>
           <t>Think Fast Talk Smart</t>
@@ -17532,13 +17528,11 @@
           <t>YouTube search</t>
         </is>
       </c>
-      <c r="W292" t="inlineStr"/>
       <c r="X292" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -17561,13 +17555,11 @@
           <t>Pioneer of presentation design; author of Resonate and Slide:ology</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr"/>
       <c r="F293" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G293" t="inlineStr"/>
       <c r="H293" t="inlineStr">
         <is>
           <t>@duarteinc</t>
@@ -17583,13 +17575,11 @@
           <t>Instagram search (company)</t>
         </is>
       </c>
-      <c r="K293" t="inlineStr"/>
       <c r="L293" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M293" t="inlineStr"/>
       <c r="N293" t="inlineStr">
         <is>
           <t>@nancyduarte</t>
@@ -17605,27 +17595,21 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q293" t="inlineStr"/>
       <c r="R293" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S293" t="inlineStr"/>
-      <c r="T293" t="inlineStr"/>
       <c r="U293" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V293" t="inlineStr"/>
-      <c r="W293" t="inlineStr"/>
       <c r="X293" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -17648,13 +17632,11 @@
           <t>Author of Talk Like TED; communication advisor to Google, Intel, LinkedIn</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr"/>
       <c r="F294" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G294" t="inlineStr"/>
       <c r="H294" t="inlineStr">
         <is>
           <t>@carminegallospeaker</t>
@@ -17670,13 +17652,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K294" t="inlineStr"/>
       <c r="L294" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M294" t="inlineStr"/>
       <c r="N294" t="inlineStr">
         <is>
           <t>@CarmineGallo14</t>
@@ -17707,20 +17687,16 @@
           <t>TikTok search</t>
         </is>
       </c>
-      <c r="T294" t="inlineStr"/>
       <c r="U294" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V294" t="inlineStr"/>
-      <c r="W294" t="inlineStr"/>
       <c r="X294" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -17833,13 +17809,11 @@
           <t>YouTube search</t>
         </is>
       </c>
-      <c r="W295" t="inlineStr"/>
       <c r="X295" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -17862,13 +17836,11 @@
           <t>Former magician; 6M+ IG followers; communication teacher based in Australia</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr"/>
       <c r="F296" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G296" t="inlineStr"/>
       <c r="H296" t="inlineStr">
         <is>
           <t>@askvinh</t>
@@ -17884,13 +17856,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K296" t="inlineStr"/>
       <c r="L296" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M296" t="inlineStr"/>
       <c r="N296" t="inlineStr">
         <is>
           <t>@AskVinh</t>
@@ -17936,13 +17906,11 @@
           <t>YouTube search</t>
         </is>
       </c>
-      <c r="W296" t="inlineStr"/>
       <c r="X296" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -17995,13 +17963,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K297" t="inlineStr"/>
       <c r="L297" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M297" t="inlineStr"/>
       <c r="N297" t="inlineStr">
         <is>
           <t>@DiannaBooher</t>
@@ -18017,13 +17983,11 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q297" t="inlineStr"/>
       <c r="R297" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S297" t="inlineStr"/>
       <c r="T297" t="inlineStr">
         <is>
           <t>DiannaBooher</t>
@@ -18039,13 +18003,11 @@
           <t>YouTube search</t>
         </is>
       </c>
-      <c r="W297" t="inlineStr"/>
       <c r="X297" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -18068,41 +18030,31 @@
           <t>Creator of 500K+ subscriber YouTube channel Communication Coach Alex Lyon</t>
         </is>
       </c>
-      <c r="E298" t="inlineStr"/>
       <c r="F298" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G298" t="inlineStr"/>
-      <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J298" t="inlineStr"/>
-      <c r="K298" t="inlineStr"/>
       <c r="L298" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M298" t="inlineStr"/>
-      <c r="N298" t="inlineStr"/>
       <c r="O298" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P298" t="inlineStr"/>
-      <c r="Q298" t="inlineStr"/>
       <c r="R298" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S298" t="inlineStr"/>
       <c r="T298" t="inlineStr">
         <is>
           <t>Communication Coach Alex Lyon</t>
@@ -18118,13 +18070,11 @@
           <t>YouTube channel</t>
         </is>
       </c>
-      <c r="W298" t="inlineStr"/>
       <c r="X298" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -18147,13 +18097,11 @@
           <t>21 years teaching leadership communication at IESE; 230K YouTube subs</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr"/>
       <c r="F299" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G299" t="inlineStr"/>
       <c r="H299" t="inlineStr">
         <is>
           <t>@cuchullainn</t>
@@ -18169,13 +18117,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K299" t="inlineStr"/>
       <c r="L299" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M299" t="inlineStr"/>
       <c r="N299" t="inlineStr">
         <is>
           <t>@conorneill</t>
@@ -18191,13 +18137,11 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q299" t="inlineStr"/>
       <c r="R299" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S299" t="inlineStr"/>
       <c r="T299" t="inlineStr">
         <is>
           <t>Conor Neill</t>
@@ -18213,13 +18157,11 @@
           <t>YouTube channel 230K</t>
         </is>
       </c>
-      <c r="W299" t="inlineStr"/>
       <c r="X299" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -18242,13 +18184,11 @@
           <t>Author of Get to the Point! and The Language of Leadership</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr"/>
       <c r="F300" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G300" t="inlineStr"/>
       <c r="H300" t="inlineStr">
         <is>
           <t>@thejoeltruth</t>
@@ -18264,13 +18204,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K300" t="inlineStr"/>
       <c r="L300" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M300" t="inlineStr"/>
       <c r="N300" t="inlineStr">
         <is>
           <t>@TheJoelTruth</t>
@@ -18286,27 +18224,21 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q300" t="inlineStr"/>
       <c r="R300" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S300" t="inlineStr"/>
-      <c r="T300" t="inlineStr"/>
       <c r="U300" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V300" t="inlineStr"/>
-      <c r="W300" t="inlineStr"/>
       <c r="X300" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -18329,13 +18261,11 @@
           <t>Author of Managing Up; Forbes and HBR contributor; coaches at Google, JP Morgan</t>
         </is>
       </c>
-      <c r="E301" t="inlineStr"/>
       <c r="F301" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G301" t="inlineStr"/>
       <c r="H301" t="inlineStr">
         <is>
           <t>@melodywilding</t>
@@ -18351,13 +18281,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K301" t="inlineStr"/>
       <c r="L301" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M301" t="inlineStr"/>
       <c r="N301" t="inlineStr">
         <is>
           <t>@MelodyWilding</t>
@@ -18373,27 +18301,21 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q301" t="inlineStr"/>
       <c r="R301" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S301" t="inlineStr"/>
-      <c r="T301" t="inlineStr"/>
       <c r="U301" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V301" t="inlineStr"/>
-      <c r="W301" t="inlineStr"/>
       <c r="X301" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -18416,13 +18338,11 @@
           <t>Host of Speak Up podcast (#3 worldwide for communication); PhD</t>
         </is>
       </c>
-      <c r="E302" t="inlineStr"/>
       <c r="F302" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G302" t="inlineStr"/>
       <c r="H302" t="inlineStr">
         <is>
           <t>@speakupwithlaura</t>
@@ -18438,13 +18358,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K302" t="inlineStr"/>
       <c r="L302" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M302" t="inlineStr"/>
       <c r="N302" t="inlineStr">
         <is>
           <t>@lauramcamacho</t>
@@ -18460,27 +18378,21 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q302" t="inlineStr"/>
       <c r="R302" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S302" t="inlineStr"/>
-      <c r="T302" t="inlineStr"/>
       <c r="U302" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V302" t="inlineStr"/>
-      <c r="W302" t="inlineStr"/>
       <c r="X302" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -18503,55 +18415,41 @@
           <t>Coached hundreds of TED speakers plus CEOs of Facebook, Ford, Levi's</t>
         </is>
       </c>
-      <c r="E303" t="inlineStr"/>
       <c r="F303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G303" t="inlineStr"/>
-      <c r="H303" t="inlineStr"/>
       <c r="I303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J303" t="inlineStr"/>
-      <c r="K303" t="inlineStr"/>
       <c r="L303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M303" t="inlineStr"/>
-      <c r="N303" t="inlineStr"/>
       <c r="O303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P303" t="inlineStr"/>
-      <c r="Q303" t="inlineStr"/>
       <c r="R303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S303" t="inlineStr"/>
-      <c r="T303" t="inlineStr"/>
       <c r="U303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V303" t="inlineStr"/>
-      <c r="W303" t="inlineStr"/>
       <c r="X303" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -18574,55 +18472,41 @@
           <t>Ranked #7 globally by Global Gurus; only African in top 30 communication</t>
         </is>
       </c>
-      <c r="E304" t="inlineStr"/>
       <c r="F304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G304" t="inlineStr"/>
-      <c r="H304" t="inlineStr"/>
       <c r="I304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J304" t="inlineStr"/>
-      <c r="K304" t="inlineStr"/>
       <c r="L304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M304" t="inlineStr"/>
-      <c r="N304" t="inlineStr"/>
       <c r="O304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P304" t="inlineStr"/>
-      <c r="Q304" t="inlineStr"/>
       <c r="R304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S304" t="inlineStr"/>
-      <c r="T304" t="inlineStr"/>
       <c r="U304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V304" t="inlineStr"/>
-      <c r="W304" t="inlineStr"/>
       <c r="X304" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -18645,27 +18529,21 @@
           <t>Author of 22 Talk SHIFTs; former CEO who grew company 3000%</t>
         </is>
       </c>
-      <c r="E305" t="inlineStr"/>
       <c r="F305" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G305" t="inlineStr"/>
-      <c r="H305" t="inlineStr"/>
       <c r="I305" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J305" t="inlineStr"/>
-      <c r="K305" t="inlineStr"/>
       <c r="L305" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M305" t="inlineStr"/>
       <c r="N305" t="inlineStr">
         <is>
           <t>@meetkrister</t>
@@ -18681,27 +18559,21 @@
           <t>Twitter/X profile</t>
         </is>
       </c>
-      <c r="Q305" t="inlineStr"/>
       <c r="R305" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S305" t="inlineStr"/>
-      <c r="T305" t="inlineStr"/>
       <c r="U305" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V305" t="inlineStr"/>
-      <c r="W305" t="inlineStr"/>
       <c r="X305" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -18724,13 +18596,11 @@
           <t>Host of Speaking and Communicating Podcast; South African; cross-cultural leadership</t>
         </is>
       </c>
-      <c r="E306" t="inlineStr"/>
       <c r="F306" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G306" t="inlineStr"/>
       <c r="H306" t="inlineStr">
         <is>
           <t>@coachandspeaker</t>
@@ -18746,41 +18616,31 @@
           <t>Instagram search</t>
         </is>
       </c>
-      <c r="K306" t="inlineStr"/>
       <c r="L306" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M306" t="inlineStr"/>
-      <c r="N306" t="inlineStr"/>
       <c r="O306" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P306" t="inlineStr"/>
-      <c r="Q306" t="inlineStr"/>
       <c r="R306" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S306" t="inlineStr"/>
-      <c r="T306" t="inlineStr"/>
       <c r="U306" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V306" t="inlineStr"/>
-      <c r="W306" t="inlineStr"/>
       <c r="X306" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -18803,55 +18663,41 @@
           <t>Leading researcher on leadership communication and internal comms</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr"/>
       <c r="F307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G307" t="inlineStr"/>
-      <c r="H307" t="inlineStr"/>
       <c r="I307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J307" t="inlineStr"/>
-      <c r="K307" t="inlineStr"/>
       <c r="L307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M307" t="inlineStr"/>
-      <c r="N307" t="inlineStr"/>
       <c r="O307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P307" t="inlineStr"/>
-      <c r="Q307" t="inlineStr"/>
       <c r="R307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S307" t="inlineStr"/>
-      <c r="T307" t="inlineStr"/>
       <c r="U307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V307" t="inlineStr"/>
-      <c r="W307" t="inlineStr"/>
       <c r="X307" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -18874,55 +18720,1320 @@
           <t>Author of The Art of Positive Communication</t>
         </is>
       </c>
-      <c r="E308" t="inlineStr"/>
       <c r="F308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr"/>
-      <c r="H308" t="inlineStr"/>
       <c r="I308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr"/>
-      <c r="K308" t="inlineStr"/>
       <c r="L308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M308" t="inlineStr"/>
-      <c r="N308" t="inlineStr"/>
       <c r="O308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P308" t="inlineStr"/>
-      <c r="Q308" t="inlineStr"/>
       <c r="R308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S308" t="inlineStr"/>
-      <c r="T308" t="inlineStr"/>
       <c r="U308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V308" t="inlineStr"/>
-      <c r="W308" t="inlineStr"/>
       <c r="X308" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Christina Maslach</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Professor Emerita of Psychology</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>UC Berkeley</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Creator of Maslach Burnout Inventory, the world's most widely used burnout measurement tool</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>@CMaslach</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>x.com profile</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U309" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X309" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Emily Nagoski</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Author &amp; Health Educator</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Co-author of Burnout: The Secret to Unlocking the Stress Cycle</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>emilynagoskiphd</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>@enagoski</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>@enagoski</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>inferred from IG</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>@emilynagoski</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S310" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="U310" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X310" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Jennifer Moss</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Author &amp; Workplace Expert</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Work Better Institute</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Author of The Burnout Epidemic (HBR Press), 2026 Golden Gavel Honoree</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>@jleighmoss</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>@jleighmoss</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>inferred from IG</t>
+        </is>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U311" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X311" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Paula Davis</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Stress &amp; Resilience Institute</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Author of Beating Burnout at Work and Lead Well</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>@pauladavisSRI</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>x.com profile</t>
+        </is>
+      </c>
+      <c r="R312" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U312" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X312" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Cait Donovan</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Host &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>FRIED Podcast / BurnBOLD</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Host of top 1% global burnout podcast FRIED with 300+ episodes</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>@caitdonovanspeaks</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>@caitdonovanspeaks</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>inferred from IG</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U313" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X313" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Michael Leiter</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Professor of Organisational Psychology</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Deakin University</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Co-author of The Burnout Challenge with Maslach, coined 'work engagement'</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X314" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Dr. Jacinta Jiménez</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Psychologist &amp; Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Independent (ex-BetterUp)</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Author of award-winning The Burnout Fix, former Global Head of Coaching at BetterUp</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X315" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Dr. Susan Biali Haas</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Medical Doctor &amp; Resilience Expert</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Author of The Resilient Life, Psychology Today blogger with 11M+ views</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>DrSusanBiali</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>@drsusanbiali</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>@drsusanbiali</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>inferred from IG</t>
+        </is>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R316" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U316" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X316" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Jonathan Malesic</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Author &amp; Journalist</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Author of The End of Burnout, named best book of 2022 by Amazon</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>@jonmalesic</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>@JonMalesic</t>
+        </is>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>x.com profile</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U317" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X317" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Rachel Montañez</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Burnout &amp; Career Expert</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Rachel Montanez LLC</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Forbes burnout columnist with 2M+ global readers, HBR author</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N318" t="inlineStr">
+        <is>
+          <t>@RachelSMontanez</t>
+        </is>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>x.com profile</t>
+        </is>
+      </c>
+      <c r="R318" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U318" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X318" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Nina Nesdoly</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Neuroscience-Based Burnout Speaker</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Canadian keynote speaker, TEDx Editor's Pick, pursuing PhD in work-related stress</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>@ninanesdoly</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>@ninanesdoly</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>inferred from IG</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>@ninanesdoly</t>
+        </is>
+      </c>
+      <c r="R319" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>website bio</t>
+        </is>
+      </c>
+      <c r="U319" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X319" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Leanne Spencer</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Bodyshot Performance</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>UK-based author of Cadence, creator of Six Signals methodology</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R320" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U320" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X320" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Kelley Bonner</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Licensed Therapist &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Black Girl Burnout</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Host of Black Girl Burnout podcast with 120K+ downloads</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>blackgirlburnout</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>kelleybonner.com</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>@blackgirlburnout</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>kelleybonner.com</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>@blkgirlburnout</t>
+        </is>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>kelleybonner.com</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>@blackgirlburnout</t>
+        </is>
+      </c>
+      <c r="R321" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S321" t="inlineStr">
+        <is>
+          <t>kelleybonner.com</t>
+        </is>
+      </c>
+      <c r="T321" t="inlineStr">
+        <is>
+          <t>@blackgirlburnout</t>
+        </is>
+      </c>
+      <c r="U321" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V321" t="inlineStr">
+        <is>
+          <t>kelleybonner.com</t>
+        </is>
+      </c>
+      <c r="X321" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Sarai Marie</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Content Creator</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Independent (@saraisthreads)</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>TikTok creator with 3M+ followers, corporate burnout humor</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>@saraisthreads</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S322" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="U322" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X322" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Siobhán Murray</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Psychotherapist &amp; Author</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Twisting the Jar</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Irish author of The Burnout Solution, works with Google, PayPal, HubSpot</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>@twistingthejar</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>@twistingthejar</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>inferred from IG</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R323" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U323" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X323" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Dex Randall</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Executive Burnout Coach &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Host of Burnout Recovery podcast with 244 episodes</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>coachdexrandall</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>linktree</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N324" t="inlineStr">
+        <is>
+          <t>@coachdexrandall</t>
+        </is>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P324" t="inlineStr">
+        <is>
+          <t>x.com profile</t>
+        </is>
+      </c>
+      <c r="R324" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U324" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X324" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Jani Konjedic</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Burnout Awareness Advocate</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Conquering Burnout (Substack)</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Slovenian, former pro volleyball player, burnout newsletter creator</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="X325" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -18936,7 +20047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -19344,6 +20455,26 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>leadership-communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>17</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>burnout-prevention</t>
         </is>
       </c>
     </row>
@@ -19359,7 +20490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -24937,6 +26068,302 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>69c3a7efecfc8d3950f4765d</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>2026-04-01T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>69c3a805dc7f763f71a451ca</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>2026-04-01T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>69c3a817dc7f763f71a45219</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>2026-04-20T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>69c3a832ecfc8d3950f47786</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>2026-04-01T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>69c3a83becfc8d3950f477bc</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>2026-04-01T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>69c3a846ecfc8d3950f47811</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>2026-04-20T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>69c3a851dc7f763f71a4531c</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2026-04-01T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Burnout Prevention</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>69c3a85adc7f763f71a45342</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>2026-04-01T13:02:00Z</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update data/handle-database.xlsx — First-Time Managers
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -974,10 +974,14 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1115,7 +1119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y325"/>
+  <dimension ref="A1:Y342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20035,6 +20039,1485 @@
         </is>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Linda Hill</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Author of 'Becoming a Manager' — definitive study on new manager transitions</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr"/>
+      <c r="H326" t="inlineStr"/>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr"/>
+      <c r="K326" t="inlineStr"/>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr"/>
+      <c r="N326" t="inlineStr">
+        <is>
+          <t>@Linda_A_Hill</t>
+        </is>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P326" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q326" t="inlineStr"/>
+      <c r="R326" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S326" t="inlineStr"/>
+      <c r="T326" t="inlineStr"/>
+      <c r="U326" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V326" t="inlineStr"/>
+      <c r="W326" t="inlineStr"/>
+      <c r="X326" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Lia Garvin</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Founder, Team Whisperer</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Team Whisperer</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>3x bestselling author of 'The New Manager Playbook', TEDx speaker, ex-Google/Microsoft/Apple</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr"/>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr"/>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>@lia.garvin</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr"/>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr"/>
+      <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P327" t="inlineStr"/>
+      <c r="Q327" t="inlineStr"/>
+      <c r="R327" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S327" t="inlineStr"/>
+      <c r="T327" t="inlineStr"/>
+      <c r="U327" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V327" t="inlineStr"/>
+      <c r="W327" t="inlineStr"/>
+      <c r="X327" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Ramona Shaw</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Leadership Accelerator</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Host of The Manager Track podcast, author of 'The Confident &amp; Competent New Manager'</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>ramona.live.lead.succeed</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>@ramona.shaw.leadership</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr"/>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr"/>
+      <c r="N328" t="inlineStr">
+        <is>
+          <t>@shaw_lead</t>
+        </is>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P328" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q328" t="inlineStr"/>
+      <c r="R328" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S328" t="inlineStr"/>
+      <c r="T328" t="inlineStr"/>
+      <c r="U328" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V328" t="inlineStr"/>
+      <c r="W328" t="inlineStr"/>
+      <c r="X328" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Lara Hogan</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Wherewithall</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Author of 'Resilient Management', former VP Engineering at Kickstarter</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>@_wherewithall_</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>Business IG</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr"/>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr"/>
+      <c r="N329" t="inlineStr">
+        <is>
+          <t>@lara_hogan</t>
+        </is>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P329" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q329" t="inlineStr"/>
+      <c r="R329" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S329" t="inlineStr"/>
+      <c r="T329" t="inlineStr"/>
+      <c r="U329" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V329" t="inlineStr"/>
+      <c r="W329" t="inlineStr"/>
+      <c r="X329" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Camille Fournier</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Author &amp; Former CTO</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Rent the Runway (former)</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Wrote 'The Manager's Path' — go-to guide for IC-to-manager transitions in tech</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr"/>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr"/>
+      <c r="K330" t="inlineStr"/>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr"/>
+      <c r="N330" t="inlineStr">
+        <is>
+          <t>@skamille</t>
+        </is>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q330" t="inlineStr"/>
+      <c r="R330" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S330" t="inlineStr"/>
+      <c r="T330" t="inlineStr"/>
+      <c r="U330" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V330" t="inlineStr"/>
+      <c r="W330" t="inlineStr">
+        <is>
+          <t>@skamille.themanagerswrath.com</t>
+        </is>
+      </c>
+      <c r="X330" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y330" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Scott Jeffrey Miller</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Senior Advisor</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>FranklinCovey</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Co-author of WSJ bestseller 'Everyone Deserves a Great Manager', 7x bestselling author</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>@scottmillerj1</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>@scottjeffreymiller</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr"/>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr"/>
+      <c r="N331" t="inlineStr"/>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P331" t="inlineStr"/>
+      <c r="Q331" t="inlineStr">
+        <is>
+          <t>@scottjeffreymiller</t>
+        </is>
+      </c>
+      <c r="R331" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S331" t="inlineStr">
+        <is>
+          <t>LinkedIn post</t>
+        </is>
+      </c>
+      <c r="T331" t="inlineStr">
+        <is>
+          <t>@scottjeffreymiller</t>
+        </is>
+      </c>
+      <c r="U331" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V331" t="inlineStr">
+        <is>
+          <t>LinkedIn post</t>
+        </is>
+      </c>
+      <c r="W331" t="inlineStr"/>
+      <c r="X331" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Jim McCormick</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Author &amp; Executive Coach</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Research Institute for Risk Intelligence</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Author of 'The First-Time Manager' — 500K+ copies sold across seven editions</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr"/>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr"/>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr"/>
+      <c r="K332" t="inlineStr"/>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr"/>
+      <c r="N332" t="inlineStr"/>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P332" t="inlineStr"/>
+      <c r="Q332" t="inlineStr"/>
+      <c r="R332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S332" t="inlineStr"/>
+      <c r="T332" t="inlineStr"/>
+      <c r="U332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V332" t="inlineStr"/>
+      <c r="W332" t="inlineStr"/>
+      <c r="X332" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Mamie Kanfer Stewart</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Host, The Modern Manager</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Meeteor</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Founder of Meeteor, author of 'Momentum', practical management podcast host</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr"/>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>@leadershipwithmamie</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Website link</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr"/>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr"/>
+      <c r="N333" t="inlineStr">
+        <is>
+          <t>@mamieks</t>
+        </is>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q333" t="inlineStr"/>
+      <c r="R333" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S333" t="inlineStr"/>
+      <c r="T333" t="inlineStr"/>
+      <c r="U333" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V333" t="inlineStr"/>
+      <c r="W333" t="inlineStr"/>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Dr. Tacy Byham</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>DDI</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Author of 'Your First Leadership Job', leads world's largest leadership assessment firm</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr"/>
+      <c r="H334" t="inlineStr"/>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr"/>
+      <c r="K334" t="inlineStr"/>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr"/>
+      <c r="N334" t="inlineStr">
+        <is>
+          <t>@TacyByham</t>
+        </is>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q334" t="inlineStr"/>
+      <c r="R334" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S334" t="inlineStr"/>
+      <c r="T334" t="inlineStr"/>
+      <c r="U334" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V334" t="inlineStr"/>
+      <c r="W334" t="inlineStr"/>
+      <c r="X334" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Molly Graham</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Glue Club</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Coined 'Give Away Your Legos' framework, former Ops at Facebook/Google/CZI</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr"/>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr"/>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr"/>
+      <c r="K335" t="inlineStr"/>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr"/>
+      <c r="N335" t="inlineStr">
+        <is>
+          <t>@molly_g</t>
+        </is>
+      </c>
+      <c r="O335" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P335" t="inlineStr">
+        <is>
+          <t>X profile (inactive)</t>
+        </is>
+      </c>
+      <c r="Q335" t="inlineStr"/>
+      <c r="R335" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S335" t="inlineStr"/>
+      <c r="T335" t="inlineStr"/>
+      <c r="U335" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V335" t="inlineStr"/>
+      <c r="W335" t="inlineStr"/>
+      <c r="X335" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>David Burkus</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Organizational Psychologist</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Author of 'Under New Management', TED speaker with 2M+ views</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr"/>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>@davidburkus</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr"/>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr"/>
+      <c r="N336" t="inlineStr">
+        <is>
+          <t>@davidburkus</t>
+        </is>
+      </c>
+      <c r="O336" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P336" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q336" t="inlineStr">
+        <is>
+          <t>@davidburkus</t>
+        </is>
+      </c>
+      <c r="R336" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S336" t="inlineStr">
+        <is>
+          <t>TikTok profile</t>
+        </is>
+      </c>
+      <c r="T336" t="inlineStr">
+        <is>
+          <t>@davidburkus</t>
+        </is>
+      </c>
+      <c r="U336" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V336" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="W336" t="inlineStr"/>
+      <c r="X336" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Wanda Wallace</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Leadership Forum Inc.</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Author of 'You Can't Know It All', former Associate Dean at Duke</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>WallaceOutoftheComfortZone</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>@wandatwallace</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr"/>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr"/>
+      <c r="N337" t="inlineStr">
+        <is>
+          <t>@askWanda</t>
+        </is>
+      </c>
+      <c r="O337" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P337" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q337" t="inlineStr"/>
+      <c r="R337" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S337" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="T337" t="inlineStr"/>
+      <c r="U337" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V337" t="inlineStr"/>
+      <c r="W337" t="inlineStr"/>
+      <c r="X337" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Mary Abbajay</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Careerstone Group</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Author of bestselling 'Managing Up', host of Cubicle Confidential podcast</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr"/>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr"/>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>@maryabbajay</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>Linktree</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr"/>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr"/>
+      <c r="N338" t="inlineStr">
+        <is>
+          <t>@maryabbajay</t>
+        </is>
+      </c>
+      <c r="O338" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P338" t="inlineStr">
+        <is>
+          <t>Linktree</t>
+        </is>
+      </c>
+      <c r="Q338" t="inlineStr"/>
+      <c r="R338" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S338" t="inlineStr"/>
+      <c r="T338" t="inlineStr">
+        <is>
+          <t>@maryabbajay</t>
+        </is>
+      </c>
+      <c r="U338" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V338" t="inlineStr">
+        <is>
+          <t>Linktree</t>
+        </is>
+      </c>
+      <c r="W338" t="inlineStr"/>
+      <c r="X338" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Jen Dary</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Plucky</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Creator of 'So Now You're a Manager' workshop, coached at 200+ companies</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr"/>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr"/>
+      <c r="K339" t="inlineStr"/>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr"/>
+      <c r="N339" t="inlineStr">
+        <is>
+          <t>@jenniferdary</t>
+        </is>
+      </c>
+      <c r="O339" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P339" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q339" t="inlineStr"/>
+      <c r="R339" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S339" t="inlineStr"/>
+      <c r="T339" t="inlineStr"/>
+      <c r="U339" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V339" t="inlineStr"/>
+      <c r="W339" t="inlineStr"/>
+      <c r="X339" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Kim Nicol</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Executive Mindfulness Coach</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Host of 'The New Manager Podcast', human-centered leadership since 2017</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr"/>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr"/>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr"/>
+      <c r="K340" t="inlineStr"/>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr"/>
+      <c r="N340" t="inlineStr"/>
+      <c r="O340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P340" t="inlineStr"/>
+      <c r="Q340" t="inlineStr"/>
+      <c r="R340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S340" t="inlineStr"/>
+      <c r="T340" t="inlineStr"/>
+      <c r="U340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V340" t="inlineStr"/>
+      <c r="W340" t="inlineStr"/>
+      <c r="X340" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Herminia Ibarra</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>London Business School</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Expert on leadership transitions, author of 'Act Like a Leader Think Like a Leader'</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr"/>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr"/>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr"/>
+      <c r="K341" t="inlineStr"/>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr"/>
+      <c r="N341" t="inlineStr">
+        <is>
+          <t>@HerminiaIbarra</t>
+        </is>
+      </c>
+      <c r="O341" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P341" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q341" t="inlineStr"/>
+      <c r="R341" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S341" t="inlineStr"/>
+      <c r="T341" t="inlineStr"/>
+      <c r="U341" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V341" t="inlineStr"/>
+      <c r="W341" t="inlineStr"/>
+      <c r="X341" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Mark Horstman</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Manager Tools</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Created world's #1 management podcast (1.4M+ monthly listeners), author of 'The Effective Manager'</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>@managertools</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Brand account</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>@managertools</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>Brand account</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr"/>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr"/>
+      <c r="N342" t="inlineStr">
+        <is>
+          <t>@managertools</t>
+        </is>
+      </c>
+      <c r="O342" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P342" t="inlineStr">
+        <is>
+          <t>Brand account</t>
+        </is>
+      </c>
+      <c r="Q342" t="inlineStr"/>
+      <c r="R342" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S342" t="inlineStr"/>
+      <c r="T342" t="inlineStr">
+        <is>
+          <t>@managertools</t>
+        </is>
+      </c>
+      <c r="U342" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V342" t="inlineStr">
+        <is>
+          <t>Brand account</t>
+        </is>
+      </c>
+      <c r="W342" t="inlineStr"/>
+      <c r="X342" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y342" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20047,7 +21530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -20475,6 +21958,26 @@
       <c r="D21" t="inlineStr">
         <is>
           <t>burnout-prevention</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>17</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>first-time-managers</t>
         </is>
       </c>
     </row>
@@ -20490,7 +21993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G161"/>
+  <dimension ref="A1:G169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -26364,6 +27867,302 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>69c3ac84ecfc8d3950f4a180</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>2026-04-02T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>69c3ac87dc7f763f71a47a64</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>2026-04-02T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>69c3aca6ecfc8d3950f4a23e</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>2026-04-01T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>69c3aca7dc7f763f71a47ad6</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>2026-04-01T23:01:00Z</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>69c3aca8dc7f763f71a47afc</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>2026-04-02T03:01:00Z</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>69c3aca9ecfc8d3950f4a264</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>2026-04-01T21:02:00Z</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>69c3acc0dc7f763f71a47b71</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>2026-04-21T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>First-Time Managers</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>69c3acb8dc7f763f71a47b4b</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>2026-04-21T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Feedback Culture
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -995,10 +995,14 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1119,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y342"/>
+  <dimension ref="A1:Y357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20060,27 +20064,21 @@
           <t>Author of 'Becoming a Manager' — definitive study on new manager transitions</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr"/>
       <c r="F326" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G326" t="inlineStr"/>
-      <c r="H326" t="inlineStr"/>
       <c r="I326" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J326" t="inlineStr"/>
-      <c r="K326" t="inlineStr"/>
       <c r="L326" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M326" t="inlineStr"/>
       <c r="N326" t="inlineStr">
         <is>
           <t>@Linda_A_Hill</t>
@@ -20096,27 +20094,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q326" t="inlineStr"/>
       <c r="R326" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S326" t="inlineStr"/>
-      <c r="T326" t="inlineStr"/>
       <c r="U326" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V326" t="inlineStr"/>
-      <c r="W326" t="inlineStr"/>
       <c r="X326" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -20139,13 +20131,11 @@
           <t>3x bestselling author of 'The New Manager Playbook', TEDx speaker, ex-Google/Microsoft/Apple</t>
         </is>
       </c>
-      <c r="E327" t="inlineStr"/>
       <c r="F327" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G327" t="inlineStr"/>
       <c r="H327" t="inlineStr">
         <is>
           <t>@lia.garvin</t>
@@ -20161,41 +20151,31 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K327" t="inlineStr"/>
       <c r="L327" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M327" t="inlineStr"/>
-      <c r="N327" t="inlineStr"/>
       <c r="O327" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P327" t="inlineStr"/>
-      <c r="Q327" t="inlineStr"/>
       <c r="R327" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S327" t="inlineStr"/>
-      <c r="T327" t="inlineStr"/>
       <c r="U327" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V327" t="inlineStr"/>
-      <c r="W327" t="inlineStr"/>
       <c r="X327" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -20248,13 +20228,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K328" t="inlineStr"/>
       <c r="L328" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M328" t="inlineStr"/>
       <c r="N328" t="inlineStr">
         <is>
           <t>@shaw_lead</t>
@@ -20270,27 +20248,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q328" t="inlineStr"/>
       <c r="R328" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S328" t="inlineStr"/>
-      <c r="T328" t="inlineStr"/>
       <c r="U328" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V328" t="inlineStr"/>
-      <c r="W328" t="inlineStr"/>
       <c r="X328" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -20313,13 +20285,11 @@
           <t>Author of 'Resilient Management', former VP Engineering at Kickstarter</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr"/>
       <c r="F329" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr">
         <is>
           <t>@_wherewithall_</t>
@@ -20335,13 +20305,11 @@
           <t>Business IG</t>
         </is>
       </c>
-      <c r="K329" t="inlineStr"/>
       <c r="L329" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M329" t="inlineStr"/>
       <c r="N329" t="inlineStr">
         <is>
           <t>@lara_hogan</t>
@@ -20357,27 +20325,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q329" t="inlineStr"/>
       <c r="R329" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S329" t="inlineStr"/>
-      <c r="T329" t="inlineStr"/>
       <c r="U329" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V329" t="inlineStr"/>
-      <c r="W329" t="inlineStr"/>
       <c r="X329" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -20400,27 +20362,21 @@
           <t>Wrote 'The Manager's Path' — go-to guide for IC-to-manager transitions in tech</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr"/>
       <c r="F330" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G330" t="inlineStr"/>
-      <c r="H330" t="inlineStr"/>
       <c r="I330" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" t="inlineStr"/>
       <c r="L330" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M330" t="inlineStr"/>
       <c r="N330" t="inlineStr">
         <is>
           <t>@skamille</t>
@@ -20436,20 +20392,16 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q330" t="inlineStr"/>
       <c r="R330" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S330" t="inlineStr"/>
-      <c r="T330" t="inlineStr"/>
       <c r="U330" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V330" t="inlineStr"/>
       <c r="W330" t="inlineStr">
         <is>
           <t>@skamille.themanagerswrath.com</t>
@@ -20517,20 +20469,16 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K331" t="inlineStr"/>
       <c r="L331" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M331" t="inlineStr"/>
-      <c r="N331" t="inlineStr"/>
       <c r="O331" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="P331" t="inlineStr"/>
       <c r="Q331" t="inlineStr">
         <is>
           <t>@scottjeffreymiller</t>
@@ -20561,13 +20509,11 @@
           <t>LinkedIn post</t>
         </is>
       </c>
-      <c r="W331" t="inlineStr"/>
       <c r="X331" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -20590,55 +20536,41 @@
           <t>Author of 'The First-Time Manager' — 500K+ copies sold across seven editions</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr"/>
       <c r="F332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G332" t="inlineStr"/>
-      <c r="H332" t="inlineStr"/>
       <c r="I332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J332" t="inlineStr"/>
-      <c r="K332" t="inlineStr"/>
       <c r="L332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M332" t="inlineStr"/>
-      <c r="N332" t="inlineStr"/>
       <c r="O332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P332" t="inlineStr"/>
-      <c r="Q332" t="inlineStr"/>
       <c r="R332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S332" t="inlineStr"/>
-      <c r="T332" t="inlineStr"/>
       <c r="U332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V332" t="inlineStr"/>
-      <c r="W332" t="inlineStr"/>
       <c r="X332" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -20661,7 +20593,6 @@
           <t>Founder of Meeteor, author of 'Momentum', practical management podcast host</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr"/>
       <c r="F333" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -20687,13 +20618,11 @@
           <t>Website link</t>
         </is>
       </c>
-      <c r="K333" t="inlineStr"/>
       <c r="L333" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M333" t="inlineStr"/>
       <c r="N333" t="inlineStr">
         <is>
           <t>@mamieks</t>
@@ -20709,27 +20638,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q333" t="inlineStr"/>
       <c r="R333" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S333" t="inlineStr"/>
-      <c r="T333" t="inlineStr"/>
       <c r="U333" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V333" t="inlineStr"/>
-      <c r="W333" t="inlineStr"/>
       <c r="X333" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -20752,27 +20675,21 @@
           <t>Author of 'Your First Leadership Job', leads world's largest leadership assessment firm</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr"/>
       <c r="F334" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G334" t="inlineStr"/>
-      <c r="H334" t="inlineStr"/>
       <c r="I334" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J334" t="inlineStr"/>
-      <c r="K334" t="inlineStr"/>
       <c r="L334" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M334" t="inlineStr"/>
       <c r="N334" t="inlineStr">
         <is>
           <t>@TacyByham</t>
@@ -20788,27 +20705,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q334" t="inlineStr"/>
       <c r="R334" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S334" t="inlineStr"/>
-      <c r="T334" t="inlineStr"/>
       <c r="U334" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V334" t="inlineStr"/>
-      <c r="W334" t="inlineStr"/>
       <c r="X334" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -20831,27 +20742,21 @@
           <t>Coined 'Give Away Your Legos' framework, former Ops at Facebook/Google/CZI</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G335" t="inlineStr"/>
-      <c r="H335" t="inlineStr"/>
       <c r="I335" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J335" t="inlineStr"/>
-      <c r="K335" t="inlineStr"/>
       <c r="L335" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M335" t="inlineStr"/>
       <c r="N335" t="inlineStr">
         <is>
           <t>@molly_g</t>
@@ -20867,27 +20772,21 @@
           <t>X profile (inactive)</t>
         </is>
       </c>
-      <c r="Q335" t="inlineStr"/>
       <c r="R335" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S335" t="inlineStr"/>
-      <c r="T335" t="inlineStr"/>
       <c r="U335" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V335" t="inlineStr"/>
-      <c r="W335" t="inlineStr"/>
       <c r="X335" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -20910,13 +20809,11 @@
           <t>Author of 'Under New Management', TED speaker with 2M+ views</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr"/>
       <c r="F336" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr">
         <is>
           <t>@davidburkus</t>
@@ -20932,13 +20829,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K336" t="inlineStr"/>
       <c r="L336" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M336" t="inlineStr"/>
       <c r="N336" t="inlineStr">
         <is>
           <t>@davidburkus</t>
@@ -20984,13 +20879,11 @@
           <t>YouTube channel</t>
         </is>
       </c>
-      <c r="W336" t="inlineStr"/>
       <c r="X336" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -21043,13 +20936,11 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="K337" t="inlineStr"/>
       <c r="L337" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M337" t="inlineStr"/>
       <c r="N337" t="inlineStr">
         <is>
           <t>@askWanda</t>
@@ -21065,7 +20956,6 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q337" t="inlineStr"/>
       <c r="R337" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -21076,20 +20966,16 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="T337" t="inlineStr"/>
       <c r="U337" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V337" t="inlineStr"/>
-      <c r="W337" t="inlineStr"/>
       <c r="X337" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -21112,13 +20998,11 @@
           <t>Author of bestselling 'Managing Up', host of Cubicle Confidential podcast</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G338" t="inlineStr"/>
       <c r="H338" t="inlineStr">
         <is>
           <t>@maryabbajay</t>
@@ -21134,13 +21018,11 @@
           <t>Linktree</t>
         </is>
       </c>
-      <c r="K338" t="inlineStr"/>
       <c r="L338" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M338" t="inlineStr"/>
       <c r="N338" t="inlineStr">
         <is>
           <t>@maryabbajay</t>
@@ -21156,13 +21038,11 @@
           <t>Linktree</t>
         </is>
       </c>
-      <c r="Q338" t="inlineStr"/>
       <c r="R338" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S338" t="inlineStr"/>
       <c r="T338" t="inlineStr">
         <is>
           <t>@maryabbajay</t>
@@ -21178,13 +21058,11 @@
           <t>Linktree</t>
         </is>
       </c>
-      <c r="W338" t="inlineStr"/>
       <c r="X338" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -21207,27 +21085,21 @@
           <t>Creator of 'So Now You're a Manager' workshop, coached at 200+ companies</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr"/>
       <c r="F339" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G339" t="inlineStr"/>
-      <c r="H339" t="inlineStr"/>
       <c r="I339" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J339" t="inlineStr"/>
-      <c r="K339" t="inlineStr"/>
       <c r="L339" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M339" t="inlineStr"/>
       <c r="N339" t="inlineStr">
         <is>
           <t>@jenniferdary</t>
@@ -21243,27 +21115,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q339" t="inlineStr"/>
       <c r="R339" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S339" t="inlineStr"/>
-      <c r="T339" t="inlineStr"/>
       <c r="U339" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V339" t="inlineStr"/>
-      <c r="W339" t="inlineStr"/>
       <c r="X339" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -21286,55 +21152,41 @@
           <t>Host of 'The New Manager Podcast', human-centered leadership since 2017</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr"/>
       <c r="F340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G340" t="inlineStr"/>
-      <c r="H340" t="inlineStr"/>
       <c r="I340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J340" t="inlineStr"/>
-      <c r="K340" t="inlineStr"/>
       <c r="L340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M340" t="inlineStr"/>
-      <c r="N340" t="inlineStr"/>
       <c r="O340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P340" t="inlineStr"/>
-      <c r="Q340" t="inlineStr"/>
       <c r="R340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S340" t="inlineStr"/>
-      <c r="T340" t="inlineStr"/>
       <c r="U340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V340" t="inlineStr"/>
-      <c r="W340" t="inlineStr"/>
       <c r="X340" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -21357,27 +21209,21 @@
           <t>Expert on leadership transitions, author of 'Act Like a Leader Think Like a Leader'</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr"/>
       <c r="F341" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G341" t="inlineStr"/>
-      <c r="H341" t="inlineStr"/>
       <c r="I341" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J341" t="inlineStr"/>
-      <c r="K341" t="inlineStr"/>
       <c r="L341" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M341" t="inlineStr"/>
       <c r="N341" t="inlineStr">
         <is>
           <t>@HerminiaIbarra</t>
@@ -21393,27 +21239,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q341" t="inlineStr"/>
       <c r="R341" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S341" t="inlineStr"/>
-      <c r="T341" t="inlineStr"/>
       <c r="U341" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V341" t="inlineStr"/>
-      <c r="W341" t="inlineStr"/>
       <c r="X341" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -21466,13 +21306,11 @@
           <t>Brand account</t>
         </is>
       </c>
-      <c r="K342" t="inlineStr"/>
       <c r="L342" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M342" t="inlineStr"/>
       <c r="N342" t="inlineStr">
         <is>
           <t>@managertools</t>
@@ -21488,13 +21326,11 @@
           <t>Brand account</t>
         </is>
       </c>
-      <c r="Q342" t="inlineStr"/>
       <c r="R342" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S342" t="inlineStr"/>
       <c r="T342" t="inlineStr">
         <is>
           <t>@managertools</t>
@@ -21510,13 +21346,1244 @@
           <t>Brand account</t>
         </is>
       </c>
-      <c r="W342" t="inlineStr"/>
       <c r="X342" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Douglas Stone</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Lecturer, Harvard Law School</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Triad Consulting / Harvard</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Co-author 'Thanks for the Feedback'. 30+ years teaching negotiation at Harvard.</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr"/>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr"/>
+      <c r="H343" t="inlineStr"/>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr"/>
+      <c r="K343" t="inlineStr"/>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr"/>
+      <c r="N343" t="inlineStr"/>
+      <c r="O343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P343" t="inlineStr"/>
+      <c r="Q343" t="inlineStr"/>
+      <c r="R343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S343" t="inlineStr"/>
+      <c r="T343" t="inlineStr"/>
+      <c r="U343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V343" t="inlineStr"/>
+      <c r="W343" t="inlineStr"/>
+      <c r="X343" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Joe Hirsch</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Author &amp; TEDx Speaker</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>joehirsch.me</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Author 'The Feedback Fix'. Pioneer of feedforward approach.</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr"/>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr"/>
+      <c r="H344" t="inlineStr"/>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr"/>
+      <c r="K344" t="inlineStr"/>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr"/>
+      <c r="N344" t="inlineStr">
+        <is>
+          <t>@joemhirsch</t>
+        </is>
+      </c>
+      <c r="O344" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P344" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="Q344" t="inlineStr"/>
+      <c r="R344" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S344" t="inlineStr"/>
+      <c r="T344" t="inlineStr"/>
+      <c r="U344" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V344" t="inlineStr"/>
+      <c r="W344" t="inlineStr"/>
+      <c r="X344" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>M. Tamra Chandler</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Author &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>PeopleWyze</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Author 'Feedback (and Other Dirty Words)'. Decades transforming performance management.</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr"/>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr"/>
+      <c r="H345" t="inlineStr"/>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr"/>
+      <c r="K345" t="inlineStr"/>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr"/>
+      <c r="N345" t="inlineStr">
+        <is>
+          <t>@mtchandler</t>
+        </is>
+      </c>
+      <c r="O345" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P345" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q345" t="inlineStr"/>
+      <c r="R345" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S345" t="inlineStr"/>
+      <c r="T345" t="inlineStr"/>
+      <c r="U345" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V345" t="inlineStr"/>
+      <c r="W345" t="inlineStr"/>
+      <c r="X345" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Therese Huston</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Cognitive Scientist</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Seattle University</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Author 'Let's Talk: Make Effective Feedback Your Superpower'. Research-backed feedback strategies.</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>@drtheresehuston</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr"/>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr"/>
+      <c r="N346" t="inlineStr">
+        <is>
+          <t>@ThereseHuston</t>
+        </is>
+      </c>
+      <c r="O346" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P346" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q346" t="inlineStr"/>
+      <c r="R346" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S346" t="inlineStr"/>
+      <c r="T346" t="inlineStr"/>
+      <c r="U346" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V346" t="inlineStr"/>
+      <c r="W346" t="inlineStr"/>
+      <c r="X346" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Georgia Murch</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Feedback Culture Expert</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Georgia Murch / Can We Talk</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Australia's leading expert on embedding feedback cultures. Author 'Fixing Feedback'.</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>wwwgeorgiamurchcom</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>@georgiamurch</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr"/>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr"/>
+      <c r="N347" t="inlineStr">
+        <is>
+          <t>@GeorgiaMurch</t>
+        </is>
+      </c>
+      <c r="O347" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P347" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q347" t="inlineStr"/>
+      <c r="R347" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S347" t="inlineStr"/>
+      <c r="T347" t="inlineStr"/>
+      <c r="U347" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V347" t="inlineStr"/>
+      <c r="W347" t="inlineStr"/>
+      <c r="X347" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>LeeAnn Renninger</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>LifeLabs Learning</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>TED talk on feedback with 1.4M+ views. PhD cognitive psychology.</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>@leeann_renn</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="K348" t="inlineStr"/>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr"/>
+      <c r="N348" t="inlineStr"/>
+      <c r="O348" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P348" t="inlineStr"/>
+      <c r="Q348" t="inlineStr"/>
+      <c r="R348" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S348" t="inlineStr"/>
+      <c r="T348" t="inlineStr"/>
+      <c r="U348" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V348" t="inlineStr"/>
+      <c r="W348" t="inlineStr"/>
+      <c r="X348" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Tania Luna</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>LifeLabs Learning / Scarlet Spark</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Co-author 'The Leader Lab'. Researcher turning feedback into scalable skill.</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr"/>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr"/>
+      <c r="K349" t="inlineStr"/>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr"/>
+      <c r="N349" t="inlineStr">
+        <is>
+          <t>@Surprisology</t>
+        </is>
+      </c>
+      <c r="O349" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P349" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="Q349" t="inlineStr"/>
+      <c r="R349" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S349" t="inlineStr"/>
+      <c r="T349" t="inlineStr"/>
+      <c r="U349" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V349" t="inlineStr"/>
+      <c r="W349" t="inlineStr"/>
+      <c r="X349" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Ashley Goodall</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Author &amp; Researcher</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Co-author HBR 'The Feedback Fallacy'. Porchlight Best Management Book 2024.</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr"/>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>@ashley_goodall</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr"/>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr"/>
+      <c r="N350" t="inlineStr">
+        <is>
+          <t>@ashleygoodall</t>
+        </is>
+      </c>
+      <c r="O350" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P350" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="Q350" t="inlineStr"/>
+      <c r="R350" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S350" t="inlineStr"/>
+      <c r="T350" t="inlineStr"/>
+      <c r="U350" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V350" t="inlineStr"/>
+      <c r="W350" t="inlineStr"/>
+      <c r="X350" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Marcus Buckingham</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Head of Research</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>ADP Research Institute</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Co-author 'The Feedback Fallacy'. Champion of strengths-based feedback.</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>@marcusbuckingham</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr"/>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr"/>
+      <c r="N351" t="inlineStr">
+        <is>
+          <t>@mwbuckingham</t>
+        </is>
+      </c>
+      <c r="O351" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P351" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q351" t="inlineStr">
+        <is>
+          <t>@marcus_buckingham</t>
+        </is>
+      </c>
+      <c r="R351" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S351" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="T351" t="inlineStr"/>
+      <c r="U351" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V351" t="inlineStr"/>
+      <c r="W351" t="inlineStr"/>
+      <c r="X351" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Jeff Wetzler</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>The Ask Approach</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Author 'Ask'. Top Leadership Book 2024. Surfaces hidden feedback.</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr"/>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>@askapproach</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr"/>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr"/>
+      <c r="N352" t="inlineStr">
+        <is>
+          <t>@jeffreywetzler</t>
+        </is>
+      </c>
+      <c r="O352" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P352" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="Q352" t="inlineStr"/>
+      <c r="R352" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S352" t="inlineStr"/>
+      <c r="T352" t="inlineStr"/>
+      <c r="U352" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V352" t="inlineStr"/>
+      <c r="W352" t="inlineStr"/>
+      <c r="X352" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Ed Batista</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Executive Coach &amp; Lecturer</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Stanford GSB</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>15 years teaching feedback at Stanford. HBR contributor. 9000+ coaching sessions.</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr"/>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr"/>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>@edbatista</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr"/>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr"/>
+      <c r="N353" t="inlineStr">
+        <is>
+          <t>@edbatista</t>
+        </is>
+      </c>
+      <c r="O353" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P353" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q353" t="inlineStr"/>
+      <c r="R353" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S353" t="inlineStr"/>
+      <c r="T353" t="inlineStr"/>
+      <c r="U353" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V353" t="inlineStr"/>
+      <c r="W353" t="inlineStr"/>
+      <c r="X353" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Anna Carroll</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Everyday Feedback</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Author 'The Feedback Imperative'. Creator of the COIN feedback model.</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr"/>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr"/>
+      <c r="H354" t="inlineStr"/>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr"/>
+      <c r="K354" t="inlineStr"/>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr"/>
+      <c r="N354" t="inlineStr">
+        <is>
+          <t>@annacarrollMSSW</t>
+        </is>
+      </c>
+      <c r="O354" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P354" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q354" t="inlineStr"/>
+      <c r="R354" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S354" t="inlineStr"/>
+      <c r="T354" t="inlineStr"/>
+      <c r="U354" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V354" t="inlineStr"/>
+      <c r="W354" t="inlineStr"/>
+      <c r="X354" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y354" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Deborah Grayson Riegel</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Keynote Speaker &amp; Professor</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Wharton / Columbia</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Teaches feedback at Wharton and Columbia. Regular HBR, Forbes contributor.</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr"/>
+      <c r="H355" t="inlineStr"/>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr"/>
+      <c r="K355" t="inlineStr"/>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M355" t="inlineStr"/>
+      <c r="N355" t="inlineStr">
+        <is>
+          <t>@DeborahGRiegel</t>
+        </is>
+      </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P355" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="Q355" t="inlineStr"/>
+      <c r="R355" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S355" t="inlineStr"/>
+      <c r="T355" t="inlineStr"/>
+      <c r="U355" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V355" t="inlineStr"/>
+      <c r="W355" t="inlineStr"/>
+      <c r="X355" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y355" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Jen Ostrich</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Grow Collective</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Co-creator Shift Positive feedback method. Co-author 'Feedback Reimagined'.</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr"/>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr"/>
+      <c r="H356" t="inlineStr"/>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr"/>
+      <c r="K356" t="inlineStr"/>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M356" t="inlineStr"/>
+      <c r="N356" t="inlineStr"/>
+      <c r="O356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P356" t="inlineStr"/>
+      <c r="Q356" t="inlineStr"/>
+      <c r="R356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S356" t="inlineStr"/>
+      <c r="T356" t="inlineStr"/>
+      <c r="U356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V356" t="inlineStr"/>
+      <c r="W356" t="inlineStr"/>
+      <c r="X356" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y356" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>William Ferriter</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>National Board Certified Teacher</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Solution Tree</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Co-author 'Creating a Culture of Feedback' in education. 29 years in classrooms.</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr"/>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr"/>
+      <c r="K357" t="inlineStr"/>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M357" t="inlineStr"/>
+      <c r="N357" t="inlineStr">
+        <is>
+          <t>@plugusin</t>
+        </is>
+      </c>
+      <c r="O357" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P357" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="Q357" t="inlineStr"/>
+      <c r="R357" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S357" t="inlineStr"/>
+      <c r="T357" t="inlineStr"/>
+      <c r="U357" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V357" t="inlineStr"/>
+      <c r="W357" t="inlineStr"/>
+      <c r="X357" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y357" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -21530,7 +22597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -21978,6 +23045,26 @@
       <c r="D22" t="inlineStr">
         <is>
           <t>first-time-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>17</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>feedback-culture</t>
         </is>
       </c>
     </row>
@@ -21993,7 +23080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G169"/>
+  <dimension ref="A1:G177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -28163,6 +29250,302 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>69c3b38aecfc8d3950f4e082</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>2026-04-02T02:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>69c3b38cecfc8d3950f4e0a8</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>2026-04-02T03:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>69c3b3d2dc7f763f71a4b821</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>2026-04-05T23:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>69c3b3a9dc7f763f71a4b456</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>2026-04-01T18:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>69c3b3aaecfc8d3950f4e303</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>2026-04-02T01:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>69c3b3bfecfc8d3950f4e455</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>2026-03-27T23:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>69c3b3c2dc7f763f71a4b568</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>2026-04-02T05:01:00.000Z</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Feedback Culture</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>69c3b3c3dc7f763f71a4b58f</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>2026-04-01T23:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Authentic Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1016,10 +1016,14 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1123,7 +1127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y357"/>
+  <dimension ref="A1:Y373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -21373,55 +21377,41 @@
           <t>Co-author 'Thanks for the Feedback'. 30+ years teaching negotiation at Harvard.</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr"/>
       <c r="F343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G343" t="inlineStr"/>
-      <c r="H343" t="inlineStr"/>
       <c r="I343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J343" t="inlineStr"/>
-      <c r="K343" t="inlineStr"/>
       <c r="L343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M343" t="inlineStr"/>
-      <c r="N343" t="inlineStr"/>
       <c r="O343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P343" t="inlineStr"/>
-      <c r="Q343" t="inlineStr"/>
       <c r="R343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S343" t="inlineStr"/>
-      <c r="T343" t="inlineStr"/>
       <c r="U343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V343" t="inlineStr"/>
-      <c r="W343" t="inlineStr"/>
       <c r="X343" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -21444,27 +21434,21 @@
           <t>Author 'The Feedback Fix'. Pioneer of feedforward approach.</t>
         </is>
       </c>
-      <c r="E344" t="inlineStr"/>
       <c r="F344" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G344" t="inlineStr"/>
-      <c r="H344" t="inlineStr"/>
       <c r="I344" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J344" t="inlineStr"/>
-      <c r="K344" t="inlineStr"/>
       <c r="L344" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M344" t="inlineStr"/>
       <c r="N344" t="inlineStr">
         <is>
           <t>@joemhirsch</t>
@@ -21480,27 +21464,21 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="Q344" t="inlineStr"/>
       <c r="R344" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S344" t="inlineStr"/>
-      <c r="T344" t="inlineStr"/>
       <c r="U344" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V344" t="inlineStr"/>
-      <c r="W344" t="inlineStr"/>
       <c r="X344" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -21523,27 +21501,21 @@
           <t>Author 'Feedback (and Other Dirty Words)'. Decades transforming performance management.</t>
         </is>
       </c>
-      <c r="E345" t="inlineStr"/>
       <c r="F345" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G345" t="inlineStr"/>
-      <c r="H345" t="inlineStr"/>
       <c r="I345" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J345" t="inlineStr"/>
-      <c r="K345" t="inlineStr"/>
       <c r="L345" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M345" t="inlineStr"/>
       <c r="N345" t="inlineStr">
         <is>
           <t>@mtchandler</t>
@@ -21559,27 +21531,21 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q345" t="inlineStr"/>
       <c r="R345" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S345" t="inlineStr"/>
-      <c r="T345" t="inlineStr"/>
       <c r="U345" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V345" t="inlineStr"/>
-      <c r="W345" t="inlineStr"/>
       <c r="X345" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -21602,13 +21568,11 @@
           <t>Author 'Let's Talk: Make Effective Feedback Your Superpower'. Research-backed feedback strategies.</t>
         </is>
       </c>
-      <c r="E346" t="inlineStr"/>
       <c r="F346" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G346" t="inlineStr"/>
       <c r="H346" t="inlineStr">
         <is>
           <t>@drtheresehuston</t>
@@ -21624,13 +21588,11 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="K346" t="inlineStr"/>
       <c r="L346" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M346" t="inlineStr"/>
       <c r="N346" t="inlineStr">
         <is>
           <t>@ThereseHuston</t>
@@ -21646,27 +21608,21 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q346" t="inlineStr"/>
       <c r="R346" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S346" t="inlineStr"/>
-      <c r="T346" t="inlineStr"/>
       <c r="U346" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V346" t="inlineStr"/>
-      <c r="W346" t="inlineStr"/>
       <c r="X346" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -21719,13 +21675,11 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="K347" t="inlineStr"/>
       <c r="L347" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M347" t="inlineStr"/>
       <c r="N347" t="inlineStr">
         <is>
           <t>@GeorgiaMurch</t>
@@ -21741,27 +21695,21 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q347" t="inlineStr"/>
       <c r="R347" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S347" t="inlineStr"/>
-      <c r="T347" t="inlineStr"/>
       <c r="U347" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V347" t="inlineStr"/>
-      <c r="W347" t="inlineStr"/>
       <c r="X347" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -21784,13 +21732,11 @@
           <t>TED talk on feedback with 1.4M+ views. PhD cognitive psychology.</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr"/>
       <c r="F348" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr">
         <is>
           <t>@leeann_renn</t>
@@ -21806,41 +21752,31 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="K348" t="inlineStr"/>
       <c r="L348" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M348" t="inlineStr"/>
-      <c r="N348" t="inlineStr"/>
       <c r="O348" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P348" t="inlineStr"/>
-      <c r="Q348" t="inlineStr"/>
       <c r="R348" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S348" t="inlineStr"/>
-      <c r="T348" t="inlineStr"/>
       <c r="U348" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V348" t="inlineStr"/>
-      <c r="W348" t="inlineStr"/>
       <c r="X348" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -21863,27 +21799,21 @@
           <t>Co-author 'The Leader Lab'. Researcher turning feedback into scalable skill.</t>
         </is>
       </c>
-      <c r="E349" t="inlineStr"/>
       <c r="F349" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G349" t="inlineStr"/>
-      <c r="H349" t="inlineStr"/>
       <c r="I349" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J349" t="inlineStr"/>
-      <c r="K349" t="inlineStr"/>
       <c r="L349" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M349" t="inlineStr"/>
       <c r="N349" t="inlineStr">
         <is>
           <t>@Surprisology</t>
@@ -21899,27 +21829,21 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="Q349" t="inlineStr"/>
       <c r="R349" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S349" t="inlineStr"/>
-      <c r="T349" t="inlineStr"/>
       <c r="U349" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V349" t="inlineStr"/>
-      <c r="W349" t="inlineStr"/>
       <c r="X349" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -21942,13 +21866,11 @@
           <t>Co-author HBR 'The Feedback Fallacy'. Porchlight Best Management Book 2024.</t>
         </is>
       </c>
-      <c r="E350" t="inlineStr"/>
       <c r="F350" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G350" t="inlineStr"/>
       <c r="H350" t="inlineStr">
         <is>
           <t>@ashley_goodall</t>
@@ -21964,13 +21886,11 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="K350" t="inlineStr"/>
       <c r="L350" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M350" t="inlineStr"/>
       <c r="N350" t="inlineStr">
         <is>
           <t>@ashleygoodall</t>
@@ -21986,27 +21906,21 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="Q350" t="inlineStr"/>
       <c r="R350" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S350" t="inlineStr"/>
-      <c r="T350" t="inlineStr"/>
       <c r="U350" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V350" t="inlineStr"/>
-      <c r="W350" t="inlineStr"/>
       <c r="X350" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -22029,13 +21943,11 @@
           <t>Co-author 'The Feedback Fallacy'. Champion of strengths-based feedback.</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr"/>
       <c r="F351" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G351" t="inlineStr"/>
       <c r="H351" t="inlineStr">
         <is>
           <t>@marcusbuckingham</t>
@@ -22051,13 +21963,11 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="K351" t="inlineStr"/>
       <c r="L351" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M351" t="inlineStr"/>
       <c r="N351" t="inlineStr">
         <is>
           <t>@mwbuckingham</t>
@@ -22088,20 +21998,16 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="T351" t="inlineStr"/>
       <c r="U351" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V351" t="inlineStr"/>
-      <c r="W351" t="inlineStr"/>
       <c r="X351" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -22124,13 +22030,11 @@
           <t>Author 'Ask'. Top Leadership Book 2024. Surfaces hidden feedback.</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr"/>
       <c r="F352" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G352" t="inlineStr"/>
       <c r="H352" t="inlineStr">
         <is>
           <t>@askapproach</t>
@@ -22146,13 +22050,11 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="K352" t="inlineStr"/>
       <c r="L352" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M352" t="inlineStr"/>
       <c r="N352" t="inlineStr">
         <is>
           <t>@jeffreywetzler</t>
@@ -22168,27 +22070,21 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="Q352" t="inlineStr"/>
       <c r="R352" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S352" t="inlineStr"/>
-      <c r="T352" t="inlineStr"/>
       <c r="U352" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V352" t="inlineStr"/>
-      <c r="W352" t="inlineStr"/>
       <c r="X352" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -22211,13 +22107,11 @@
           <t>15 years teaching feedback at Stanford. HBR contributor. 9000+ coaching sessions.</t>
         </is>
       </c>
-      <c r="E353" t="inlineStr"/>
       <c r="F353" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G353" t="inlineStr"/>
       <c r="H353" t="inlineStr">
         <is>
           <t>@edbatista</t>
@@ -22233,13 +22127,11 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="K353" t="inlineStr"/>
       <c r="L353" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M353" t="inlineStr"/>
       <c r="N353" t="inlineStr">
         <is>
           <t>@edbatista</t>
@@ -22255,27 +22147,21 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q353" t="inlineStr"/>
       <c r="R353" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S353" t="inlineStr"/>
-      <c r="T353" t="inlineStr"/>
       <c r="U353" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V353" t="inlineStr"/>
-      <c r="W353" t="inlineStr"/>
       <c r="X353" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -22298,27 +22184,21 @@
           <t>Author 'The Feedback Imperative'. Creator of the COIN feedback model.</t>
         </is>
       </c>
-      <c r="E354" t="inlineStr"/>
       <c r="F354" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G354" t="inlineStr"/>
-      <c r="H354" t="inlineStr"/>
       <c r="I354" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J354" t="inlineStr"/>
-      <c r="K354" t="inlineStr"/>
       <c r="L354" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M354" t="inlineStr"/>
       <c r="N354" t="inlineStr">
         <is>
           <t>@annacarrollMSSW</t>
@@ -22334,27 +22214,21 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q354" t="inlineStr"/>
       <c r="R354" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S354" t="inlineStr"/>
-      <c r="T354" t="inlineStr"/>
       <c r="U354" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V354" t="inlineStr"/>
-      <c r="W354" t="inlineStr"/>
       <c r="X354" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -22377,27 +22251,21 @@
           <t>Teaches feedback at Wharton and Columbia. Regular HBR, Forbes contributor.</t>
         </is>
       </c>
-      <c r="E355" t="inlineStr"/>
       <c r="F355" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G355" t="inlineStr"/>
-      <c r="H355" t="inlineStr"/>
       <c r="I355" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J355" t="inlineStr"/>
-      <c r="K355" t="inlineStr"/>
       <c r="L355" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M355" t="inlineStr"/>
       <c r="N355" t="inlineStr">
         <is>
           <t>@DeborahGRiegel</t>
@@ -22413,27 +22281,21 @@
           <t>Website</t>
         </is>
       </c>
-      <c r="Q355" t="inlineStr"/>
       <c r="R355" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S355" t="inlineStr"/>
-      <c r="T355" t="inlineStr"/>
       <c r="U355" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V355" t="inlineStr"/>
-      <c r="W355" t="inlineStr"/>
       <c r="X355" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -22456,55 +22318,41 @@
           <t>Co-creator Shift Positive feedback method. Co-author 'Feedback Reimagined'.</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr"/>
       <c r="F356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G356" t="inlineStr"/>
-      <c r="H356" t="inlineStr"/>
       <c r="I356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J356" t="inlineStr"/>
-      <c r="K356" t="inlineStr"/>
       <c r="L356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M356" t="inlineStr"/>
-      <c r="N356" t="inlineStr"/>
       <c r="O356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P356" t="inlineStr"/>
-      <c r="Q356" t="inlineStr"/>
       <c r="R356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S356" t="inlineStr"/>
-      <c r="T356" t="inlineStr"/>
       <c r="U356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V356" t="inlineStr"/>
-      <c r="W356" t="inlineStr"/>
       <c r="X356" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -22527,27 +22375,21 @@
           <t>Co-author 'Creating a Culture of Feedback' in education. 29 years in classrooms.</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr"/>
       <c r="F357" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G357" t="inlineStr"/>
-      <c r="H357" t="inlineStr"/>
       <c r="I357" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J357" t="inlineStr"/>
-      <c r="K357" t="inlineStr"/>
       <c r="L357" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M357" t="inlineStr"/>
       <c r="N357" t="inlineStr">
         <is>
           <t>@plugusin</t>
@@ -22563,27 +22405,1285 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="Q357" t="inlineStr"/>
       <c r="R357" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S357" t="inlineStr"/>
-      <c r="T357" t="inlineStr"/>
       <c r="U357" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V357" t="inlineStr"/>
-      <c r="W357" t="inlineStr"/>
       <c r="X357" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Bill George</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Harvard Business School Professor</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Harvard Business School / Medtronic</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Author of 'Authentic Leadership' and 'True North' — the foundational texts that defined authentic leadership</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr"/>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr"/>
+      <c r="H358" t="inlineStr"/>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr"/>
+      <c r="K358" t="inlineStr"/>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M358" t="inlineStr"/>
+      <c r="N358" t="inlineStr">
+        <is>
+          <t>@Bill_George</t>
+        </is>
+      </c>
+      <c r="O358" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P358" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q358" t="inlineStr"/>
+      <c r="R358" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S358" t="inlineStr"/>
+      <c r="T358" t="inlineStr"/>
+      <c r="U358" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V358" t="inlineStr"/>
+      <c r="W358" t="inlineStr"/>
+      <c r="X358" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y358" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Bruce Avolio</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>University of Washington Foster School of Business</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Co-developed the Authentic Leadership Questionnaire (ALQ)</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr"/>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr"/>
+      <c r="H359" t="inlineStr"/>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr"/>
+      <c r="K359" t="inlineStr"/>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M359" t="inlineStr"/>
+      <c r="N359" t="inlineStr">
+        <is>
+          <t>@bavolio</t>
+        </is>
+      </c>
+      <c r="O359" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P359" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q359" t="inlineStr"/>
+      <c r="R359" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S359" t="inlineStr"/>
+      <c r="T359" t="inlineStr"/>
+      <c r="U359" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V359" t="inlineStr"/>
+      <c r="W359" t="inlineStr"/>
+      <c r="X359" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>William Gardner</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Jerry S. Rawls Chair in Leadership</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Texas Tech University</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Co-created the self-based model of authentic leadership</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr"/>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr"/>
+      <c r="H360" t="inlineStr"/>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr"/>
+      <c r="K360" t="inlineStr"/>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr"/>
+      <c r="N360" t="inlineStr"/>
+      <c r="O360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P360" t="inlineStr"/>
+      <c r="Q360" t="inlineStr"/>
+      <c r="R360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S360" t="inlineStr"/>
+      <c r="T360" t="inlineStr"/>
+      <c r="U360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V360" t="inlineStr"/>
+      <c r="W360" t="inlineStr"/>
+      <c r="X360" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y360" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Fred Walumbwa</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Co-developed the ALQ across China, Kenya, and the US</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr"/>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr"/>
+      <c r="H361" t="inlineStr"/>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr"/>
+      <c r="K361" t="inlineStr"/>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr"/>
+      <c r="N361" t="inlineStr"/>
+      <c r="O361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P361" t="inlineStr"/>
+      <c r="Q361" t="inlineStr"/>
+      <c r="R361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S361" t="inlineStr"/>
+      <c r="T361" t="inlineStr"/>
+      <c r="U361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V361" t="inlineStr"/>
+      <c r="W361" t="inlineStr"/>
+      <c r="X361" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y361" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Rob Goffee</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Emeritus Professor</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>London Business School</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Co-author of 'Why Should Anyone Be Led by You?'</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr"/>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr"/>
+      <c r="H362" t="inlineStr"/>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr"/>
+      <c r="K362" t="inlineStr"/>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr"/>
+      <c r="N362" t="inlineStr"/>
+      <c r="O362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P362" t="inlineStr"/>
+      <c r="Q362" t="inlineStr"/>
+      <c r="R362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S362" t="inlineStr"/>
+      <c r="T362" t="inlineStr"/>
+      <c r="U362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V362" t="inlineStr"/>
+      <c r="W362" t="inlineStr"/>
+      <c r="X362" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y362" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Gareth Jones</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Fellow</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>London Business School / IE Business School</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Co-author of 'Why Should Anyone Be Led by You?'</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr"/>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr"/>
+      <c r="H363" t="inlineStr"/>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr"/>
+      <c r="K363" t="inlineStr"/>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr"/>
+      <c r="N363" t="inlineStr"/>
+      <c r="O363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P363" t="inlineStr"/>
+      <c r="Q363" t="inlineStr"/>
+      <c r="R363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S363" t="inlineStr"/>
+      <c r="T363" t="inlineStr"/>
+      <c r="U363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V363" t="inlineStr"/>
+      <c r="W363" t="inlineStr"/>
+      <c r="X363" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y363" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Nick Craig</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Founder &amp; President</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Core Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Founded the Authentic Leadership Institute, co-authored 'Finding Your True North'</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr"/>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr"/>
+      <c r="H364" t="inlineStr"/>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr"/>
+      <c r="K364" t="inlineStr"/>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr"/>
+      <c r="N364" t="inlineStr">
+        <is>
+          <t>@NickCraig1</t>
+        </is>
+      </c>
+      <c r="O364" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P364" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q364" t="inlineStr"/>
+      <c r="R364" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S364" t="inlineStr"/>
+      <c r="T364" t="inlineStr"/>
+      <c r="U364" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V364" t="inlineStr"/>
+      <c r="W364" t="inlineStr"/>
+      <c r="X364" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Henna Inam</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Transformational Leadership Inc</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Author of 'Wired for Authenticity', neuroscience-based authentic leadership</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr"/>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr"/>
+      <c r="H365" t="inlineStr"/>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr"/>
+      <c r="K365" t="inlineStr"/>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr"/>
+      <c r="N365" t="inlineStr">
+        <is>
+          <t>@hennainam</t>
+        </is>
+      </c>
+      <c r="O365" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P365" t="inlineStr">
+        <is>
+          <t>X profile / Forbes</t>
+        </is>
+      </c>
+      <c r="Q365" t="inlineStr"/>
+      <c r="R365" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S365" t="inlineStr"/>
+      <c r="T365" t="inlineStr"/>
+      <c r="U365" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V365" t="inlineStr"/>
+      <c r="W365" t="inlineStr"/>
+      <c r="X365" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Karissa Thacker</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Management Psychologist</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Strategic Performance Solutions</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Author of 'The Art of Authenticity'</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr"/>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr"/>
+      <c r="H366" t="inlineStr"/>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr"/>
+      <c r="K366" t="inlineStr"/>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr"/>
+      <c r="N366" t="inlineStr">
+        <is>
+          <t>@karissathacker</t>
+        </is>
+      </c>
+      <c r="O366" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P366" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q366" t="inlineStr"/>
+      <c r="R366" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S366" t="inlineStr"/>
+      <c r="T366" t="inlineStr"/>
+      <c r="U366" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V366" t="inlineStr"/>
+      <c r="W366" t="inlineStr"/>
+      <c r="X366" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y366" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Kevin Cashman</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Global Leader of CEO Development</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Korn Ferry</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Author of 'Leadership from the Inside Out'</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr"/>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr"/>
+      <c r="H367" t="inlineStr"/>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr"/>
+      <c r="K367" t="inlineStr"/>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M367" t="inlineStr"/>
+      <c r="N367" t="inlineStr"/>
+      <c r="O367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P367" t="inlineStr"/>
+      <c r="Q367" t="inlineStr"/>
+      <c r="R367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S367" t="inlineStr"/>
+      <c r="T367" t="inlineStr"/>
+      <c r="U367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V367" t="inlineStr"/>
+      <c r="W367" t="inlineStr"/>
+      <c r="X367" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Jeff Davis</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Author &amp; Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Mr. Mountaintop</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Author of 'The Power of Authentic Leadership', TEDx speaker</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr"/>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr"/>
+      <c r="H368" t="inlineStr"/>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr"/>
+      <c r="K368" t="inlineStr"/>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M368" t="inlineStr"/>
+      <c r="N368" t="inlineStr">
+        <is>
+          <t>@JeffDavis027</t>
+        </is>
+      </c>
+      <c r="O368" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P368" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q368" t="inlineStr"/>
+      <c r="R368" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S368" t="inlineStr"/>
+      <c r="T368" t="inlineStr"/>
+      <c r="U368" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V368" t="inlineStr"/>
+      <c r="W368" t="inlineStr"/>
+      <c r="X368" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y368" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Dan Owolabi</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Author &amp; Executive Director</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Branches Worldwide / Owolabi Leadership</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Author of 'Authentic Leadership', works with leaders in 20+ countries</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>iamdanowolabi</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>@iamdanowolabi</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K369" t="inlineStr"/>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr"/>
+      <c r="N369" t="inlineStr">
+        <is>
+          <t>@iamdanowolabi</t>
+        </is>
+      </c>
+      <c r="O369" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P369" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q369" t="inlineStr"/>
+      <c r="R369" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S369" t="inlineStr"/>
+      <c r="T369" t="inlineStr"/>
+      <c r="U369" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V369" t="inlineStr"/>
+      <c r="W369" t="inlineStr"/>
+      <c r="X369" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y369" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Marsha Clark</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Marsha Clark &amp; Associates</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Author of 'Embracing Your Power: A Woman's Path to Authentic Leadership'</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>MarshaClarkAssociates</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr"/>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr"/>
+      <c r="K370" t="inlineStr"/>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M370" t="inlineStr"/>
+      <c r="N370" t="inlineStr"/>
+      <c r="O370" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P370" t="inlineStr"/>
+      <c r="Q370" t="inlineStr"/>
+      <c r="R370" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S370" t="inlineStr"/>
+      <c r="T370" t="inlineStr"/>
+      <c r="U370" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V370" t="inlineStr"/>
+      <c r="W370" t="inlineStr"/>
+      <c r="X370" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y370" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Dino Cattaneo</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Host &amp; Executive Coach</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Authentic Leadership for Everyday People Podcast</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>183+ episodes exploring authenticity in leadership</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr"/>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr"/>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>@al4edp</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Podcast website</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>@al4edp</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>Podcast website</t>
+        </is>
+      </c>
+      <c r="N371" t="inlineStr">
+        <is>
+          <t>@al4edp</t>
+        </is>
+      </c>
+      <c r="O371" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P371" t="inlineStr">
+        <is>
+          <t>Podcast website</t>
+        </is>
+      </c>
+      <c r="Q371" t="inlineStr"/>
+      <c r="R371" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S371" t="inlineStr"/>
+      <c r="T371" t="inlineStr"/>
+      <c r="U371" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V371" t="inlineStr"/>
+      <c r="W371" t="inlineStr"/>
+      <c r="X371" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y371" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Zach Clayton</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Three Ships</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Co-author of 'True North: Emerging Leader Edition' with Bill George</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr"/>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr"/>
+      <c r="H372" t="inlineStr"/>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr"/>
+      <c r="K372" t="inlineStr"/>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M372" t="inlineStr"/>
+      <c r="N372" t="inlineStr">
+        <is>
+          <t>@zsclayton</t>
+        </is>
+      </c>
+      <c r="O372" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P372" t="inlineStr">
+        <is>
+          <t>X profile link</t>
+        </is>
+      </c>
+      <c r="Q372" t="inlineStr"/>
+      <c r="R372" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S372" t="inlineStr"/>
+      <c r="T372" t="inlineStr"/>
+      <c r="U372" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V372" t="inlineStr"/>
+      <c r="W372" t="inlineStr"/>
+      <c r="X372" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Mike Robbins</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Author &amp; Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Mike Robbins Inc</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Author of 'Bring Your Whole Self to Work', 25 years helping leaders lead with authenticity</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>mikerobbinspage</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>@mikedrobbins</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr"/>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr"/>
+      <c r="N373" t="inlineStr"/>
+      <c r="O373" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P373" t="inlineStr"/>
+      <c r="Q373" t="inlineStr"/>
+      <c r="R373" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S373" t="inlineStr"/>
+      <c r="T373" t="inlineStr"/>
+      <c r="U373" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V373" t="inlineStr"/>
+      <c r="W373" t="inlineStr"/>
+      <c r="X373" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y373" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -22597,7 +23697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -23065,6 +24165,26 @@
       <c r="D23" t="inlineStr">
         <is>
           <t>feedback-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>16</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>authentic-leadership</t>
         </is>
       </c>
     </row>
@@ -23080,7 +24200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G177"/>
+  <dimension ref="A1:G185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -29546,6 +30666,302 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>69c3b980dc7f763f71a4dfae</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>2026-04-02T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>69c3b982ecfc8d3950f5126e</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>2026-04-02T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>69c3b9c8dc7f763f71a4e27b</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>2026-04-01T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>69c3b99ddc7f763f71a4e1b0</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>2026-04-02T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>69c3b9bfdc7f763f71a4e255</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>2026-03-28T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>69c3b99fdc7f763f71a4e1d6</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>2026-04-02T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>69c3b99fecfc8d3950f513da</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>2026-04-02T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Authentic Leadership</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>69c3b9b3ecfc8d3950f514d8</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>2026-04-02T05:20:00Z</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Principal Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1037,10 +1037,14 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Education footer variant</t>
@@ -1127,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y373"/>
+  <dimension ref="A1:Y390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22442,27 +22446,21 @@
           <t>Author of 'Authentic Leadership' and 'True North' — the foundational texts that defined authentic leadership</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr"/>
       <c r="F358" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G358" t="inlineStr"/>
-      <c r="H358" t="inlineStr"/>
       <c r="I358" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J358" t="inlineStr"/>
-      <c r="K358" t="inlineStr"/>
       <c r="L358" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M358" t="inlineStr"/>
       <c r="N358" t="inlineStr">
         <is>
           <t>@Bill_George</t>
@@ -22478,27 +22476,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q358" t="inlineStr"/>
       <c r="R358" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S358" t="inlineStr"/>
-      <c r="T358" t="inlineStr"/>
       <c r="U358" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V358" t="inlineStr"/>
-      <c r="W358" t="inlineStr"/>
       <c r="X358" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -22521,27 +22513,21 @@
           <t>Co-developed the Authentic Leadership Questionnaire (ALQ)</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr"/>
       <c r="F359" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G359" t="inlineStr"/>
-      <c r="H359" t="inlineStr"/>
       <c r="I359" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J359" t="inlineStr"/>
-      <c r="K359" t="inlineStr"/>
       <c r="L359" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M359" t="inlineStr"/>
       <c r="N359" t="inlineStr">
         <is>
           <t>@bavolio</t>
@@ -22557,27 +22543,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q359" t="inlineStr"/>
       <c r="R359" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S359" t="inlineStr"/>
-      <c r="T359" t="inlineStr"/>
       <c r="U359" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V359" t="inlineStr"/>
-      <c r="W359" t="inlineStr"/>
       <c r="X359" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -22600,55 +22580,41 @@
           <t>Co-created the self-based model of authentic leadership</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr"/>
       <c r="F360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G360" t="inlineStr"/>
-      <c r="H360" t="inlineStr"/>
       <c r="I360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J360" t="inlineStr"/>
-      <c r="K360" t="inlineStr"/>
       <c r="L360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M360" t="inlineStr"/>
-      <c r="N360" t="inlineStr"/>
       <c r="O360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P360" t="inlineStr"/>
-      <c r="Q360" t="inlineStr"/>
       <c r="R360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S360" t="inlineStr"/>
-      <c r="T360" t="inlineStr"/>
       <c r="U360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V360" t="inlineStr"/>
-      <c r="W360" t="inlineStr"/>
       <c r="X360" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -22671,55 +22637,41 @@
           <t>Co-developed the ALQ across China, Kenya, and the US</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr"/>
       <c r="F361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G361" t="inlineStr"/>
-      <c r="H361" t="inlineStr"/>
       <c r="I361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J361" t="inlineStr"/>
-      <c r="K361" t="inlineStr"/>
       <c r="L361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M361" t="inlineStr"/>
-      <c r="N361" t="inlineStr"/>
       <c r="O361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P361" t="inlineStr"/>
-      <c r="Q361" t="inlineStr"/>
       <c r="R361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S361" t="inlineStr"/>
-      <c r="T361" t="inlineStr"/>
       <c r="U361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V361" t="inlineStr"/>
-      <c r="W361" t="inlineStr"/>
       <c r="X361" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -22742,55 +22694,41 @@
           <t>Co-author of 'Why Should Anyone Be Led by You?'</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr"/>
       <c r="F362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G362" t="inlineStr"/>
-      <c r="H362" t="inlineStr"/>
       <c r="I362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J362" t="inlineStr"/>
-      <c r="K362" t="inlineStr"/>
       <c r="L362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M362" t="inlineStr"/>
-      <c r="N362" t="inlineStr"/>
       <c r="O362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P362" t="inlineStr"/>
-      <c r="Q362" t="inlineStr"/>
       <c r="R362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S362" t="inlineStr"/>
-      <c r="T362" t="inlineStr"/>
       <c r="U362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V362" t="inlineStr"/>
-      <c r="W362" t="inlineStr"/>
       <c r="X362" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -22813,55 +22751,41 @@
           <t>Co-author of 'Why Should Anyone Be Led by You?'</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr"/>
       <c r="F363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G363" t="inlineStr"/>
-      <c r="H363" t="inlineStr"/>
       <c r="I363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J363" t="inlineStr"/>
-      <c r="K363" t="inlineStr"/>
       <c r="L363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M363" t="inlineStr"/>
-      <c r="N363" t="inlineStr"/>
       <c r="O363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P363" t="inlineStr"/>
-      <c r="Q363" t="inlineStr"/>
       <c r="R363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S363" t="inlineStr"/>
-      <c r="T363" t="inlineStr"/>
       <c r="U363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V363" t="inlineStr"/>
-      <c r="W363" t="inlineStr"/>
       <c r="X363" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -22884,27 +22808,21 @@
           <t>Founded the Authentic Leadership Institute, co-authored 'Finding Your True North'</t>
         </is>
       </c>
-      <c r="E364" t="inlineStr"/>
       <c r="F364" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G364" t="inlineStr"/>
-      <c r="H364" t="inlineStr"/>
       <c r="I364" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J364" t="inlineStr"/>
-      <c r="K364" t="inlineStr"/>
       <c r="L364" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M364" t="inlineStr"/>
       <c r="N364" t="inlineStr">
         <is>
           <t>@NickCraig1</t>
@@ -22920,27 +22838,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q364" t="inlineStr"/>
       <c r="R364" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S364" t="inlineStr"/>
-      <c r="T364" t="inlineStr"/>
       <c r="U364" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V364" t="inlineStr"/>
-      <c r="W364" t="inlineStr"/>
       <c r="X364" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -22963,27 +22875,21 @@
           <t>Author of 'Wired for Authenticity', neuroscience-based authentic leadership</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr"/>
       <c r="F365" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G365" t="inlineStr"/>
-      <c r="H365" t="inlineStr"/>
       <c r="I365" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J365" t="inlineStr"/>
-      <c r="K365" t="inlineStr"/>
       <c r="L365" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M365" t="inlineStr"/>
       <c r="N365" t="inlineStr">
         <is>
           <t>@hennainam</t>
@@ -22999,27 +22905,21 @@
           <t>X profile / Forbes</t>
         </is>
       </c>
-      <c r="Q365" t="inlineStr"/>
       <c r="R365" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S365" t="inlineStr"/>
-      <c r="T365" t="inlineStr"/>
       <c r="U365" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V365" t="inlineStr"/>
-      <c r="W365" t="inlineStr"/>
       <c r="X365" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -23042,27 +22942,21 @@
           <t>Author of 'The Art of Authenticity'</t>
         </is>
       </c>
-      <c r="E366" t="inlineStr"/>
       <c r="F366" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G366" t="inlineStr"/>
-      <c r="H366" t="inlineStr"/>
       <c r="I366" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J366" t="inlineStr"/>
-      <c r="K366" t="inlineStr"/>
       <c r="L366" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M366" t="inlineStr"/>
       <c r="N366" t="inlineStr">
         <is>
           <t>@karissathacker</t>
@@ -23078,27 +22972,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q366" t="inlineStr"/>
       <c r="R366" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S366" t="inlineStr"/>
-      <c r="T366" t="inlineStr"/>
       <c r="U366" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V366" t="inlineStr"/>
-      <c r="W366" t="inlineStr"/>
       <c r="X366" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -23121,55 +23009,41 @@
           <t>Author of 'Leadership from the Inside Out'</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr"/>
       <c r="F367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G367" t="inlineStr"/>
-      <c r="H367" t="inlineStr"/>
       <c r="I367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J367" t="inlineStr"/>
-      <c r="K367" t="inlineStr"/>
       <c r="L367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M367" t="inlineStr"/>
-      <c r="N367" t="inlineStr"/>
       <c r="O367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P367" t="inlineStr"/>
-      <c r="Q367" t="inlineStr"/>
       <c r="R367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S367" t="inlineStr"/>
-      <c r="T367" t="inlineStr"/>
       <c r="U367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V367" t="inlineStr"/>
-      <c r="W367" t="inlineStr"/>
       <c r="X367" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -23192,27 +23066,21 @@
           <t>Author of 'The Power of Authentic Leadership', TEDx speaker</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr"/>
       <c r="F368" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G368" t="inlineStr"/>
-      <c r="H368" t="inlineStr"/>
       <c r="I368" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J368" t="inlineStr"/>
-      <c r="K368" t="inlineStr"/>
       <c r="L368" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M368" t="inlineStr"/>
       <c r="N368" t="inlineStr">
         <is>
           <t>@JeffDavis027</t>
@@ -23228,27 +23096,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q368" t="inlineStr"/>
       <c r="R368" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S368" t="inlineStr"/>
-      <c r="T368" t="inlineStr"/>
       <c r="U368" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V368" t="inlineStr"/>
-      <c r="W368" t="inlineStr"/>
       <c r="X368" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -23301,13 +23163,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K369" t="inlineStr"/>
       <c r="L369" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M369" t="inlineStr"/>
       <c r="N369" t="inlineStr">
         <is>
           <t>@iamdanowolabi</t>
@@ -23323,27 +23183,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q369" t="inlineStr"/>
       <c r="R369" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S369" t="inlineStr"/>
-      <c r="T369" t="inlineStr"/>
       <c r="U369" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V369" t="inlineStr"/>
-      <c r="W369" t="inlineStr"/>
       <c r="X369" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -23381,48 +23235,36 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H370" t="inlineStr"/>
       <c r="I370" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J370" t="inlineStr"/>
-      <c r="K370" t="inlineStr"/>
       <c r="L370" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M370" t="inlineStr"/>
-      <c r="N370" t="inlineStr"/>
       <c r="O370" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P370" t="inlineStr"/>
-      <c r="Q370" t="inlineStr"/>
       <c r="R370" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S370" t="inlineStr"/>
-      <c r="T370" t="inlineStr"/>
       <c r="U370" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V370" t="inlineStr"/>
-      <c r="W370" t="inlineStr"/>
       <c r="X370" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -23445,13 +23287,11 @@
           <t>183+ episodes exploring authenticity in leadership</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr"/>
       <c r="F371" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G371" t="inlineStr"/>
       <c r="H371" t="inlineStr">
         <is>
           <t>@al4edp</t>
@@ -23497,27 +23337,21 @@
           <t>Podcast website</t>
         </is>
       </c>
-      <c r="Q371" t="inlineStr"/>
       <c r="R371" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S371" t="inlineStr"/>
-      <c r="T371" t="inlineStr"/>
       <c r="U371" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V371" t="inlineStr"/>
-      <c r="W371" t="inlineStr"/>
       <c r="X371" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -23540,27 +23374,21 @@
           <t>Co-author of 'True North: Emerging Leader Edition' with Bill George</t>
         </is>
       </c>
-      <c r="E372" t="inlineStr"/>
       <c r="F372" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G372" t="inlineStr"/>
-      <c r="H372" t="inlineStr"/>
       <c r="I372" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J372" t="inlineStr"/>
-      <c r="K372" t="inlineStr"/>
       <c r="L372" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M372" t="inlineStr"/>
       <c r="N372" t="inlineStr">
         <is>
           <t>@zsclayton</t>
@@ -23576,27 +23404,21 @@
           <t>X profile link</t>
         </is>
       </c>
-      <c r="Q372" t="inlineStr"/>
       <c r="R372" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S372" t="inlineStr"/>
-      <c r="T372" t="inlineStr"/>
       <c r="U372" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V372" t="inlineStr"/>
-      <c r="W372" t="inlineStr"/>
       <c r="X372" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -23649,41 +23471,1478 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K373" t="inlineStr"/>
       <c r="L373" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M373" t="inlineStr"/>
-      <c r="N373" t="inlineStr"/>
       <c r="O373" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P373" t="inlineStr"/>
-      <c r="Q373" t="inlineStr"/>
       <c r="R373" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S373" t="inlineStr"/>
-      <c r="T373" t="inlineStr"/>
       <c r="U373" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V373" t="inlineStr"/>
-      <c r="W373" t="inlineStr"/>
       <c r="X373" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y373" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Eric Sheninger</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Former Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Aspire Change EDU</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Author of Digital Leadership. NASSP Digital Principal Award winner.</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>EricCSheninger</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>esheninger</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr"/>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr"/>
+      <c r="N374" t="inlineStr">
+        <is>
+          <t>E_Sheninger</t>
+        </is>
+      </c>
+      <c r="O374" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P374" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="Q374" t="inlineStr"/>
+      <c r="R374" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S374" t="inlineStr"/>
+      <c r="T374" t="inlineStr"/>
+      <c r="U374" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V374" t="inlineStr"/>
+      <c r="W374" t="inlineStr"/>
+      <c r="X374" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y374" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Anthony Muhammad</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Former Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>New Frontier 21 Consulting</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Author of Transforming School Culture. Global Gurus Top 30.</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Dr. Anthony Muhammad</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr"/>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr"/>
+      <c r="K375" t="inlineStr"/>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr"/>
+      <c r="N375" t="inlineStr">
+        <is>
+          <t>newfrontier21</t>
+        </is>
+      </c>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P375" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q375" t="inlineStr"/>
+      <c r="R375" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S375" t="inlineStr"/>
+      <c r="T375" t="inlineStr"/>
+      <c r="U375" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V375" t="inlineStr"/>
+      <c r="W375" t="inlineStr"/>
+      <c r="X375" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y375" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Jethro Jones</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Podcast Host &amp; Author</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Transformative Principal</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Host of longest-running ed leadership podcast. 2017 NASSP Digital Principal.</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr"/>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr"/>
+      <c r="H376" t="inlineStr"/>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr"/>
+      <c r="K376" t="inlineStr"/>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr"/>
+      <c r="N376" t="inlineStr">
+        <is>
+          <t>jethrojones</t>
+        </is>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P376" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q376" t="inlineStr"/>
+      <c r="R376" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S376" t="inlineStr"/>
+      <c r="T376" t="inlineStr"/>
+      <c r="U376" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V376" t="inlineStr"/>
+      <c r="W376" t="inlineStr"/>
+      <c r="X376" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Justin Baeder</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Director, The Principal Center</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>The Principal Center</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Author of Now We're Talking. Helped 10,000+ leaders in 50 countries.</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr"/>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr"/>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>principalcenter</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr"/>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr"/>
+      <c r="N377" t="inlineStr">
+        <is>
+          <t>eduleadership</t>
+        </is>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P377" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q377" t="inlineStr"/>
+      <c r="R377" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S377" t="inlineStr"/>
+      <c r="T377" t="inlineStr"/>
+      <c r="U377" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V377" t="inlineStr"/>
+      <c r="W377" t="inlineStr"/>
+      <c r="X377" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Dwight Carter</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Former Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>2013 NASSP Digital Principal of the Year. Author of Be GREAT.</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr"/>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr"/>
+      <c r="H378" t="inlineStr"/>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr"/>
+      <c r="K378" t="inlineStr"/>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr"/>
+      <c r="N378" t="inlineStr">
+        <is>
+          <t>Dwight_Carter</t>
+        </is>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P378" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q378" t="inlineStr"/>
+      <c r="R378" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S378" t="inlineStr"/>
+      <c r="T378" t="inlineStr"/>
+      <c r="U378" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V378" t="inlineStr"/>
+      <c r="W378" t="inlineStr"/>
+      <c r="X378" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Gerry Brooks</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Principal &amp; Educator-Comedian</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Educator</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Over 1.1M TikTok followers. Viral school humor videos.</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>gerrybrooksprin</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>gerrybrooksprin</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr"/>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr"/>
+      <c r="N379" t="inlineStr">
+        <is>
+          <t>gerrybrooksprin</t>
+        </is>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P379" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q379" t="inlineStr">
+        <is>
+          <t>gerrybrooksprin</t>
+        </is>
+      </c>
+      <c r="R379" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S379" t="inlineStr">
+        <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="T379" t="inlineStr"/>
+      <c r="U379" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V379" t="inlineStr"/>
+      <c r="W379" t="inlineStr"/>
+      <c r="X379" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Dr. Brad Johnson</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Education Speaker &amp; Author</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Education Speaker</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Global Gurus #3 in Education 2025. Author of 20+ books.</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>drbradjohnson</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>drbradjohnson</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr"/>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr"/>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>DrBradJohnson</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q380" t="inlineStr"/>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S380" t="inlineStr"/>
+      <c r="T380" t="inlineStr"/>
+      <c r="U380" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V380" t="inlineStr"/>
+      <c r="W380" t="inlineStr"/>
+      <c r="X380" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Peter DeWitt</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Former Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Instructional Leadership Collective</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>EdWeek Finding Common Ground blogger. Multiple Corwin books.</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr"/>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr"/>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>peter_dewitt518</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr"/>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr"/>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>PeterMDeWitt</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P381" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q381" t="inlineStr"/>
+      <c r="R381" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S381" t="inlineStr"/>
+      <c r="T381" t="inlineStr"/>
+      <c r="U381" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V381" t="inlineStr"/>
+      <c r="W381" t="inlineStr"/>
+      <c r="X381" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y381" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>George Couros</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Former School Admin &amp; Author</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Author</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Author of The Innovator's Mindset. Worldwide speaker.</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr"/>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr"/>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>gcouros</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr"/>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr"/>
+      <c r="N382" t="inlineStr">
+        <is>
+          <t>gcouros</t>
+        </is>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P382" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q382" t="inlineStr"/>
+      <c r="R382" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S382" t="inlineStr"/>
+      <c r="T382" t="inlineStr"/>
+      <c r="U382" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V382" t="inlineStr"/>
+      <c r="W382" t="inlineStr"/>
+      <c r="X382" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y382" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Salome Thomas-EL</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Award-Winning Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Author of I Choose to Stay. Eight-time national chess champions coach.</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr"/>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr"/>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>dr.principalel</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr"/>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr"/>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>Principal_EL</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P383" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q383" t="inlineStr"/>
+      <c r="R383" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S383" t="inlineStr"/>
+      <c r="T383" t="inlineStr"/>
+      <c r="U383" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V383" t="inlineStr"/>
+      <c r="W383" t="inlineStr"/>
+      <c r="X383" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y383" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Tony Cattani</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Principal, Lenape HS</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Lenape High School</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>NASSP 2025-26 National HS Principal of the Year. Proud Principals Podcast host.</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr"/>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr"/>
+      <c r="H384" t="inlineStr"/>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr"/>
+      <c r="K384" t="inlineStr"/>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr"/>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t>CattaniTony</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P384" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q384" t="inlineStr"/>
+      <c r="R384" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S384" t="inlineStr"/>
+      <c r="T384" t="inlineStr"/>
+      <c r="U384" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V384" t="inlineStr"/>
+      <c r="W384" t="inlineStr"/>
+      <c r="X384" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y384" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>William D. Parker</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Podcast Host &amp; Author</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Principal Matters LLC</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Host of Principal Matters podcast with 1.5M+ downloads.</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr"/>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr"/>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>william_d_parker</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr"/>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr"/>
+      <c r="N385" t="inlineStr"/>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P385" t="inlineStr"/>
+      <c r="Q385" t="inlineStr"/>
+      <c r="R385" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S385" t="inlineStr"/>
+      <c r="T385" t="inlineStr"/>
+      <c r="U385" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V385" t="inlineStr"/>
+      <c r="W385" t="inlineStr"/>
+      <c r="X385" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y385" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Deborah Netolicky</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Walford Anglican School for Girls</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Host of The Edu Salon podcast. Australian principal and PhD researcher.</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr"/>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr"/>
+      <c r="H386" t="inlineStr"/>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr"/>
+      <c r="K386" t="inlineStr"/>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr"/>
+      <c r="N386" t="inlineStr">
+        <is>
+          <t>debsnet</t>
+        </is>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P386" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q386" t="inlineStr"/>
+      <c r="R386" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S386" t="inlineStr"/>
+      <c r="T386" t="inlineStr"/>
+      <c r="U386" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V386" t="inlineStr"/>
+      <c r="W386" t="inlineStr"/>
+      <c r="X386" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y386" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Viviane Robinson</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Distinguished Professor</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>University of Auckland</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Author of Student-Centered Leadership. AERA Fellow.</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr"/>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr"/>
+      <c r="H387" t="inlineStr"/>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr"/>
+      <c r="K387" t="inlineStr"/>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr"/>
+      <c r="N387" t="inlineStr">
+        <is>
+          <t>RobinsonViviane</t>
+        </is>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P387" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q387" t="inlineStr"/>
+      <c r="R387" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S387" t="inlineStr"/>
+      <c r="T387" t="inlineStr"/>
+      <c r="U387" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V387" t="inlineStr"/>
+      <c r="W387" t="inlineStr"/>
+      <c r="X387" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Alma Harris</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Swansea University</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>World-leading distributed leadership researcher. Past President ICSEI.</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr"/>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr"/>
+      <c r="H388" t="inlineStr"/>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr"/>
+      <c r="K388" t="inlineStr"/>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr"/>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t>AlmaHarris1</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P388" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q388" t="inlineStr"/>
+      <c r="R388" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S388" t="inlineStr"/>
+      <c r="T388" t="inlineStr"/>
+      <c r="U388" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V388" t="inlineStr"/>
+      <c r="W388" t="inlineStr"/>
+      <c r="X388" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Dr. Gastrid Harrigan</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>High School Principal</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Broward County Public Schools</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Host of The School Leader's Podcast. Professor at Broward College.</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>gastrid.harrigan</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr"/>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr"/>
+      <c r="K389" t="inlineStr"/>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr"/>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t>DrGHarrigan</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P389" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q389" t="inlineStr"/>
+      <c r="R389" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S389" t="inlineStr"/>
+      <c r="T389" t="inlineStr"/>
+      <c r="U389" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V389" t="inlineStr"/>
+      <c r="W389" t="inlineStr"/>
+      <c r="X389" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Jeffrey Zoul</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Former Asst. Superintendent &amp; Author</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Educator &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Co-author of The Principled Principal. Leadership values expert.</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr"/>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr"/>
+      <c r="H390" t="inlineStr"/>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr"/>
+      <c r="K390" t="inlineStr"/>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr"/>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t>Jeff_Zoul</t>
+        </is>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P390" t="inlineStr">
+        <is>
+          <t>twitter</t>
+        </is>
+      </c>
+      <c r="Q390" t="inlineStr"/>
+      <c r="R390" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S390" t="inlineStr"/>
+      <c r="T390" t="inlineStr"/>
+      <c r="U390" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V390" t="inlineStr"/>
+      <c r="W390" t="inlineStr"/>
+      <c r="X390" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y390" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -23697,7 +24956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -24185,6 +25444,26 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>authentic-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>principal-leadership</t>
         </is>
       </c>
     </row>
@@ -24200,7 +25479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -30962,6 +32241,302 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>69c3c4a7ecfc8d3950f55cf3</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>2026-04-02T20:30:00Z</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>69c3c4a9dc7f763f71a52874</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>2026-04-02T20:30:00Z</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>69c3c4bdecfc8d3950f55e85</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>2026-04-02T12:45:00Z</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>69c3c4beecfc8d3950f55eaf</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>2026-04-02T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>69c3c4dbdc7f763f71a52aa7</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>2026-04-28T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>69c3c4ccecfc8d3950f55efd</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>2026-04-03T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>69c3c4ddecfc8d3950f55f3d</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>2026-04-28T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Principal Leadership</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>69c3c4dfdc7f763f71a52ace</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>2026-04-02T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update topics queue — add 20 engagement-optimized topics, revise queue 27-50
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Vulnerability in Leadership</t>
+          <t>Courage &amp; Vulnerability in Leadership</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1066,7 +1066,11 @@
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Search around Dare to Lead community, courage-based leadership practitioners</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1074,7 +1078,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>High-Performing Teams</t>
+          <t>Instructional Coaching</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1083,7 +1087,11 @@
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Education footer variant. Active niche: coaches in schools, PD specialists, edtech creators</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1100,7 +1108,11 @@
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Strong niche with own conferences, podcasts, and communities</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1108,7 +1120,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Leadership During Crisis</t>
+          <t>Neurodiversity in the Workplace</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1117,7 +1129,411 @@
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Growing niche with active creators, advocates, and workplace consultants</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Education footer variant. Patrick Lencioni's framework — active facilitator community</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Education footer variant. Active community of educators, wellbeing coordinators</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CliftonStrengths / Gallup community — very active coaches and creators</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Niche but growing: people who specifically help orgs fix meetings</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Nurse leaders, physician leaders, healthcare admin — distinct community</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Huge active community: pastors, ministry leaders, church planters</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Coaches, athlete development, sports psychology — active on social</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Introverted Leadership</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Niche but passionate community with active creators</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>IDEO/d.school community — practitioners, facilitators, creators</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Middle Management</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Growing niche: sandwich leaders, first-time directors, skip-level management</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Active community: IAF members, experience designers, session facilitators</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Meta-post: people who HOST leadership podcasts — they'll definitely reshare</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Veteran transition community — very engaged, active on social</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>EdTech Leadership</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Education footer variant. Tech-forward school leaders, LMS creators</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Positive Psychology in Leadership</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PERMA/flourishing community — researchers + practitioners</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Systems Thinking</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Distinct methodology community with active practitioners</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Succession Planning</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Niche HR/leadership topic with specialist consultants</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Cross-Cultural Leadership</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Global/expat leadership community — active international voices</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Mindful Leadership</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Meditation + leadership intersection — active wellness/leadership creators</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Leadership Book Authors 2024-2025</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Meta-post: people who published leadership books recently — they'll reshare</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E31"/>
@@ -23548,13 +23964,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K374" t="inlineStr"/>
       <c r="L374" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M374" t="inlineStr"/>
       <c r="N374" t="inlineStr">
         <is>
           <t>E_Sheninger</t>
@@ -23570,27 +23984,21 @@
           <t>website</t>
         </is>
       </c>
-      <c r="Q374" t="inlineStr"/>
       <c r="R374" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S374" t="inlineStr"/>
-      <c r="T374" t="inlineStr"/>
       <c r="U374" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V374" t="inlineStr"/>
-      <c r="W374" t="inlineStr"/>
       <c r="X374" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -23628,20 +24036,16 @@
           <t>facebook</t>
         </is>
       </c>
-      <c r="H375" t="inlineStr"/>
       <c r="I375" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J375" t="inlineStr"/>
-      <c r="K375" t="inlineStr"/>
       <c r="L375" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M375" t="inlineStr"/>
       <c r="N375" t="inlineStr">
         <is>
           <t>newfrontier21</t>
@@ -23657,27 +24061,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q375" t="inlineStr"/>
       <c r="R375" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S375" t="inlineStr"/>
-      <c r="T375" t="inlineStr"/>
       <c r="U375" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V375" t="inlineStr"/>
-      <c r="W375" t="inlineStr"/>
       <c r="X375" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -23700,27 +24098,21 @@
           <t>Host of longest-running ed leadership podcast. 2017 NASSP Digital Principal.</t>
         </is>
       </c>
-      <c r="E376" t="inlineStr"/>
       <c r="F376" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G376" t="inlineStr"/>
-      <c r="H376" t="inlineStr"/>
       <c r="I376" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J376" t="inlineStr"/>
-      <c r="K376" t="inlineStr"/>
       <c r="L376" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M376" t="inlineStr"/>
       <c r="N376" t="inlineStr">
         <is>
           <t>jethrojones</t>
@@ -23736,27 +24128,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q376" t="inlineStr"/>
       <c r="R376" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S376" t="inlineStr"/>
-      <c r="T376" t="inlineStr"/>
       <c r="U376" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V376" t="inlineStr"/>
-      <c r="W376" t="inlineStr"/>
       <c r="X376" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -23779,13 +24165,11 @@
           <t>Author of Now We're Talking. Helped 10,000+ leaders in 50 countries.</t>
         </is>
       </c>
-      <c r="E377" t="inlineStr"/>
       <c r="F377" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G377" t="inlineStr"/>
       <c r="H377" t="inlineStr">
         <is>
           <t>principalcenter</t>
@@ -23801,13 +24185,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K377" t="inlineStr"/>
       <c r="L377" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M377" t="inlineStr"/>
       <c r="N377" t="inlineStr">
         <is>
           <t>eduleadership</t>
@@ -23823,27 +24205,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q377" t="inlineStr"/>
       <c r="R377" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S377" t="inlineStr"/>
-      <c r="T377" t="inlineStr"/>
       <c r="U377" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V377" t="inlineStr"/>
-      <c r="W377" t="inlineStr"/>
       <c r="X377" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -23866,27 +24242,21 @@
           <t>2013 NASSP Digital Principal of the Year. Author of Be GREAT.</t>
         </is>
       </c>
-      <c r="E378" t="inlineStr"/>
       <c r="F378" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G378" t="inlineStr"/>
-      <c r="H378" t="inlineStr"/>
       <c r="I378" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J378" t="inlineStr"/>
-      <c r="K378" t="inlineStr"/>
       <c r="L378" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M378" t="inlineStr"/>
       <c r="N378" t="inlineStr">
         <is>
           <t>Dwight_Carter</t>
@@ -23902,27 +24272,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q378" t="inlineStr"/>
       <c r="R378" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S378" t="inlineStr"/>
-      <c r="T378" t="inlineStr"/>
       <c r="U378" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V378" t="inlineStr"/>
-      <c r="W378" t="inlineStr"/>
       <c r="X378" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -23975,13 +24339,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K379" t="inlineStr"/>
       <c r="L379" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M379" t="inlineStr"/>
       <c r="N379" t="inlineStr">
         <is>
           <t>gerrybrooksprin</t>
@@ -24012,20 +24374,16 @@
           <t>tiktok</t>
         </is>
       </c>
-      <c r="T379" t="inlineStr"/>
       <c r="U379" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V379" t="inlineStr"/>
-      <c r="W379" t="inlineStr"/>
       <c r="X379" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -24078,13 +24436,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K380" t="inlineStr"/>
       <c r="L380" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M380" t="inlineStr"/>
       <c r="N380" t="inlineStr">
         <is>
           <t>DrBradJohnson</t>
@@ -24100,27 +24456,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q380" t="inlineStr"/>
       <c r="R380" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S380" t="inlineStr"/>
-      <c r="T380" t="inlineStr"/>
       <c r="U380" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V380" t="inlineStr"/>
-      <c r="W380" t="inlineStr"/>
       <c r="X380" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -24143,13 +24493,11 @@
           <t>EdWeek Finding Common Ground blogger. Multiple Corwin books.</t>
         </is>
       </c>
-      <c r="E381" t="inlineStr"/>
       <c r="F381" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G381" t="inlineStr"/>
       <c r="H381" t="inlineStr">
         <is>
           <t>peter_dewitt518</t>
@@ -24165,13 +24513,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K381" t="inlineStr"/>
       <c r="L381" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M381" t="inlineStr"/>
       <c r="N381" t="inlineStr">
         <is>
           <t>PeterMDeWitt</t>
@@ -24187,27 +24533,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q381" t="inlineStr"/>
       <c r="R381" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S381" t="inlineStr"/>
-      <c r="T381" t="inlineStr"/>
       <c r="U381" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V381" t="inlineStr"/>
-      <c r="W381" t="inlineStr"/>
       <c r="X381" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -24230,13 +24570,11 @@
           <t>Author of The Innovator's Mindset. Worldwide speaker.</t>
         </is>
       </c>
-      <c r="E382" t="inlineStr"/>
       <c r="F382" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G382" t="inlineStr"/>
       <c r="H382" t="inlineStr">
         <is>
           <t>gcouros</t>
@@ -24252,13 +24590,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K382" t="inlineStr"/>
       <c r="L382" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M382" t="inlineStr"/>
       <c r="N382" t="inlineStr">
         <is>
           <t>gcouros</t>
@@ -24274,27 +24610,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q382" t="inlineStr"/>
       <c r="R382" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S382" t="inlineStr"/>
-      <c r="T382" t="inlineStr"/>
       <c r="U382" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V382" t="inlineStr"/>
-      <c r="W382" t="inlineStr"/>
       <c r="X382" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -24317,13 +24647,11 @@
           <t>Author of I Choose to Stay. Eight-time national chess champions coach.</t>
         </is>
       </c>
-      <c r="E383" t="inlineStr"/>
       <c r="F383" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G383" t="inlineStr"/>
       <c r="H383" t="inlineStr">
         <is>
           <t>dr.principalel</t>
@@ -24339,13 +24667,11 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K383" t="inlineStr"/>
       <c r="L383" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M383" t="inlineStr"/>
       <c r="N383" t="inlineStr">
         <is>
           <t>Principal_EL</t>
@@ -24361,27 +24687,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q383" t="inlineStr"/>
       <c r="R383" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S383" t="inlineStr"/>
-      <c r="T383" t="inlineStr"/>
       <c r="U383" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V383" t="inlineStr"/>
-      <c r="W383" t="inlineStr"/>
       <c r="X383" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -24404,27 +24724,21 @@
           <t>NASSP 2025-26 National HS Principal of the Year. Proud Principals Podcast host.</t>
         </is>
       </c>
-      <c r="E384" t="inlineStr"/>
       <c r="F384" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G384" t="inlineStr"/>
-      <c r="H384" t="inlineStr"/>
       <c r="I384" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="J384" t="inlineStr"/>
-      <c r="K384" t="inlineStr"/>
       <c r="L384" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M384" t="inlineStr"/>
       <c r="N384" t="inlineStr">
         <is>
           <t>CattaniTony</t>
@@ -24440,27 +24754,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q384" t="inlineStr"/>
       <c r="R384" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S384" t="inlineStr"/>
-      <c r="T384" t="inlineStr"/>
       <c r="U384" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V384" t="inlineStr"/>
-      <c r="W384" t="inlineStr"/>
       <c r="X384" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -24483,13 +24791,11 @@
           <t>Host of Principal Matters podcast with 1.5M+ downloads.</t>
         </is>
       </c>
-      <c r="E385" t="inlineStr"/>
       <c r="F385" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G385" t="inlineStr"/>
       <c r="H385" t="inlineStr">
         <is>
           <t>william_d_parker</t>
@@ -24505,41 +24811,31 @@
           <t>instagram</t>
         </is>
       </c>
-      <c r="K385" t="inlineStr"/>
       <c r="L385" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M385" t="inlineStr"/>
-      <c r="N385" t="inlineStr"/>
       <c r="O385" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P385" t="inlineStr"/>
-      <c r="Q385" t="inlineStr"/>
       <c r="R385" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S385" t="inlineStr"/>
-      <c r="T385" t="inlineStr"/>
       <c r="U385" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V385" t="inlineStr"/>
-      <c r="W385" t="inlineStr"/>
       <c r="X385" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -24562,27 +24858,21 @@
           <t>Host of The Edu Salon podcast. Australian principal and PhD researcher.</t>
         </is>
       </c>
-      <c r="E386" t="inlineStr"/>
       <c r="F386" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G386" t="inlineStr"/>
-      <c r="H386" t="inlineStr"/>
       <c r="I386" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J386" t="inlineStr"/>
-      <c r="K386" t="inlineStr"/>
       <c r="L386" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M386" t="inlineStr"/>
       <c r="N386" t="inlineStr">
         <is>
           <t>debsnet</t>
@@ -24598,27 +24888,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q386" t="inlineStr"/>
       <c r="R386" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S386" t="inlineStr"/>
-      <c r="T386" t="inlineStr"/>
       <c r="U386" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V386" t="inlineStr"/>
-      <c r="W386" t="inlineStr"/>
       <c r="X386" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -24641,27 +24925,21 @@
           <t>Author of Student-Centered Leadership. AERA Fellow.</t>
         </is>
       </c>
-      <c r="E387" t="inlineStr"/>
       <c r="F387" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G387" t="inlineStr"/>
-      <c r="H387" t="inlineStr"/>
       <c r="I387" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J387" t="inlineStr"/>
-      <c r="K387" t="inlineStr"/>
       <c r="L387" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M387" t="inlineStr"/>
       <c r="N387" t="inlineStr">
         <is>
           <t>RobinsonViviane</t>
@@ -24677,27 +24955,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q387" t="inlineStr"/>
       <c r="R387" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S387" t="inlineStr"/>
-      <c r="T387" t="inlineStr"/>
       <c r="U387" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V387" t="inlineStr"/>
-      <c r="W387" t="inlineStr"/>
       <c r="X387" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -24720,27 +24992,21 @@
           <t>World-leading distributed leadership researcher. Past President ICSEI.</t>
         </is>
       </c>
-      <c r="E388" t="inlineStr"/>
       <c r="F388" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G388" t="inlineStr"/>
-      <c r="H388" t="inlineStr"/>
       <c r="I388" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J388" t="inlineStr"/>
-      <c r="K388" t="inlineStr"/>
       <c r="L388" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M388" t="inlineStr"/>
       <c r="N388" t="inlineStr">
         <is>
           <t>AlmaHarris1</t>
@@ -24756,27 +25022,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q388" t="inlineStr"/>
       <c r="R388" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S388" t="inlineStr"/>
-      <c r="T388" t="inlineStr"/>
       <c r="U388" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V388" t="inlineStr"/>
-      <c r="W388" t="inlineStr"/>
       <c r="X388" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -24814,20 +25074,16 @@
           <t>facebook</t>
         </is>
       </c>
-      <c r="H389" t="inlineStr"/>
       <c r="I389" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="J389" t="inlineStr"/>
-      <c r="K389" t="inlineStr"/>
       <c r="L389" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M389" t="inlineStr"/>
       <c r="N389" t="inlineStr">
         <is>
           <t>DrGHarrigan</t>
@@ -24843,27 +25099,21 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q389" t="inlineStr"/>
       <c r="R389" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S389" t="inlineStr"/>
-      <c r="T389" t="inlineStr"/>
       <c r="U389" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V389" t="inlineStr"/>
-      <c r="W389" t="inlineStr"/>
       <c r="X389" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -24886,27 +25136,21 @@
           <t>Co-author of The Principled Principal. Leadership values expert.</t>
         </is>
       </c>
-      <c r="E390" t="inlineStr"/>
       <c r="F390" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G390" t="inlineStr"/>
-      <c r="H390" t="inlineStr"/>
       <c r="I390" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J390" t="inlineStr"/>
-      <c r="K390" t="inlineStr"/>
       <c r="L390" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M390" t="inlineStr"/>
       <c r="N390" t="inlineStr">
         <is>
           <t>Jeff_Zoul</t>
@@ -24922,27 +25166,21 @@
           <t>twitter</t>
         </is>
       </c>
-      <c r="Q390" t="inlineStr"/>
       <c r="R390" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S390" t="inlineStr"/>
-      <c r="T390" t="inlineStr"/>
       <c r="U390" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V390" t="inlineStr"/>
-      <c r="W390" t="inlineStr"/>
       <c r="X390" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y390" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>

</xml_diff>

<commit_message>
Update handle database — Courage & Vulnerability in Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1062,10 +1062,14 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Search around Dare to Lead community, courage-based leadership practitioners</t>
@@ -1547,7 +1551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y390"/>
+  <dimension ref="A1:Y406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -25182,6 +25186,1302 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Jim Detert</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Professor of Business Admin</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>UVA Darden School of Business</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>World's foremost expert on workplace courage. Author of Choosing Courage (HBR Press).</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr"/>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr"/>
+      <c r="H391" t="inlineStr"/>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr"/>
+      <c r="K391" t="inlineStr"/>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr"/>
+      <c r="N391" t="inlineStr"/>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P391" t="inlineStr"/>
+      <c r="Q391" t="inlineStr"/>
+      <c r="R391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S391" t="inlineStr"/>
+      <c r="T391" t="inlineStr"/>
+      <c r="U391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V391" t="inlineStr"/>
+      <c r="W391" t="inlineStr"/>
+      <c r="X391" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Jacob Morgan</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>5x Bestselling Author &amp; Futurist</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>The Future Organization</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Author of Leading with Vulnerability. Interviewed 100+ CEOs, surveyed 14,000 employees.</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr"/>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr"/>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>jacobmorgan8</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr"/>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr"/>
+      <c r="N392" t="inlineStr"/>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P392" t="inlineStr"/>
+      <c r="Q392" t="inlineStr"/>
+      <c r="R392" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S392" t="inlineStr"/>
+      <c r="T392" t="inlineStr"/>
+      <c r="U392" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V392" t="inlineStr"/>
+      <c r="W392" t="inlineStr"/>
+      <c r="X392" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Bill Treasurer</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>CEO &amp; Chief Encouragement Officer</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Giant Leap Consulting</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Pioneer of courage-building as org development. Author of Courage Goes to Work. 6 books.</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr"/>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr"/>
+      <c r="H393" t="inlineStr"/>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr"/>
+      <c r="K393" t="inlineStr"/>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr"/>
+      <c r="N393" t="inlineStr"/>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P393" t="inlineStr"/>
+      <c r="Q393" t="inlineStr"/>
+      <c r="R393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S393" t="inlineStr"/>
+      <c r="T393" t="inlineStr"/>
+      <c r="U393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V393" t="inlineStr"/>
+      <c r="W393" t="inlineStr"/>
+      <c r="X393" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Cindy Solomon</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Courageous Leadership Institute</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>TED talks 3M+ views. Global Gurus Top 10. Courage frameworks for Google, Gates Foundation.</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>CindySolomonAssociates</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr"/>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr"/>
+      <c r="K394" t="inlineStr"/>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr"/>
+      <c r="N394" t="inlineStr"/>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P394" t="inlineStr"/>
+      <c r="Q394" t="inlineStr"/>
+      <c r="R394" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S394" t="inlineStr"/>
+      <c r="T394" t="inlineStr"/>
+      <c r="U394" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V394" t="inlineStr"/>
+      <c r="W394" t="inlineStr"/>
+      <c r="X394" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Margie Warrell</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>5x Bestselling Author &amp; Courage Expert</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Dr Margie Warrell</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Australia's leading voice on brave leadership. Author of The Courage Gap, Stop Playing Safe.</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>margiewarrell</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>margiewarrell</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr"/>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr"/>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>margiewarrell</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P395" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q395" t="inlineStr"/>
+      <c r="R395" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S395" t="inlineStr"/>
+      <c r="T395" t="inlineStr">
+        <is>
+          <t>margiewarrell</t>
+        </is>
+      </c>
+      <c r="U395" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V395" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="W395" t="inlineStr"/>
+      <c r="X395" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y395" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Ryan Holiday</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Author &amp; Host</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Daily Stoic</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Author of Courage Is Calling (Stoic Virtues Series). Brought stoic courage to millions.</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr"/>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr"/>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>ryanholiday</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr"/>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr"/>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>RyanHoliday</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P396" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q396" t="inlineStr">
+        <is>
+          <t>ryan_holiday</t>
+        </is>
+      </c>
+      <c r="R396" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t>TikTok profile</t>
+        </is>
+      </c>
+      <c r="T396" t="inlineStr">
+        <is>
+          <t>dailystoic</t>
+        </is>
+      </c>
+      <c r="U396" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>YouTube channel</t>
+        </is>
+      </c>
+      <c r="W396" t="inlineStr"/>
+      <c r="X396" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Karin Hurt</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Let's Grow Leaders</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Co-author of Courageous Cultures. Inc Top 100 Leadership Speaker. Helps teams speak up.</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr"/>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr"/>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>karinbhurt</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr"/>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr"/>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>LetsGrowLeaders</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P397" t="inlineStr">
+        <is>
+          <t>Twitter (shared)</t>
+        </is>
+      </c>
+      <c r="Q397" t="inlineStr"/>
+      <c r="R397" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S397" t="inlineStr"/>
+      <c r="T397" t="inlineStr"/>
+      <c r="U397" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V397" t="inlineStr"/>
+      <c r="W397" t="inlineStr"/>
+      <c r="X397" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y397" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>David Dye</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Let's Grow Leaders</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Co-author of Courageous Cultures and Winning Well. Builds cultures where people share ideas.</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr"/>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr"/>
+      <c r="H398" t="inlineStr"/>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr"/>
+      <c r="K398" t="inlineStr"/>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr"/>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>LetsGrowLeaders</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P398" t="inlineStr">
+        <is>
+          <t>Twitter (shared)</t>
+        </is>
+      </c>
+      <c r="Q398" t="inlineStr"/>
+      <c r="R398" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S398" t="inlineStr"/>
+      <c r="T398" t="inlineStr"/>
+      <c r="U398" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V398" t="inlineStr"/>
+      <c r="W398" t="inlineStr"/>
+      <c r="X398" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y398" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Jill Schulman</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Founder, Breakthrough Leadership Group</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>USMC Veteran &amp; Bravery Expert</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Former Marine turned positive psychology practitioner. Author of The Bravery Effect.</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr"/>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr"/>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>jillschulman</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr"/>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr"/>
+      <c r="N399" t="inlineStr"/>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P399" t="inlineStr"/>
+      <c r="Q399" t="inlineStr"/>
+      <c r="R399" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S399" t="inlineStr"/>
+      <c r="T399" t="inlineStr"/>
+      <c r="U399" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V399" t="inlineStr"/>
+      <c r="W399" t="inlineStr"/>
+      <c r="X399" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Kathy Caprino</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Finding Brave / Kathy Caprino LLC</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Author of The Most Powerful You. Finding Brave podcast (Top 100 Apple). Champions bravery for women.</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr"/>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr"/>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>kathycaprino</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Instagram profile</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr"/>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr"/>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>kathycaprino</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P400" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q400" t="inlineStr"/>
+      <c r="R400" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S400" t="inlineStr"/>
+      <c r="T400" t="inlineStr"/>
+      <c r="U400" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V400" t="inlineStr"/>
+      <c r="W400" t="inlineStr"/>
+      <c r="X400" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y400" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Margareta Kull</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Kull Leadership AB</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>20+ years training leaders from 30+ countries to make courageous decisions. Based in Sweden.</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr"/>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr"/>
+      <c r="H401" t="inlineStr"/>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr"/>
+      <c r="K401" t="inlineStr"/>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr"/>
+      <c r="N401" t="inlineStr"/>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P401" t="inlineStr"/>
+      <c r="Q401" t="inlineStr"/>
+      <c r="R401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S401" t="inlineStr"/>
+      <c r="T401" t="inlineStr"/>
+      <c r="U401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V401" t="inlineStr"/>
+      <c r="W401" t="inlineStr"/>
+      <c r="X401" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Annabel Beerel</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Author &amp; Executive Consultant</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Author of Courage: The Heart of Leadership (Routledge, 2025). 10 books. Former AI CEO.</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr"/>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr"/>
+      <c r="H402" t="inlineStr"/>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr"/>
+      <c r="K402" t="inlineStr"/>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr"/>
+      <c r="N402" t="inlineStr"/>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P402" t="inlineStr"/>
+      <c r="Q402" t="inlineStr"/>
+      <c r="R402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S402" t="inlineStr"/>
+      <c r="T402" t="inlineStr"/>
+      <c r="U402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V402" t="inlineStr"/>
+      <c r="W402" t="inlineStr"/>
+      <c r="X402" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y402" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Angela Sebaly</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Personify Leadership</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Author of The Courageous Leader (Wiley). Created Spine of a Leader framework.</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>asebaly</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr"/>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr"/>
+      <c r="K403" t="inlineStr"/>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr"/>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>AngelaSebaly</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P403" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q403" t="inlineStr"/>
+      <c r="R403" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S403" t="inlineStr"/>
+      <c r="T403" t="inlineStr"/>
+      <c r="U403" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V403" t="inlineStr"/>
+      <c r="W403" t="inlineStr"/>
+      <c r="X403" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y403" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>David McQueen</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Author &amp; 3x TEDx Speaker</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Q Squared Ltd</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Author of The BRAVE Leader. Hosts BRAVE Leader podcast. Coaches at Google, Bloomberg, JPM.</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr"/>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr"/>
+      <c r="H404" t="inlineStr"/>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr"/>
+      <c r="K404" t="inlineStr"/>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr"/>
+      <c r="N404" t="inlineStr"/>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P404" t="inlineStr"/>
+      <c r="Q404" t="inlineStr"/>
+      <c r="R404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S404" t="inlineStr"/>
+      <c r="T404" t="inlineStr"/>
+      <c r="U404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V404" t="inlineStr"/>
+      <c r="W404" t="inlineStr"/>
+      <c r="X404" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y404" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Michelle Gibbings</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Certified Dare to Lead Facilitator</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Michelle Gibbings Pty Ltd</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Award-winning Australian author and workplace expert. 3 books. Helps build courage-driven cultures.</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>MichelleGibbing</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr"/>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr"/>
+      <c r="K405" t="inlineStr"/>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr"/>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>MichelleGibbing</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P405" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q405" t="inlineStr"/>
+      <c r="R405" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S405" t="inlineStr"/>
+      <c r="T405" t="inlineStr"/>
+      <c r="U405" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V405" t="inlineStr"/>
+      <c r="W405" t="inlineStr"/>
+      <c r="X405" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y405" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Manley Hopkinson</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Compassionate Leadership Academy</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Ex-Royal Navy officer, ocean rower. Author of Compassionate Leadership. Courage through adventure.</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr"/>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr"/>
+      <c r="H406" t="inlineStr"/>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr"/>
+      <c r="K406" t="inlineStr"/>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr"/>
+      <c r="N406" t="inlineStr"/>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P406" t="inlineStr"/>
+      <c r="Q406" t="inlineStr"/>
+      <c r="R406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S406" t="inlineStr"/>
+      <c r="T406" t="inlineStr"/>
+      <c r="U406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V406" t="inlineStr"/>
+      <c r="W406" t="inlineStr"/>
+      <c r="X406" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y406" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25194,7 +26494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -25702,6 +27002,26 @@
       <c r="D25" t="inlineStr">
         <is>
           <t>principal-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>17</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>courage-vulnerability-leadership</t>
         </is>
       </c>
     </row>
@@ -25717,7 +27037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G193"/>
+  <dimension ref="A1:G201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -32775,6 +34095,302 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>69c3d1cddc7f763f71a5895a</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>2026-04-03T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>69c3d1cfecfc8d3950f5b9d4</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>2026-04-03T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>69c3d1eaecfc8d3950f5bb01</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>2026-03-29T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>69c3d1eddc7f763f71a58b45</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>2026-04-03T03:01:00Z</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>69c3d1eedc7f763f71a58b6b</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>2026-04-03T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>69c3d1eeecfc8d3950f5bb9d</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>2026-04-03T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>69c3d1fddc7f763f71a58beb</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>2026-04-30T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>69c3d200ecfc8d3950f5bc13</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>2026-04-03T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx — Instructional Coaching
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1087,10 +1087,14 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Education footer variant. Active niche: coaches in schools, PD specialists, edtech creators</t>
@@ -1551,7 +1555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y406"/>
+  <dimension ref="A1:Y421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -25207,55 +25211,41 @@
           <t>World's foremost expert on workplace courage. Author of Choosing Courage (HBR Press).</t>
         </is>
       </c>
-      <c r="E391" t="inlineStr"/>
       <c r="F391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G391" t="inlineStr"/>
-      <c r="H391" t="inlineStr"/>
       <c r="I391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J391" t="inlineStr"/>
-      <c r="K391" t="inlineStr"/>
       <c r="L391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M391" t="inlineStr"/>
-      <c r="N391" t="inlineStr"/>
       <c r="O391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P391" t="inlineStr"/>
-      <c r="Q391" t="inlineStr"/>
       <c r="R391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S391" t="inlineStr"/>
-      <c r="T391" t="inlineStr"/>
       <c r="U391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V391" t="inlineStr"/>
-      <c r="W391" t="inlineStr"/>
       <c r="X391" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -25278,13 +25268,11 @@
           <t>Author of Leading with Vulnerability. Interviewed 100+ CEOs, surveyed 14,000 employees.</t>
         </is>
       </c>
-      <c r="E392" t="inlineStr"/>
       <c r="F392" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G392" t="inlineStr"/>
       <c r="H392" t="inlineStr">
         <is>
           <t>jacobmorgan8</t>
@@ -25300,41 +25288,31 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K392" t="inlineStr"/>
       <c r="L392" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M392" t="inlineStr"/>
-      <c r="N392" t="inlineStr"/>
       <c r="O392" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P392" t="inlineStr"/>
-      <c r="Q392" t="inlineStr"/>
       <c r="R392" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S392" t="inlineStr"/>
-      <c r="T392" t="inlineStr"/>
       <c r="U392" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V392" t="inlineStr"/>
-      <c r="W392" t="inlineStr"/>
       <c r="X392" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -25357,55 +25335,41 @@
           <t>Pioneer of courage-building as org development. Author of Courage Goes to Work. 6 books.</t>
         </is>
       </c>
-      <c r="E393" t="inlineStr"/>
       <c r="F393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G393" t="inlineStr"/>
-      <c r="H393" t="inlineStr"/>
       <c r="I393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J393" t="inlineStr"/>
-      <c r="K393" t="inlineStr"/>
       <c r="L393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M393" t="inlineStr"/>
-      <c r="N393" t="inlineStr"/>
       <c r="O393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P393" t="inlineStr"/>
-      <c r="Q393" t="inlineStr"/>
       <c r="R393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S393" t="inlineStr"/>
-      <c r="T393" t="inlineStr"/>
       <c r="U393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V393" t="inlineStr"/>
-      <c r="W393" t="inlineStr"/>
       <c r="X393" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -25443,48 +25407,36 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H394" t="inlineStr"/>
       <c r="I394" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J394" t="inlineStr"/>
-      <c r="K394" t="inlineStr"/>
       <c r="L394" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M394" t="inlineStr"/>
-      <c r="N394" t="inlineStr"/>
       <c r="O394" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P394" t="inlineStr"/>
-      <c r="Q394" t="inlineStr"/>
       <c r="R394" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S394" t="inlineStr"/>
-      <c r="T394" t="inlineStr"/>
       <c r="U394" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V394" t="inlineStr"/>
-      <c r="W394" t="inlineStr"/>
       <c r="X394" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -25537,13 +25489,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K395" t="inlineStr"/>
       <c r="L395" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M395" t="inlineStr"/>
       <c r="N395" t="inlineStr">
         <is>
           <t>margiewarrell</t>
@@ -25559,13 +25509,11 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q395" t="inlineStr"/>
       <c r="R395" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S395" t="inlineStr"/>
       <c r="T395" t="inlineStr">
         <is>
           <t>margiewarrell</t>
@@ -25581,13 +25529,11 @@
           <t>YouTube channel</t>
         </is>
       </c>
-      <c r="W395" t="inlineStr"/>
       <c r="X395" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -25610,13 +25556,11 @@
           <t>Author of Courage Is Calling (Stoic Virtues Series). Brought stoic courage to millions.</t>
         </is>
       </c>
-      <c r="E396" t="inlineStr"/>
       <c r="F396" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="G396" t="inlineStr"/>
       <c r="H396" t="inlineStr">
         <is>
           <t>ryanholiday</t>
@@ -25632,13 +25576,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K396" t="inlineStr"/>
       <c r="L396" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M396" t="inlineStr"/>
       <c r="N396" t="inlineStr">
         <is>
           <t>RyanHoliday</t>
@@ -25684,13 +25626,11 @@
           <t>YouTube channel</t>
         </is>
       </c>
-      <c r="W396" t="inlineStr"/>
       <c r="X396" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -25713,13 +25653,11 @@
           <t>Co-author of Courageous Cultures. Inc Top 100 Leadership Speaker. Helps teams speak up.</t>
         </is>
       </c>
-      <c r="E397" t="inlineStr"/>
       <c r="F397" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G397" t="inlineStr"/>
       <c r="H397" t="inlineStr">
         <is>
           <t>karinbhurt</t>
@@ -25735,13 +25673,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K397" t="inlineStr"/>
       <c r="L397" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M397" t="inlineStr"/>
       <c r="N397" t="inlineStr">
         <is>
           <t>LetsGrowLeaders</t>
@@ -25757,27 +25693,21 @@
           <t>Twitter (shared)</t>
         </is>
       </c>
-      <c r="Q397" t="inlineStr"/>
       <c r="R397" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S397" t="inlineStr"/>
-      <c r="T397" t="inlineStr"/>
       <c r="U397" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V397" t="inlineStr"/>
-      <c r="W397" t="inlineStr"/>
       <c r="X397" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -25800,27 +25730,21 @@
           <t>Co-author of Courageous Cultures and Winning Well. Builds cultures where people share ideas.</t>
         </is>
       </c>
-      <c r="E398" t="inlineStr"/>
       <c r="F398" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G398" t="inlineStr"/>
-      <c r="H398" t="inlineStr"/>
       <c r="I398" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J398" t="inlineStr"/>
-      <c r="K398" t="inlineStr"/>
       <c r="L398" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M398" t="inlineStr"/>
       <c r="N398" t="inlineStr">
         <is>
           <t>LetsGrowLeaders</t>
@@ -25836,27 +25760,21 @@
           <t>Twitter (shared)</t>
         </is>
       </c>
-      <c r="Q398" t="inlineStr"/>
       <c r="R398" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S398" t="inlineStr"/>
-      <c r="T398" t="inlineStr"/>
       <c r="U398" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V398" t="inlineStr"/>
-      <c r="W398" t="inlineStr"/>
       <c r="X398" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -25879,13 +25797,11 @@
           <t>Former Marine turned positive psychology practitioner. Author of The Bravery Effect.</t>
         </is>
       </c>
-      <c r="E399" t="inlineStr"/>
       <c r="F399" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="G399" t="inlineStr"/>
       <c r="H399" t="inlineStr">
         <is>
           <t>jillschulman</t>
@@ -25901,41 +25817,31 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K399" t="inlineStr"/>
       <c r="L399" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M399" t="inlineStr"/>
-      <c r="N399" t="inlineStr"/>
       <c r="O399" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P399" t="inlineStr"/>
-      <c r="Q399" t="inlineStr"/>
       <c r="R399" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S399" t="inlineStr"/>
-      <c r="T399" t="inlineStr"/>
       <c r="U399" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="V399" t="inlineStr"/>
-      <c r="W399" t="inlineStr"/>
       <c r="X399" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -25958,13 +25864,11 @@
           <t>Author of The Most Powerful You. Finding Brave podcast (Top 100 Apple). Champions bravery for women.</t>
         </is>
       </c>
-      <c r="E400" t="inlineStr"/>
       <c r="F400" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="G400" t="inlineStr"/>
       <c r="H400" t="inlineStr">
         <is>
           <t>kathycaprino</t>
@@ -25980,13 +25884,11 @@
           <t>Instagram profile</t>
         </is>
       </c>
-      <c r="K400" t="inlineStr"/>
       <c r="L400" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M400" t="inlineStr"/>
       <c r="N400" t="inlineStr">
         <is>
           <t>kathycaprino</t>
@@ -26002,27 +25904,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q400" t="inlineStr"/>
       <c r="R400" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S400" t="inlineStr"/>
-      <c r="T400" t="inlineStr"/>
       <c r="U400" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="V400" t="inlineStr"/>
-      <c r="W400" t="inlineStr"/>
       <c r="X400" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -26045,55 +25941,41 @@
           <t>20+ years training leaders from 30+ countries to make courageous decisions. Based in Sweden.</t>
         </is>
       </c>
-      <c r="E401" t="inlineStr"/>
       <c r="F401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G401" t="inlineStr"/>
-      <c r="H401" t="inlineStr"/>
       <c r="I401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J401" t="inlineStr"/>
-      <c r="K401" t="inlineStr"/>
       <c r="L401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M401" t="inlineStr"/>
-      <c r="N401" t="inlineStr"/>
       <c r="O401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P401" t="inlineStr"/>
-      <c r="Q401" t="inlineStr"/>
       <c r="R401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S401" t="inlineStr"/>
-      <c r="T401" t="inlineStr"/>
       <c r="U401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V401" t="inlineStr"/>
-      <c r="W401" t="inlineStr"/>
       <c r="X401" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -26116,55 +25998,41 @@
           <t>Author of Courage: The Heart of Leadership (Routledge, 2025). 10 books. Former AI CEO.</t>
         </is>
       </c>
-      <c r="E402" t="inlineStr"/>
       <c r="F402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G402" t="inlineStr"/>
-      <c r="H402" t="inlineStr"/>
       <c r="I402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J402" t="inlineStr"/>
-      <c r="K402" t="inlineStr"/>
       <c r="L402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M402" t="inlineStr"/>
-      <c r="N402" t="inlineStr"/>
       <c r="O402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P402" t="inlineStr"/>
-      <c r="Q402" t="inlineStr"/>
       <c r="R402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S402" t="inlineStr"/>
-      <c r="T402" t="inlineStr"/>
       <c r="U402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V402" t="inlineStr"/>
-      <c r="W402" t="inlineStr"/>
       <c r="X402" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -26202,20 +26070,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H403" t="inlineStr"/>
       <c r="I403" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J403" t="inlineStr"/>
-      <c r="K403" t="inlineStr"/>
       <c r="L403" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M403" t="inlineStr"/>
       <c r="N403" t="inlineStr">
         <is>
           <t>AngelaSebaly</t>
@@ -26231,27 +26095,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q403" t="inlineStr"/>
       <c r="R403" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S403" t="inlineStr"/>
-      <c r="T403" t="inlineStr"/>
       <c r="U403" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V403" t="inlineStr"/>
-      <c r="W403" t="inlineStr"/>
       <c r="X403" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -26274,55 +26132,41 @@
           <t>Author of The BRAVE Leader. Hosts BRAVE Leader podcast. Coaches at Google, Bloomberg, JPM.</t>
         </is>
       </c>
-      <c r="E404" t="inlineStr"/>
       <c r="F404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G404" t="inlineStr"/>
-      <c r="H404" t="inlineStr"/>
       <c r="I404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J404" t="inlineStr"/>
-      <c r="K404" t="inlineStr"/>
       <c r="L404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M404" t="inlineStr"/>
-      <c r="N404" t="inlineStr"/>
       <c r="O404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P404" t="inlineStr"/>
-      <c r="Q404" t="inlineStr"/>
       <c r="R404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S404" t="inlineStr"/>
-      <c r="T404" t="inlineStr"/>
       <c r="U404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V404" t="inlineStr"/>
-      <c r="W404" t="inlineStr"/>
       <c r="X404" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -26360,20 +26204,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H405" t="inlineStr"/>
       <c r="I405" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J405" t="inlineStr"/>
-      <c r="K405" t="inlineStr"/>
       <c r="L405" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M405" t="inlineStr"/>
       <c r="N405" t="inlineStr">
         <is>
           <t>MichelleGibbing</t>
@@ -26389,27 +26229,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q405" t="inlineStr"/>
       <c r="R405" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S405" t="inlineStr"/>
-      <c r="T405" t="inlineStr"/>
       <c r="U405" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V405" t="inlineStr"/>
-      <c r="W405" t="inlineStr"/>
       <c r="X405" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -26432,55 +26266,1254 @@
           <t>Ex-Royal Navy officer, ocean rower. Author of Compassionate Leadership. Courage through adventure.</t>
         </is>
       </c>
-      <c r="E406" t="inlineStr"/>
       <c r="F406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G406" t="inlineStr"/>
-      <c r="H406" t="inlineStr"/>
       <c r="I406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J406" t="inlineStr"/>
-      <c r="K406" t="inlineStr"/>
       <c r="L406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M406" t="inlineStr"/>
-      <c r="N406" t="inlineStr"/>
       <c r="O406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P406" t="inlineStr"/>
-      <c r="Q406" t="inlineStr"/>
       <c r="R406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S406" t="inlineStr"/>
-      <c r="T406" t="inlineStr"/>
       <c r="U406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V406" t="inlineStr"/>
-      <c r="W406" t="inlineStr"/>
       <c r="X406" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y406" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Jim Knight</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Founder &amp; Senior Partner</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Instructional Coaching Group</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Wrote first major work on instructional coaching. Author of The Impact Cycle, Data Rules (2024), IC Toolkit (2024)</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr"/>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr"/>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>jimknight99</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>ICG website</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>jimknight99</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>Inferred from IG</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t>jimknight99</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P407" t="inlineStr">
+        <is>
+          <t>Official website/X</t>
+        </is>
+      </c>
+      <c r="Q407" t="inlineStr">
+        <is>
+          <t>brightmorningtm</t>
+        </is>
+      </c>
+      <c r="R407" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S407" t="inlineStr"/>
+      <c r="T407" t="inlineStr"/>
+      <c r="U407" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V407" t="inlineStr"/>
+      <c r="W407" t="inlineStr"/>
+      <c r="X407" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y407" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Chrissy Beltran</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Instructional Coach &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Buzzing with Ms. B</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Hosts Instructional Coaching with Ms. B podcast. Teaches coaches to design coaching programs</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>BuzzingWithMsB</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>buzzingwithmsb</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Website/search</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr"/>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr"/>
+      <c r="N408" t="inlineStr"/>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P408" t="inlineStr"/>
+      <c r="Q408" t="inlineStr"/>
+      <c r="R408" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S408" t="inlineStr"/>
+      <c r="T408" t="inlineStr"/>
+      <c r="U408" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V408" t="inlineStr"/>
+      <c r="W408" t="inlineStr"/>
+      <c r="X408" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Steve Barkley</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Executive VP</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>PLS 3rd Learning</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>35+ years supporting educators globally. Hosts Ponders Out Loud podcast. Author of Quality Teaching in a Culture of Coaching</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr"/>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr"/>
+      <c r="H409" t="inlineStr"/>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr"/>
+      <c r="K409" t="inlineStr"/>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr"/>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>stevebarkley</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P409" t="inlineStr">
+        <is>
+          <t>barkleypd.com</t>
+        </is>
+      </c>
+      <c r="Q409" t="inlineStr"/>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S409" t="inlineStr"/>
+      <c r="T409" t="inlineStr"/>
+      <c r="U409" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V409" t="inlineStr"/>
+      <c r="W409" t="inlineStr"/>
+      <c r="X409" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Joellen Killion</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Senior Advisor</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Learning Forward</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Defined the 10 roles of a coach in Taking the Lead. 45+ years shaping professional learning standards</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr"/>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr"/>
+      <c r="H410" t="inlineStr"/>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr"/>
+      <c r="K410" t="inlineStr"/>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr"/>
+      <c r="N410" t="inlineStr"/>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P410" t="inlineStr"/>
+      <c r="Q410" t="inlineStr"/>
+      <c r="R410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S410" t="inlineStr"/>
+      <c r="T410" t="inlineStr"/>
+      <c r="U410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V410" t="inlineStr"/>
+      <c r="W410" t="inlineStr"/>
+      <c r="X410" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Jennifer Serravallo</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Founder &amp; President</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Literacy Strategies Consulting</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>NYT bestselling author of The Reading Strategies Book. Coaches literacy educators worldwide</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr"/>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr"/>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>jenniferserravallo</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr"/>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr"/>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t>jserravallo</t>
+        </is>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P411" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+      <c r="Q411" t="inlineStr"/>
+      <c r="R411" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S411" t="inlineStr"/>
+      <c r="T411" t="inlineStr"/>
+      <c r="U411" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V411" t="inlineStr"/>
+      <c r="W411" t="inlineStr"/>
+      <c r="X411" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y411" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Nicole Turner</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Simply Instructional Coaching Inc.</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Created Simply Coaching Summit and Accelerator. Author and podcast host with 19 years in education</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr"/>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>Facebook group</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr"/>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr"/>
+      <c r="K412" t="inlineStr"/>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr"/>
+      <c r="N412" t="inlineStr"/>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P412" t="inlineStr"/>
+      <c r="Q412" t="inlineStr"/>
+      <c r="R412" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S412" t="inlineStr"/>
+      <c r="T412" t="inlineStr"/>
+      <c r="U412" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V412" t="inlineStr"/>
+      <c r="W412" t="inlineStr"/>
+      <c r="X412" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y412" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Sherry St. Clair</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Reflective Learning LLC</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Author of Coaching Redefined and Intentional Instructional Moves (2024). Works with schools worldwide</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr"/>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr"/>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>sherryst.clair</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>Instagram search</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr"/>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr"/>
+      <c r="N413" t="inlineStr"/>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P413" t="inlineStr"/>
+      <c r="Q413" t="inlineStr"/>
+      <c r="R413" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S413" t="inlineStr"/>
+      <c r="T413" t="inlineStr"/>
+      <c r="U413" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V413" t="inlineStr"/>
+      <c r="W413" t="inlineStr"/>
+      <c r="X413" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Vicki Collet</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>University of Arkansas</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Created the GIR Coaching Model. Author of Differentiated Mentoring and Coaching. Weekly blog for coaches</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>My Coaches Couch</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Blog reference</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr"/>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr"/>
+      <c r="K414" t="inlineStr"/>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr"/>
+      <c r="N414" t="inlineStr"/>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P414" t="inlineStr"/>
+      <c r="Q414" t="inlineStr"/>
+      <c r="R414" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S414" t="inlineStr"/>
+      <c r="T414" t="inlineStr"/>
+      <c r="U414" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V414" t="inlineStr"/>
+      <c r="W414" t="inlineStr"/>
+      <c r="X414" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Kathy Perret</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Instructional Coaching Trainer</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Kathy Perret Consulting</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Co-founded #EduCoach, first Twitter chat for instructional coaches. Co-author of Compassionate Coaching</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr"/>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr"/>
+      <c r="H415" t="inlineStr"/>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr"/>
+      <c r="K415" t="inlineStr"/>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr"/>
+      <c r="N415" t="inlineStr">
+        <is>
+          <t>KathyPerret</t>
+        </is>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P415" t="inlineStr">
+        <is>
+          <t>Twitter profile</t>
+        </is>
+      </c>
+      <c r="Q415" t="inlineStr"/>
+      <c r="R415" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S415" t="inlineStr"/>
+      <c r="T415" t="inlineStr"/>
+      <c r="U415" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V415" t="inlineStr"/>
+      <c r="W415" t="inlineStr"/>
+      <c r="X415" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Jan Hasbrouck</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Educational Consultant &amp; Researcher</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Developed Student-Focused Coaching model. 15 years as reading specialist and coach. Co-founded Read Washington</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr"/>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr"/>
+      <c r="H416" t="inlineStr"/>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr"/>
+      <c r="K416" t="inlineStr"/>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr"/>
+      <c r="N416" t="inlineStr">
+        <is>
+          <t>janhasbrouck</t>
+        </is>
+      </c>
+      <c r="O416" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P416" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q416" t="inlineStr"/>
+      <c r="R416" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S416" t="inlineStr"/>
+      <c r="T416" t="inlineStr"/>
+      <c r="U416" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V416" t="inlineStr"/>
+      <c r="W416" t="inlineStr"/>
+      <c r="X416" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y416" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Katie Ritter</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Chief Learning Officer</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Forward Edge</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Top 100 EdTech Influencer 2023. Hosts Restart Recharge podcast. Former ISTE Coaching PLN President</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr"/>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr"/>
+      <c r="H417" t="inlineStr"/>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>Linktree</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr"/>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr"/>
+      <c r="N417" t="inlineStr">
+        <is>
+          <t>Katie_M_Ritter</t>
+        </is>
+      </c>
+      <c r="O417" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P417" t="inlineStr">
+        <is>
+          <t>X profile/Linktree</t>
+        </is>
+      </c>
+      <c r="Q417" t="inlineStr"/>
+      <c r="R417" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S417" t="inlineStr"/>
+      <c r="T417" t="inlineStr"/>
+      <c r="U417" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V417" t="inlineStr"/>
+      <c r="W417" t="inlineStr"/>
+      <c r="X417" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Gravity Goldberg</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Educational Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Gravity Goldberg LLC / Wesleyan University</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Author of Mindsets &amp; Moves and 8 other books. Specialises in side-by-side literacy coaching</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr"/>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr"/>
+      <c r="H418" t="inlineStr"/>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr"/>
+      <c r="K418" t="inlineStr"/>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr"/>
+      <c r="N418" t="inlineStr">
+        <is>
+          <t>drgravityg</t>
+        </is>
+      </c>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P418" t="inlineStr">
+        <is>
+          <t>Search results</t>
+        </is>
+      </c>
+      <c r="Q418" t="inlineStr"/>
+      <c r="R418" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S418" t="inlineStr"/>
+      <c r="T418" t="inlineStr"/>
+      <c r="U418" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V418" t="inlineStr"/>
+      <c r="W418" t="inlineStr"/>
+      <c r="X418" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Jessica Johnson</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Elementary Principal &amp; Author</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Dodgeland School District</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>WI Principal of the Year. Co-author Coach Approach to School Leadership. Co-hosts PrincipalPLN podcast</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr"/>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr"/>
+      <c r="H419" t="inlineStr"/>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr"/>
+      <c r="K419" t="inlineStr"/>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr"/>
+      <c r="N419" t="inlineStr">
+        <is>
+          <t>PrincipalJ</t>
+        </is>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P419" t="inlineStr">
+        <is>
+          <t>Book bio/Twitter</t>
+        </is>
+      </c>
+      <c r="Q419" t="inlineStr"/>
+      <c r="R419" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S419" t="inlineStr"/>
+      <c r="T419" t="inlineStr"/>
+      <c r="U419" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V419" t="inlineStr"/>
+      <c r="W419" t="inlineStr"/>
+      <c r="X419" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y419" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Tonya Ward Singer</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Courageous Literacy LLC</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Equity-focused coaching specialist. Author of EL Excellence Every Day and Opening Doors to Equity</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>TonyaWardSinger</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr"/>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr"/>
+      <c r="K420" t="inlineStr"/>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr"/>
+      <c r="N420" t="inlineStr">
+        <is>
+          <t>TonyaWardSinger</t>
+        </is>
+      </c>
+      <c r="O420" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P420" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q420" t="inlineStr"/>
+      <c r="R420" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S420" t="inlineStr"/>
+      <c r="T420" t="inlineStr"/>
+      <c r="U420" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V420" t="inlineStr"/>
+      <c r="W420" t="inlineStr"/>
+      <c r="X420" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Kristin Anderson</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>The Brilliance Project</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Brought Visible Learning to North America. Researches trust between adults in schools and coaching impact</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr"/>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr"/>
+      <c r="H421" t="inlineStr"/>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr"/>
+      <c r="K421" t="inlineStr"/>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr"/>
+      <c r="N421" t="inlineStr"/>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P421" t="inlineStr"/>
+      <c r="Q421" t="inlineStr"/>
+      <c r="R421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S421" t="inlineStr"/>
+      <c r="T421" t="inlineStr"/>
+      <c r="U421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V421" t="inlineStr"/>
+      <c r="W421" t="inlineStr"/>
+      <c r="X421" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y421" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -26494,7 +27527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -27022,6 +28055,26 @@
       <c r="D26" t="inlineStr">
         <is>
           <t>courage-vulnerability-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>17</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>instructional-coaching</t>
         </is>
       </c>
     </row>
@@ -27037,7 +28090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G201"/>
+  <dimension ref="A1:G209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -34391,6 +35444,302 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>69c3d6addc7f763f71a5adb7</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>2026-04-03T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>69c3d6afecfc8d3950f5e8c2</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>2026-04-03T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>69c3d6b2dc7f763f71a5ae03</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>2026-04-03T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>69c3d6b3ecfc8d3950f5e8e8</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>2026-04-03T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>69c3d6cadc7f763f71a5ae98</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>2026-03-29T05:01:00Z</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>69c3d6cbecfc8d3950f5e968</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>2026-05-01T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>69c3d6cddc7f763f71a5aebe</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>2026-04-03T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Instructional Coaching</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>69c3d6ceecfc8d3950f5e98f</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>2026-04-03T12:15:00Z</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Nonprofit Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1112,10 +1112,14 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
           <t>Strong niche with own conferences, podcasts, and communities</t>
@@ -1555,7 +1559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y421"/>
+  <dimension ref="A1:Y438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -26323,13 +26327,11 @@
           <t>Wrote first major work on instructional coaching. Author of The Impact Cycle, Data Rules (2024), IC Toolkit (2024)</t>
         </is>
       </c>
-      <c r="E407" t="inlineStr"/>
       <c r="F407" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G407" t="inlineStr"/>
       <c r="H407" t="inlineStr">
         <is>
           <t>jimknight99</t>
@@ -26385,21 +26387,16 @@
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S407" t="inlineStr"/>
-      <c r="T407" t="inlineStr"/>
       <c r="U407" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V407" t="inlineStr"/>
-      <c r="W407" t="inlineStr"/>
       <c r="X407" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -26452,41 +26449,31 @@
           <t>Website/search</t>
         </is>
       </c>
-      <c r="K408" t="inlineStr"/>
       <c r="L408" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M408" t="inlineStr"/>
-      <c r="N408" t="inlineStr"/>
       <c r="O408" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P408" t="inlineStr"/>
-      <c r="Q408" t="inlineStr"/>
       <c r="R408" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S408" t="inlineStr"/>
-      <c r="T408" t="inlineStr"/>
       <c r="U408" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V408" t="inlineStr"/>
-      <c r="W408" t="inlineStr"/>
       <c r="X408" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -26509,27 +26496,21 @@
           <t>35+ years supporting educators globally. Hosts Ponders Out Loud podcast. Author of Quality Teaching in a Culture of Coaching</t>
         </is>
       </c>
-      <c r="E409" t="inlineStr"/>
       <c r="F409" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G409" t="inlineStr"/>
-      <c r="H409" t="inlineStr"/>
       <c r="I409" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J409" t="inlineStr"/>
-      <c r="K409" t="inlineStr"/>
       <c r="L409" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M409" t="inlineStr"/>
       <c r="N409" t="inlineStr">
         <is>
           <t>stevebarkley</t>
@@ -26545,27 +26526,21 @@
           <t>barkleypd.com</t>
         </is>
       </c>
-      <c r="Q409" t="inlineStr"/>
       <c r="R409" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S409" t="inlineStr"/>
-      <c r="T409" t="inlineStr"/>
       <c r="U409" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V409" t="inlineStr"/>
-      <c r="W409" t="inlineStr"/>
       <c r="X409" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -26588,55 +26563,41 @@
           <t>Defined the 10 roles of a coach in Taking the Lead. 45+ years shaping professional learning standards</t>
         </is>
       </c>
-      <c r="E410" t="inlineStr"/>
       <c r="F410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G410" t="inlineStr"/>
-      <c r="H410" t="inlineStr"/>
       <c r="I410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J410" t="inlineStr"/>
-      <c r="K410" t="inlineStr"/>
       <c r="L410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M410" t="inlineStr"/>
-      <c r="N410" t="inlineStr"/>
       <c r="O410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P410" t="inlineStr"/>
-      <c r="Q410" t="inlineStr"/>
       <c r="R410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S410" t="inlineStr"/>
-      <c r="T410" t="inlineStr"/>
       <c r="U410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V410" t="inlineStr"/>
-      <c r="W410" t="inlineStr"/>
       <c r="X410" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -26659,13 +26620,11 @@
           <t>NYT bestselling author of The Reading Strategies Book. Coaches literacy educators worldwide</t>
         </is>
       </c>
-      <c r="E411" t="inlineStr"/>
       <c r="F411" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G411" t="inlineStr"/>
       <c r="H411" t="inlineStr">
         <is>
           <t>jenniferserravallo</t>
@@ -26681,13 +26640,11 @@
           <t>Official website</t>
         </is>
       </c>
-      <c r="K411" t="inlineStr"/>
       <c r="L411" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M411" t="inlineStr"/>
       <c r="N411" t="inlineStr">
         <is>
           <t>jserravallo</t>
@@ -26703,27 +26660,21 @@
           <t>Official website</t>
         </is>
       </c>
-      <c r="Q411" t="inlineStr"/>
       <c r="R411" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S411" t="inlineStr"/>
-      <c r="T411" t="inlineStr"/>
       <c r="U411" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V411" t="inlineStr"/>
-      <c r="W411" t="inlineStr"/>
       <c r="X411" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -26746,7 +26697,6 @@
           <t>Created Simply Coaching Summit and Accelerator. Author and podcast host with 19 years in education</t>
         </is>
       </c>
-      <c r="E412" t="inlineStr"/>
       <c r="F412" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -26757,48 +26707,36 @@
           <t>Facebook group</t>
         </is>
       </c>
-      <c r="H412" t="inlineStr"/>
       <c r="I412" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J412" t="inlineStr"/>
-      <c r="K412" t="inlineStr"/>
       <c r="L412" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M412" t="inlineStr"/>
-      <c r="N412" t="inlineStr"/>
       <c r="O412" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P412" t="inlineStr"/>
-      <c r="Q412" t="inlineStr"/>
       <c r="R412" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S412" t="inlineStr"/>
-      <c r="T412" t="inlineStr"/>
       <c r="U412" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V412" t="inlineStr"/>
-      <c r="W412" t="inlineStr"/>
       <c r="X412" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -26821,13 +26759,11 @@
           <t>Author of Coaching Redefined and Intentional Instructional Moves (2024). Works with schools worldwide</t>
         </is>
       </c>
-      <c r="E413" t="inlineStr"/>
       <c r="F413" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G413" t="inlineStr"/>
       <c r="H413" t="inlineStr">
         <is>
           <t>sherryst.clair</t>
@@ -26843,41 +26779,31 @@
           <t>Instagram search</t>
         </is>
       </c>
-      <c r="K413" t="inlineStr"/>
       <c r="L413" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M413" t="inlineStr"/>
-      <c r="N413" t="inlineStr"/>
       <c r="O413" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P413" t="inlineStr"/>
-      <c r="Q413" t="inlineStr"/>
       <c r="R413" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S413" t="inlineStr"/>
-      <c r="T413" t="inlineStr"/>
       <c r="U413" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V413" t="inlineStr"/>
-      <c r="W413" t="inlineStr"/>
       <c r="X413" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -26915,48 +26841,36 @@
           <t>Blog reference</t>
         </is>
       </c>
-      <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J414" t="inlineStr"/>
-      <c r="K414" t="inlineStr"/>
       <c r="L414" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M414" t="inlineStr"/>
-      <c r="N414" t="inlineStr"/>
       <c r="O414" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P414" t="inlineStr"/>
-      <c r="Q414" t="inlineStr"/>
       <c r="R414" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S414" t="inlineStr"/>
-      <c r="T414" t="inlineStr"/>
       <c r="U414" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V414" t="inlineStr"/>
-      <c r="W414" t="inlineStr"/>
       <c r="X414" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -26979,27 +26893,21 @@
           <t>Co-founded #EduCoach, first Twitter chat for instructional coaches. Co-author of Compassionate Coaching</t>
         </is>
       </c>
-      <c r="E415" t="inlineStr"/>
       <c r="F415" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G415" t="inlineStr"/>
-      <c r="H415" t="inlineStr"/>
       <c r="I415" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J415" t="inlineStr"/>
-      <c r="K415" t="inlineStr"/>
       <c r="L415" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M415" t="inlineStr"/>
       <c r="N415" t="inlineStr">
         <is>
           <t>KathyPerret</t>
@@ -27015,27 +26923,21 @@
           <t>Twitter profile</t>
         </is>
       </c>
-      <c r="Q415" t="inlineStr"/>
       <c r="R415" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S415" t="inlineStr"/>
-      <c r="T415" t="inlineStr"/>
       <c r="U415" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V415" t="inlineStr"/>
-      <c r="W415" t="inlineStr"/>
       <c r="X415" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -27058,27 +26960,21 @@
           <t>Developed Student-Focused Coaching model. 15 years as reading specialist and coach. Co-founded Read Washington</t>
         </is>
       </c>
-      <c r="E416" t="inlineStr"/>
       <c r="F416" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G416" t="inlineStr"/>
-      <c r="H416" t="inlineStr"/>
       <c r="I416" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J416" t="inlineStr"/>
-      <c r="K416" t="inlineStr"/>
       <c r="L416" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M416" t="inlineStr"/>
       <c r="N416" t="inlineStr">
         <is>
           <t>janhasbrouck</t>
@@ -27094,27 +26990,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q416" t="inlineStr"/>
       <c r="R416" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S416" t="inlineStr"/>
-      <c r="T416" t="inlineStr"/>
       <c r="U416" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V416" t="inlineStr"/>
-      <c r="W416" t="inlineStr"/>
       <c r="X416" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -27137,14 +27027,11 @@
           <t>Top 100 EdTech Influencer 2023. Hosts Restart Recharge podcast. Former ISTE Coaching PLN President</t>
         </is>
       </c>
-      <c r="E417" t="inlineStr"/>
       <c r="F417" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G417" t="inlineStr"/>
-      <c r="H417" t="inlineStr"/>
       <c r="I417" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -27155,13 +27042,11 @@
           <t>Linktree</t>
         </is>
       </c>
-      <c r="K417" t="inlineStr"/>
       <c r="L417" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M417" t="inlineStr"/>
       <c r="N417" t="inlineStr">
         <is>
           <t>Katie_M_Ritter</t>
@@ -27177,27 +27062,21 @@
           <t>X profile/Linktree</t>
         </is>
       </c>
-      <c r="Q417" t="inlineStr"/>
       <c r="R417" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S417" t="inlineStr"/>
-      <c r="T417" t="inlineStr"/>
       <c r="U417" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V417" t="inlineStr"/>
-      <c r="W417" t="inlineStr"/>
       <c r="X417" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -27220,27 +27099,21 @@
           <t>Author of Mindsets &amp; Moves and 8 other books. Specialises in side-by-side literacy coaching</t>
         </is>
       </c>
-      <c r="E418" t="inlineStr"/>
       <c r="F418" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G418" t="inlineStr"/>
-      <c r="H418" t="inlineStr"/>
       <c r="I418" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J418" t="inlineStr"/>
-      <c r="K418" t="inlineStr"/>
       <c r="L418" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M418" t="inlineStr"/>
       <c r="N418" t="inlineStr">
         <is>
           <t>drgravityg</t>
@@ -27256,27 +27129,21 @@
           <t>Search results</t>
         </is>
       </c>
-      <c r="Q418" t="inlineStr"/>
       <c r="R418" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S418" t="inlineStr"/>
-      <c r="T418" t="inlineStr"/>
       <c r="U418" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V418" t="inlineStr"/>
-      <c r="W418" t="inlineStr"/>
       <c r="X418" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -27299,27 +27166,21 @@
           <t>WI Principal of the Year. Co-author Coach Approach to School Leadership. Co-hosts PrincipalPLN podcast</t>
         </is>
       </c>
-      <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G419" t="inlineStr"/>
-      <c r="H419" t="inlineStr"/>
       <c r="I419" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J419" t="inlineStr"/>
-      <c r="K419" t="inlineStr"/>
       <c r="L419" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M419" t="inlineStr"/>
       <c r="N419" t="inlineStr">
         <is>
           <t>PrincipalJ</t>
@@ -27335,27 +27196,21 @@
           <t>Book bio/Twitter</t>
         </is>
       </c>
-      <c r="Q419" t="inlineStr"/>
       <c r="R419" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S419" t="inlineStr"/>
-      <c r="T419" t="inlineStr"/>
       <c r="U419" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V419" t="inlineStr"/>
-      <c r="W419" t="inlineStr"/>
       <c r="X419" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -27393,20 +27248,16 @@
           <t>Facebook page</t>
         </is>
       </c>
-      <c r="H420" t="inlineStr"/>
       <c r="I420" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J420" t="inlineStr"/>
-      <c r="K420" t="inlineStr"/>
       <c r="L420" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M420" t="inlineStr"/>
       <c r="N420" t="inlineStr">
         <is>
           <t>TonyaWardSinger</t>
@@ -27422,27 +27273,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q420" t="inlineStr"/>
       <c r="R420" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S420" t="inlineStr"/>
-      <c r="T420" t="inlineStr"/>
       <c r="U420" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V420" t="inlineStr"/>
-      <c r="W420" t="inlineStr"/>
       <c r="X420" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -27465,55 +27310,1448 @@
           <t>Brought Visible Learning to North America. Researches trust between adults in schools and coaching impact</t>
         </is>
       </c>
-      <c r="E421" t="inlineStr"/>
       <c r="F421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G421" t="inlineStr"/>
-      <c r="H421" t="inlineStr"/>
       <c r="I421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J421" t="inlineStr"/>
-      <c r="K421" t="inlineStr"/>
       <c r="L421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M421" t="inlineStr"/>
-      <c r="N421" t="inlineStr"/>
       <c r="O421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P421" t="inlineStr"/>
-      <c r="Q421" t="inlineStr"/>
       <c r="R421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S421" t="inlineStr"/>
-      <c r="T421" t="inlineStr"/>
       <c r="U421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V421" t="inlineStr"/>
-      <c r="W421" t="inlineStr"/>
       <c r="X421" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y421" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Joan Garry</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Joan Garry Consulting</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Former GLAAD CEO, #1 nonprofit podcast host, author of Joan Garry's Guide to Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>joangarry</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>joangarryconsulting</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>joangarryconsulting</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N422" t="inlineStr">
+        <is>
+          <t>joangarry</t>
+        </is>
+      </c>
+      <c r="O422" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P422" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q422" t="inlineStr"/>
+      <c r="R422" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S422" t="inlineStr"/>
+      <c r="T422" t="inlineStr"/>
+      <c r="U422" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V422" t="inlineStr"/>
+      <c r="W422" t="inlineStr"/>
+      <c r="X422" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Beth Kanter</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Author &amp; Nonprofit Innovator</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Named most influential woman in tech by Fast Company, pioneer in nonprofit digital transformation</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>bethkanter</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>kanter</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr"/>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr"/>
+      <c r="N423" t="inlineStr">
+        <is>
+          <t>kanter</t>
+        </is>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P423" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q423" t="inlineStr"/>
+      <c r="R423" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S423" t="inlineStr"/>
+      <c r="T423" t="inlineStr"/>
+      <c r="U423" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V423" t="inlineStr"/>
+      <c r="W423" t="inlineStr"/>
+      <c r="X423" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Vu Le</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Nonprofit AF</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Internationally known speaker using humor to tackle nonprofit equity and systems change</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>nonprofitAF</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>nonprofitaf</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>nonprofitaf</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N424" t="inlineStr">
+        <is>
+          <t>NonprofitAF</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P424" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="Q424" t="inlineStr"/>
+      <c r="R424" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S424" t="inlineStr"/>
+      <c r="T424" t="inlineStr"/>
+      <c r="U424" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V424" t="inlineStr"/>
+      <c r="W424" t="inlineStr"/>
+      <c r="X424" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Julia Campbell</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>J Campbell Social Marketing</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Author of Storytelling in the Digital Age, Nonprofit Nation podcast, Forbes top thought leader</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>jcsocialmarketing</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>juliacampbell77</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr"/>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr"/>
+      <c r="N425" t="inlineStr">
+        <is>
+          <t>JuliaCSocial</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P425" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q425" t="inlineStr"/>
+      <c r="R425" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S425" t="inlineStr"/>
+      <c r="T425" t="inlineStr"/>
+      <c r="U425" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V425" t="inlineStr"/>
+      <c r="W425" t="inlineStr"/>
+      <c r="X425" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y425" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Mallory Erickson</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Practivated</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Power Partners Formula creator, What the Fundraising podcast host, trained 60K+ fundraisers</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>malloryericksoncoach</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>_malloryerickson</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>_malloryerickson</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N426" t="inlineStr"/>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P426" t="inlineStr"/>
+      <c r="Q426" t="inlineStr"/>
+      <c r="R426" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S426" t="inlineStr"/>
+      <c r="T426" t="inlineStr"/>
+      <c r="U426" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V426" t="inlineStr"/>
+      <c r="W426" t="inlineStr"/>
+      <c r="X426" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Dana Snyder</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Positive Equation</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Monthly giving specialist, Missions to Movements podcast host, nonprofit social media expert</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>positiveequation</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr"/>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr"/>
+      <c r="K427" t="inlineStr"/>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr"/>
+      <c r="N427" t="inlineStr"/>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P427" t="inlineStr"/>
+      <c r="Q427" t="inlineStr"/>
+      <c r="R427" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S427" t="inlineStr"/>
+      <c r="T427" t="inlineStr"/>
+      <c r="U427" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V427" t="inlineStr"/>
+      <c r="W427" t="inlineStr"/>
+      <c r="X427" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Kishshana Palmer</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>ManageMint</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>SPARK Framework creator, 20+ years fundraising and talent management, CFRE</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>iamkishshanapalmer</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>kishshana</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr"/>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr"/>
+      <c r="N428" t="inlineStr"/>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P428" t="inlineStr"/>
+      <c r="Q428" t="inlineStr"/>
+      <c r="R428" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S428" t="inlineStr"/>
+      <c r="T428" t="inlineStr"/>
+      <c r="U428" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V428" t="inlineStr"/>
+      <c r="W428" t="inlineStr"/>
+      <c r="X428" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Rhea Wong</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Rhea Wong Consulting</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Major gifts and board development expert, Nonprofit Lowdown podcast host</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>rheawongconsulting</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>rheawongconsulting</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr"/>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr"/>
+      <c r="N429" t="inlineStr"/>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P429" t="inlineStr"/>
+      <c r="Q429" t="inlineStr"/>
+      <c r="R429" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S429" t="inlineStr"/>
+      <c r="T429" t="inlineStr"/>
+      <c r="U429" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V429" t="inlineStr"/>
+      <c r="W429" t="inlineStr"/>
+      <c r="X429" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Claire Axelrad</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Clairification</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>AFP Outstanding Fundraising Professional, donor retention specialist and coach, CFRE</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr"/>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr"/>
+      <c r="H430" t="inlineStr"/>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr"/>
+      <c r="K430" t="inlineStr"/>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr"/>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t>CharityClairity</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P430" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q430" t="inlineStr"/>
+      <c r="R430" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S430" t="inlineStr"/>
+      <c r="T430" t="inlineStr"/>
+      <c r="U430" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V430" t="inlineStr"/>
+      <c r="W430" t="inlineStr"/>
+      <c r="X430" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Brooke Richie-Babbage</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Bending Arc</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Harvard JD/MPP, nonprofit growth strategist, Nonprofit Mastermind Podcast host</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>richiebabbage</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr"/>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr"/>
+      <c r="K431" t="inlineStr"/>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr"/>
+      <c r="N431" t="inlineStr"/>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P431" t="inlineStr"/>
+      <c r="Q431" t="inlineStr"/>
+      <c r="R431" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S431" t="inlineStr"/>
+      <c r="T431" t="inlineStr"/>
+      <c r="U431" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V431" t="inlineStr"/>
+      <c r="W431" t="inlineStr"/>
+      <c r="X431" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Patton McDowell</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>PMA Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Bestselling author, Your Path to Nonprofit Leadership podcast, Ed.D/CFRE</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr"/>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr"/>
+      <c r="H432" t="inlineStr"/>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr"/>
+      <c r="K432" t="inlineStr"/>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr"/>
+      <c r="N432" t="inlineStr"/>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P432" t="inlineStr"/>
+      <c r="Q432" t="inlineStr"/>
+      <c r="R432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S432" t="inlineStr"/>
+      <c r="T432" t="inlineStr"/>
+      <c r="U432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V432" t="inlineStr"/>
+      <c r="W432" t="inlineStr"/>
+      <c r="X432" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Tosha Anderson</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>The Charity CFO</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Nonprofit financial specialist, A Modern Nonprofit podcast host, CPA</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr"/>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr"/>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr"/>
+      <c r="K433" t="inlineStr"/>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr"/>
+      <c r="N433" t="inlineStr"/>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P433" t="inlineStr"/>
+      <c r="Q433" t="inlineStr"/>
+      <c r="R433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S433" t="inlineStr"/>
+      <c r="T433" t="inlineStr"/>
+      <c r="U433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V433" t="inlineStr"/>
+      <c r="W433" t="inlineStr"/>
+      <c r="X433" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Jon McCoy</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>We Are For Good</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>CFRE with 20+ years in development, co-host of top-rated nonprofit podcast</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr"/>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr"/>
+      <c r="H434" t="inlineStr"/>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr"/>
+      <c r="K434" t="inlineStr"/>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr"/>
+      <c r="N434" t="inlineStr"/>
+      <c r="O434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P434" t="inlineStr"/>
+      <c r="Q434" t="inlineStr"/>
+      <c r="R434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S434" t="inlineStr"/>
+      <c r="T434" t="inlineStr"/>
+      <c r="U434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V434" t="inlineStr"/>
+      <c r="W434" t="inlineStr"/>
+      <c r="X434" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Becky Endicott</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>We Are For Good</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>CFRE and Chief Storyteller, co-host of 400+ episode nonprofit podcast</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr"/>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr"/>
+      <c r="H435" t="inlineStr"/>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr"/>
+      <c r="K435" t="inlineStr"/>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr"/>
+      <c r="N435" t="inlineStr"/>
+      <c r="O435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P435" t="inlineStr"/>
+      <c r="Q435" t="inlineStr"/>
+      <c r="R435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S435" t="inlineStr"/>
+      <c r="T435" t="inlineStr"/>
+      <c r="U435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V435" t="inlineStr"/>
+      <c r="W435" t="inlineStr"/>
+      <c r="X435" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Dennis C. Miller</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Board Governance Expert</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Author of 5 books on nonprofit success, 40+ years coaching boards and executives</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr"/>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr"/>
+      <c r="H436" t="inlineStr"/>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr"/>
+      <c r="K436" t="inlineStr"/>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr"/>
+      <c r="N436" t="inlineStr"/>
+      <c r="O436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P436" t="inlineStr"/>
+      <c r="Q436" t="inlineStr"/>
+      <c r="R436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S436" t="inlineStr"/>
+      <c r="T436" t="inlineStr"/>
+      <c r="U436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V436" t="inlineStr"/>
+      <c r="W436" t="inlineStr"/>
+      <c r="X436" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>David Renz</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Professor Emeritus</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>UMKC</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Editor of The Jossey-Bass Handbook of Nonprofit Leadership and Management (5th ed)</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr"/>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr"/>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr"/>
+      <c r="K437" t="inlineStr"/>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr"/>
+      <c r="N437" t="inlineStr"/>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P437" t="inlineStr"/>
+      <c r="Q437" t="inlineStr"/>
+      <c r="R437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S437" t="inlineStr"/>
+      <c r="T437" t="inlineStr"/>
+      <c r="U437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V437" t="inlineStr"/>
+      <c r="W437" t="inlineStr"/>
+      <c r="X437" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Dr. Rob Harter</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>30+ years social impact experience, keynote speaker and executive coach</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr"/>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr"/>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr"/>
+      <c r="K438" t="inlineStr"/>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr"/>
+      <c r="N438" t="inlineStr">
+        <is>
+          <t>robharter</t>
+        </is>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P438" t="inlineStr">
+        <is>
+          <t>X profile</t>
+        </is>
+      </c>
+      <c r="Q438" t="inlineStr"/>
+      <c r="R438" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S438" t="inlineStr"/>
+      <c r="T438" t="inlineStr"/>
+      <c r="U438" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V438" t="inlineStr"/>
+      <c r="W438" t="inlineStr"/>
+      <c r="X438" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y438" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -27527,7 +28765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -28075,6 +29313,46 @@
       <c r="D27" t="inlineStr">
         <is>
           <t>instructional-coaching</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>17</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>courage-vulnerability-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>17</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nonprofit-leadership</t>
         </is>
       </c>
     </row>
@@ -28090,7 +29368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G209"/>
+  <dimension ref="A1:G225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -35740,6 +37018,598 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>69c3d1cddc7f763f71a5895a</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>2026-04-03T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>69c3d1cfecfc8d3950f5b9d4</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>2026-04-03T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>69c3d1eaecfc8d3950f5bb01</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>2026-03-29T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>69c3d1eddc7f763f71a58b45</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>2026-04-03T03:01:00Z</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>69c3d1eedc7f763f71a58b6b</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>2026-04-03T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>69c3d1eeecfc8d3950f5bb9d</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>2026-04-03T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>69c3d1fddc7f763f71a58beb</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>2026-04-30T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Courage &amp; Vulnerability in Leadership</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>69c3d200ecfc8d3950f5bc13</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>2026-04-03T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>69c3e486a916f74f97753e8f</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>2026-04-03T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>69c3e48aa916f74f97753ec8</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>2026-04-03T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>69c3e48ca916f74f97753eee</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>2026-04-03T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>69c3e48daf1ab213a2f440a0</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>2026-04-03T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>69c3e4a4a916f74f97753f25</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>2026-05-03T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>69c3e4a6af1ab213a2f440f7</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>2026-05-03T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>69c3e4a9af1ab213a2f4411e</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>2026-04-03T21:15:00Z</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>69c3e4aaa916f74f97753f58</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>2026-04-03T14:01:00Z</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update data/handle-database.xlsx — neurodiversity-in-the-workplace
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1137,10 +1137,14 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Growing niche with active creators, advocates, and workplace consultants</t>
@@ -1559,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y438"/>
+  <dimension ref="A1:Y455"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -27427,27 +27431,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q422" t="inlineStr"/>
       <c r="R422" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S422" t="inlineStr"/>
-      <c r="T422" t="inlineStr"/>
       <c r="U422" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V422" t="inlineStr"/>
-      <c r="W422" t="inlineStr"/>
       <c r="X422" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -27500,13 +27498,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K423" t="inlineStr"/>
       <c r="L423" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M423" t="inlineStr"/>
       <c r="N423" t="inlineStr">
         <is>
           <t>kanter</t>
@@ -27522,27 +27518,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q423" t="inlineStr"/>
       <c r="R423" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S423" t="inlineStr"/>
-      <c r="T423" t="inlineStr"/>
       <c r="U423" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V423" t="inlineStr"/>
-      <c r="W423" t="inlineStr"/>
       <c r="X423" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -27625,27 +27615,21 @@
           <t>website</t>
         </is>
       </c>
-      <c r="Q424" t="inlineStr"/>
       <c r="R424" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S424" t="inlineStr"/>
-      <c r="T424" t="inlineStr"/>
       <c r="U424" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V424" t="inlineStr"/>
-      <c r="W424" t="inlineStr"/>
       <c r="X424" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -27698,13 +27682,11 @@
           <t>search</t>
         </is>
       </c>
-      <c r="K425" t="inlineStr"/>
       <c r="L425" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M425" t="inlineStr"/>
       <c r="N425" t="inlineStr">
         <is>
           <t>JuliaCSocial</t>
@@ -27720,27 +27702,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q425" t="inlineStr"/>
       <c r="R425" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S425" t="inlineStr"/>
-      <c r="T425" t="inlineStr"/>
       <c r="U425" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V425" t="inlineStr"/>
-      <c r="W425" t="inlineStr"/>
       <c r="X425" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -27808,34 +27784,26 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N426" t="inlineStr"/>
       <c r="O426" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P426" t="inlineStr"/>
-      <c r="Q426" t="inlineStr"/>
       <c r="R426" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S426" t="inlineStr"/>
-      <c r="T426" t="inlineStr"/>
       <c r="U426" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V426" t="inlineStr"/>
-      <c r="W426" t="inlineStr"/>
       <c r="X426" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -27873,48 +27841,36 @@
           <t>search</t>
         </is>
       </c>
-      <c r="H427" t="inlineStr"/>
       <c r="I427" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J427" t="inlineStr"/>
-      <c r="K427" t="inlineStr"/>
       <c r="L427" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M427" t="inlineStr"/>
-      <c r="N427" t="inlineStr"/>
       <c r="O427" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P427" t="inlineStr"/>
-      <c r="Q427" t="inlineStr"/>
       <c r="R427" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S427" t="inlineStr"/>
-      <c r="T427" t="inlineStr"/>
       <c r="U427" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V427" t="inlineStr"/>
-      <c r="W427" t="inlineStr"/>
       <c r="X427" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -27967,41 +27923,31 @@
           <t>search</t>
         </is>
       </c>
-      <c r="K428" t="inlineStr"/>
       <c r="L428" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M428" t="inlineStr"/>
-      <c r="N428" t="inlineStr"/>
       <c r="O428" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P428" t="inlineStr"/>
-      <c r="Q428" t="inlineStr"/>
       <c r="R428" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S428" t="inlineStr"/>
-      <c r="T428" t="inlineStr"/>
       <c r="U428" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V428" t="inlineStr"/>
-      <c r="W428" t="inlineStr"/>
       <c r="X428" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -28054,41 +28000,31 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K429" t="inlineStr"/>
       <c r="L429" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M429" t="inlineStr"/>
-      <c r="N429" t="inlineStr"/>
       <c r="O429" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P429" t="inlineStr"/>
-      <c r="Q429" t="inlineStr"/>
       <c r="R429" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S429" t="inlineStr"/>
-      <c r="T429" t="inlineStr"/>
       <c r="U429" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V429" t="inlineStr"/>
-      <c r="W429" t="inlineStr"/>
       <c r="X429" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -28111,27 +28047,21 @@
           <t>AFP Outstanding Fundraising Professional, donor retention specialist and coach, CFRE</t>
         </is>
       </c>
-      <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G430" t="inlineStr"/>
-      <c r="H430" t="inlineStr"/>
       <c r="I430" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J430" t="inlineStr"/>
-      <c r="K430" t="inlineStr"/>
       <c r="L430" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M430" t="inlineStr"/>
       <c r="N430" t="inlineStr">
         <is>
           <t>CharityClairity</t>
@@ -28147,27 +28077,21 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q430" t="inlineStr"/>
       <c r="R430" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S430" t="inlineStr"/>
-      <c r="T430" t="inlineStr"/>
       <c r="U430" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V430" t="inlineStr"/>
-      <c r="W430" t="inlineStr"/>
       <c r="X430" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -28205,48 +28129,36 @@
           <t>Facebook</t>
         </is>
       </c>
-      <c r="H431" t="inlineStr"/>
       <c r="I431" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J431" t="inlineStr"/>
-      <c r="K431" t="inlineStr"/>
       <c r="L431" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M431" t="inlineStr"/>
-      <c r="N431" t="inlineStr"/>
       <c r="O431" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P431" t="inlineStr"/>
-      <c r="Q431" t="inlineStr"/>
       <c r="R431" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S431" t="inlineStr"/>
-      <c r="T431" t="inlineStr"/>
       <c r="U431" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V431" t="inlineStr"/>
-      <c r="W431" t="inlineStr"/>
       <c r="X431" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -28269,55 +28181,41 @@
           <t>Bestselling author, Your Path to Nonprofit Leadership podcast, Ed.D/CFRE</t>
         </is>
       </c>
-      <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G432" t="inlineStr"/>
-      <c r="H432" t="inlineStr"/>
       <c r="I432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J432" t="inlineStr"/>
-      <c r="K432" t="inlineStr"/>
       <c r="L432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M432" t="inlineStr"/>
-      <c r="N432" t="inlineStr"/>
       <c r="O432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P432" t="inlineStr"/>
-      <c r="Q432" t="inlineStr"/>
       <c r="R432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S432" t="inlineStr"/>
-      <c r="T432" t="inlineStr"/>
       <c r="U432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V432" t="inlineStr"/>
-      <c r="W432" t="inlineStr"/>
       <c r="X432" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -28340,55 +28238,41 @@
           <t>Nonprofit financial specialist, A Modern Nonprofit podcast host, CPA</t>
         </is>
       </c>
-      <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G433" t="inlineStr"/>
-      <c r="H433" t="inlineStr"/>
       <c r="I433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J433" t="inlineStr"/>
-      <c r="K433" t="inlineStr"/>
       <c r="L433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M433" t="inlineStr"/>
-      <c r="N433" t="inlineStr"/>
       <c r="O433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P433" t="inlineStr"/>
-      <c r="Q433" t="inlineStr"/>
       <c r="R433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S433" t="inlineStr"/>
-      <c r="T433" t="inlineStr"/>
       <c r="U433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V433" t="inlineStr"/>
-      <c r="W433" t="inlineStr"/>
       <c r="X433" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -28411,55 +28295,41 @@
           <t>CFRE with 20+ years in development, co-host of top-rated nonprofit podcast</t>
         </is>
       </c>
-      <c r="E434" t="inlineStr"/>
       <c r="F434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G434" t="inlineStr"/>
-      <c r="H434" t="inlineStr"/>
       <c r="I434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J434" t="inlineStr"/>
-      <c r="K434" t="inlineStr"/>
       <c r="L434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M434" t="inlineStr"/>
-      <c r="N434" t="inlineStr"/>
       <c r="O434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P434" t="inlineStr"/>
-      <c r="Q434" t="inlineStr"/>
       <c r="R434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S434" t="inlineStr"/>
-      <c r="T434" t="inlineStr"/>
       <c r="U434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V434" t="inlineStr"/>
-      <c r="W434" t="inlineStr"/>
       <c r="X434" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -28482,55 +28352,41 @@
           <t>CFRE and Chief Storyteller, co-host of 400+ episode nonprofit podcast</t>
         </is>
       </c>
-      <c r="E435" t="inlineStr"/>
       <c r="F435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G435" t="inlineStr"/>
-      <c r="H435" t="inlineStr"/>
       <c r="I435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J435" t="inlineStr"/>
-      <c r="K435" t="inlineStr"/>
       <c r="L435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M435" t="inlineStr"/>
-      <c r="N435" t="inlineStr"/>
       <c r="O435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P435" t="inlineStr"/>
-      <c r="Q435" t="inlineStr"/>
       <c r="R435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S435" t="inlineStr"/>
-      <c r="T435" t="inlineStr"/>
       <c r="U435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V435" t="inlineStr"/>
-      <c r="W435" t="inlineStr"/>
       <c r="X435" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -28553,55 +28409,41 @@
           <t>Author of 5 books on nonprofit success, 40+ years coaching boards and executives</t>
         </is>
       </c>
-      <c r="E436" t="inlineStr"/>
       <c r="F436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G436" t="inlineStr"/>
-      <c r="H436" t="inlineStr"/>
       <c r="I436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J436" t="inlineStr"/>
-      <c r="K436" t="inlineStr"/>
       <c r="L436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M436" t="inlineStr"/>
-      <c r="N436" t="inlineStr"/>
       <c r="O436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P436" t="inlineStr"/>
-      <c r="Q436" t="inlineStr"/>
       <c r="R436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S436" t="inlineStr"/>
-      <c r="T436" t="inlineStr"/>
       <c r="U436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V436" t="inlineStr"/>
-      <c r="W436" t="inlineStr"/>
       <c r="X436" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -28624,55 +28466,41 @@
           <t>Editor of The Jossey-Bass Handbook of Nonprofit Leadership and Management (5th ed)</t>
         </is>
       </c>
-      <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G437" t="inlineStr"/>
-      <c r="H437" t="inlineStr"/>
       <c r="I437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J437" t="inlineStr"/>
-      <c r="K437" t="inlineStr"/>
       <c r="L437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M437" t="inlineStr"/>
-      <c r="N437" t="inlineStr"/>
       <c r="O437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P437" t="inlineStr"/>
-      <c r="Q437" t="inlineStr"/>
       <c r="R437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S437" t="inlineStr"/>
-      <c r="T437" t="inlineStr"/>
       <c r="U437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V437" t="inlineStr"/>
-      <c r="W437" t="inlineStr"/>
       <c r="X437" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -28695,27 +28523,21 @@
           <t>30+ years social impact experience, keynote speaker and executive coach</t>
         </is>
       </c>
-      <c r="E438" t="inlineStr"/>
       <c r="F438" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G438" t="inlineStr"/>
-      <c r="H438" t="inlineStr"/>
       <c r="I438" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J438" t="inlineStr"/>
-      <c r="K438" t="inlineStr"/>
       <c r="L438" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M438" t="inlineStr"/>
       <c r="N438" t="inlineStr">
         <is>
           <t>robharter</t>
@@ -28731,27 +28553,395 @@
           <t>X profile</t>
         </is>
       </c>
-      <c r="Q438" t="inlineStr"/>
       <c r="R438" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S438" t="inlineStr"/>
-      <c r="T438" t="inlineStr"/>
       <c r="U438" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V438" t="inlineStr"/>
-      <c r="W438" t="inlineStr"/>
       <c r="X438" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Amanda Kirby</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Do-IT Solutions</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Co-author 'Neurodiversity at Work', 100+ research papers, 25+ years in neurodiversity field</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Theo Smith</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Neurodiversity at Work Ltd</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Co-author 'Neurodiversity at Work', podcast host, LinkedIn Top Voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Nancy Doyle</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Founder &amp; CRO</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Genius Within</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Occupational psychologist, Birkbeck Professor, BPS Working Group founder, spoken at UN</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Ludmila Praslova</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Vanguard University</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Author 'The Canary Code', Thinkers50 Talent Award, first autistic HBR author</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Ed Thompson</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Uptimize</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Author 'A Hidden Force', leads neurodiversity training for Salesforce/JPMorgan/Deloitte</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Jessica McCabe</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>How to ADHD</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>YouTube channel with 2M+ subscribers, bestselling author 'How to ADHD'</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Lyric Rivera</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>NeuroDivergent Consulting</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>NeuroDivergent Rebel, author 'Workplace NeuroDiversity Rising', creator #AskingAutistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Haley Moss</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Attorney &amp; Advocate</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>First openly autistic female attorney in Florida, author of 4 books</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Kate Griggs</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Made By Dyslexia</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Global charity reframing dyslexia, author, podcast host 'Lessons In Dyslexic Thinking'</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Kelly Grainger</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Perfectly Autistic</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Diagnosed autistic ADHDer, 300+ talks for BBC, Red Bull Racing, UN</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Joe Riddle</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>NITW</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Nonprofit behind Fortune 500 neurodivergent hiring programs at SAP, Dell, EY</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Emily Kircher-Morris</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Neurodiversity Podcast</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Licensed counselor, podcast host exploring neurodivergent lives at work</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Noelle Sinclair</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>TEDx speaker, autistic ADHD professional championing cognitive diversity at work</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Brett Whitmarsh</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>VP &amp; Host</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Heinemann Publishing / AuDHD Boss</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Autistic ADHD corporate leader, podcast host sharing workplace strategies</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Daniel M. Jones</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>The Aspie World</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Largest autism-focused YouTube channel globally, 700K+ followers</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Jhillika Kumar</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Mentra</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Forbes 30 Under 30, world's largest neurodiversity employment network</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Susanne Bruyère</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Cornell University</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Director Yang-Tan Institute, co-editor 'Neurodiversity in the Workplace', 120+ publications</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -28765,7 +28955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -29353,6 +29543,26 @@
       <c r="D29" t="inlineStr">
         <is>
           <t>nonprofit-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>17</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>neurodiversity-in-the-workplace</t>
         </is>
       </c>
     </row>
@@ -29368,7 +29578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G225"/>
+  <dimension ref="A1:G233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -37610,6 +37820,302 @@
         </is>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>69c3f1d930396998263ddf1b</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>2026-04-04T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>69c3f1ff30396998263de108</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>2026-04-04T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>69c3f20d30396998263de159</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>2026-05-04T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>69c3f1dc30396998263ddf73</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>2026-04-03T23:01:00Z</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>69c3f20230396998263de12d</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>2026-05-04T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>69c3f1dd30396998263ddfc0</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>2026-04-04T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>69c3f2009e7cfc33a35b8941</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>2026-04-04T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Neurodiversity in the Workplace</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>69c3f1de9e7cfc33a35b87f8</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>2026-04-04T04:30:00Z</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Working Genius
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1162,7 +1162,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1563,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y455"/>
+  <dimension ref="A1:Y471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -28943,6 +28948,1622 @@
         </is>
       </c>
     </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Cody Thompson</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>The Table Group</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Co-host of Working Genius Podcast. Leads content &amp; strategy for the WG framework</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr"/>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr"/>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K456" t="inlineStr"/>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N456" t="inlineStr"/>
+      <c r="O456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q456" t="inlineStr"/>
+      <c r="R456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T456" t="inlineStr"/>
+      <c r="U456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W456" t="inlineStr"/>
+      <c r="X456" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y456" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Tracy Noble</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CDO</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>The Table Group</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Chief Development Officer. Oversees all Table Group products including Working Genius</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr"/>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr"/>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K457" t="inlineStr"/>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N457" t="inlineStr"/>
+      <c r="O457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q457" t="inlineStr"/>
+      <c r="R457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T457" t="inlineStr"/>
+      <c r="U457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W457" t="inlineStr"/>
+      <c r="X457" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y457" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Matt Lencioni</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Content &amp; Podcast Specialist</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>The Table Group</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Podcast specialist &amp; key voice on Working Genius show. Translates ideas into practice</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr"/>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr"/>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K458" t="inlineStr"/>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N458" t="inlineStr"/>
+      <c r="O458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q458" t="inlineStr"/>
+      <c r="R458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T458" t="inlineStr"/>
+      <c r="U458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W458" t="inlineStr"/>
+      <c r="X458" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y458" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Jonathan Bissell</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>CEO &amp; Executive Coach</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>High Performance Impact</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Working Genius Master Facilitator. Director of WG global certification program at The Table Group</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr"/>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr"/>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K459" t="inlineStr"/>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N459" t="inlineStr"/>
+      <c r="O459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q459" t="inlineStr"/>
+      <c r="R459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T459" t="inlineStr"/>
+      <c r="U459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W459" t="inlineStr"/>
+      <c r="X459" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y459" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Kristin Arnold</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>CEO &amp; Master Facilitator</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>The Extraordinary Team</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Certified WG facilitator. Award-winning author &amp; high-stakes meeting facilitator for 27+ years</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr"/>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr"/>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K460" t="inlineStr"/>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N460" t="inlineStr"/>
+      <c r="O460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q460" t="inlineStr"/>
+      <c r="R460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T460" t="inlineStr"/>
+      <c r="U460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W460" t="inlineStr"/>
+      <c r="X460" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y460" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Justin Self</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Founder &amp; Executive Coach</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Continuity Consulting</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Working Genius Master Facilitator. Executive team coach specialising in org health</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr"/>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K461" t="inlineStr"/>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr"/>
+      <c r="O461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q461" t="inlineStr"/>
+      <c r="R461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T461" t="inlineStr"/>
+      <c r="U461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W461" t="inlineStr"/>
+      <c r="X461" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y461" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Jeremy Podany</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Career Leadership Collective</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>WG facilitator for higher education. Serves 1000+ colleges &amp; universities</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr"/>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr"/>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr"/>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr">
+        <is>
+          <t>jeremypodany</t>
+        </is>
+      </c>
+      <c r="O462" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q462" t="inlineStr"/>
+      <c r="R462" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T462" t="inlineStr"/>
+      <c r="U462" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W462" t="inlineStr"/>
+      <c r="X462" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y462" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Dr. Katie Ervin</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Catalyst Development</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>WG facilitator &amp; workplace culture expert. Author of You Might Be An Asshole</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr"/>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr"/>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr"/>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr"/>
+      <c r="O463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q463" t="inlineStr"/>
+      <c r="R463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T463" t="inlineStr"/>
+      <c r="U463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W463" t="inlineStr"/>
+      <c r="X463" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y463" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Greg Harrod</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Executive Business Consultant</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Greg Harrod Enterprises</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Certified WG Facilitator with 30+ years leadership experience. Podcast host</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr"/>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr"/>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr"/>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N464" t="inlineStr"/>
+      <c r="O464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q464" t="inlineStr"/>
+      <c r="R464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T464" t="inlineStr"/>
+      <c r="U464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W464" t="inlineStr"/>
+      <c r="X464" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y464" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Roger Fairhead</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Leadership Specialist</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Roger Fairhead Ltd (UK)</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Certified WG Facilitator. Former CEO of Global Leadership Network UK &amp; Ireland</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>rogerfairhead</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr"/>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N465" t="inlineStr">
+        <is>
+          <t>rogerfairhead</t>
+        </is>
+      </c>
+      <c r="O465" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q465" t="inlineStr"/>
+      <c r="R465" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T465" t="inlineStr"/>
+      <c r="U465" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W465" t="inlineStr"/>
+      <c r="X465" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y465" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Tracy Winkler</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>CEO &amp; Leadership Facilitator</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Elevate2Grow</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Certified WG Facilitator with 30+ years building leaders &amp; high-performing teams</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>TracyWinklerCoach</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr"/>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr"/>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N466" t="inlineStr"/>
+      <c r="O466" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q466" t="inlineStr"/>
+      <c r="R466" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T466" t="inlineStr"/>
+      <c r="U466" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W466" t="inlineStr"/>
+      <c r="X466" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y466" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Cindy Bultema</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Bultema Impact Group</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>WG Facilitator &amp; leadership consultant. 25+ years in ministry &amp; nonprofit leadership</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>CindyBultemaspeaker</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>cindybultema</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr"/>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N467" t="inlineStr">
+        <is>
+          <t>CindyBultema</t>
+        </is>
+      </c>
+      <c r="O467" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q467" t="inlineStr"/>
+      <c r="R467" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T467" t="inlineStr"/>
+      <c r="U467" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W467" t="inlineStr"/>
+      <c r="X467" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y467" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Dr. Candace Goodwin</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Executive Leadership Consultant</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Dr. Candace L. Goodwin LLC</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>WG Facilitator specialising in culture &amp; change management in higher education</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr"/>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr"/>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr"/>
+      <c r="O468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q468" t="inlineStr"/>
+      <c r="R468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T468" t="inlineStr"/>
+      <c r="U468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W468" t="inlineStr"/>
+      <c r="X468" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y468" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Krissy Lewis</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Founder &amp; Communication Coach</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>A Good Work Co</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Certified WG Facilitator with 27+ years coaching speakers &amp; teams on communication</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr"/>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr"/>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr"/>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr"/>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q469" t="inlineStr"/>
+      <c r="R469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T469" t="inlineStr"/>
+      <c r="U469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W469" t="inlineStr"/>
+      <c r="X469" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y469" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Dennis McIntee</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>CEO &amp; Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Leadership Development Group</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>WG certified team. Author of Drama Free Teams. 2000+ companies served</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>LeadershipDevGrp</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr"/>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr"/>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N470" t="inlineStr"/>
+      <c r="O470" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q470" t="inlineStr"/>
+      <c r="R470" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T470" t="inlineStr"/>
+      <c r="U470" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W470" t="inlineStr"/>
+      <c r="X470" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y470" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Larry Collett</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>AI Consultant &amp; WG Trainer</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Automation Captain</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Certified WG trainer who bridges AI innovation with team productivity</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr"/>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr"/>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr"/>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N471" t="inlineStr"/>
+      <c r="O471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q471" t="inlineStr"/>
+      <c r="R471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T471" t="inlineStr"/>
+      <c r="U471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W471" t="inlineStr"/>
+      <c r="X471" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28955,7 +30576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -29563,6 +31184,26 @@
       <c r="D30" t="inlineStr">
         <is>
           <t>neurodiversity-in-the-workplace</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>17</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>working-genius</t>
         </is>
       </c>
     </row>
@@ -29578,7 +31219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G233"/>
+  <dimension ref="A1:G241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38116,6 +39757,302 @@
         </is>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>69c40f40da2cbd2f2bec028e</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>2026-04-04T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>69c40f442af55555f07047b5</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>2026-04-04T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>69c40f7f2af55555f0704999</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>2026-05-05T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>69c40f672af55555f07048de</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>2026-04-04T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>69c40f682af55555f0704915</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>2026-04-04T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>69c40f812af55555f07049bf</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>2026-05-05T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>69c40f692af55555f070493b</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>2026-04-04T13:30:00Z</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Working Genius</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>69c40f852af55555f07049f4</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>2026-04-04T06:12:00Z</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Teacher Wellbeing
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1187,7 +1187,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1568,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y471"/>
+  <dimension ref="A1:Y488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -28969,7 +28974,6 @@
           <t>Co-host of Working Genius Podcast. Leads content &amp; strategy for the WG framework</t>
         </is>
       </c>
-      <c r="E456" t="inlineStr"/>
       <c r="F456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -28980,7 +28984,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H456" t="inlineStr"/>
       <c r="I456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -28991,7 +28994,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K456" t="inlineStr"/>
       <c r="L456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29002,7 +29004,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N456" t="inlineStr"/>
       <c r="O456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29013,7 +29014,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q456" t="inlineStr"/>
       <c r="R456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29024,7 +29024,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T456" t="inlineStr"/>
       <c r="U456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29035,7 +29034,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W456" t="inlineStr"/>
       <c r="X456" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29068,7 +29066,6 @@
           <t>Chief Development Officer. Oversees all Table Group products including Working Genius</t>
         </is>
       </c>
-      <c r="E457" t="inlineStr"/>
       <c r="F457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29079,7 +29076,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H457" t="inlineStr"/>
       <c r="I457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29090,7 +29086,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K457" t="inlineStr"/>
       <c r="L457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29101,7 +29096,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N457" t="inlineStr"/>
       <c r="O457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29112,7 +29106,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q457" t="inlineStr"/>
       <c r="R457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29123,7 +29116,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T457" t="inlineStr"/>
       <c r="U457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29134,7 +29126,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W457" t="inlineStr"/>
       <c r="X457" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29167,7 +29158,6 @@
           <t>Podcast specialist &amp; key voice on Working Genius show. Translates ideas into practice</t>
         </is>
       </c>
-      <c r="E458" t="inlineStr"/>
       <c r="F458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29178,7 +29168,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H458" t="inlineStr"/>
       <c r="I458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29189,7 +29178,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K458" t="inlineStr"/>
       <c r="L458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29200,7 +29188,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N458" t="inlineStr"/>
       <c r="O458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29211,7 +29198,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q458" t="inlineStr"/>
       <c r="R458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29222,7 +29208,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T458" t="inlineStr"/>
       <c r="U458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29233,7 +29218,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W458" t="inlineStr"/>
       <c r="X458" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29266,7 +29250,6 @@
           <t>Working Genius Master Facilitator. Director of WG global certification program at The Table Group</t>
         </is>
       </c>
-      <c r="E459" t="inlineStr"/>
       <c r="F459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29277,7 +29260,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H459" t="inlineStr"/>
       <c r="I459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29288,7 +29270,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K459" t="inlineStr"/>
       <c r="L459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29299,7 +29280,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N459" t="inlineStr"/>
       <c r="O459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29310,7 +29290,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q459" t="inlineStr"/>
       <c r="R459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29321,7 +29300,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T459" t="inlineStr"/>
       <c r="U459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29332,7 +29310,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W459" t="inlineStr"/>
       <c r="X459" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29365,7 +29342,6 @@
           <t>Certified WG facilitator. Award-winning author &amp; high-stakes meeting facilitator for 27+ years</t>
         </is>
       </c>
-      <c r="E460" t="inlineStr"/>
       <c r="F460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29376,7 +29352,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H460" t="inlineStr"/>
       <c r="I460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29387,7 +29362,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K460" t="inlineStr"/>
       <c r="L460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29398,7 +29372,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N460" t="inlineStr"/>
       <c r="O460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29409,7 +29382,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q460" t="inlineStr"/>
       <c r="R460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29420,7 +29392,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T460" t="inlineStr"/>
       <c r="U460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29431,7 +29402,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W460" t="inlineStr"/>
       <c r="X460" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29464,7 +29434,6 @@
           <t>Working Genius Master Facilitator. Executive team coach specialising in org health</t>
         </is>
       </c>
-      <c r="E461" t="inlineStr"/>
       <c r="F461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29475,7 +29444,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H461" t="inlineStr"/>
       <c r="I461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29486,7 +29454,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K461" t="inlineStr"/>
       <c r="L461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29497,7 +29464,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N461" t="inlineStr"/>
       <c r="O461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29508,7 +29474,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q461" t="inlineStr"/>
       <c r="R461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29519,7 +29484,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T461" t="inlineStr"/>
       <c r="U461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29530,7 +29494,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W461" t="inlineStr"/>
       <c r="X461" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29563,7 +29526,6 @@
           <t>WG facilitator for higher education. Serves 1000+ colleges &amp; universities</t>
         </is>
       </c>
-      <c r="E462" t="inlineStr"/>
       <c r="F462" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29574,7 +29536,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H462" t="inlineStr"/>
       <c r="I462" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29585,7 +29546,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K462" t="inlineStr"/>
       <c r="L462" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29611,7 +29571,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q462" t="inlineStr"/>
       <c r="R462" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29622,7 +29581,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T462" t="inlineStr"/>
       <c r="U462" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29633,7 +29591,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W462" t="inlineStr"/>
       <c r="X462" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29666,7 +29623,6 @@
           <t>WG facilitator &amp; workplace culture expert. Author of You Might Be An Asshole</t>
         </is>
       </c>
-      <c r="E463" t="inlineStr"/>
       <c r="F463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29677,7 +29633,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H463" t="inlineStr"/>
       <c r="I463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29688,7 +29643,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K463" t="inlineStr"/>
       <c r="L463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29699,7 +29653,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N463" t="inlineStr"/>
       <c r="O463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29710,7 +29663,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q463" t="inlineStr"/>
       <c r="R463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29721,7 +29673,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T463" t="inlineStr"/>
       <c r="U463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29732,7 +29683,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W463" t="inlineStr"/>
       <c r="X463" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29765,7 +29715,6 @@
           <t>Certified WG Facilitator with 30+ years leadership experience. Podcast host</t>
         </is>
       </c>
-      <c r="E464" t="inlineStr"/>
       <c r="F464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29776,7 +29725,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H464" t="inlineStr"/>
       <c r="I464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29787,7 +29735,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K464" t="inlineStr"/>
       <c r="L464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29798,7 +29745,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N464" t="inlineStr"/>
       <c r="O464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29809,7 +29755,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q464" t="inlineStr"/>
       <c r="R464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29820,7 +29765,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T464" t="inlineStr"/>
       <c r="U464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29831,7 +29775,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W464" t="inlineStr"/>
       <c r="X464" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29879,7 +29822,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H465" t="inlineStr"/>
       <c r="I465" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29890,7 +29832,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K465" t="inlineStr"/>
       <c r="L465" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29916,7 +29857,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q465" t="inlineStr"/>
       <c r="R465" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29927,7 +29867,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T465" t="inlineStr"/>
       <c r="U465" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29938,7 +29877,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W465" t="inlineStr"/>
       <c r="X465" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29986,7 +29924,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H466" t="inlineStr"/>
       <c r="I466" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -29997,7 +29934,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K466" t="inlineStr"/>
       <c r="L466" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30008,7 +29944,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N466" t="inlineStr"/>
       <c r="O466" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30019,7 +29954,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q466" t="inlineStr"/>
       <c r="R466" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30030,7 +29964,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T466" t="inlineStr"/>
       <c r="U466" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30041,7 +29974,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W466" t="inlineStr"/>
       <c r="X466" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30104,7 +30036,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K467" t="inlineStr"/>
       <c r="L467" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30130,7 +30061,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q467" t="inlineStr"/>
       <c r="R467" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30141,7 +30071,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T467" t="inlineStr"/>
       <c r="U467" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30152,7 +30081,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W467" t="inlineStr"/>
       <c r="X467" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30185,7 +30113,6 @@
           <t>WG Facilitator specialising in culture &amp; change management in higher education</t>
         </is>
       </c>
-      <c r="E468" t="inlineStr"/>
       <c r="F468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30196,7 +30123,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H468" t="inlineStr"/>
       <c r="I468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30207,7 +30133,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K468" t="inlineStr"/>
       <c r="L468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30218,7 +30143,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N468" t="inlineStr"/>
       <c r="O468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30229,7 +30153,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q468" t="inlineStr"/>
       <c r="R468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30240,7 +30163,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T468" t="inlineStr"/>
       <c r="U468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30251,7 +30173,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W468" t="inlineStr"/>
       <c r="X468" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30284,7 +30205,6 @@
           <t>Certified WG Facilitator with 27+ years coaching speakers &amp; teams on communication</t>
         </is>
       </c>
-      <c r="E469" t="inlineStr"/>
       <c r="F469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30295,7 +30215,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H469" t="inlineStr"/>
       <c r="I469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30306,7 +30225,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K469" t="inlineStr"/>
       <c r="L469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30317,7 +30235,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N469" t="inlineStr"/>
       <c r="O469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30328,7 +30245,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q469" t="inlineStr"/>
       <c r="R469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30339,7 +30255,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T469" t="inlineStr"/>
       <c r="U469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30350,7 +30265,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W469" t="inlineStr"/>
       <c r="X469" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30398,7 +30312,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H470" t="inlineStr"/>
       <c r="I470" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30409,7 +30322,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K470" t="inlineStr"/>
       <c r="L470" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30420,7 +30332,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N470" t="inlineStr"/>
       <c r="O470" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30431,7 +30342,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q470" t="inlineStr"/>
       <c r="R470" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30442,7 +30352,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T470" t="inlineStr"/>
       <c r="U470" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30453,7 +30362,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W470" t="inlineStr"/>
       <c r="X470" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30486,7 +30394,6 @@
           <t>Certified WG trainer who bridges AI innovation with team productivity</t>
         </is>
       </c>
-      <c r="E471" t="inlineStr"/>
       <c r="F471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30497,7 +30404,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H471" t="inlineStr"/>
       <c r="I471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30508,7 +30414,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K471" t="inlineStr"/>
       <c r="L471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30519,7 +30424,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N471" t="inlineStr"/>
       <c r="O471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30530,7 +30434,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q471" t="inlineStr"/>
       <c r="R471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30541,7 +30444,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T471" t="inlineStr"/>
       <c r="U471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30552,13 +30454,1847 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W471" t="inlineStr"/>
       <c r="X471" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
       <c r="Y471" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Dr. Tina H. Boogren</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Author &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Solution Tree</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Global Gurus #5 Education. 180 Days of Self-Care for Busy Educators. Self-Care for Educators podcast host.</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>selfcareforeducators</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>selfcareforeducators</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>selfcareforeducators</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N472" t="inlineStr">
+        <is>
+          <t>THBoogren</t>
+        </is>
+      </c>
+      <c r="O472" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q472" t="inlineStr"/>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T472" t="inlineStr"/>
+      <c r="U472" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W472" t="inlineStr"/>
+      <c r="X472" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y472" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Angela Watson</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>40 Hour Teacher Workweek</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Truth for Teachers podcast 9M+ downloads. 40 Hour Teacher Workweek program. National Board Certified teacher.</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>TruthForTeachers</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr"/>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr"/>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N473" t="inlineStr">
+        <is>
+          <t>Angela_Watson</t>
+        </is>
+      </c>
+      <c r="O473" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q473" t="inlineStr"/>
+      <c r="R473" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T473" t="inlineStr"/>
+      <c r="U473" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W473" t="inlineStr"/>
+      <c r="X473" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y473" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Adrian Bethune</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Founder of Teachappy</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Teachappy</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>UK teacher. Wellbeing in the Primary Classroom author. Happy Hero medal at House of Lords. Spoke with the Dalai Lama.</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr"/>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>teachappyuk</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr"/>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N474" t="inlineStr">
+        <is>
+          <t>AdrianBethune</t>
+        </is>
+      </c>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q474" t="inlineStr"/>
+      <c r="R474" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T474" t="inlineStr"/>
+      <c r="U474" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W474" t="inlineStr"/>
+      <c r="X474" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y474" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Chase Mielke</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>ASCD</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>The Burnout Cure &amp; Illuminate the Way author. Educator Happy Hour podcast. Featured on CNN, Edutopia.</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>chasemielkespeaker</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>chasemielke</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>chasemielke</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N475" t="inlineStr">
+        <is>
+          <t>ChaseMielke</t>
+        </is>
+      </c>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q475" t="inlineStr"/>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T475" t="inlineStr"/>
+      <c r="U475" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W475" t="inlineStr"/>
+      <c r="X475" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y475" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Daniela Falecki</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Australian educator. 25+ years experience. Trained 7,000+ educators in wellbeing intelligence.</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>teacherwellbeing</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>teacherwellbeing</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>teacherwellbeing</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N476" t="inlineStr">
+        <is>
+          <t>dfalecki</t>
+        </is>
+      </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q476" t="inlineStr"/>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T476" t="inlineStr"/>
+      <c r="U476" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W476" t="inlineStr"/>
+      <c r="X476" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y476" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Dr. Julie Schmidt Hasson</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Professor &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Appalachian State University</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Teacher Recharge Framework creator. TEDx speaker. Author of four books including Pause, Ponder, and Persist.</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr"/>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>julieshasson</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr"/>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N477" t="inlineStr">
+        <is>
+          <t>JulieSHasson</t>
+        </is>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q477" t="inlineStr"/>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T477" t="inlineStr"/>
+      <c r="U477" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W477" t="inlineStr"/>
+      <c r="X477" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y477" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Mandy Froehlich</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Divergent EDU</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>The Fire Within &amp; Reignite the Flames author. Pioneering human sustainability for educator wellness.</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr"/>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>froehlichmandy</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr"/>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N478" t="inlineStr">
+        <is>
+          <t>froehlichm</t>
+        </is>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q478" t="inlineStr"/>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr"/>
+      <c r="U478" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W478" t="inlineStr"/>
+      <c r="X478" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y478" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Meg Durham</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Wellbeing Speaker</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Open Mind Education</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Australian. School of Wellbeing podcast host. M.Ed in Student Wellbeing. National speaker.</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>openmindeduau</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>megdurham__</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr"/>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N479" t="inlineStr"/>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q479" t="inlineStr"/>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T479" t="inlineStr"/>
+      <c r="U479" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W479" t="inlineStr"/>
+      <c r="X479" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y479" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Adrienne Hornby</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Staff Wellbeing Consultant</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Well-Led Schools</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Australian. Worked with 60+ schools. Well-Led Schools podcast host. 6 Steps to Well-Led Schools model.</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr"/>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>adriennehornby_coach</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr"/>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N480" t="inlineStr"/>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q480" t="inlineStr"/>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T480" t="inlineStr"/>
+      <c r="U480" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W480" t="inlineStr"/>
+      <c r="X480" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y480" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Charlie Burley</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Teacher Health Coach</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>The Teachers' Health Coach</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>UK nutritionist and coach. 47K IG followers. Rewriting Wellbeing podcast. Healthy Habits for Teacher Life author.</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>charlie.burley.teachers.health.coach</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>the.teachers.health.coach</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>the.teachers.health.coach</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N481" t="inlineStr">
+        <is>
+          <t>CharlieBurley_</t>
+        </is>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q481" t="inlineStr"/>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T481" t="inlineStr"/>
+      <c r="U481" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W481" t="inlineStr"/>
+      <c r="X481" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y481" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Ellen Ronalds Keene</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Self-Care for Teachers</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Australian teacher and wellbeing coach. Teacher Wellbeing Podcast 119 episodes. Self-Care for Teachers founder.</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr"/>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>selfcareforteachers</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr"/>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N482" t="inlineStr"/>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q482" t="inlineStr"/>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr"/>
+      <c r="U482" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W482" t="inlineStr"/>
+      <c r="X482" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y482" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Dr. Timothy D. Kanold</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Solution Tree</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Co-author of Educator Wellness and HEART! Gold Medal IPPY Award winner. Former superintendent.</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr"/>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr"/>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr"/>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N483" t="inlineStr">
+        <is>
+          <t>tkanold</t>
+        </is>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q483" t="inlineStr"/>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr"/>
+      <c r="U483" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W483" t="inlineStr"/>
+      <c r="X483" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y483" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Dr. Jenny Grant Rankin</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Author &amp; Researcher</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Psychology Today</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Two doctorates. First Aid for Teacher Burnout author. Fulbright Specialist. Taught at Cambridge and Columbia.</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr"/>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>jennygrankin</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr"/>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N484" t="inlineStr">
+        <is>
+          <t>JennyGRankin</t>
+        </is>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q484" t="inlineStr"/>
+      <c r="R484" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T484" t="inlineStr"/>
+      <c r="U484" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W484" t="inlineStr"/>
+      <c r="X484" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y484" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Rae Hughart</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Teachers Deserve It</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>TEDx speaker. Henry Ford Teacher Innovator Award. Empowers educators with sustainable wellness strategies.</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>TeachFurther</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr"/>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr"/>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N485" t="inlineStr">
+        <is>
+          <t>RaeHughart</t>
+        </is>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q485" t="inlineStr">
+        <is>
+          <t>RaeHughart.edu</t>
+        </is>
+      </c>
+      <c r="R485" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T485" t="inlineStr"/>
+      <c r="U485" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W485" t="inlineStr"/>
+      <c r="X485" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y485" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Dr. Emma Kell</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Those That Can</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>UK teacher with doctorate on teacher wellbeing. How To Survive in Teaching author. TEDx Norwich speaker.</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>emmakell</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>thosethatcan</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr"/>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N486" t="inlineStr">
+        <is>
+          <t>thosethatcan</t>
+        </is>
+      </c>
+      <c r="O486" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q486" t="inlineStr"/>
+      <c r="R486" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T486" t="inlineStr"/>
+      <c r="U486" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W486" t="inlineStr">
+        <is>
+          <t>thosethatcan.bsky.social</t>
+        </is>
+      </c>
+      <c r="X486" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="Y486" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Prof. Faye McCallum</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Professor of Education</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>University of Adelaide</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Award-winning Australian researcher on teacher wellbeing. Alby Jones Gold Medal for educational leadership.</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr"/>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr"/>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr"/>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N487" t="inlineStr"/>
+      <c r="O487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q487" t="inlineStr"/>
+      <c r="R487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T487" t="inlineStr"/>
+      <c r="U487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W487" t="inlineStr"/>
+      <c r="X487" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y487" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Dr. Kari Vogelgesang</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Podcast Host &amp; Professor</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>University of Iowa</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Educator Wellness Podcast host. Scanlan Center for School Mental Health. Former elementary teacher.</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr"/>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr"/>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr"/>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N488" t="inlineStr"/>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P488" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q488" t="inlineStr"/>
+      <c r="R488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S488" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T488" t="inlineStr"/>
+      <c r="U488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V488" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W488" t="inlineStr"/>
+      <c r="X488" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y488" t="inlineStr">
         <is>
           <t>Web search</t>
         </is>
@@ -30576,7 +32312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -31204,6 +32940,26 @@
       <c r="D31" t="inlineStr">
         <is>
           <t>working-genius</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>17</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>teacher-wellbeing</t>
         </is>
       </c>
     </row>
@@ -31219,7 +32975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G241"/>
+  <dimension ref="A1:G249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -40053,6 +41809,302 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>69c42b9e21b4a7b258e68297</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>2026-04-04T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>69c42ba121b4a7b258e682bd</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>2026-04-04T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>69c42bd921b4a7b258e683a2</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>2026-05-06T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>69c42bdc2af55555f070d7fa</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>2026-04-04T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>69c42bb921b4a7b258e682f1</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>2026-04-04T14:20:00Z</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>69c42bdd2af55555f070d81f</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>2026-05-06T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>69c42bdf2af55555f070d846</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>2026-04-04T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Teacher Wellbeing</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>69c42be021b4a7b258e683f4</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>2026-04-04T11:30:00Z</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update data/handle-database.xlsx — strengths-based-leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1212,7 +1212,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1573,7 +1578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y488"/>
+  <dimension ref="A1:Y504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30546,7 +30551,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q472" t="inlineStr"/>
       <c r="R472" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30557,7 +30561,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T472" t="inlineStr"/>
       <c r="U472" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30568,7 +30571,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W472" t="inlineStr"/>
       <c r="X472" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30616,7 +30618,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H473" t="inlineStr"/>
       <c r="I473" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30627,7 +30628,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K473" t="inlineStr"/>
       <c r="L473" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30653,7 +30653,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q473" t="inlineStr"/>
       <c r="R473" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30664,7 +30663,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T473" t="inlineStr"/>
       <c r="U473" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30675,7 +30673,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W473" t="inlineStr"/>
       <c r="X473" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30708,7 +30705,6 @@
           <t>UK teacher. Wellbeing in the Primary Classroom author. Happy Hero medal at House of Lords. Spoke with the Dalai Lama.</t>
         </is>
       </c>
-      <c r="E474" t="inlineStr"/>
       <c r="F474" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30734,7 +30730,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K474" t="inlineStr"/>
       <c r="L474" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30760,7 +30755,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q474" t="inlineStr"/>
       <c r="R474" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30771,7 +30765,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T474" t="inlineStr"/>
       <c r="U474" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30782,7 +30775,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W474" t="inlineStr"/>
       <c r="X474" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30875,7 +30867,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q475" t="inlineStr"/>
       <c r="R475" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30886,7 +30877,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T475" t="inlineStr"/>
       <c r="U475" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30897,7 +30887,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W475" t="inlineStr"/>
       <c r="X475" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -30990,7 +30979,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q476" t="inlineStr"/>
       <c r="R476" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31001,7 +30989,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T476" t="inlineStr"/>
       <c r="U476" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31012,7 +30999,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W476" t="inlineStr"/>
       <c r="X476" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31045,7 +31031,6 @@
           <t>Teacher Recharge Framework creator. TEDx speaker. Author of four books including Pause, Ponder, and Persist.</t>
         </is>
       </c>
-      <c r="E477" t="inlineStr"/>
       <c r="F477" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31071,7 +31056,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K477" t="inlineStr"/>
       <c r="L477" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31097,7 +31081,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q477" t="inlineStr"/>
       <c r="R477" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31108,7 +31091,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T477" t="inlineStr"/>
       <c r="U477" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31119,7 +31101,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W477" t="inlineStr"/>
       <c r="X477" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31152,7 +31133,6 @@
           <t>The Fire Within &amp; Reignite the Flames author. Pioneering human sustainability for educator wellness.</t>
         </is>
       </c>
-      <c r="E478" t="inlineStr"/>
       <c r="F478" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31178,7 +31158,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K478" t="inlineStr"/>
       <c r="L478" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31204,7 +31183,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q478" t="inlineStr"/>
       <c r="R478" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31215,7 +31193,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T478" t="inlineStr"/>
       <c r="U478" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31226,7 +31203,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W478" t="inlineStr"/>
       <c r="X478" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31289,7 +31265,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K479" t="inlineStr"/>
       <c r="L479" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31300,7 +31275,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N479" t="inlineStr"/>
       <c r="O479" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31311,7 +31285,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q479" t="inlineStr"/>
       <c r="R479" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31322,7 +31295,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T479" t="inlineStr"/>
       <c r="U479" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31333,7 +31305,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W479" t="inlineStr"/>
       <c r="X479" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31366,7 +31337,6 @@
           <t>Australian. Worked with 60+ schools. Well-Led Schools podcast host. 6 Steps to Well-Led Schools model.</t>
         </is>
       </c>
-      <c r="E480" t="inlineStr"/>
       <c r="F480" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31392,7 +31362,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K480" t="inlineStr"/>
       <c r="L480" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31403,7 +31372,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N480" t="inlineStr"/>
       <c r="O480" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31414,7 +31382,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q480" t="inlineStr"/>
       <c r="R480" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31425,7 +31392,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T480" t="inlineStr"/>
       <c r="U480" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31436,7 +31402,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W480" t="inlineStr"/>
       <c r="X480" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31529,7 +31494,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q481" t="inlineStr"/>
       <c r="R481" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31540,7 +31504,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T481" t="inlineStr"/>
       <c r="U481" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31551,7 +31514,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W481" t="inlineStr"/>
       <c r="X481" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31584,7 +31546,6 @@
           <t>Australian teacher and wellbeing coach. Teacher Wellbeing Podcast 119 episodes. Self-Care for Teachers founder.</t>
         </is>
       </c>
-      <c r="E482" t="inlineStr"/>
       <c r="F482" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31610,7 +31571,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K482" t="inlineStr"/>
       <c r="L482" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31621,7 +31581,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N482" t="inlineStr"/>
       <c r="O482" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31632,7 +31591,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q482" t="inlineStr"/>
       <c r="R482" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31643,7 +31601,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T482" t="inlineStr"/>
       <c r="U482" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31654,7 +31611,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W482" t="inlineStr"/>
       <c r="X482" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31687,7 +31643,6 @@
           <t>Co-author of Educator Wellness and HEART! Gold Medal IPPY Award winner. Former superintendent.</t>
         </is>
       </c>
-      <c r="E483" t="inlineStr"/>
       <c r="F483" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31698,7 +31653,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H483" t="inlineStr"/>
       <c r="I483" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31709,7 +31663,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K483" t="inlineStr"/>
       <c r="L483" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31735,7 +31688,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q483" t="inlineStr"/>
       <c r="R483" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31746,7 +31698,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T483" t="inlineStr"/>
       <c r="U483" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31757,7 +31708,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W483" t="inlineStr"/>
       <c r="X483" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31790,7 +31740,6 @@
           <t>Two doctorates. First Aid for Teacher Burnout author. Fulbright Specialist. Taught at Cambridge and Columbia.</t>
         </is>
       </c>
-      <c r="E484" t="inlineStr"/>
       <c r="F484" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31816,7 +31765,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K484" t="inlineStr"/>
       <c r="L484" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31842,7 +31790,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q484" t="inlineStr"/>
       <c r="R484" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31853,7 +31800,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T484" t="inlineStr"/>
       <c r="U484" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31864,7 +31810,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W484" t="inlineStr"/>
       <c r="X484" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31912,7 +31857,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H485" t="inlineStr"/>
       <c r="I485" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31923,7 +31867,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K485" t="inlineStr"/>
       <c r="L485" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31964,7 +31907,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T485" t="inlineStr"/>
       <c r="U485" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -31975,7 +31917,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W485" t="inlineStr"/>
       <c r="X485" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32038,7 +31979,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K486" t="inlineStr"/>
       <c r="L486" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32064,7 +32004,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q486" t="inlineStr"/>
       <c r="R486" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32075,7 +32014,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T486" t="inlineStr"/>
       <c r="U486" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32123,7 +32061,6 @@
           <t>Award-winning Australian researcher on teacher wellbeing. Alby Jones Gold Medal for educational leadership.</t>
         </is>
       </c>
-      <c r="E487" t="inlineStr"/>
       <c r="F487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32134,7 +32071,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H487" t="inlineStr"/>
       <c r="I487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32145,7 +32081,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K487" t="inlineStr"/>
       <c r="L487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32156,7 +32091,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N487" t="inlineStr"/>
       <c r="O487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32167,7 +32101,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q487" t="inlineStr"/>
       <c r="R487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32178,7 +32111,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T487" t="inlineStr"/>
       <c r="U487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32189,7 +32121,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W487" t="inlineStr"/>
       <c r="X487" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32222,7 +32153,6 @@
           <t>Educator Wellness Podcast host. Scanlan Center for School Mental Health. Former elementary teacher.</t>
         </is>
       </c>
-      <c r="E488" t="inlineStr"/>
       <c r="F488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32233,7 +32163,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H488" t="inlineStr"/>
       <c r="I488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32244,7 +32173,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K488" t="inlineStr"/>
       <c r="L488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32255,7 +32183,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N488" t="inlineStr"/>
       <c r="O488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32266,7 +32193,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q488" t="inlineStr"/>
       <c r="R488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32277,7 +32203,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T488" t="inlineStr"/>
       <c r="U488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32288,7 +32213,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W488" t="inlineStr"/>
       <c r="X488" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -32299,6 +32223,1278 @@
           <t>Web search</t>
         </is>
       </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Tom Rath</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Author &amp; Researcher</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Former Gallup Senior Scientist</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Co-author of Strengths Based Leadership and StrengthsFinder 2.0</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>authortomrath</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>facebook.com/authortomrath</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>tomrath</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>instagram.com/tomrath</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr"/>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr"/>
+      <c r="N489" t="inlineStr">
+        <is>
+          <t>TomCRath</t>
+        </is>
+      </c>
+      <c r="O489" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P489" t="inlineStr">
+        <is>
+          <t>x.com/TomCRath</t>
+        </is>
+      </c>
+      <c r="Q489" t="inlineStr"/>
+      <c r="R489" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S489" t="inlineStr"/>
+      <c r="T489" t="inlineStr"/>
+      <c r="U489" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V489" t="inlineStr"/>
+      <c r="W489" t="inlineStr"/>
+      <c r="X489" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y489" t="inlineStr"/>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Barry Conchie</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Leadership Consultant</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Conchie Associates</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Co-author of Strengths Based Leadership, 35 years in executive assessment</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr"/>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr"/>
+      <c r="H490" t="inlineStr"/>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr"/>
+      <c r="K490" t="inlineStr"/>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr"/>
+      <c r="N490" t="inlineStr">
+        <is>
+          <t>BarryConchie</t>
+        </is>
+      </c>
+      <c r="O490" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P490" t="inlineStr">
+        <is>
+          <t>x.com/BarryConchie</t>
+        </is>
+      </c>
+      <c r="Q490" t="inlineStr"/>
+      <c r="R490" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S490" t="inlineStr"/>
+      <c r="T490" t="inlineStr"/>
+      <c r="U490" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V490" t="inlineStr"/>
+      <c r="W490" t="inlineStr"/>
+      <c r="X490" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y490" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Ryan Niemiec</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Chief Science Officer</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>VIA Institute on Character</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>World's leading expert on character strengths science</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr"/>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr"/>
+      <c r="H491" t="inlineStr"/>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr"/>
+      <c r="K491" t="inlineStr"/>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr"/>
+      <c r="N491" t="inlineStr">
+        <is>
+          <t>ryanVIA</t>
+        </is>
+      </c>
+      <c r="O491" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P491" t="inlineStr">
+        <is>
+          <t>x.com/ryanVIA</t>
+        </is>
+      </c>
+      <c r="Q491" t="inlineStr"/>
+      <c r="R491" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S491" t="inlineStr"/>
+      <c r="T491" t="inlineStr"/>
+      <c r="U491" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V491" t="inlineStr"/>
+      <c r="W491" t="inlineStr"/>
+      <c r="X491" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y491" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Lisa Cummings</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>CEO &amp; Strengths Trainer</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Lead Through Strengths</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Gallup Certified Coach, 20,500+ participants across 14 countries</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr"/>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr"/>
+      <c r="H492" t="inlineStr"/>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr"/>
+      <c r="K492" t="inlineStr"/>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr"/>
+      <c r="N492" t="inlineStr"/>
+      <c r="O492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P492" t="inlineStr"/>
+      <c r="Q492" t="inlineStr"/>
+      <c r="R492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S492" t="inlineStr"/>
+      <c r="T492" t="inlineStr"/>
+      <c r="U492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V492" t="inlineStr"/>
+      <c r="W492" t="inlineStr"/>
+      <c r="X492" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y492" t="inlineStr"/>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Brent O'Bannon</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Strengths Coach</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Strengths Champion Solutions</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>First Gallup-Certified Strengths Coach in the world, 27,000+ hours</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>brentobannonstrengthschampionsolutions</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr"/>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr"/>
+      <c r="K493" t="inlineStr"/>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr"/>
+      <c r="N493" t="inlineStr"/>
+      <c r="O493" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P493" t="inlineStr"/>
+      <c r="Q493" t="inlineStr"/>
+      <c r="R493" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S493" t="inlineStr"/>
+      <c r="T493" t="inlineStr"/>
+      <c r="U493" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V493" t="inlineStr"/>
+      <c r="W493" t="inlineStr"/>
+      <c r="X493" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y493" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Brandon Miller</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>CEO &amp; Co-Founder</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>34 Strong</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>One of the first seven certified Gallup CliftonStrengths coaches</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr"/>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr"/>
+      <c r="H494" t="inlineStr"/>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr"/>
+      <c r="K494" t="inlineStr"/>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr"/>
+      <c r="N494" t="inlineStr"/>
+      <c r="O494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P494" t="inlineStr"/>
+      <c r="Q494" t="inlineStr"/>
+      <c r="R494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S494" t="inlineStr"/>
+      <c r="T494" t="inlineStr"/>
+      <c r="U494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V494" t="inlineStr"/>
+      <c r="W494" t="inlineStr"/>
+      <c r="X494" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y494" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Chuen Chuen Yeo</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Author &amp; Executive Coach</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>ACESENCE, Singapore</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Penguin author of Leaders People Love, CliftonStrengths Coach, 40 countries</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr"/>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr"/>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>yeochuenchuen</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>instagram.com/yeochuenchuen</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr"/>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr"/>
+      <c r="N495" t="inlineStr"/>
+      <c r="O495" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P495" t="inlineStr"/>
+      <c r="Q495" t="inlineStr"/>
+      <c r="R495" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S495" t="inlineStr"/>
+      <c r="T495" t="inlineStr"/>
+      <c r="U495" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V495" t="inlineStr"/>
+      <c r="W495" t="inlineStr"/>
+      <c r="X495" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y495" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Victor Seet</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>StrengthsTransform, Singapore</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>World's first Gold and Platinum Gallup CliftonStrengths Coach</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr"/>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr"/>
+      <c r="H496" t="inlineStr"/>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>victor-seet.com</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr"/>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr"/>
+      <c r="N496" t="inlineStr"/>
+      <c r="O496" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P496" t="inlineStr"/>
+      <c r="Q496" t="inlineStr"/>
+      <c r="R496" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S496" t="inlineStr"/>
+      <c r="T496" t="inlineStr"/>
+      <c r="U496" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V496" t="inlineStr"/>
+      <c r="W496" t="inlineStr"/>
+      <c r="X496" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y496" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Marianne van Woerkom</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Tilburg University</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Leading researcher on strengths-based leadership</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr"/>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr"/>
+      <c r="H497" t="inlineStr"/>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr"/>
+      <c r="K497" t="inlineStr"/>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr"/>
+      <c r="N497" t="inlineStr"/>
+      <c r="O497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P497" t="inlineStr"/>
+      <c r="Q497" t="inlineStr"/>
+      <c r="R497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S497" t="inlineStr"/>
+      <c r="T497" t="inlineStr"/>
+      <c r="U497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V497" t="inlineStr"/>
+      <c r="W497" t="inlineStr"/>
+      <c r="X497" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y497" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Sally Bibb</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>PA Consulting</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Author of The Strengths Book and Strengths-Based Recruitment</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>sallybibbauthorpage</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>sallybibb.com</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>sallybibbauthor</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>sallybibb.com</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr"/>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr"/>
+      <c r="N498" t="inlineStr">
+        <is>
+          <t>sallybibb</t>
+        </is>
+      </c>
+      <c r="O498" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P498" t="inlineStr">
+        <is>
+          <t>sallybibb.com</t>
+        </is>
+      </c>
+      <c r="Q498" t="inlineStr"/>
+      <c r="R498" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S498" t="inlineStr"/>
+      <c r="T498" t="inlineStr"/>
+      <c r="U498" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V498" t="inlineStr"/>
+      <c r="W498" t="inlineStr"/>
+      <c r="X498" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y498" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Jim Collison</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Community Manager</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Gallup</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Host of Called to Coach and The CliftonStrengths Podcast</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr"/>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr"/>
+      <c r="H499" t="inlineStr"/>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr"/>
+      <c r="K499" t="inlineStr"/>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr"/>
+      <c r="N499" t="inlineStr">
+        <is>
+          <t>jcollison</t>
+        </is>
+      </c>
+      <c r="O499" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P499" t="inlineStr">
+        <is>
+          <t>x.com/jcollison</t>
+        </is>
+      </c>
+      <c r="Q499" t="inlineStr"/>
+      <c r="R499" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S499" t="inlineStr"/>
+      <c r="T499" t="inlineStr"/>
+      <c r="U499" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V499" t="inlineStr"/>
+      <c r="W499" t="inlineStr"/>
+      <c r="X499" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y499" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Becky Hammond</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Strengths Maven</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Isogo Strong</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Among original 100 Gallup Certified Coaches, healthcare specialisation</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>isogostrong</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>isogostrong.com</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>isogostrong</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>isogostrong.com</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr"/>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr"/>
+      <c r="N500" t="inlineStr">
+        <is>
+          <t>IsogoStrong</t>
+        </is>
+      </c>
+      <c r="O500" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P500" t="inlineStr">
+        <is>
+          <t>x.com/IsogoStrong</t>
+        </is>
+      </c>
+      <c r="Q500" t="inlineStr"/>
+      <c r="R500" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S500" t="inlineStr"/>
+      <c r="T500" t="inlineStr"/>
+      <c r="U500" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V500" t="inlineStr"/>
+      <c r="W500" t="inlineStr"/>
+      <c r="X500" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y500" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>TyAnn Osborn</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Coach</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Osborn Consulting Group</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>One of first Gallup-Certified coaches worldwide, author A Life Aligned</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr"/>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr"/>
+      <c r="H501" t="inlineStr"/>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>tyannosborn.com</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr"/>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr"/>
+      <c r="N501" t="inlineStr"/>
+      <c r="O501" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P501" t="inlineStr"/>
+      <c r="Q501" t="inlineStr">
+        <is>
+          <t>tyannosborn</t>
+        </is>
+      </c>
+      <c r="R501" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S501" t="inlineStr">
+        <is>
+          <t>tiktok.com/@tyannosborn</t>
+        </is>
+      </c>
+      <c r="T501" t="inlineStr"/>
+      <c r="U501" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V501" t="inlineStr"/>
+      <c r="W501" t="inlineStr"/>
+      <c r="X501" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y501" t="inlineStr"/>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Murray Guest</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Strengths Coach</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Inspire My Business, Australia</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Only coach to speak at all three Gallup Strengths Summits</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr"/>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr"/>
+      <c r="H502" t="inlineStr"/>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr"/>
+      <c r="K502" t="inlineStr"/>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr"/>
+      <c r="N502" t="inlineStr"/>
+      <c r="O502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P502" t="inlineStr"/>
+      <c r="Q502" t="inlineStr"/>
+      <c r="R502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S502" t="inlineStr"/>
+      <c r="T502" t="inlineStr"/>
+      <c r="U502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V502" t="inlineStr"/>
+      <c r="W502" t="inlineStr"/>
+      <c r="X502" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y502" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Alex Linley</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>CEO &amp; Psychologist</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Cappfinity</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Created the Strengths Profile assessment, founder CAPP</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr"/>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr"/>
+      <c r="H503" t="inlineStr"/>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr"/>
+      <c r="K503" t="inlineStr"/>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr"/>
+      <c r="N503" t="inlineStr">
+        <is>
+          <t>AlexLinley</t>
+        </is>
+      </c>
+      <c r="O503" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P503" t="inlineStr">
+        <is>
+          <t>x.com/AlexLinley</t>
+        </is>
+      </c>
+      <c r="Q503" t="inlineStr"/>
+      <c r="R503" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S503" t="inlineStr"/>
+      <c r="T503" t="inlineStr"/>
+      <c r="U503" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V503" t="inlineStr"/>
+      <c r="W503" t="inlineStr"/>
+      <c r="X503" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y503" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Sara Regan</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Strengths Now</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>One of the first dozen Gallup Certified CliftonStrengths Coaches</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr"/>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr"/>
+      <c r="H504" t="inlineStr"/>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr"/>
+      <c r="K504" t="inlineStr"/>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr"/>
+      <c r="N504" t="inlineStr"/>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P504" t="inlineStr"/>
+      <c r="Q504" t="inlineStr"/>
+      <c r="R504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S504" t="inlineStr"/>
+      <c r="T504" t="inlineStr"/>
+      <c r="U504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V504" t="inlineStr"/>
+      <c r="W504" t="inlineStr"/>
+      <c r="X504" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y504" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -32312,7 +33508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -32960,6 +34156,26 @@
       <c r="D32" t="inlineStr">
         <is>
           <t>teacher-wellbeing</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>17</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>strengths-based-leadership</t>
         </is>
       </c>
     </row>
@@ -32975,7 +34191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G249"/>
+  <dimension ref="A1:G257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -42105,6 +43321,298 @@
         </is>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>69c4395921b4a7b258e6d0a9</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>2026-04-04T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>69c4395c2af55555f0712942</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>2026-04-04T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>69c439a921b4a7b258e6e029</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>2026-04-05T04:00:00Z</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>69c439792af55555f07130c8</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>2026-04-04T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>69c4397a2af55555f071313e</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>2026-04-04T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>69c439c92af55555f071384d</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr"/>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>69c4397a21b4a7b258e6d92d</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>2026-04-04T20:30:00Z</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Strengths-Based Leadership</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>69c439922af55555f0713713</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>2026-04-04T13:02:00Z</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Meeting Culture
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1237,7 +1237,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1578,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y504"/>
+  <dimension ref="A1:Y520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -32275,13 +32280,11 @@
           <t>instagram.com/tomrath</t>
         </is>
       </c>
-      <c r="K489" t="inlineStr"/>
       <c r="L489" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M489" t="inlineStr"/>
       <c r="N489" t="inlineStr">
         <is>
           <t>TomCRath</t>
@@ -32297,27 +32300,21 @@
           <t>x.com/TomCRath</t>
         </is>
       </c>
-      <c r="Q489" t="inlineStr"/>
       <c r="R489" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S489" t="inlineStr"/>
-      <c r="T489" t="inlineStr"/>
       <c r="U489" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V489" t="inlineStr"/>
-      <c r="W489" t="inlineStr"/>
       <c r="X489" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -32340,27 +32337,21 @@
           <t>Co-author of Strengths Based Leadership, 35 years in executive assessment</t>
         </is>
       </c>
-      <c r="E490" t="inlineStr"/>
       <c r="F490" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G490" t="inlineStr"/>
-      <c r="H490" t="inlineStr"/>
       <c r="I490" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J490" t="inlineStr"/>
-      <c r="K490" t="inlineStr"/>
       <c r="L490" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M490" t="inlineStr"/>
       <c r="N490" t="inlineStr">
         <is>
           <t>BarryConchie</t>
@@ -32376,27 +32367,21 @@
           <t>x.com/BarryConchie</t>
         </is>
       </c>
-      <c r="Q490" t="inlineStr"/>
       <c r="R490" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S490" t="inlineStr"/>
-      <c r="T490" t="inlineStr"/>
       <c r="U490" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V490" t="inlineStr"/>
-      <c r="W490" t="inlineStr"/>
       <c r="X490" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -32419,27 +32404,21 @@
           <t>World's leading expert on character strengths science</t>
         </is>
       </c>
-      <c r="E491" t="inlineStr"/>
       <c r="F491" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G491" t="inlineStr"/>
-      <c r="H491" t="inlineStr"/>
       <c r="I491" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J491" t="inlineStr"/>
-      <c r="K491" t="inlineStr"/>
       <c r="L491" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M491" t="inlineStr"/>
       <c r="N491" t="inlineStr">
         <is>
           <t>ryanVIA</t>
@@ -32455,27 +32434,21 @@
           <t>x.com/ryanVIA</t>
         </is>
       </c>
-      <c r="Q491" t="inlineStr"/>
       <c r="R491" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S491" t="inlineStr"/>
-      <c r="T491" t="inlineStr"/>
       <c r="U491" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V491" t="inlineStr"/>
-      <c r="W491" t="inlineStr"/>
       <c r="X491" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y491" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -32498,55 +32471,41 @@
           <t>Gallup Certified Coach, 20,500+ participants across 14 countries</t>
         </is>
       </c>
-      <c r="E492" t="inlineStr"/>
       <c r="F492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G492" t="inlineStr"/>
-      <c r="H492" t="inlineStr"/>
       <c r="I492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J492" t="inlineStr"/>
-      <c r="K492" t="inlineStr"/>
       <c r="L492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M492" t="inlineStr"/>
-      <c r="N492" t="inlineStr"/>
       <c r="O492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P492" t="inlineStr"/>
-      <c r="Q492" t="inlineStr"/>
       <c r="R492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S492" t="inlineStr"/>
-      <c r="T492" t="inlineStr"/>
       <c r="U492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V492" t="inlineStr"/>
-      <c r="W492" t="inlineStr"/>
       <c r="X492" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -32584,48 +32543,36 @@
           <t>facebook.com</t>
         </is>
       </c>
-      <c r="H493" t="inlineStr"/>
       <c r="I493" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J493" t="inlineStr"/>
-      <c r="K493" t="inlineStr"/>
       <c r="L493" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M493" t="inlineStr"/>
-      <c r="N493" t="inlineStr"/>
       <c r="O493" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P493" t="inlineStr"/>
-      <c r="Q493" t="inlineStr"/>
       <c r="R493" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S493" t="inlineStr"/>
-      <c r="T493" t="inlineStr"/>
       <c r="U493" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V493" t="inlineStr"/>
-      <c r="W493" t="inlineStr"/>
       <c r="X493" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -32648,55 +32595,41 @@
           <t>One of the first seven certified Gallup CliftonStrengths coaches</t>
         </is>
       </c>
-      <c r="E494" t="inlineStr"/>
       <c r="F494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G494" t="inlineStr"/>
-      <c r="H494" t="inlineStr"/>
       <c r="I494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J494" t="inlineStr"/>
-      <c r="K494" t="inlineStr"/>
       <c r="L494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M494" t="inlineStr"/>
-      <c r="N494" t="inlineStr"/>
       <c r="O494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P494" t="inlineStr"/>
-      <c r="Q494" t="inlineStr"/>
       <c r="R494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S494" t="inlineStr"/>
-      <c r="T494" t="inlineStr"/>
       <c r="U494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V494" t="inlineStr"/>
-      <c r="W494" t="inlineStr"/>
       <c r="X494" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -32719,13 +32652,11 @@
           <t>Penguin author of Leaders People Love, CliftonStrengths Coach, 40 countries</t>
         </is>
       </c>
-      <c r="E495" t="inlineStr"/>
       <c r="F495" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G495" t="inlineStr"/>
       <c r="H495" t="inlineStr">
         <is>
           <t>yeochuenchuen</t>
@@ -32741,41 +32672,31 @@
           <t>instagram.com/yeochuenchuen</t>
         </is>
       </c>
-      <c r="K495" t="inlineStr"/>
       <c r="L495" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M495" t="inlineStr"/>
-      <c r="N495" t="inlineStr"/>
       <c r="O495" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P495" t="inlineStr"/>
-      <c r="Q495" t="inlineStr"/>
       <c r="R495" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S495" t="inlineStr"/>
-      <c r="T495" t="inlineStr"/>
       <c r="U495" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V495" t="inlineStr"/>
-      <c r="W495" t="inlineStr"/>
       <c r="X495" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -32798,14 +32719,11 @@
           <t>World's first Gold and Platinum Gallup CliftonStrengths Coach</t>
         </is>
       </c>
-      <c r="E496" t="inlineStr"/>
       <c r="F496" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G496" t="inlineStr"/>
-      <c r="H496" t="inlineStr"/>
       <c r="I496" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -32816,41 +32734,31 @@
           <t>victor-seet.com</t>
         </is>
       </c>
-      <c r="K496" t="inlineStr"/>
       <c r="L496" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M496" t="inlineStr"/>
-      <c r="N496" t="inlineStr"/>
       <c r="O496" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P496" t="inlineStr"/>
-      <c r="Q496" t="inlineStr"/>
       <c r="R496" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S496" t="inlineStr"/>
-      <c r="T496" t="inlineStr"/>
       <c r="U496" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V496" t="inlineStr"/>
-      <c r="W496" t="inlineStr"/>
       <c r="X496" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -32873,55 +32781,41 @@
           <t>Leading researcher on strengths-based leadership</t>
         </is>
       </c>
-      <c r="E497" t="inlineStr"/>
       <c r="F497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G497" t="inlineStr"/>
-      <c r="H497" t="inlineStr"/>
       <c r="I497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J497" t="inlineStr"/>
-      <c r="K497" t="inlineStr"/>
       <c r="L497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M497" t="inlineStr"/>
-      <c r="N497" t="inlineStr"/>
       <c r="O497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P497" t="inlineStr"/>
-      <c r="Q497" t="inlineStr"/>
       <c r="R497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S497" t="inlineStr"/>
-      <c r="T497" t="inlineStr"/>
       <c r="U497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V497" t="inlineStr"/>
-      <c r="W497" t="inlineStr"/>
       <c r="X497" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -32974,13 +32868,11 @@
           <t>sallybibb.com</t>
         </is>
       </c>
-      <c r="K498" t="inlineStr"/>
       <c r="L498" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M498" t="inlineStr"/>
       <c r="N498" t="inlineStr">
         <is>
           <t>sallybibb</t>
@@ -32996,27 +32888,21 @@
           <t>sallybibb.com</t>
         </is>
       </c>
-      <c r="Q498" t="inlineStr"/>
       <c r="R498" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S498" t="inlineStr"/>
-      <c r="T498" t="inlineStr"/>
       <c r="U498" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V498" t="inlineStr"/>
-      <c r="W498" t="inlineStr"/>
       <c r="X498" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -33039,27 +32925,21 @@
           <t>Host of Called to Coach and The CliftonStrengths Podcast</t>
         </is>
       </c>
-      <c r="E499" t="inlineStr"/>
       <c r="F499" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G499" t="inlineStr"/>
-      <c r="H499" t="inlineStr"/>
       <c r="I499" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J499" t="inlineStr"/>
-      <c r="K499" t="inlineStr"/>
       <c r="L499" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M499" t="inlineStr"/>
       <c r="N499" t="inlineStr">
         <is>
           <t>jcollison</t>
@@ -33075,27 +32955,21 @@
           <t>x.com/jcollison</t>
         </is>
       </c>
-      <c r="Q499" t="inlineStr"/>
       <c r="R499" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S499" t="inlineStr"/>
-      <c r="T499" t="inlineStr"/>
       <c r="U499" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V499" t="inlineStr"/>
-      <c r="W499" t="inlineStr"/>
       <c r="X499" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -33148,13 +33022,11 @@
           <t>isogostrong.com</t>
         </is>
       </c>
-      <c r="K500" t="inlineStr"/>
       <c r="L500" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M500" t="inlineStr"/>
       <c r="N500" t="inlineStr">
         <is>
           <t>IsogoStrong</t>
@@ -33170,27 +33042,21 @@
           <t>x.com/IsogoStrong</t>
         </is>
       </c>
-      <c r="Q500" t="inlineStr"/>
       <c r="R500" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S500" t="inlineStr"/>
-      <c r="T500" t="inlineStr"/>
       <c r="U500" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V500" t="inlineStr"/>
-      <c r="W500" t="inlineStr"/>
       <c r="X500" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -33213,14 +33079,11 @@
           <t>One of first Gallup-Certified coaches worldwide, author A Life Aligned</t>
         </is>
       </c>
-      <c r="E501" t="inlineStr"/>
       <c r="F501" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G501" t="inlineStr"/>
-      <c r="H501" t="inlineStr"/>
       <c r="I501" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -33231,20 +33094,16 @@
           <t>tyannosborn.com</t>
         </is>
       </c>
-      <c r="K501" t="inlineStr"/>
       <c r="L501" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M501" t="inlineStr"/>
-      <c r="N501" t="inlineStr"/>
       <c r="O501" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P501" t="inlineStr"/>
       <c r="Q501" t="inlineStr">
         <is>
           <t>tyannosborn</t>
@@ -33260,20 +33119,16 @@
           <t>tiktok.com/@tyannosborn</t>
         </is>
       </c>
-      <c r="T501" t="inlineStr"/>
       <c r="U501" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V501" t="inlineStr"/>
-      <c r="W501" t="inlineStr"/>
       <c r="X501" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -33296,55 +33151,41 @@
           <t>Only coach to speak at all three Gallup Strengths Summits</t>
         </is>
       </c>
-      <c r="E502" t="inlineStr"/>
       <c r="F502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G502" t="inlineStr"/>
-      <c r="H502" t="inlineStr"/>
       <c r="I502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J502" t="inlineStr"/>
-      <c r="K502" t="inlineStr"/>
       <c r="L502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M502" t="inlineStr"/>
-      <c r="N502" t="inlineStr"/>
       <c r="O502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P502" t="inlineStr"/>
-      <c r="Q502" t="inlineStr"/>
       <c r="R502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S502" t="inlineStr"/>
-      <c r="T502" t="inlineStr"/>
       <c r="U502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V502" t="inlineStr"/>
-      <c r="W502" t="inlineStr"/>
       <c r="X502" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y502" t="inlineStr"/>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -33367,27 +33208,21 @@
           <t>Created the Strengths Profile assessment, founder CAPP</t>
         </is>
       </c>
-      <c r="E503" t="inlineStr"/>
       <c r="F503" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G503" t="inlineStr"/>
-      <c r="H503" t="inlineStr"/>
       <c r="I503" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J503" t="inlineStr"/>
-      <c r="K503" t="inlineStr"/>
       <c r="L503" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M503" t="inlineStr"/>
       <c r="N503" t="inlineStr">
         <is>
           <t>AlexLinley</t>
@@ -33403,27 +33238,21 @@
           <t>x.com/AlexLinley</t>
         </is>
       </c>
-      <c r="Q503" t="inlineStr"/>
       <c r="R503" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S503" t="inlineStr"/>
-      <c r="T503" t="inlineStr"/>
       <c r="U503" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V503" t="inlineStr"/>
-      <c r="W503" t="inlineStr"/>
       <c r="X503" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y503" t="inlineStr"/>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
@@ -33446,55 +33275,1701 @@
           <t>One of the first dozen Gallup Certified CliftonStrengths Coaches</t>
         </is>
       </c>
-      <c r="E504" t="inlineStr"/>
       <c r="F504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G504" t="inlineStr"/>
-      <c r="H504" t="inlineStr"/>
       <c r="I504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J504" t="inlineStr"/>
-      <c r="K504" t="inlineStr"/>
       <c r="L504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M504" t="inlineStr"/>
-      <c r="N504" t="inlineStr"/>
       <c r="O504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="P504" t="inlineStr"/>
-      <c r="Q504" t="inlineStr"/>
       <c r="R504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="S504" t="inlineStr"/>
-      <c r="T504" t="inlineStr"/>
       <c r="U504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V504" t="inlineStr"/>
-      <c r="W504" t="inlineStr"/>
       <c r="X504" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y504" t="inlineStr"/>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Dr. Steven Rogelberg</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Chancellor's Professor</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>UNC Charlotte</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>The world's leading meeting scientist. Author of The Surprising Science of Meetings and Glad We Met.</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr"/>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr"/>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K505" t="inlineStr"/>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N505" t="inlineStr">
+        <is>
+          <t>@stevenrogelberg</t>
+        </is>
+      </c>
+      <c r="O505" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q505" t="inlineStr"/>
+      <c r="R505" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T505" t="inlineStr"/>
+      <c r="U505" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W505" t="inlineStr"/>
+      <c r="X505" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y505" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Rebecca Hinds</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Head of Work AI Institute</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Glean</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Stanford PhD. Author of Your Best Meeting Ever (2026). Founded Asana's Work Innovation Lab.</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr"/>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr"/>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr"/>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N506" t="inlineStr">
+        <is>
+          <t>@RebHinds</t>
+        </is>
+      </c>
+      <c r="O506" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q506" t="inlineStr"/>
+      <c r="R506" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T506" t="inlineStr"/>
+      <c r="U506" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W506" t="inlineStr"/>
+      <c r="X506" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y506" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Elise Keith</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Lucid Meetings</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>The Meeting Maven. Author of Where the Action Is. Inc.com columnist on meeting culture.</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr"/>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr"/>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K507" t="inlineStr"/>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N507" t="inlineStr">
+        <is>
+          <t>@EliseID8</t>
+        </is>
+      </c>
+      <c r="O507" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q507" t="inlineStr"/>
+      <c r="R507" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T507" t="inlineStr"/>
+      <c r="U507" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W507" t="inlineStr"/>
+      <c r="X507" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y507" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Dr. Joseph Allen</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>University of Utah</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>The Meeting Doctor. Co-author of Suddenly Virtual. Has written 25% of all meeting science research.</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr"/>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr"/>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr"/>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N508" t="inlineStr"/>
+      <c r="O508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q508" t="inlineStr"/>
+      <c r="R508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T508" t="inlineStr"/>
+      <c r="U508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W508" t="inlineStr"/>
+      <c r="X508" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y508" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Al Pittampalli</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Modern Meeting Company</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Author of Read This Before Our Next Meeting. Meeting culture warrior. Helped NASA, IBM fix meetings.</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr"/>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr"/>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr"/>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N509" t="inlineStr">
+        <is>
+          <t>@pittampalli</t>
+        </is>
+      </c>
+      <c r="O509" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q509" t="inlineStr"/>
+      <c r="R509" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T509" t="inlineStr"/>
+      <c r="U509" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W509" t="inlineStr"/>
+      <c r="X509" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y509" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Karin Reed</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Speaker Dynamics</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Emmy-winning journalist. Co-author of Suddenly Virtual. Leading voice on virtual meeting presence.</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr"/>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>@speakerdynamics</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr"/>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N510" t="inlineStr">
+        <is>
+          <t>@karin_reed</t>
+        </is>
+      </c>
+      <c r="O510" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q510" t="inlineStr"/>
+      <c r="R510" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T510" t="inlineStr"/>
+      <c r="U510" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W510" t="inlineStr"/>
+      <c r="X510" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y510" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Paul Axtell</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Meeting Effectiveness Consultant</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Contextual Program Designs</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Author of award-winning Meetings Matter and Make Meetings Matter.</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr"/>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr"/>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr"/>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N511" t="inlineStr"/>
+      <c r="O511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q511" t="inlineStr"/>
+      <c r="R511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T511" t="inlineStr"/>
+      <c r="U511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W511" t="inlineStr"/>
+      <c r="X511" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y511" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Douglas Ferguson</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Voltage Control</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Author of Magical Meetings. Hosts Facilitation Lab Podcast. Runs global facilitation certification.</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>@douglasvoltagecontrol</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr"/>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr"/>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N512" t="inlineStr"/>
+      <c r="O512" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q512" t="inlineStr"/>
+      <c r="R512" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T512" t="inlineStr"/>
+      <c r="U512" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W512" t="inlineStr"/>
+      <c r="X512" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y512" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Donna McGeorge</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Keynote Speaker &amp; Author</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Independent (Australia)</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Author of The 25 Minute Meeting. Helps organisations reclaim time with shorter meetings.</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>@makingworkwork</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>@dmcgeorge</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K513" t="inlineStr"/>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N513" t="inlineStr">
+        <is>
+          <t>@DonnaMcGeorge</t>
+        </is>
+      </c>
+      <c r="O513" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q513" t="inlineStr"/>
+      <c r="R513" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T513" t="inlineStr"/>
+      <c r="U513" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W513" t="inlineStr"/>
+      <c r="X513" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y513" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Cameron Herold</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>COO Alliance</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>The CEO Whisperer. Author of Meetings Suck. Teaches leaders to run meetings that drive action.</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr"/>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>@cameronherold</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr"/>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N514" t="inlineStr">
+        <is>
+          <t>@CameronHerold</t>
+        </is>
+      </c>
+      <c r="O514" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q514" t="inlineStr"/>
+      <c r="R514" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T514" t="inlineStr"/>
+      <c r="U514" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W514" t="inlineStr"/>
+      <c r="X514" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y514" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Jason Fried</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Co-founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>37signals / Basecamp</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Champion of meetings-as-last-resort. Author of It Doesn't Have to Be Crazy at Work.</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr"/>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr"/>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K515" t="inlineStr"/>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N515" t="inlineStr">
+        <is>
+          <t>@jasonfried</t>
+        </is>
+      </c>
+      <c r="O515" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q515" t="inlineStr"/>
+      <c r="R515" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T515" t="inlineStr"/>
+      <c r="U515" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W515" t="inlineStr">
+        <is>
+          <t>@jasonfried.bsky.social</t>
+        </is>
+      </c>
+      <c r="X515" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="Y515" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Dr. Liana Kreamer</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Florida Institute of Technology</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Rising meeting science researcher. Studies meeting scheduling and hybrid meeting effectiveness.</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr"/>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr"/>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr"/>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N516" t="inlineStr"/>
+      <c r="O516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q516" t="inlineStr"/>
+      <c r="R516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T516" t="inlineStr"/>
+      <c r="U516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W516" t="inlineStr"/>
+      <c r="X516" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y516" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Graham Allcott</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Think Productive</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Co-author of How to Fix Meetings. Hosts Beyond Busy podcast. UK-based productivity expert.</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr"/>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>@grahamallcott</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K517" t="inlineStr"/>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N517" t="inlineStr">
+        <is>
+          <t>@grahamallcott</t>
+        </is>
+      </c>
+      <c r="O517" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q517" t="inlineStr"/>
+      <c r="R517" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T517" t="inlineStr"/>
+      <c r="U517" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W517" t="inlineStr"/>
+      <c r="X517" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y517" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Lauren Green</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>MeetingMakers</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Host of This Meeting Sucks podcast. Certified facilitator on a mission to fix meetings everywhere.</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr"/>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>@dancingwithmarkers</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr"/>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N518" t="inlineStr">
+        <is>
+          <t>@dancing_markers</t>
+        </is>
+      </c>
+      <c r="O518" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q518" t="inlineStr"/>
+      <c r="R518" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T518" t="inlineStr"/>
+      <c r="U518" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W518" t="inlineStr"/>
+      <c r="X518" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y518" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Sahil Lavingia</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Gumroad</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Runs a company with zero meetings. Pioneer of async-first culture. Author of The Minimalist Entrepreneur.</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr"/>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr"/>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr"/>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N519" t="inlineStr">
+        <is>
+          <t>@shl</t>
+        </is>
+      </c>
+      <c r="O519" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q519" t="inlineStr"/>
+      <c r="R519" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T519" t="inlineStr"/>
+      <c r="U519" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W519" t="inlineStr"/>
+      <c r="X519" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y519" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Helen Chapman</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Co-founder &amp; Director</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>The Facilitation Partnership</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Author of The Meeting Book. Designs powerful business conversations that create action.</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr"/>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr"/>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr"/>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="N520" t="inlineStr"/>
+      <c r="O520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="Q520" t="inlineStr"/>
+      <c r="R520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="T520" t="inlineStr"/>
+      <c r="U520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="W520" t="inlineStr"/>
+      <c r="X520" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y520" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -33508,7 +34983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -34176,6 +35651,26 @@
       <c r="D33" t="inlineStr">
         <is>
           <t>strengths-based-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>17</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>meeting-culture</t>
         </is>
       </c>
     </row>
@@ -34191,7 +35686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G257"/>
+  <dimension ref="A1:G265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -43532,7 +45027,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>draft</t>
@@ -43608,6 +45102,302 @@
         </is>
       </c>
       <c r="G257" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>69c44a677a3b9076bfbf1a9e</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>2026-04-05T05:01:00Z</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>69c44a69fc62f8daf548bc98</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>2026-04-05T05:01:00Z</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>69c44ab57a3b9076bfbf1c19</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>2026-04-04T20:00:00Z</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>69c44a86fc62f8daf548bd3c</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>2026-04-04T20:30:00Z</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>69c44abffc62f8daf548be0f</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>2026-04-10T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>69c44a9d7a3b9076bfbf1ba7</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>2026-04-05T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>69c44a877a3b9076bfbf1b31</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>2026-04-05T04:02:00Z</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Meeting Culture</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>69c44a88fc62f8daf548bd72</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>2026-04-05T02:01:00Z</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
         <is>
           <t>addToQueue</t>
         </is>

</xml_diff>

<commit_message>
Update handle database — Leadership in Healthcare
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1262,7 +1262,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1583,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y520"/>
+  <dimension ref="A1:Y537"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -33332,7 +33337,6 @@
           <t>The world's leading meeting scientist. Author of The Surprising Science of Meetings and Glad We Met.</t>
         </is>
       </c>
-      <c r="E505" t="inlineStr"/>
       <c r="F505" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33343,7 +33347,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H505" t="inlineStr"/>
       <c r="I505" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33354,7 +33357,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K505" t="inlineStr"/>
       <c r="L505" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33380,7 +33382,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q505" t="inlineStr"/>
       <c r="R505" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33391,7 +33392,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T505" t="inlineStr"/>
       <c r="U505" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33402,7 +33402,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W505" t="inlineStr"/>
       <c r="X505" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33435,7 +33434,6 @@
           <t>Stanford PhD. Author of Your Best Meeting Ever (2026). Founded Asana's Work Innovation Lab.</t>
         </is>
       </c>
-      <c r="E506" t="inlineStr"/>
       <c r="F506" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33446,7 +33444,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H506" t="inlineStr"/>
       <c r="I506" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33457,7 +33454,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K506" t="inlineStr"/>
       <c r="L506" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33483,7 +33479,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q506" t="inlineStr"/>
       <c r="R506" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33494,7 +33489,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T506" t="inlineStr"/>
       <c r="U506" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33505,7 +33499,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W506" t="inlineStr"/>
       <c r="X506" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33538,7 +33531,6 @@
           <t>The Meeting Maven. Author of Where the Action Is. Inc.com columnist on meeting culture.</t>
         </is>
       </c>
-      <c r="E507" t="inlineStr"/>
       <c r="F507" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33549,7 +33541,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H507" t="inlineStr"/>
       <c r="I507" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33560,7 +33551,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K507" t="inlineStr"/>
       <c r="L507" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33586,7 +33576,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q507" t="inlineStr"/>
       <c r="R507" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33597,7 +33586,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T507" t="inlineStr"/>
       <c r="U507" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33608,7 +33596,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W507" t="inlineStr"/>
       <c r="X507" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33641,7 +33628,6 @@
           <t>The Meeting Doctor. Co-author of Suddenly Virtual. Has written 25% of all meeting science research.</t>
         </is>
       </c>
-      <c r="E508" t="inlineStr"/>
       <c r="F508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33652,7 +33638,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H508" t="inlineStr"/>
       <c r="I508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33663,7 +33648,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K508" t="inlineStr"/>
       <c r="L508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33674,7 +33658,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N508" t="inlineStr"/>
       <c r="O508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33685,7 +33668,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q508" t="inlineStr"/>
       <c r="R508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33696,7 +33678,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T508" t="inlineStr"/>
       <c r="U508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33707,7 +33688,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W508" t="inlineStr"/>
       <c r="X508" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33740,7 +33720,6 @@
           <t>Author of Read This Before Our Next Meeting. Meeting culture warrior. Helped NASA, IBM fix meetings.</t>
         </is>
       </c>
-      <c r="E509" t="inlineStr"/>
       <c r="F509" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33751,7 +33730,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H509" t="inlineStr"/>
       <c r="I509" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33762,7 +33740,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K509" t="inlineStr"/>
       <c r="L509" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33788,7 +33765,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q509" t="inlineStr"/>
       <c r="R509" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33799,7 +33775,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T509" t="inlineStr"/>
       <c r="U509" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33810,7 +33785,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W509" t="inlineStr"/>
       <c r="X509" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33843,7 +33817,6 @@
           <t>Emmy-winning journalist. Co-author of Suddenly Virtual. Leading voice on virtual meeting presence.</t>
         </is>
       </c>
-      <c r="E510" t="inlineStr"/>
       <c r="F510" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33869,7 +33842,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K510" t="inlineStr"/>
       <c r="L510" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33895,7 +33867,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q510" t="inlineStr"/>
       <c r="R510" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33906,7 +33877,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T510" t="inlineStr"/>
       <c r="U510" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33917,7 +33887,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W510" t="inlineStr"/>
       <c r="X510" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33950,7 +33919,6 @@
           <t>Author of award-winning Meetings Matter and Make Meetings Matter.</t>
         </is>
       </c>
-      <c r="E511" t="inlineStr"/>
       <c r="F511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33961,7 +33929,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H511" t="inlineStr"/>
       <c r="I511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33972,7 +33939,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K511" t="inlineStr"/>
       <c r="L511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33983,7 +33949,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N511" t="inlineStr"/>
       <c r="O511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -33994,7 +33959,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q511" t="inlineStr"/>
       <c r="R511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34005,7 +33969,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T511" t="inlineStr"/>
       <c r="U511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34016,7 +33979,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W511" t="inlineStr"/>
       <c r="X511" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34064,7 +34026,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H512" t="inlineStr"/>
       <c r="I512" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34075,7 +34036,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K512" t="inlineStr"/>
       <c r="L512" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34086,7 +34046,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N512" t="inlineStr"/>
       <c r="O512" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34097,7 +34056,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q512" t="inlineStr"/>
       <c r="R512" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34108,7 +34066,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T512" t="inlineStr"/>
       <c r="U512" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34119,7 +34076,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W512" t="inlineStr"/>
       <c r="X512" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34182,7 +34138,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K513" t="inlineStr"/>
       <c r="L513" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34208,7 +34163,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q513" t="inlineStr"/>
       <c r="R513" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34219,7 +34173,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T513" t="inlineStr"/>
       <c r="U513" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34230,7 +34183,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W513" t="inlineStr"/>
       <c r="X513" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34263,7 +34215,6 @@
           <t>The CEO Whisperer. Author of Meetings Suck. Teaches leaders to run meetings that drive action.</t>
         </is>
       </c>
-      <c r="E514" t="inlineStr"/>
       <c r="F514" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34289,7 +34240,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K514" t="inlineStr"/>
       <c r="L514" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34315,7 +34265,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q514" t="inlineStr"/>
       <c r="R514" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34326,7 +34275,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T514" t="inlineStr"/>
       <c r="U514" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34337,7 +34285,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W514" t="inlineStr"/>
       <c r="X514" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34370,7 +34317,6 @@
           <t>Champion of meetings-as-last-resort. Author of It Doesn't Have to Be Crazy at Work.</t>
         </is>
       </c>
-      <c r="E515" t="inlineStr"/>
       <c r="F515" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34381,7 +34327,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H515" t="inlineStr"/>
       <c r="I515" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34392,7 +34337,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K515" t="inlineStr"/>
       <c r="L515" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34418,7 +34362,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q515" t="inlineStr"/>
       <c r="R515" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34429,7 +34372,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T515" t="inlineStr"/>
       <c r="U515" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34477,7 +34419,6 @@
           <t>Rising meeting science researcher. Studies meeting scheduling and hybrid meeting effectiveness.</t>
         </is>
       </c>
-      <c r="E516" t="inlineStr"/>
       <c r="F516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34488,7 +34429,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H516" t="inlineStr"/>
       <c r="I516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34499,7 +34439,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K516" t="inlineStr"/>
       <c r="L516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34510,7 +34449,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N516" t="inlineStr"/>
       <c r="O516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34521,7 +34459,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q516" t="inlineStr"/>
       <c r="R516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34532,7 +34469,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T516" t="inlineStr"/>
       <c r="U516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34543,7 +34479,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W516" t="inlineStr"/>
       <c r="X516" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34576,7 +34511,6 @@
           <t>Co-author of How to Fix Meetings. Hosts Beyond Busy podcast. UK-based productivity expert.</t>
         </is>
       </c>
-      <c r="E517" t="inlineStr"/>
       <c r="F517" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34602,7 +34536,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K517" t="inlineStr"/>
       <c r="L517" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34628,7 +34561,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q517" t="inlineStr"/>
       <c r="R517" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34639,7 +34571,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T517" t="inlineStr"/>
       <c r="U517" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34650,7 +34581,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W517" t="inlineStr"/>
       <c r="X517" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34683,7 +34613,6 @@
           <t>Host of This Meeting Sucks podcast. Certified facilitator on a mission to fix meetings everywhere.</t>
         </is>
       </c>
-      <c r="E518" t="inlineStr"/>
       <c r="F518" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34709,7 +34638,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K518" t="inlineStr"/>
       <c r="L518" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34735,7 +34663,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q518" t="inlineStr"/>
       <c r="R518" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34746,7 +34673,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T518" t="inlineStr"/>
       <c r="U518" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34757,7 +34683,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W518" t="inlineStr"/>
       <c r="X518" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34790,7 +34715,6 @@
           <t>Runs a company with zero meetings. Pioneer of async-first culture. Author of The Minimalist Entrepreneur.</t>
         </is>
       </c>
-      <c r="E519" t="inlineStr"/>
       <c r="F519" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34801,7 +34725,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H519" t="inlineStr"/>
       <c r="I519" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34812,7 +34735,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K519" t="inlineStr"/>
       <c r="L519" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34838,7 +34760,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q519" t="inlineStr"/>
       <c r="R519" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34849,7 +34770,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T519" t="inlineStr"/>
       <c r="U519" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34860,7 +34780,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W519" t="inlineStr"/>
       <c r="X519" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34893,7 +34812,6 @@
           <t>Author of The Meeting Book. Designs powerful business conversations that create action.</t>
         </is>
       </c>
-      <c r="E520" t="inlineStr"/>
       <c r="F520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34904,7 +34822,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="H520" t="inlineStr"/>
       <c r="I520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34915,7 +34832,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="K520" t="inlineStr"/>
       <c r="L520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34926,7 +34842,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="N520" t="inlineStr"/>
       <c r="O520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34937,7 +34852,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="Q520" t="inlineStr"/>
       <c r="R520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34948,7 +34862,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="T520" t="inlineStr"/>
       <c r="U520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34959,7 +34872,6 @@
           <t>Web search</t>
         </is>
       </c>
-      <c r="W520" t="inlineStr"/>
       <c r="X520" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34968,6 +34880,1793 @@
       <c r="Y520" t="inlineStr">
         <is>
           <t>Web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Quint Studer</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Healthcare Plus Solutions Group</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Created Hardwiring Excellence framework used by 1,000+ hospitals. Malcolm Baldrige Award winner.</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>QuintStuder</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>qdstuder</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K521" t="inlineStr"/>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N521" t="inlineStr">
+        <is>
+          <t>quint_studer</t>
+        </is>
+      </c>
+      <c r="O521" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q521" t="inlineStr"/>
+      <c r="R521" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T521" t="inlineStr"/>
+      <c r="U521" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W521" t="inlineStr"/>
+      <c r="X521" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y521" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Eric Topol</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Scripps Research Translational Institute</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Pioneering AI in medicine. Author of Deep Medicine. Time 100 Health honoree.</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr"/>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>erictopol1</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr"/>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N522" t="inlineStr">
+        <is>
+          <t>EricTopol</t>
+        </is>
+      </c>
+      <c r="O522" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q522" t="inlineStr"/>
+      <c r="R522" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T522" t="inlineStr"/>
+      <c r="U522" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W522" t="inlineStr"/>
+      <c r="X522" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y522" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Atul Gawande</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Surgeon &amp; Author</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Brigham and Women's Hospital</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Wrote The Checklist Manifesto reducing surgical deaths by 47%.</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>AtulGawandeOfficial</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr"/>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K523" t="inlineStr"/>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N523" t="inlineStr">
+        <is>
+          <t>Atul_Gawande</t>
+        </is>
+      </c>
+      <c r="O523" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q523" t="inlineStr"/>
+      <c r="R523" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T523" t="inlineStr"/>
+      <c r="U523" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W523" t="inlineStr"/>
+      <c r="X523" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y523" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Dr. Renee Thompson</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Healthy Workforce Institute</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Leading authority on eradicating bullying and incivility in healthcare.</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>HealthyWorkforceInstitute</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr"/>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K524" t="inlineStr"/>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N524" t="inlineStr">
+        <is>
+          <t>RTConnections</t>
+        </is>
+      </c>
+      <c r="O524" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q524" t="inlineStr"/>
+      <c r="R524" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T524" t="inlineStr"/>
+      <c r="U524" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W524" t="inlineStr"/>
+      <c r="X524" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y524" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Rose Sherman</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Editor in Chief</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Nurse Leader Journal</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Author of The Nurse Leader Coach. Runs emergingrnleader.com blog.</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr"/>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr"/>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K525" t="inlineStr"/>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N525" t="inlineStr"/>
+      <c r="O525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q525" t="inlineStr"/>
+      <c r="R525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T525" t="inlineStr"/>
+      <c r="U525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W525" t="inlineStr"/>
+      <c r="X525" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y525" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Kevin Pho</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>KevinMD.com</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Social media's leading physician voice. 3M+ monthly readers.</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>KevinMD</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>kevinphomd</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K526" t="inlineStr"/>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N526" t="inlineStr">
+        <is>
+          <t>KevinMD</t>
+        </is>
+      </c>
+      <c r="O526" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q526" t="inlineStr"/>
+      <c r="R526" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T526" t="inlineStr"/>
+      <c r="U526" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W526" t="inlineStr"/>
+      <c r="X526" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y526" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Dike Drummond</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>TheHappyMD.com</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Physician burnout prevention specialist. Created the Burnout Prevention Matrix.</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>thehappymd</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr"/>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K527" t="inlineStr"/>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N527" t="inlineStr">
+        <is>
+          <t>thehappymd</t>
+        </is>
+      </c>
+      <c r="O527" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q527" t="inlineStr"/>
+      <c r="R527" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T527" t="inlineStr"/>
+      <c r="U527" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W527" t="inlineStr"/>
+      <c r="X527" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y527" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Bonnie Clipper</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Innovation Advantage</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>First VP of Innovation at ANA. Author of The Nurse's Guide to Innovation.</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr"/>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr"/>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K528" t="inlineStr"/>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N528" t="inlineStr">
+        <is>
+          <t>thoughtleaderRN</t>
+        </is>
+      </c>
+      <c r="O528" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q528" t="inlineStr"/>
+      <c r="R528" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T528" t="inlineStr"/>
+      <c r="U528" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W528" t="inlineStr"/>
+      <c r="X528" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y528" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Agnes Binagwaho</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>University of Global Health Equity</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Former Rwanda Minister of Health who transformed a nation's healthcare system.</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr"/>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr"/>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K529" t="inlineStr"/>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N529" t="inlineStr">
+        <is>
+          <t>agnesbinagwaho</t>
+        </is>
+      </c>
+      <c r="O529" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q529" t="inlineStr"/>
+      <c r="R529" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T529" t="inlineStr"/>
+      <c r="U529" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W529" t="inlineStr"/>
+      <c r="X529" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y529" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Tim Porter-O'Grady</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Senior Partner</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>TPOG Associates</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Created the shared governance model. Author of 26 books on healthcare leadership.</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr"/>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr"/>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K530" t="inlineStr"/>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N530" t="inlineStr"/>
+      <c r="O530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q530" t="inlineStr"/>
+      <c r="R530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T530" t="inlineStr"/>
+      <c r="U530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W530" t="inlineStr"/>
+      <c r="X530" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y530" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Donald Berwick</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>President Emeritus</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>IHI</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Founded the Institute for Healthcare Improvement. Quality improvement pioneer.</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr"/>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr"/>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K531" t="inlineStr"/>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N531" t="inlineStr">
+        <is>
+          <t>donberwick</t>
+        </is>
+      </c>
+      <c r="O531" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q531" t="inlineStr"/>
+      <c r="R531" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T531" t="inlineStr"/>
+      <c r="U531" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W531" t="inlineStr"/>
+      <c r="X531" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y531" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Kay Kennedy</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>uLeadership</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Developed the Human-Centered Leadership model for healthcare.</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr"/>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr"/>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K532" t="inlineStr"/>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N532" t="inlineStr"/>
+      <c r="O532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q532" t="inlineStr"/>
+      <c r="R532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T532" t="inlineStr"/>
+      <c r="U532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W532" t="inlineStr"/>
+      <c r="X532" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y532" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Dr. Kojo Sarfo</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Psychiatric NP &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Uses TikTok and podcasting to make mental health accessible. 2M+ followers.</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr"/>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>drkojosarfo</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>drkojosarfo</t>
+        </is>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N533" t="inlineStr"/>
+      <c r="O533" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q533" t="inlineStr">
+        <is>
+          <t>dr.kojosarfo</t>
+        </is>
+      </c>
+      <c r="R533" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T533" t="inlineStr"/>
+      <c r="U533" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W533" t="inlineStr"/>
+      <c r="X533" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y533" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Nurse Blake</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Nurse Advocate &amp; Comedian</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>4M+ followers using comedy to spotlight nursing issues.</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>NurseBlake</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>nurse.blake</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>nurse.blake</t>
+        </is>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N534" t="inlineStr"/>
+      <c r="O534" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q534" t="inlineStr">
+        <is>
+          <t>nurseblake</t>
+        </is>
+      </c>
+      <c r="R534" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T534" t="inlineStr">
+        <is>
+          <t>NurseBlake</t>
+        </is>
+      </c>
+      <c r="U534" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W534" t="inlineStr"/>
+      <c r="X534" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y534" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Kedar Mate</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Founder &amp; CMO</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Qualified Health</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Former IHI CEO now building AI for healthcare. Weill Cornell faculty.</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr"/>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr"/>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K535" t="inlineStr"/>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N535" t="inlineStr">
+        <is>
+          <t>KedarMate</t>
+        </is>
+      </c>
+      <c r="O535" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q535" t="inlineStr"/>
+      <c r="R535" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T535" t="inlineStr"/>
+      <c r="U535" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W535" t="inlineStr"/>
+      <c r="X535" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y535" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Karl Pister</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>The Coaching Group Inc.</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Hosts the Healthcare Leadership Excellence podcast. 30+ years coaching.</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr"/>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr"/>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K536" t="inlineStr"/>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N536" t="inlineStr"/>
+      <c r="O536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q536" t="inlineStr"/>
+      <c r="R536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T536" t="inlineStr"/>
+      <c r="U536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W536" t="inlineStr"/>
+      <c r="X536" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y536" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Lisa Miller</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>VIE Healthcare Consulting</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Host of Healthcare Leadership Experience podcast. $720M+ in hospital savings.</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr"/>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr"/>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="K537" t="inlineStr"/>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M537" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="N537" t="inlineStr"/>
+      <c r="O537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P537" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="Q537" t="inlineStr"/>
+      <c r="R537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S537" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="T537" t="inlineStr"/>
+      <c r="U537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V537" t="inlineStr">
+        <is>
+          <t>web search</t>
+        </is>
+      </c>
+      <c r="W537" t="inlineStr"/>
+      <c r="X537" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y537" t="inlineStr">
+        <is>
+          <t>web search</t>
         </is>
       </c>
     </row>
@@ -34983,7 +36682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -35671,6 +37370,26 @@
       <c r="D34" t="inlineStr">
         <is>
           <t>meeting-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>17</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>leadership-in-healthcare</t>
         </is>
       </c>
     </row>
@@ -35686,7 +37405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -45403,6 +47122,302 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>69c455eea944ef6d1634475f</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>2026-04-05T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>69c455f06e5c468ed6e79837</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>2026-04-05T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>69c456256e5c468ed6e79a14</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>2026-03-29T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>69c455f2a944ef6d16344785</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>2026-04-05T01:02:00Z</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>69c4561a6e5c468ed6e799c6</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>2026-03-28T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>69c4560e6e5c468ed6e79950</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>2026-04-05T13:30:00Z</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>69c4560d6e5c468ed6e7992a</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>2026-04-05T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Leadership in Healthcare</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>69c4560fa944ef6d1634485d</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>2026-04-05T06:12:00Z</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx with Church Leadership data
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1287,7 +1287,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1588,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y537"/>
+  <dimension ref="A1:Y572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34934,7 +34939,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K521" t="inlineStr"/>
       <c r="L521" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34960,7 +34964,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q521" t="inlineStr"/>
       <c r="R521" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34971,7 +34974,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T521" t="inlineStr"/>
       <c r="U521" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -34982,7 +34984,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W521" t="inlineStr"/>
       <c r="X521" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35015,7 +35016,6 @@
           <t>Pioneering AI in medicine. Author of Deep Medicine. Time 100 Health honoree.</t>
         </is>
       </c>
-      <c r="E522" t="inlineStr"/>
       <c r="F522" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35041,7 +35041,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K522" t="inlineStr"/>
       <c r="L522" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35067,7 +35066,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q522" t="inlineStr"/>
       <c r="R522" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35078,7 +35076,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T522" t="inlineStr"/>
       <c r="U522" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35089,7 +35086,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W522" t="inlineStr"/>
       <c r="X522" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35137,7 +35133,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H523" t="inlineStr"/>
       <c r="I523" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35148,7 +35143,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K523" t="inlineStr"/>
       <c r="L523" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35174,7 +35168,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q523" t="inlineStr"/>
       <c r="R523" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35185,7 +35178,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T523" t="inlineStr"/>
       <c r="U523" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35196,7 +35188,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W523" t="inlineStr"/>
       <c r="X523" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35244,7 +35235,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H524" t="inlineStr"/>
       <c r="I524" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -35255,7 +35245,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K524" t="inlineStr"/>
       <c r="L524" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35281,7 +35270,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q524" t="inlineStr"/>
       <c r="R524" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35292,7 +35280,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T524" t="inlineStr"/>
       <c r="U524" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35303,7 +35290,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W524" t="inlineStr"/>
       <c r="X524" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35336,7 +35322,6 @@
           <t>Author of The Nurse Leader Coach. Runs emergingrnleader.com blog.</t>
         </is>
       </c>
-      <c r="E525" t="inlineStr"/>
       <c r="F525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35347,7 +35332,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H525" t="inlineStr"/>
       <c r="I525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35358,7 +35342,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K525" t="inlineStr"/>
       <c r="L525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35369,7 +35352,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N525" t="inlineStr"/>
       <c r="O525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35380,7 +35362,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q525" t="inlineStr"/>
       <c r="R525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35391,7 +35372,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T525" t="inlineStr"/>
       <c r="U525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35402,7 +35382,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W525" t="inlineStr"/>
       <c r="X525" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35465,7 +35444,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K526" t="inlineStr"/>
       <c r="L526" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35491,7 +35469,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q526" t="inlineStr"/>
       <c r="R526" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35502,7 +35479,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T526" t="inlineStr"/>
       <c r="U526" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -35513,7 +35489,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W526" t="inlineStr"/>
       <c r="X526" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35561,7 +35536,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H527" t="inlineStr"/>
       <c r="I527" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35572,7 +35546,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K527" t="inlineStr"/>
       <c r="L527" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35598,7 +35571,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q527" t="inlineStr"/>
       <c r="R527" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35609,7 +35581,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T527" t="inlineStr"/>
       <c r="U527" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35620,7 +35591,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W527" t="inlineStr"/>
       <c r="X527" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35653,7 +35623,6 @@
           <t>First VP of Innovation at ANA. Author of The Nurse's Guide to Innovation.</t>
         </is>
       </c>
-      <c r="E528" t="inlineStr"/>
       <c r="F528" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35664,7 +35633,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H528" t="inlineStr"/>
       <c r="I528" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -35675,7 +35643,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K528" t="inlineStr"/>
       <c r="L528" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35701,7 +35668,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q528" t="inlineStr"/>
       <c r="R528" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35712,7 +35678,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T528" t="inlineStr"/>
       <c r="U528" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35723,7 +35688,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W528" t="inlineStr"/>
       <c r="X528" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35756,7 +35720,6 @@
           <t>Former Rwanda Minister of Health who transformed a nation's healthcare system.</t>
         </is>
       </c>
-      <c r="E529" t="inlineStr"/>
       <c r="F529" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35767,7 +35730,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H529" t="inlineStr"/>
       <c r="I529" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35778,7 +35740,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K529" t="inlineStr"/>
       <c r="L529" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35804,7 +35765,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q529" t="inlineStr"/>
       <c r="R529" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35815,7 +35775,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T529" t="inlineStr"/>
       <c r="U529" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35826,7 +35785,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W529" t="inlineStr"/>
       <c r="X529" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35859,7 +35817,6 @@
           <t>Created the shared governance model. Author of 26 books on healthcare leadership.</t>
         </is>
       </c>
-      <c r="E530" t="inlineStr"/>
       <c r="F530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35870,7 +35827,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H530" t="inlineStr"/>
       <c r="I530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35881,7 +35837,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K530" t="inlineStr"/>
       <c r="L530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35892,7 +35847,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N530" t="inlineStr"/>
       <c r="O530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35903,7 +35857,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q530" t="inlineStr"/>
       <c r="R530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35914,7 +35867,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T530" t="inlineStr"/>
       <c r="U530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35925,7 +35877,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W530" t="inlineStr"/>
       <c r="X530" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35958,7 +35909,6 @@
           <t>Founded the Institute for Healthcare Improvement. Quality improvement pioneer.</t>
         </is>
       </c>
-      <c r="E531" t="inlineStr"/>
       <c r="F531" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35969,7 +35919,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H531" t="inlineStr"/>
       <c r="I531" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -35980,7 +35929,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K531" t="inlineStr"/>
       <c r="L531" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36006,7 +35954,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q531" t="inlineStr"/>
       <c r="R531" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36017,7 +35964,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T531" t="inlineStr"/>
       <c r="U531" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36028,7 +35974,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W531" t="inlineStr"/>
       <c r="X531" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36061,7 +36006,6 @@
           <t>Developed the Human-Centered Leadership model for healthcare.</t>
         </is>
       </c>
-      <c r="E532" t="inlineStr"/>
       <c r="F532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36072,7 +36016,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H532" t="inlineStr"/>
       <c r="I532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36083,7 +36026,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K532" t="inlineStr"/>
       <c r="L532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36094,7 +36036,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N532" t="inlineStr"/>
       <c r="O532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36105,7 +36046,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q532" t="inlineStr"/>
       <c r="R532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36116,7 +36056,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T532" t="inlineStr"/>
       <c r="U532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36127,7 +36066,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W532" t="inlineStr"/>
       <c r="X532" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36160,7 +36098,6 @@
           <t>Uses TikTok and podcasting to make mental health accessible. 2M+ followers.</t>
         </is>
       </c>
-      <c r="E533" t="inlineStr"/>
       <c r="F533" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36201,7 +36138,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N533" t="inlineStr"/>
       <c r="O533" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36227,7 +36163,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T533" t="inlineStr"/>
       <c r="U533" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -36238,7 +36173,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W533" t="inlineStr"/>
       <c r="X533" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36316,7 +36250,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N534" t="inlineStr"/>
       <c r="O534" t="inlineStr">
         <is>
           <t>LIKELY</t>
@@ -36357,7 +36290,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W534" t="inlineStr"/>
       <c r="X534" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36390,7 +36322,6 @@
           <t>Former IHI CEO now building AI for healthcare. Weill Cornell faculty.</t>
         </is>
       </c>
-      <c r="E535" t="inlineStr"/>
       <c r="F535" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36401,7 +36332,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H535" t="inlineStr"/>
       <c r="I535" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36412,7 +36342,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K535" t="inlineStr"/>
       <c r="L535" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36438,7 +36367,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q535" t="inlineStr"/>
       <c r="R535" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36449,7 +36377,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T535" t="inlineStr"/>
       <c r="U535" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36460,7 +36387,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W535" t="inlineStr"/>
       <c r="X535" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36493,7 +36419,6 @@
           <t>Hosts the Healthcare Leadership Excellence podcast. 30+ years coaching.</t>
         </is>
       </c>
-      <c r="E536" t="inlineStr"/>
       <c r="F536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36504,7 +36429,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H536" t="inlineStr"/>
       <c r="I536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36515,7 +36439,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K536" t="inlineStr"/>
       <c r="L536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36526,7 +36449,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N536" t="inlineStr"/>
       <c r="O536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36537,7 +36459,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q536" t="inlineStr"/>
       <c r="R536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36548,7 +36469,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T536" t="inlineStr"/>
       <c r="U536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36559,7 +36479,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W536" t="inlineStr"/>
       <c r="X536" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36592,7 +36511,6 @@
           <t>Host of Healthcare Leadership Experience podcast. $720M+ in hospital savings.</t>
         </is>
       </c>
-      <c r="E537" t="inlineStr"/>
       <c r="F537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36603,7 +36521,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="H537" t="inlineStr"/>
       <c r="I537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36614,7 +36531,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="K537" t="inlineStr"/>
       <c r="L537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36625,7 +36541,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="N537" t="inlineStr"/>
       <c r="O537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36636,7 +36551,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="Q537" t="inlineStr"/>
       <c r="R537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36647,7 +36561,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="T537" t="inlineStr"/>
       <c r="U537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36658,7 +36571,6 @@
           <t>web search</t>
         </is>
       </c>
-      <c r="W537" t="inlineStr"/>
       <c r="X537" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -36669,6 +36581,2431 @@
           <t>web search</t>
         </is>
       </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Steven Furtick</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Elevation Church</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Author, sermon clips, motivational content</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>stevenfurtick</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>stevenfurtick</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>stevenfurtick</t>
+        </is>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M538" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N538" t="inlineStr"/>
+      <c r="O538" t="inlineStr"/>
+      <c r="P538" t="inlineStr"/>
+      <c r="Q538" t="inlineStr">
+        <is>
+          <t>stevenfurtick</t>
+        </is>
+      </c>
+      <c r="R538" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S538" t="inlineStr">
+        <is>
+          <t>feedspot</t>
+        </is>
+      </c>
+      <c r="T538" t="inlineStr">
+        <is>
+          <t>elevationchurch</t>
+        </is>
+      </c>
+      <c r="U538" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V538" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W538" t="inlineStr"/>
+      <c r="X538" t="inlineStr"/>
+      <c r="Y538" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Carey Nieuwhof</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Author &amp; Podcaster</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Carey Nieuwhof Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>37M+ downloads podcast, church leadership strategy</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr"/>
+      <c r="F539" t="inlineStr"/>
+      <c r="G539" t="inlineStr"/>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>caborneuf</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>caborneuf</t>
+        </is>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M539" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N539" t="inlineStr">
+        <is>
+          <t>caborneuf</t>
+        </is>
+      </c>
+      <c r="O539" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P539" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q539" t="inlineStr"/>
+      <c r="R539" t="inlineStr"/>
+      <c r="S539" t="inlineStr"/>
+      <c r="T539" t="inlineStr">
+        <is>
+          <t>CareyNieuwhof</t>
+        </is>
+      </c>
+      <c r="U539" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V539" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W539" t="inlineStr">
+        <is>
+          <t>careynieuwhof.bsky.social</t>
+        </is>
+      </c>
+      <c r="X539" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y539" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Priscilla Shirer</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Going Beyond Ministries</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Bible teacher, War Room actress</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>priscillashirer</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>priscillashirer</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>priscillashirer</t>
+        </is>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N540" t="inlineStr"/>
+      <c r="O540" t="inlineStr"/>
+      <c r="P540" t="inlineStr"/>
+      <c r="Q540" t="inlineStr"/>
+      <c r="R540" t="inlineStr"/>
+      <c r="S540" t="inlineStr"/>
+      <c r="T540" t="inlineStr">
+        <is>
+          <t>GoingBeyondMinistries</t>
+        </is>
+      </c>
+      <c r="U540" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V540" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W540" t="inlineStr"/>
+      <c r="X540" t="inlineStr"/>
+      <c r="Y540" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Sadie Robertson Huff</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Live Original</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Reaching younger generations with faith leadership</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr"/>
+      <c r="F541" t="inlineStr"/>
+      <c r="G541" t="inlineStr"/>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>legitsadierob</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K541" t="inlineStr"/>
+      <c r="L541" t="inlineStr"/>
+      <c r="M541" t="inlineStr"/>
+      <c r="N541" t="inlineStr"/>
+      <c r="O541" t="inlineStr"/>
+      <c r="P541" t="inlineStr"/>
+      <c r="Q541" t="inlineStr">
+        <is>
+          <t>sadierob</t>
+        </is>
+      </c>
+      <c r="R541" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S541" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="T541" t="inlineStr"/>
+      <c r="U541" t="inlineStr"/>
+      <c r="V541" t="inlineStr"/>
+      <c r="W541" t="inlineStr"/>
+      <c r="X541" t="inlineStr"/>
+      <c r="Y541" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Christine Caine</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>A21 &amp; Propel Women</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Anti-trafficking advocate, women in ministry</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>ChristineCaine</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>christinecaine</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>christinecaine</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M542" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N542" t="inlineStr"/>
+      <c r="O542" t="inlineStr"/>
+      <c r="P542" t="inlineStr"/>
+      <c r="Q542" t="inlineStr"/>
+      <c r="R542" t="inlineStr"/>
+      <c r="S542" t="inlineStr"/>
+      <c r="T542" t="inlineStr"/>
+      <c r="U542" t="inlineStr"/>
+      <c r="V542" t="inlineStr"/>
+      <c r="W542" t="inlineStr"/>
+      <c r="X542" t="inlineStr"/>
+      <c r="Y542" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Louie Giglio</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Pastor</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Passion City Church</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Passion Conferences founder, worship leadership</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>louiegiglio</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>louiegiglio</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K543" t="inlineStr">
+        <is>
+          <t>louiegiglio</t>
+        </is>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M543" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N543" t="inlineStr"/>
+      <c r="O543" t="inlineStr"/>
+      <c r="P543" t="inlineStr"/>
+      <c r="Q543" t="inlineStr"/>
+      <c r="R543" t="inlineStr"/>
+      <c r="S543" t="inlineStr"/>
+      <c r="T543" t="inlineStr">
+        <is>
+          <t>louiegiglio</t>
+        </is>
+      </c>
+      <c r="U543" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V543" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W543" t="inlineStr"/>
+      <c r="X543" t="inlineStr"/>
+      <c r="Y543" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Levi Lusko</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Fresh Life Church</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Creative communicator reaching young adults</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr"/>
+      <c r="F544" t="inlineStr"/>
+      <c r="G544" t="inlineStr"/>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>levilusko</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>levilusko</t>
+        </is>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N544" t="inlineStr"/>
+      <c r="O544" t="inlineStr"/>
+      <c r="P544" t="inlineStr"/>
+      <c r="Q544" t="inlineStr">
+        <is>
+          <t>levilusko</t>
+        </is>
+      </c>
+      <c r="R544" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S544" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="T544" t="inlineStr"/>
+      <c r="U544" t="inlineStr"/>
+      <c r="V544" t="inlineStr"/>
+      <c r="W544" t="inlineStr"/>
+      <c r="X544" t="inlineStr"/>
+      <c r="Y544" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Rich Wilkerson Jr</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>VOUS Church</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Miami pastor, culturally relevant ministry</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr"/>
+      <c r="F545" t="inlineStr"/>
+      <c r="G545" t="inlineStr"/>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>richwilkersonjr</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K545" t="inlineStr"/>
+      <c r="L545" t="inlineStr"/>
+      <c r="M545" t="inlineStr"/>
+      <c r="N545" t="inlineStr"/>
+      <c r="O545" t="inlineStr"/>
+      <c r="P545" t="inlineStr"/>
+      <c r="Q545" t="inlineStr">
+        <is>
+          <t>richwilkersonjr</t>
+        </is>
+      </c>
+      <c r="R545" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S545" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="T545" t="inlineStr"/>
+      <c r="U545" t="inlineStr"/>
+      <c r="V545" t="inlineStr"/>
+      <c r="W545" t="inlineStr"/>
+      <c r="X545" t="inlineStr"/>
+      <c r="Y545" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Chad Veach</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Zoe Church</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>LA pastor, engaging visual content</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr"/>
+      <c r="F546" t="inlineStr"/>
+      <c r="G546" t="inlineStr"/>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>chadveach</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr"/>
+      <c r="L546" t="inlineStr"/>
+      <c r="M546" t="inlineStr"/>
+      <c r="N546" t="inlineStr"/>
+      <c r="O546" t="inlineStr"/>
+      <c r="P546" t="inlineStr"/>
+      <c r="Q546" t="inlineStr">
+        <is>
+          <t>chadveach</t>
+        </is>
+      </c>
+      <c r="R546" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S546" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="T546" t="inlineStr"/>
+      <c r="U546" t="inlineStr"/>
+      <c r="V546" t="inlineStr"/>
+      <c r="W546" t="inlineStr"/>
+      <c r="X546" t="inlineStr"/>
+      <c r="Y546" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Jennie Allen</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>IF:Gathering</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Million-strong women's movement</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>jennieallen</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>jennieallen</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>jennieallen</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M547" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N547" t="inlineStr"/>
+      <c r="O547" t="inlineStr"/>
+      <c r="P547" t="inlineStr"/>
+      <c r="Q547" t="inlineStr"/>
+      <c r="R547" t="inlineStr"/>
+      <c r="S547" t="inlineStr"/>
+      <c r="T547" t="inlineStr"/>
+      <c r="U547" t="inlineStr"/>
+      <c r="V547" t="inlineStr"/>
+      <c r="W547" t="inlineStr"/>
+      <c r="X547" t="inlineStr"/>
+      <c r="Y547" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Albert Tate</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Fellowship Church</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Dynamic communicator, authenticity and humor</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr"/>
+      <c r="F548" t="inlineStr"/>
+      <c r="G548" t="inlineStr"/>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>alberttate</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr"/>
+      <c r="L548" t="inlineStr"/>
+      <c r="M548" t="inlineStr"/>
+      <c r="N548" t="inlineStr"/>
+      <c r="O548" t="inlineStr"/>
+      <c r="P548" t="inlineStr"/>
+      <c r="Q548" t="inlineStr">
+        <is>
+          <t>alberttate</t>
+        </is>
+      </c>
+      <c r="R548" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S548" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="T548" t="inlineStr"/>
+      <c r="U548" t="inlineStr"/>
+      <c r="V548" t="inlineStr"/>
+      <c r="W548" t="inlineStr"/>
+      <c r="X548" t="inlineStr"/>
+      <c r="Y548" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Rich Villodas</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>New Life Fellowship</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>The Deeply Formed Life author, multiracial church</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr"/>
+      <c r="F549" t="inlineStr"/>
+      <c r="G549" t="inlineStr"/>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>richvillodas</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>richvillodas</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M549" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N549" t="inlineStr">
+        <is>
+          <t>richvillodas</t>
+        </is>
+      </c>
+      <c r="O549" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P549" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q549" t="inlineStr"/>
+      <c r="R549" t="inlineStr"/>
+      <c r="S549" t="inlineStr"/>
+      <c r="T549" t="inlineStr"/>
+      <c r="U549" t="inlineStr"/>
+      <c r="V549" t="inlineStr"/>
+      <c r="W549" t="inlineStr">
+        <is>
+          <t>richvillodas.bsky.social</t>
+        </is>
+      </c>
+      <c r="X549" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y549" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Mark Batterson</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>National Community Church</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>The Circle Maker author, church planting pioneer</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>markbatterson</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>markbatterson</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>markbatterson</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M550" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="N550" t="inlineStr">
+        <is>
+          <t>MarkBatterson</t>
+        </is>
+      </c>
+      <c r="O550" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P550" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q550" t="inlineStr"/>
+      <c r="R550" t="inlineStr"/>
+      <c r="S550" t="inlineStr"/>
+      <c r="T550" t="inlineStr">
+        <is>
+          <t>MarkBatterson</t>
+        </is>
+      </c>
+      <c r="U550" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V550" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W550" t="inlineStr"/>
+      <c r="X550" t="inlineStr"/>
+      <c r="Y550" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Dharius Daniels</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Change Church</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Princeton-educated, certified coach</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr"/>
+      <c r="F551" t="inlineStr"/>
+      <c r="G551" t="inlineStr"/>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>dhariusdaniels</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr"/>
+      <c r="L551" t="inlineStr"/>
+      <c r="M551" t="inlineStr"/>
+      <c r="N551" t="inlineStr">
+        <is>
+          <t>DhariusDaniels</t>
+        </is>
+      </c>
+      <c r="O551" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P551" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q551" t="inlineStr"/>
+      <c r="R551" t="inlineStr"/>
+      <c r="S551" t="inlineStr"/>
+      <c r="T551" t="inlineStr"/>
+      <c r="U551" t="inlineStr"/>
+      <c r="V551" t="inlineStr"/>
+      <c r="W551" t="inlineStr"/>
+      <c r="X551" t="inlineStr"/>
+      <c r="Y551" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Jerry Eze</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Streams of Joy International</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>2.2M TikTok followers, viral prayer content</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr"/>
+      <c r="F552" t="inlineStr"/>
+      <c r="G552" t="inlineStr"/>
+      <c r="H552" t="inlineStr"/>
+      <c r="I552" t="inlineStr"/>
+      <c r="J552" t="inlineStr"/>
+      <c r="K552" t="inlineStr"/>
+      <c r="L552" t="inlineStr"/>
+      <c r="M552" t="inlineStr"/>
+      <c r="N552" t="inlineStr"/>
+      <c r="O552" t="inlineStr"/>
+      <c r="P552" t="inlineStr"/>
+      <c r="Q552" t="inlineStr">
+        <is>
+          <t>pastorjerryeze</t>
+        </is>
+      </c>
+      <c r="R552" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S552" t="inlineStr">
+        <is>
+          <t>feedspot</t>
+        </is>
+      </c>
+      <c r="T552" t="inlineStr"/>
+      <c r="U552" t="inlineStr"/>
+      <c r="V552" t="inlineStr"/>
+      <c r="W552" t="inlineStr"/>
+      <c r="X552" t="inlineStr"/>
+      <c r="Y552" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Michael Todd</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Transformation Church</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>1.4M TikTok, 1.7M YT subscribers</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr"/>
+      <c r="F553" t="inlineStr"/>
+      <c r="G553" t="inlineStr"/>
+      <c r="H553" t="inlineStr"/>
+      <c r="I553" t="inlineStr"/>
+      <c r="J553" t="inlineStr"/>
+      <c r="K553" t="inlineStr"/>
+      <c r="L553" t="inlineStr"/>
+      <c r="M553" t="inlineStr"/>
+      <c r="N553" t="inlineStr"/>
+      <c r="O553" t="inlineStr"/>
+      <c r="P553" t="inlineStr"/>
+      <c r="Q553" t="inlineStr">
+        <is>
+          <t>iammiketodd</t>
+        </is>
+      </c>
+      <c r="R553" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S553" t="inlineStr">
+        <is>
+          <t>feedspot</t>
+        </is>
+      </c>
+      <c r="T553" t="inlineStr">
+        <is>
+          <t>TransformationChurch</t>
+        </is>
+      </c>
+      <c r="U553" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V553" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W553" t="inlineStr"/>
+      <c r="X553" t="inlineStr"/>
+      <c r="Y553" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Pastor Mike Jr</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Pastor &amp; Author</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr"/>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>2.4M TikTok followers, faith for younger audiences</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr"/>
+      <c r="F554" t="inlineStr"/>
+      <c r="G554" t="inlineStr"/>
+      <c r="H554" t="inlineStr"/>
+      <c r="I554" t="inlineStr"/>
+      <c r="J554" t="inlineStr"/>
+      <c r="K554" t="inlineStr"/>
+      <c r="L554" t="inlineStr"/>
+      <c r="M554" t="inlineStr"/>
+      <c r="N554" t="inlineStr"/>
+      <c r="O554" t="inlineStr"/>
+      <c r="P554" t="inlineStr"/>
+      <c r="Q554" t="inlineStr">
+        <is>
+          <t>pastormikejr</t>
+        </is>
+      </c>
+      <c r="R554" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S554" t="inlineStr">
+        <is>
+          <t>feedspot</t>
+        </is>
+      </c>
+      <c r="T554" t="inlineStr"/>
+      <c r="U554" t="inlineStr"/>
+      <c r="V554" t="inlineStr"/>
+      <c r="W554" t="inlineStr"/>
+      <c r="X554" t="inlineStr"/>
+      <c r="Y554" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Sam Collier</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Hillsong Atlanta</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Church planter, racial justice voice</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr"/>
+      <c r="F555" t="inlineStr"/>
+      <c r="G555" t="inlineStr"/>
+      <c r="H555" t="inlineStr"/>
+      <c r="I555" t="inlineStr"/>
+      <c r="J555" t="inlineStr"/>
+      <c r="K555" t="inlineStr"/>
+      <c r="L555" t="inlineStr"/>
+      <c r="M555" t="inlineStr"/>
+      <c r="N555" t="inlineStr">
+        <is>
+          <t>PastorSamCollier</t>
+        </is>
+      </c>
+      <c r="O555" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P555" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q555" t="inlineStr">
+        <is>
+          <t>samcollier</t>
+        </is>
+      </c>
+      <c r="R555" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S555" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="T555" t="inlineStr"/>
+      <c r="U555" t="inlineStr"/>
+      <c r="V555" t="inlineStr"/>
+      <c r="W555" t="inlineStr"/>
+      <c r="X555" t="inlineStr"/>
+      <c r="Y555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Judah Smith</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Churchome</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Cultural commentary, faith leadership</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr"/>
+      <c r="F556" t="inlineStr"/>
+      <c r="G556" t="inlineStr"/>
+      <c r="H556" t="inlineStr"/>
+      <c r="I556" t="inlineStr"/>
+      <c r="J556" t="inlineStr"/>
+      <c r="K556" t="inlineStr"/>
+      <c r="L556" t="inlineStr"/>
+      <c r="M556" t="inlineStr"/>
+      <c r="N556" t="inlineStr"/>
+      <c r="O556" t="inlineStr"/>
+      <c r="P556" t="inlineStr"/>
+      <c r="Q556" t="inlineStr">
+        <is>
+          <t>judahsmith</t>
+        </is>
+      </c>
+      <c r="R556" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="S556" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+      <c r="T556" t="inlineStr"/>
+      <c r="U556" t="inlineStr"/>
+      <c r="V556" t="inlineStr"/>
+      <c r="W556" t="inlineStr"/>
+      <c r="X556" t="inlineStr"/>
+      <c r="Y556" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Andy Stanley</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Founding Pastor</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>North Point Community Church</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Your Move podcast, bestselling author</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>andystanley</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr"/>
+      <c r="I557" t="inlineStr"/>
+      <c r="J557" t="inlineStr"/>
+      <c r="K557" t="inlineStr"/>
+      <c r="L557" t="inlineStr"/>
+      <c r="M557" t="inlineStr"/>
+      <c r="N557" t="inlineStr">
+        <is>
+          <t>AndyStanley</t>
+        </is>
+      </c>
+      <c r="O557" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P557" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q557" t="inlineStr"/>
+      <c r="R557" t="inlineStr"/>
+      <c r="S557" t="inlineStr"/>
+      <c r="T557" t="inlineStr">
+        <is>
+          <t>AndyStanley</t>
+        </is>
+      </c>
+      <c r="U557" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V557" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W557" t="inlineStr"/>
+      <c r="X557" t="inlineStr"/>
+      <c r="Y557" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>T.D. Jakes</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Bishop</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>The Potter's House</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>1.79M YouTube subscribers, decades of teaching</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr"/>
+      <c r="F558" t="inlineStr"/>
+      <c r="G558" t="inlineStr"/>
+      <c r="H558" t="inlineStr"/>
+      <c r="I558" t="inlineStr"/>
+      <c r="J558" t="inlineStr"/>
+      <c r="K558" t="inlineStr"/>
+      <c r="L558" t="inlineStr"/>
+      <c r="M558" t="inlineStr"/>
+      <c r="N558" t="inlineStr"/>
+      <c r="O558" t="inlineStr"/>
+      <c r="P558" t="inlineStr"/>
+      <c r="Q558" t="inlineStr"/>
+      <c r="R558" t="inlineStr"/>
+      <c r="S558" t="inlineStr"/>
+      <c r="T558" t="inlineStr">
+        <is>
+          <t>TDJakesOfficial</t>
+        </is>
+      </c>
+      <c r="U558" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V558" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W558" t="inlineStr"/>
+      <c r="X558" t="inlineStr"/>
+      <c r="Y558" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Tony Evans</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Senior Pastor</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Oak Cliff Bible Fellowship</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Popular YouTube, daily devotionals</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>drtonyevans</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr"/>
+      <c r="I559" t="inlineStr"/>
+      <c r="J559" t="inlineStr"/>
+      <c r="K559" t="inlineStr"/>
+      <c r="L559" t="inlineStr"/>
+      <c r="M559" t="inlineStr"/>
+      <c r="N559" t="inlineStr"/>
+      <c r="O559" t="inlineStr"/>
+      <c r="P559" t="inlineStr"/>
+      <c r="Q559" t="inlineStr"/>
+      <c r="R559" t="inlineStr"/>
+      <c r="S559" t="inlineStr"/>
+      <c r="T559" t="inlineStr">
+        <is>
+          <t>TonyEvans</t>
+        </is>
+      </c>
+      <c r="U559" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V559" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W559" t="inlineStr"/>
+      <c r="X559" t="inlineStr"/>
+      <c r="Y559" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Francis Chan</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr"/>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Crazy Love author, church planting</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr"/>
+      <c r="F560" t="inlineStr"/>
+      <c r="G560" t="inlineStr"/>
+      <c r="H560" t="inlineStr"/>
+      <c r="I560" t="inlineStr"/>
+      <c r="J560" t="inlineStr"/>
+      <c r="K560" t="inlineStr"/>
+      <c r="L560" t="inlineStr"/>
+      <c r="M560" t="inlineStr"/>
+      <c r="N560" t="inlineStr"/>
+      <c r="O560" t="inlineStr"/>
+      <c r="P560" t="inlineStr"/>
+      <c r="Q560" t="inlineStr"/>
+      <c r="R560" t="inlineStr"/>
+      <c r="S560" t="inlineStr"/>
+      <c r="T560" t="inlineStr">
+        <is>
+          <t>FrancisChanOfficial</t>
+        </is>
+      </c>
+      <c r="U560" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V560" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W560" t="inlineStr"/>
+      <c r="X560" t="inlineStr"/>
+      <c r="Y560" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Greg Laurie</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Senior Pastor</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Harvest Christian Fellowship</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Prolific social media, evangelistic content</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>greglaurie</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr"/>
+      <c r="I561" t="inlineStr"/>
+      <c r="J561" t="inlineStr"/>
+      <c r="K561" t="inlineStr"/>
+      <c r="L561" t="inlineStr"/>
+      <c r="M561" t="inlineStr"/>
+      <c r="N561" t="inlineStr"/>
+      <c r="O561" t="inlineStr"/>
+      <c r="P561" t="inlineStr"/>
+      <c r="Q561" t="inlineStr"/>
+      <c r="R561" t="inlineStr"/>
+      <c r="S561" t="inlineStr"/>
+      <c r="T561" t="inlineStr">
+        <is>
+          <t>greglaurie</t>
+        </is>
+      </c>
+      <c r="U561" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="V561" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W561" t="inlineStr"/>
+      <c r="X561" t="inlineStr"/>
+      <c r="Y561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>David Platt</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Pastor &amp; Author</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>McLean Bible Church</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Radical author, missions and leadership</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr"/>
+      <c r="F562" t="inlineStr"/>
+      <c r="G562" t="inlineStr"/>
+      <c r="H562" t="inlineStr"/>
+      <c r="I562" t="inlineStr"/>
+      <c r="J562" t="inlineStr"/>
+      <c r="K562" t="inlineStr"/>
+      <c r="L562" t="inlineStr"/>
+      <c r="M562" t="inlineStr"/>
+      <c r="N562" t="inlineStr"/>
+      <c r="O562" t="inlineStr"/>
+      <c r="P562" t="inlineStr"/>
+      <c r="Q562" t="inlineStr"/>
+      <c r="R562" t="inlineStr"/>
+      <c r="S562" t="inlineStr"/>
+      <c r="T562" t="inlineStr">
+        <is>
+          <t>DavidPlatt</t>
+        </is>
+      </c>
+      <c r="U562" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V562" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="W562" t="inlineStr"/>
+      <c r="X562" t="inlineStr"/>
+      <c r="Y562" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Ed Stetzer</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Dean</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Talbot School of Theology</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Church researcher, trend commentator</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr"/>
+      <c r="F563" t="inlineStr"/>
+      <c r="G563" t="inlineStr"/>
+      <c r="H563" t="inlineStr"/>
+      <c r="I563" t="inlineStr"/>
+      <c r="J563" t="inlineStr"/>
+      <c r="K563" t="inlineStr"/>
+      <c r="L563" t="inlineStr"/>
+      <c r="M563" t="inlineStr"/>
+      <c r="N563" t="inlineStr">
+        <is>
+          <t>edstetzer</t>
+        </is>
+      </c>
+      <c r="O563" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P563" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q563" t="inlineStr"/>
+      <c r="R563" t="inlineStr"/>
+      <c r="S563" t="inlineStr"/>
+      <c r="T563" t="inlineStr"/>
+      <c r="U563" t="inlineStr"/>
+      <c r="V563" t="inlineStr"/>
+      <c r="W563" t="inlineStr">
+        <is>
+          <t>edstetzer.bsky.social</t>
+        </is>
+      </c>
+      <c r="X563" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y563" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Matt Chandler</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Lead Pastor</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>The Village Church</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Theological leadership voice</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr"/>
+      <c r="F564" t="inlineStr"/>
+      <c r="G564" t="inlineStr"/>
+      <c r="H564" t="inlineStr"/>
+      <c r="I564" t="inlineStr"/>
+      <c r="J564" t="inlineStr"/>
+      <c r="K564" t="inlineStr"/>
+      <c r="L564" t="inlineStr"/>
+      <c r="M564" t="inlineStr"/>
+      <c r="N564" t="inlineStr">
+        <is>
+          <t>MattChandler74</t>
+        </is>
+      </c>
+      <c r="O564" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P564" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q564" t="inlineStr"/>
+      <c r="R564" t="inlineStr"/>
+      <c r="S564" t="inlineStr"/>
+      <c r="T564" t="inlineStr"/>
+      <c r="U564" t="inlineStr"/>
+      <c r="V564" t="inlineStr"/>
+      <c r="W564" t="inlineStr"/>
+      <c r="X564" t="inlineStr"/>
+      <c r="Y564" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Bob Goff</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr"/>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Love Does author, inspirational leadership</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>bobgoff</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr"/>
+      <c r="I565" t="inlineStr"/>
+      <c r="J565" t="inlineStr"/>
+      <c r="K565" t="inlineStr"/>
+      <c r="L565" t="inlineStr"/>
+      <c r="M565" t="inlineStr"/>
+      <c r="N565" t="inlineStr">
+        <is>
+          <t>bobgoff</t>
+        </is>
+      </c>
+      <c r="O565" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P565" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q565" t="inlineStr"/>
+      <c r="R565" t="inlineStr"/>
+      <c r="S565" t="inlineStr"/>
+      <c r="T565" t="inlineStr"/>
+      <c r="U565" t="inlineStr"/>
+      <c r="V565" t="inlineStr"/>
+      <c r="W565" t="inlineStr">
+        <is>
+          <t>bobgoff.bsky.social</t>
+        </is>
+      </c>
+      <c r="X565" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y565" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Jenni Catron</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>The 4Sight Group</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Church leadership consultant</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr"/>
+      <c r="F566" t="inlineStr"/>
+      <c r="G566" t="inlineStr"/>
+      <c r="H566" t="inlineStr"/>
+      <c r="I566" t="inlineStr"/>
+      <c r="J566" t="inlineStr"/>
+      <c r="K566" t="inlineStr"/>
+      <c r="L566" t="inlineStr"/>
+      <c r="M566" t="inlineStr"/>
+      <c r="N566" t="inlineStr">
+        <is>
+          <t>jennicatron</t>
+        </is>
+      </c>
+      <c r="O566" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P566" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q566" t="inlineStr"/>
+      <c r="R566" t="inlineStr"/>
+      <c r="S566" t="inlineStr"/>
+      <c r="T566" t="inlineStr"/>
+      <c r="U566" t="inlineStr"/>
+      <c r="V566" t="inlineStr"/>
+      <c r="W566" t="inlineStr"/>
+      <c r="X566" t="inlineStr"/>
+      <c r="Y566" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Reggie Joiner</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Orange / Think Orange</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Church curriculum pioneer, next-gen ministry</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr"/>
+      <c r="F567" t="inlineStr"/>
+      <c r="G567" t="inlineStr"/>
+      <c r="H567" t="inlineStr"/>
+      <c r="I567" t="inlineStr"/>
+      <c r="J567" t="inlineStr"/>
+      <c r="K567" t="inlineStr"/>
+      <c r="L567" t="inlineStr"/>
+      <c r="M567" t="inlineStr"/>
+      <c r="N567" t="inlineStr">
+        <is>
+          <t>reggiejoiner</t>
+        </is>
+      </c>
+      <c r="O567" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P567" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q567" t="inlineStr"/>
+      <c r="R567" t="inlineStr"/>
+      <c r="S567" t="inlineStr"/>
+      <c r="T567" t="inlineStr"/>
+      <c r="U567" t="inlineStr"/>
+      <c r="V567" t="inlineStr"/>
+      <c r="W567" t="inlineStr"/>
+      <c r="X567" t="inlineStr"/>
+      <c r="Y567" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>John Mark Comer</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Author &amp; Teacher</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Practicing the Way</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Spiritual formation, bestselling author</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr"/>
+      <c r="F568" t="inlineStr"/>
+      <c r="G568" t="inlineStr"/>
+      <c r="H568" t="inlineStr"/>
+      <c r="I568" t="inlineStr"/>
+      <c r="J568" t="inlineStr"/>
+      <c r="K568" t="inlineStr"/>
+      <c r="L568" t="inlineStr"/>
+      <c r="M568" t="inlineStr"/>
+      <c r="N568" t="inlineStr">
+        <is>
+          <t>johnmarkcomer</t>
+        </is>
+      </c>
+      <c r="O568" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P568" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q568" t="inlineStr"/>
+      <c r="R568" t="inlineStr"/>
+      <c r="S568" t="inlineStr"/>
+      <c r="T568" t="inlineStr"/>
+      <c r="U568" t="inlineStr"/>
+      <c r="V568" t="inlineStr"/>
+      <c r="W568" t="inlineStr">
+        <is>
+          <t>johnmarkcomer.bsky.social</t>
+        </is>
+      </c>
+      <c r="X568" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y568" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Lisa Harper</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr"/>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Bible teacher, warm storytelling voice</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr"/>
+      <c r="F569" t="inlineStr"/>
+      <c r="G569" t="inlineStr"/>
+      <c r="H569" t="inlineStr"/>
+      <c r="I569" t="inlineStr"/>
+      <c r="J569" t="inlineStr"/>
+      <c r="K569" t="inlineStr"/>
+      <c r="L569" t="inlineStr"/>
+      <c r="M569" t="inlineStr"/>
+      <c r="N569" t="inlineStr">
+        <is>
+          <t>lisaharper</t>
+        </is>
+      </c>
+      <c r="O569" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P569" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q569" t="inlineStr"/>
+      <c r="R569" t="inlineStr"/>
+      <c r="S569" t="inlineStr"/>
+      <c r="T569" t="inlineStr"/>
+      <c r="U569" t="inlineStr"/>
+      <c r="V569" t="inlineStr"/>
+      <c r="W569" t="inlineStr"/>
+      <c r="X569" t="inlineStr"/>
+      <c r="Y569" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>J.D. Greear</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Pastor</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>The Summit Church</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Former SBC President, gospel-centered</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr"/>
+      <c r="F570" t="inlineStr"/>
+      <c r="G570" t="inlineStr"/>
+      <c r="H570" t="inlineStr"/>
+      <c r="I570" t="inlineStr"/>
+      <c r="J570" t="inlineStr"/>
+      <c r="K570" t="inlineStr"/>
+      <c r="L570" t="inlineStr"/>
+      <c r="M570" t="inlineStr"/>
+      <c r="N570" t="inlineStr">
+        <is>
+          <t>jdgreear</t>
+        </is>
+      </c>
+      <c r="O570" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P570" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="Q570" t="inlineStr"/>
+      <c r="R570" t="inlineStr"/>
+      <c r="S570" t="inlineStr"/>
+      <c r="T570" t="inlineStr"/>
+      <c r="U570" t="inlineStr"/>
+      <c r="V570" t="inlineStr"/>
+      <c r="W570" t="inlineStr">
+        <is>
+          <t>jdgreear.bsky.social</t>
+        </is>
+      </c>
+      <c r="X570" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y570" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Lysa TerKeurst</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Proverbs 31 Ministries</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Leadership and faith for women</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>OfficialLysaTerKeurst</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr"/>
+      <c r="I571" t="inlineStr"/>
+      <c r="J571" t="inlineStr"/>
+      <c r="K571" t="inlineStr"/>
+      <c r="L571" t="inlineStr"/>
+      <c r="M571" t="inlineStr"/>
+      <c r="N571" t="inlineStr"/>
+      <c r="O571" t="inlineStr"/>
+      <c r="P571" t="inlineStr"/>
+      <c r="Q571" t="inlineStr"/>
+      <c r="R571" t="inlineStr"/>
+      <c r="S571" t="inlineStr"/>
+      <c r="T571" t="inlineStr"/>
+      <c r="U571" t="inlineStr"/>
+      <c r="V571" t="inlineStr"/>
+      <c r="W571" t="inlineStr"/>
+      <c r="X571" t="inlineStr"/>
+      <c r="Y571" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>ChurchLeaders</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Ministry Resource</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>ChurchLeaders.com</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>812K+ likes, equipping ministry leaders</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>ChurchLeaders</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr"/>
+      <c r="I572" t="inlineStr"/>
+      <c r="J572" t="inlineStr"/>
+      <c r="K572" t="inlineStr"/>
+      <c r="L572" t="inlineStr"/>
+      <c r="M572" t="inlineStr"/>
+      <c r="N572" t="inlineStr"/>
+      <c r="O572" t="inlineStr"/>
+      <c r="P572" t="inlineStr"/>
+      <c r="Q572" t="inlineStr"/>
+      <c r="R572" t="inlineStr"/>
+      <c r="S572" t="inlineStr"/>
+      <c r="T572" t="inlineStr"/>
+      <c r="U572" t="inlineStr"/>
+      <c r="V572" t="inlineStr"/>
+      <c r="W572" t="inlineStr"/>
+      <c r="X572" t="inlineStr"/>
+      <c r="Y572" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -36682,7 +39019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -37390,6 +39727,26 @@
       <c r="D35" t="inlineStr">
         <is>
           <t>leadership-in-healthcare</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>17</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>church-leadership</t>
         </is>
       </c>
     </row>
@@ -37405,7 +39762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G273"/>
+  <dimension ref="A1:G281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -47418,6 +49775,302 @@
         </is>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>69c48cb3639981b8e4f29ad6</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>2026-04-05T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>69c48ccb639981b8e4f29b61</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>2026-04-05T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>69c48cd756ee505bd8c7f2ce</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>2026-04-05T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>69c48d0256ee505bd8c7f3bb</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>2026-04-05T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>69c48d0356ee505bd8c7f3e1</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>2026-04-05T14:20:00Z</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>69c48d1c639981b8e4f29c3c</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>2026-04-05T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>69c48d2d56ee505bd8c7f479</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Church Leadership</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>69c48d2f639981b8e4f29c67</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>2026-05-09T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update tracking files for sports-leadership-coaching
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1312,7 +1312,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1593,7 +1598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y572"/>
+  <dimension ref="A1:Y606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36648,9 +36653,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N538" t="inlineStr"/>
-      <c r="O538" t="inlineStr"/>
-      <c r="P538" t="inlineStr"/>
       <c r="Q538" t="inlineStr">
         <is>
           <t>stevenfurtick</t>
@@ -36681,9 +36683,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W538" t="inlineStr"/>
-      <c r="X538" t="inlineStr"/>
-      <c r="Y538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -36706,9 +36705,6 @@
           <t>37M+ downloads podcast, church leadership strategy</t>
         </is>
       </c>
-      <c r="E539" t="inlineStr"/>
-      <c r="F539" t="inlineStr"/>
-      <c r="G539" t="inlineStr"/>
       <c r="H539" t="inlineStr">
         <is>
           <t>caborneuf</t>
@@ -36754,9 +36750,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q539" t="inlineStr"/>
-      <c r="R539" t="inlineStr"/>
-      <c r="S539" t="inlineStr"/>
       <c r="T539" t="inlineStr">
         <is>
           <t>CareyNieuwhof</t>
@@ -36854,12 +36847,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N540" t="inlineStr"/>
-      <c r="O540" t="inlineStr"/>
-      <c r="P540" t="inlineStr"/>
-      <c r="Q540" t="inlineStr"/>
-      <c r="R540" t="inlineStr"/>
-      <c r="S540" t="inlineStr"/>
       <c r="T540" t="inlineStr">
         <is>
           <t>GoingBeyondMinistries</t>
@@ -36875,9 +36862,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W540" t="inlineStr"/>
-      <c r="X540" t="inlineStr"/>
-      <c r="Y540" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -36900,9 +36884,6 @@
           <t>Reaching younger generations with faith leadership</t>
         </is>
       </c>
-      <c r="E541" t="inlineStr"/>
-      <c r="F541" t="inlineStr"/>
-      <c r="G541" t="inlineStr"/>
       <c r="H541" t="inlineStr">
         <is>
           <t>legitsadierob</t>
@@ -36918,12 +36899,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="K541" t="inlineStr"/>
-      <c r="L541" t="inlineStr"/>
-      <c r="M541" t="inlineStr"/>
-      <c r="N541" t="inlineStr"/>
-      <c r="O541" t="inlineStr"/>
-      <c r="P541" t="inlineStr"/>
       <c r="Q541" t="inlineStr">
         <is>
           <t>sadierob</t>
@@ -36939,12 +36914,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="T541" t="inlineStr"/>
-      <c r="U541" t="inlineStr"/>
-      <c r="V541" t="inlineStr"/>
-      <c r="W541" t="inlineStr"/>
-      <c r="X541" t="inlineStr"/>
-      <c r="Y541" t="inlineStr"/>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -37012,18 +36981,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N542" t="inlineStr"/>
-      <c r="O542" t="inlineStr"/>
-      <c r="P542" t="inlineStr"/>
-      <c r="Q542" t="inlineStr"/>
-      <c r="R542" t="inlineStr"/>
-      <c r="S542" t="inlineStr"/>
-      <c r="T542" t="inlineStr"/>
-      <c r="U542" t="inlineStr"/>
-      <c r="V542" t="inlineStr"/>
-      <c r="W542" t="inlineStr"/>
-      <c r="X542" t="inlineStr"/>
-      <c r="Y542" t="inlineStr"/>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -37091,12 +37048,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N543" t="inlineStr"/>
-      <c r="O543" t="inlineStr"/>
-      <c r="P543" t="inlineStr"/>
-      <c r="Q543" t="inlineStr"/>
-      <c r="R543" t="inlineStr"/>
-      <c r="S543" t="inlineStr"/>
       <c r="T543" t="inlineStr">
         <is>
           <t>louiegiglio</t>
@@ -37112,9 +37063,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W543" t="inlineStr"/>
-      <c r="X543" t="inlineStr"/>
-      <c r="Y543" t="inlineStr"/>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -37137,9 +37085,6 @@
           <t>Creative communicator reaching young adults</t>
         </is>
       </c>
-      <c r="E544" t="inlineStr"/>
-      <c r="F544" t="inlineStr"/>
-      <c r="G544" t="inlineStr"/>
       <c r="H544" t="inlineStr">
         <is>
           <t>levilusko</t>
@@ -37170,9 +37115,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N544" t="inlineStr"/>
-      <c r="O544" t="inlineStr"/>
-      <c r="P544" t="inlineStr"/>
       <c r="Q544" t="inlineStr">
         <is>
           <t>levilusko</t>
@@ -37188,12 +37130,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="T544" t="inlineStr"/>
-      <c r="U544" t="inlineStr"/>
-      <c r="V544" t="inlineStr"/>
-      <c r="W544" t="inlineStr"/>
-      <c r="X544" t="inlineStr"/>
-      <c r="Y544" t="inlineStr"/>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -37216,9 +37152,6 @@
           <t>Miami pastor, culturally relevant ministry</t>
         </is>
       </c>
-      <c r="E545" t="inlineStr"/>
-      <c r="F545" t="inlineStr"/>
-      <c r="G545" t="inlineStr"/>
       <c r="H545" t="inlineStr">
         <is>
           <t>richwilkersonjr</t>
@@ -37234,12 +37167,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="K545" t="inlineStr"/>
-      <c r="L545" t="inlineStr"/>
-      <c r="M545" t="inlineStr"/>
-      <c r="N545" t="inlineStr"/>
-      <c r="O545" t="inlineStr"/>
-      <c r="P545" t="inlineStr"/>
       <c r="Q545" t="inlineStr">
         <is>
           <t>richwilkersonjr</t>
@@ -37255,12 +37182,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="T545" t="inlineStr"/>
-      <c r="U545" t="inlineStr"/>
-      <c r="V545" t="inlineStr"/>
-      <c r="W545" t="inlineStr"/>
-      <c r="X545" t="inlineStr"/>
-      <c r="Y545" t="inlineStr"/>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -37283,9 +37204,6 @@
           <t>LA pastor, engaging visual content</t>
         </is>
       </c>
-      <c r="E546" t="inlineStr"/>
-      <c r="F546" t="inlineStr"/>
-      <c r="G546" t="inlineStr"/>
       <c r="H546" t="inlineStr">
         <is>
           <t>chadveach</t>
@@ -37301,12 +37219,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="K546" t="inlineStr"/>
-      <c r="L546" t="inlineStr"/>
-      <c r="M546" t="inlineStr"/>
-      <c r="N546" t="inlineStr"/>
-      <c r="O546" t="inlineStr"/>
-      <c r="P546" t="inlineStr"/>
       <c r="Q546" t="inlineStr">
         <is>
           <t>chadveach</t>
@@ -37322,12 +37234,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="T546" t="inlineStr"/>
-      <c r="U546" t="inlineStr"/>
-      <c r="V546" t="inlineStr"/>
-      <c r="W546" t="inlineStr"/>
-      <c r="X546" t="inlineStr"/>
-      <c r="Y546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -37395,18 +37301,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="N547" t="inlineStr"/>
-      <c r="O547" t="inlineStr"/>
-      <c r="P547" t="inlineStr"/>
-      <c r="Q547" t="inlineStr"/>
-      <c r="R547" t="inlineStr"/>
-      <c r="S547" t="inlineStr"/>
-      <c r="T547" t="inlineStr"/>
-      <c r="U547" t="inlineStr"/>
-      <c r="V547" t="inlineStr"/>
-      <c r="W547" t="inlineStr"/>
-      <c r="X547" t="inlineStr"/>
-      <c r="Y547" t="inlineStr"/>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -37429,9 +37323,6 @@
           <t>Dynamic communicator, authenticity and humor</t>
         </is>
       </c>
-      <c r="E548" t="inlineStr"/>
-      <c r="F548" t="inlineStr"/>
-      <c r="G548" t="inlineStr"/>
       <c r="H548" t="inlineStr">
         <is>
           <t>alberttate</t>
@@ -37447,12 +37338,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="K548" t="inlineStr"/>
-      <c r="L548" t="inlineStr"/>
-      <c r="M548" t="inlineStr"/>
-      <c r="N548" t="inlineStr"/>
-      <c r="O548" t="inlineStr"/>
-      <c r="P548" t="inlineStr"/>
       <c r="Q548" t="inlineStr">
         <is>
           <t>alberttate</t>
@@ -37468,12 +37353,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="T548" t="inlineStr"/>
-      <c r="U548" t="inlineStr"/>
-      <c r="V548" t="inlineStr"/>
-      <c r="W548" t="inlineStr"/>
-      <c r="X548" t="inlineStr"/>
-      <c r="Y548" t="inlineStr"/>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -37496,9 +37375,6 @@
           <t>The Deeply Formed Life author, multiracial church</t>
         </is>
       </c>
-      <c r="E549" t="inlineStr"/>
-      <c r="F549" t="inlineStr"/>
-      <c r="G549" t="inlineStr"/>
       <c r="H549" t="inlineStr">
         <is>
           <t>richvillodas</t>
@@ -37544,12 +37420,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q549" t="inlineStr"/>
-      <c r="R549" t="inlineStr"/>
-      <c r="S549" t="inlineStr"/>
-      <c r="T549" t="inlineStr"/>
-      <c r="U549" t="inlineStr"/>
-      <c r="V549" t="inlineStr"/>
       <c r="W549" t="inlineStr">
         <is>
           <t>richvillodas.bsky.social</t>
@@ -37647,9 +37517,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q550" t="inlineStr"/>
-      <c r="R550" t="inlineStr"/>
-      <c r="S550" t="inlineStr"/>
       <c r="T550" t="inlineStr">
         <is>
           <t>MarkBatterson</t>
@@ -37665,9 +37532,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W550" t="inlineStr"/>
-      <c r="X550" t="inlineStr"/>
-      <c r="Y550" t="inlineStr"/>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
@@ -37690,9 +37554,6 @@
           <t>Princeton-educated, certified coach</t>
         </is>
       </c>
-      <c r="E551" t="inlineStr"/>
-      <c r="F551" t="inlineStr"/>
-      <c r="G551" t="inlineStr"/>
       <c r="H551" t="inlineStr">
         <is>
           <t>dhariusdaniels</t>
@@ -37708,9 +37569,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="K551" t="inlineStr"/>
-      <c r="L551" t="inlineStr"/>
-      <c r="M551" t="inlineStr"/>
       <c r="N551" t="inlineStr">
         <is>
           <t>DhariusDaniels</t>
@@ -37726,15 +37584,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q551" t="inlineStr"/>
-      <c r="R551" t="inlineStr"/>
-      <c r="S551" t="inlineStr"/>
-      <c r="T551" t="inlineStr"/>
-      <c r="U551" t="inlineStr"/>
-      <c r="V551" t="inlineStr"/>
-      <c r="W551" t="inlineStr"/>
-      <c r="X551" t="inlineStr"/>
-      <c r="Y551" t="inlineStr"/>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr">
@@ -37757,18 +37606,6 @@
           <t>2.2M TikTok followers, viral prayer content</t>
         </is>
       </c>
-      <c r="E552" t="inlineStr"/>
-      <c r="F552" t="inlineStr"/>
-      <c r="G552" t="inlineStr"/>
-      <c r="H552" t="inlineStr"/>
-      <c r="I552" t="inlineStr"/>
-      <c r="J552" t="inlineStr"/>
-      <c r="K552" t="inlineStr"/>
-      <c r="L552" t="inlineStr"/>
-      <c r="M552" t="inlineStr"/>
-      <c r="N552" t="inlineStr"/>
-      <c r="O552" t="inlineStr"/>
-      <c r="P552" t="inlineStr"/>
       <c r="Q552" t="inlineStr">
         <is>
           <t>pastorjerryeze</t>
@@ -37784,12 +37621,6 @@
           <t>feedspot</t>
         </is>
       </c>
-      <c r="T552" t="inlineStr"/>
-      <c r="U552" t="inlineStr"/>
-      <c r="V552" t="inlineStr"/>
-      <c r="W552" t="inlineStr"/>
-      <c r="X552" t="inlineStr"/>
-      <c r="Y552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -37812,18 +37643,6 @@
           <t>1.4M TikTok, 1.7M YT subscribers</t>
         </is>
       </c>
-      <c r="E553" t="inlineStr"/>
-      <c r="F553" t="inlineStr"/>
-      <c r="G553" t="inlineStr"/>
-      <c r="H553" t="inlineStr"/>
-      <c r="I553" t="inlineStr"/>
-      <c r="J553" t="inlineStr"/>
-      <c r="K553" t="inlineStr"/>
-      <c r="L553" t="inlineStr"/>
-      <c r="M553" t="inlineStr"/>
-      <c r="N553" t="inlineStr"/>
-      <c r="O553" t="inlineStr"/>
-      <c r="P553" t="inlineStr"/>
       <c r="Q553" t="inlineStr">
         <is>
           <t>iammiketodd</t>
@@ -37854,9 +37673,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W553" t="inlineStr"/>
-      <c r="X553" t="inlineStr"/>
-      <c r="Y553" t="inlineStr"/>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
@@ -37869,24 +37685,11 @@
           <t>Pastor &amp; Author</t>
         </is>
       </c>
-      <c r="C554" t="inlineStr"/>
       <c r="D554" t="inlineStr">
         <is>
           <t>2.4M TikTok followers, faith for younger audiences</t>
         </is>
       </c>
-      <c r="E554" t="inlineStr"/>
-      <c r="F554" t="inlineStr"/>
-      <c r="G554" t="inlineStr"/>
-      <c r="H554" t="inlineStr"/>
-      <c r="I554" t="inlineStr"/>
-      <c r="J554" t="inlineStr"/>
-      <c r="K554" t="inlineStr"/>
-      <c r="L554" t="inlineStr"/>
-      <c r="M554" t="inlineStr"/>
-      <c r="N554" t="inlineStr"/>
-      <c r="O554" t="inlineStr"/>
-      <c r="P554" t="inlineStr"/>
       <c r="Q554" t="inlineStr">
         <is>
           <t>pastormikejr</t>
@@ -37902,12 +37705,6 @@
           <t>feedspot</t>
         </is>
       </c>
-      <c r="T554" t="inlineStr"/>
-      <c r="U554" t="inlineStr"/>
-      <c r="V554" t="inlineStr"/>
-      <c r="W554" t="inlineStr"/>
-      <c r="X554" t="inlineStr"/>
-      <c r="Y554" t="inlineStr"/>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -37930,15 +37727,6 @@
           <t>Church planter, racial justice voice</t>
         </is>
       </c>
-      <c r="E555" t="inlineStr"/>
-      <c r="F555" t="inlineStr"/>
-      <c r="G555" t="inlineStr"/>
-      <c r="H555" t="inlineStr"/>
-      <c r="I555" t="inlineStr"/>
-      <c r="J555" t="inlineStr"/>
-      <c r="K555" t="inlineStr"/>
-      <c r="L555" t="inlineStr"/>
-      <c r="M555" t="inlineStr"/>
       <c r="N555" t="inlineStr">
         <is>
           <t>PastorSamCollier</t>
@@ -37969,12 +37757,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="T555" t="inlineStr"/>
-      <c r="U555" t="inlineStr"/>
-      <c r="V555" t="inlineStr"/>
-      <c r="W555" t="inlineStr"/>
-      <c r="X555" t="inlineStr"/>
-      <c r="Y555" t="inlineStr"/>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -37997,18 +37779,6 @@
           <t>Cultural commentary, faith leadership</t>
         </is>
       </c>
-      <c r="E556" t="inlineStr"/>
-      <c r="F556" t="inlineStr"/>
-      <c r="G556" t="inlineStr"/>
-      <c r="H556" t="inlineStr"/>
-      <c r="I556" t="inlineStr"/>
-      <c r="J556" t="inlineStr"/>
-      <c r="K556" t="inlineStr"/>
-      <c r="L556" t="inlineStr"/>
-      <c r="M556" t="inlineStr"/>
-      <c r="N556" t="inlineStr"/>
-      <c r="O556" t="inlineStr"/>
-      <c r="P556" t="inlineStr"/>
       <c r="Q556" t="inlineStr">
         <is>
           <t>judahsmith</t>
@@ -38024,12 +37794,6 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="T556" t="inlineStr"/>
-      <c r="U556" t="inlineStr"/>
-      <c r="V556" t="inlineStr"/>
-      <c r="W556" t="inlineStr"/>
-      <c r="X556" t="inlineStr"/>
-      <c r="Y556" t="inlineStr"/>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
@@ -38067,12 +37831,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="H557" t="inlineStr"/>
-      <c r="I557" t="inlineStr"/>
-      <c r="J557" t="inlineStr"/>
-      <c r="K557" t="inlineStr"/>
-      <c r="L557" t="inlineStr"/>
-      <c r="M557" t="inlineStr"/>
       <c r="N557" t="inlineStr">
         <is>
           <t>AndyStanley</t>
@@ -38088,9 +37846,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q557" t="inlineStr"/>
-      <c r="R557" t="inlineStr"/>
-      <c r="S557" t="inlineStr"/>
       <c r="T557" t="inlineStr">
         <is>
           <t>AndyStanley</t>
@@ -38106,9 +37861,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W557" t="inlineStr"/>
-      <c r="X557" t="inlineStr"/>
-      <c r="Y557" t="inlineStr"/>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -38131,21 +37883,6 @@
           <t>1.79M YouTube subscribers, decades of teaching</t>
         </is>
       </c>
-      <c r="E558" t="inlineStr"/>
-      <c r="F558" t="inlineStr"/>
-      <c r="G558" t="inlineStr"/>
-      <c r="H558" t="inlineStr"/>
-      <c r="I558" t="inlineStr"/>
-      <c r="J558" t="inlineStr"/>
-      <c r="K558" t="inlineStr"/>
-      <c r="L558" t="inlineStr"/>
-      <c r="M558" t="inlineStr"/>
-      <c r="N558" t="inlineStr"/>
-      <c r="O558" t="inlineStr"/>
-      <c r="P558" t="inlineStr"/>
-      <c r="Q558" t="inlineStr"/>
-      <c r="R558" t="inlineStr"/>
-      <c r="S558" t="inlineStr"/>
       <c r="T558" t="inlineStr">
         <is>
           <t>TDJakesOfficial</t>
@@ -38161,9 +37898,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W558" t="inlineStr"/>
-      <c r="X558" t="inlineStr"/>
-      <c r="Y558" t="inlineStr"/>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr">
@@ -38201,18 +37935,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="H559" t="inlineStr"/>
-      <c r="I559" t="inlineStr"/>
-      <c r="J559" t="inlineStr"/>
-      <c r="K559" t="inlineStr"/>
-      <c r="L559" t="inlineStr"/>
-      <c r="M559" t="inlineStr"/>
-      <c r="N559" t="inlineStr"/>
-      <c r="O559" t="inlineStr"/>
-      <c r="P559" t="inlineStr"/>
-      <c r="Q559" t="inlineStr"/>
-      <c r="R559" t="inlineStr"/>
-      <c r="S559" t="inlineStr"/>
       <c r="T559" t="inlineStr">
         <is>
           <t>TonyEvans</t>
@@ -38228,9 +37950,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W559" t="inlineStr"/>
-      <c r="X559" t="inlineStr"/>
-      <c r="Y559" t="inlineStr"/>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -38243,27 +37962,11 @@
           <t>Author &amp; Speaker</t>
         </is>
       </c>
-      <c r="C560" t="inlineStr"/>
       <c r="D560" t="inlineStr">
         <is>
           <t>Crazy Love author, church planting</t>
         </is>
       </c>
-      <c r="E560" t="inlineStr"/>
-      <c r="F560" t="inlineStr"/>
-      <c r="G560" t="inlineStr"/>
-      <c r="H560" t="inlineStr"/>
-      <c r="I560" t="inlineStr"/>
-      <c r="J560" t="inlineStr"/>
-      <c r="K560" t="inlineStr"/>
-      <c r="L560" t="inlineStr"/>
-      <c r="M560" t="inlineStr"/>
-      <c r="N560" t="inlineStr"/>
-      <c r="O560" t="inlineStr"/>
-      <c r="P560" t="inlineStr"/>
-      <c r="Q560" t="inlineStr"/>
-      <c r="R560" t="inlineStr"/>
-      <c r="S560" t="inlineStr"/>
       <c r="T560" t="inlineStr">
         <is>
           <t>FrancisChanOfficial</t>
@@ -38279,9 +37982,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W560" t="inlineStr"/>
-      <c r="X560" t="inlineStr"/>
-      <c r="Y560" t="inlineStr"/>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -38319,18 +38019,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="H561" t="inlineStr"/>
-      <c r="I561" t="inlineStr"/>
-      <c r="J561" t="inlineStr"/>
-      <c r="K561" t="inlineStr"/>
-      <c r="L561" t="inlineStr"/>
-      <c r="M561" t="inlineStr"/>
-      <c r="N561" t="inlineStr"/>
-      <c r="O561" t="inlineStr"/>
-      <c r="P561" t="inlineStr"/>
-      <c r="Q561" t="inlineStr"/>
-      <c r="R561" t="inlineStr"/>
-      <c r="S561" t="inlineStr"/>
       <c r="T561" t="inlineStr">
         <is>
           <t>greglaurie</t>
@@ -38346,9 +38034,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W561" t="inlineStr"/>
-      <c r="X561" t="inlineStr"/>
-      <c r="Y561" t="inlineStr"/>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -38371,21 +38056,6 @@
           <t>Radical author, missions and leadership</t>
         </is>
       </c>
-      <c r="E562" t="inlineStr"/>
-      <c r="F562" t="inlineStr"/>
-      <c r="G562" t="inlineStr"/>
-      <c r="H562" t="inlineStr"/>
-      <c r="I562" t="inlineStr"/>
-      <c r="J562" t="inlineStr"/>
-      <c r="K562" t="inlineStr"/>
-      <c r="L562" t="inlineStr"/>
-      <c r="M562" t="inlineStr"/>
-      <c r="N562" t="inlineStr"/>
-      <c r="O562" t="inlineStr"/>
-      <c r="P562" t="inlineStr"/>
-      <c r="Q562" t="inlineStr"/>
-      <c r="R562" t="inlineStr"/>
-      <c r="S562" t="inlineStr"/>
       <c r="T562" t="inlineStr">
         <is>
           <t>DavidPlatt</t>
@@ -38401,9 +38071,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="W562" t="inlineStr"/>
-      <c r="X562" t="inlineStr"/>
-      <c r="Y562" t="inlineStr"/>
     </row>
     <row r="563">
       <c r="A563" t="inlineStr">
@@ -38426,15 +38093,6 @@
           <t>Church researcher, trend commentator</t>
         </is>
       </c>
-      <c r="E563" t="inlineStr"/>
-      <c r="F563" t="inlineStr"/>
-      <c r="G563" t="inlineStr"/>
-      <c r="H563" t="inlineStr"/>
-      <c r="I563" t="inlineStr"/>
-      <c r="J563" t="inlineStr"/>
-      <c r="K563" t="inlineStr"/>
-      <c r="L563" t="inlineStr"/>
-      <c r="M563" t="inlineStr"/>
       <c r="N563" t="inlineStr">
         <is>
           <t>edstetzer</t>
@@ -38450,12 +38108,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q563" t="inlineStr"/>
-      <c r="R563" t="inlineStr"/>
-      <c r="S563" t="inlineStr"/>
-      <c r="T563" t="inlineStr"/>
-      <c r="U563" t="inlineStr"/>
-      <c r="V563" t="inlineStr"/>
       <c r="W563" t="inlineStr">
         <is>
           <t>edstetzer.bsky.social</t>
@@ -38493,15 +38145,6 @@
           <t>Theological leadership voice</t>
         </is>
       </c>
-      <c r="E564" t="inlineStr"/>
-      <c r="F564" t="inlineStr"/>
-      <c r="G564" t="inlineStr"/>
-      <c r="H564" t="inlineStr"/>
-      <c r="I564" t="inlineStr"/>
-      <c r="J564" t="inlineStr"/>
-      <c r="K564" t="inlineStr"/>
-      <c r="L564" t="inlineStr"/>
-      <c r="M564" t="inlineStr"/>
       <c r="N564" t="inlineStr">
         <is>
           <t>MattChandler74</t>
@@ -38517,15 +38160,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q564" t="inlineStr"/>
-      <c r="R564" t="inlineStr"/>
-      <c r="S564" t="inlineStr"/>
-      <c r="T564" t="inlineStr"/>
-      <c r="U564" t="inlineStr"/>
-      <c r="V564" t="inlineStr"/>
-      <c r="W564" t="inlineStr"/>
-      <c r="X564" t="inlineStr"/>
-      <c r="Y564" t="inlineStr"/>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -38538,7 +38172,6 @@
           <t>Author</t>
         </is>
       </c>
-      <c r="C565" t="inlineStr"/>
       <c r="D565" t="inlineStr">
         <is>
           <t>Love Does author, inspirational leadership</t>
@@ -38559,12 +38192,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="H565" t="inlineStr"/>
-      <c r="I565" t="inlineStr"/>
-      <c r="J565" t="inlineStr"/>
-      <c r="K565" t="inlineStr"/>
-      <c r="L565" t="inlineStr"/>
-      <c r="M565" t="inlineStr"/>
       <c r="N565" t="inlineStr">
         <is>
           <t>bobgoff</t>
@@ -38580,12 +38207,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q565" t="inlineStr"/>
-      <c r="R565" t="inlineStr"/>
-      <c r="S565" t="inlineStr"/>
-      <c r="T565" t="inlineStr"/>
-      <c r="U565" t="inlineStr"/>
-      <c r="V565" t="inlineStr"/>
       <c r="W565" t="inlineStr">
         <is>
           <t>bobgoff.bsky.social</t>
@@ -38623,15 +38244,6 @@
           <t>Church leadership consultant</t>
         </is>
       </c>
-      <c r="E566" t="inlineStr"/>
-      <c r="F566" t="inlineStr"/>
-      <c r="G566" t="inlineStr"/>
-      <c r="H566" t="inlineStr"/>
-      <c r="I566" t="inlineStr"/>
-      <c r="J566" t="inlineStr"/>
-      <c r="K566" t="inlineStr"/>
-      <c r="L566" t="inlineStr"/>
-      <c r="M566" t="inlineStr"/>
       <c r="N566" t="inlineStr">
         <is>
           <t>jennicatron</t>
@@ -38647,15 +38259,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q566" t="inlineStr"/>
-      <c r="R566" t="inlineStr"/>
-      <c r="S566" t="inlineStr"/>
-      <c r="T566" t="inlineStr"/>
-      <c r="U566" t="inlineStr"/>
-      <c r="V566" t="inlineStr"/>
-      <c r="W566" t="inlineStr"/>
-      <c r="X566" t="inlineStr"/>
-      <c r="Y566" t="inlineStr"/>
     </row>
     <row r="567">
       <c r="A567" t="inlineStr">
@@ -38678,15 +38281,6 @@
           <t>Church curriculum pioneer, next-gen ministry</t>
         </is>
       </c>
-      <c r="E567" t="inlineStr"/>
-      <c r="F567" t="inlineStr"/>
-      <c r="G567" t="inlineStr"/>
-      <c r="H567" t="inlineStr"/>
-      <c r="I567" t="inlineStr"/>
-      <c r="J567" t="inlineStr"/>
-      <c r="K567" t="inlineStr"/>
-      <c r="L567" t="inlineStr"/>
-      <c r="M567" t="inlineStr"/>
       <c r="N567" t="inlineStr">
         <is>
           <t>reggiejoiner</t>
@@ -38702,15 +38296,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q567" t="inlineStr"/>
-      <c r="R567" t="inlineStr"/>
-      <c r="S567" t="inlineStr"/>
-      <c r="T567" t="inlineStr"/>
-      <c r="U567" t="inlineStr"/>
-      <c r="V567" t="inlineStr"/>
-      <c r="W567" t="inlineStr"/>
-      <c r="X567" t="inlineStr"/>
-      <c r="Y567" t="inlineStr"/>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
@@ -38733,15 +38318,6 @@
           <t>Spiritual formation, bestselling author</t>
         </is>
       </c>
-      <c r="E568" t="inlineStr"/>
-      <c r="F568" t="inlineStr"/>
-      <c r="G568" t="inlineStr"/>
-      <c r="H568" t="inlineStr"/>
-      <c r="I568" t="inlineStr"/>
-      <c r="J568" t="inlineStr"/>
-      <c r="K568" t="inlineStr"/>
-      <c r="L568" t="inlineStr"/>
-      <c r="M568" t="inlineStr"/>
       <c r="N568" t="inlineStr">
         <is>
           <t>johnmarkcomer</t>
@@ -38757,12 +38333,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q568" t="inlineStr"/>
-      <c r="R568" t="inlineStr"/>
-      <c r="S568" t="inlineStr"/>
-      <c r="T568" t="inlineStr"/>
-      <c r="U568" t="inlineStr"/>
-      <c r="V568" t="inlineStr"/>
       <c r="W568" t="inlineStr">
         <is>
           <t>johnmarkcomer.bsky.social</t>
@@ -38790,21 +38360,11 @@
           <t>Author &amp; Speaker</t>
         </is>
       </c>
-      <c r="C569" t="inlineStr"/>
       <c r="D569" t="inlineStr">
         <is>
           <t>Bible teacher, warm storytelling voice</t>
         </is>
       </c>
-      <c r="E569" t="inlineStr"/>
-      <c r="F569" t="inlineStr"/>
-      <c r="G569" t="inlineStr"/>
-      <c r="H569" t="inlineStr"/>
-      <c r="I569" t="inlineStr"/>
-      <c r="J569" t="inlineStr"/>
-      <c r="K569" t="inlineStr"/>
-      <c r="L569" t="inlineStr"/>
-      <c r="M569" t="inlineStr"/>
       <c r="N569" t="inlineStr">
         <is>
           <t>lisaharper</t>
@@ -38820,15 +38380,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q569" t="inlineStr"/>
-      <c r="R569" t="inlineStr"/>
-      <c r="S569" t="inlineStr"/>
-      <c r="T569" t="inlineStr"/>
-      <c r="U569" t="inlineStr"/>
-      <c r="V569" t="inlineStr"/>
-      <c r="W569" t="inlineStr"/>
-      <c r="X569" t="inlineStr"/>
-      <c r="Y569" t="inlineStr"/>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -38851,15 +38402,6 @@
           <t>Former SBC President, gospel-centered</t>
         </is>
       </c>
-      <c r="E570" t="inlineStr"/>
-      <c r="F570" t="inlineStr"/>
-      <c r="G570" t="inlineStr"/>
-      <c r="H570" t="inlineStr"/>
-      <c r="I570" t="inlineStr"/>
-      <c r="J570" t="inlineStr"/>
-      <c r="K570" t="inlineStr"/>
-      <c r="L570" t="inlineStr"/>
-      <c r="M570" t="inlineStr"/>
       <c r="N570" t="inlineStr">
         <is>
           <t>jdgreear</t>
@@ -38875,12 +38417,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="Q570" t="inlineStr"/>
-      <c r="R570" t="inlineStr"/>
-      <c r="S570" t="inlineStr"/>
-      <c r="T570" t="inlineStr"/>
-      <c r="U570" t="inlineStr"/>
-      <c r="V570" t="inlineStr"/>
       <c r="W570" t="inlineStr">
         <is>
           <t>jdgreear.bsky.social</t>
@@ -38933,24 +38469,6 @@
           <t>web</t>
         </is>
       </c>
-      <c r="H571" t="inlineStr"/>
-      <c r="I571" t="inlineStr"/>
-      <c r="J571" t="inlineStr"/>
-      <c r="K571" t="inlineStr"/>
-      <c r="L571" t="inlineStr"/>
-      <c r="M571" t="inlineStr"/>
-      <c r="N571" t="inlineStr"/>
-      <c r="O571" t="inlineStr"/>
-      <c r="P571" t="inlineStr"/>
-      <c r="Q571" t="inlineStr"/>
-      <c r="R571" t="inlineStr"/>
-      <c r="S571" t="inlineStr"/>
-      <c r="T571" t="inlineStr"/>
-      <c r="U571" t="inlineStr"/>
-      <c r="V571" t="inlineStr"/>
-      <c r="W571" t="inlineStr"/>
-      <c r="X571" t="inlineStr"/>
-      <c r="Y571" t="inlineStr"/>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
@@ -38988,24 +38506,1508 @@
           <t>web</t>
         </is>
       </c>
-      <c r="H572" t="inlineStr"/>
-      <c r="I572" t="inlineStr"/>
-      <c r="J572" t="inlineStr"/>
-      <c r="K572" t="inlineStr"/>
-      <c r="L572" t="inlineStr"/>
-      <c r="M572" t="inlineStr"/>
-      <c r="N572" t="inlineStr"/>
-      <c r="O572" t="inlineStr"/>
-      <c r="P572" t="inlineStr"/>
-      <c r="Q572" t="inlineStr"/>
-      <c r="R572" t="inlineStr"/>
-      <c r="S572" t="inlineStr"/>
-      <c r="T572" t="inlineStr"/>
-      <c r="U572" t="inlineStr"/>
-      <c r="V572" t="inlineStr"/>
-      <c r="W572" t="inlineStr"/>
-      <c r="X572" t="inlineStr"/>
-      <c r="Y572" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>J.P. Nerbun</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>TOC Culture Consulting</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Sports culture consultant</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>TOCCulture</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>tocculture</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K573" t="inlineStr"/>
+      <c r="L573" t="inlineStr"/>
+      <c r="M573" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>John O'Sullivan</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Changing the Game Project</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Youth sports reform leader</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>ChangingtheGameProject</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>changingthegameproject</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr"/>
+      <c r="L574" t="inlineStr"/>
+      <c r="M574" t="inlineStr"/>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Brett Ledbetter</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>What Drives Winning</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Character-driven coaching</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>WhatDrivesWinning</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>whatdriveswinning</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K575" t="inlineStr"/>
+      <c r="L575" t="inlineStr"/>
+      <c r="M575" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Becky Burleigh</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Hall of Fame Coach</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>What Drives Winning</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>UF Soccer, 500+ wins</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr"/>
+      <c r="F576" t="inlineStr"/>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>beckyburleigh</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K576" t="inlineStr"/>
+      <c r="L576" t="inlineStr"/>
+      <c r="M576" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Gabriel Deieno</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Mental Performance Coach</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr"/>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>209K IG followers</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr"/>
+      <c r="F577" t="inlineStr"/>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>gabrieldeieno</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K577" t="inlineStr"/>
+      <c r="L577" t="inlineStr"/>
+      <c r="M577" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Brenley Shapiro</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Mental Performance Coach</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>PWHL/NHL</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Pro sports mindset</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr"/>
+      <c r="F578" t="inlineStr"/>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>brenleyshapiro</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K578" t="inlineStr"/>
+      <c r="L578" t="inlineStr"/>
+      <c r="M578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Laura Wilkinson</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Olympic Champion</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr"/>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Mindset &amp; performance coach</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr"/>
+      <c r="F579" t="inlineStr"/>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>lala_the_diver</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K579" t="inlineStr"/>
+      <c r="L579" t="inlineStr"/>
+      <c r="M579" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Eli Straw</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Sport Psychology Coach</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr"/>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>M.S. Sport Psychology</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr"/>
+      <c r="F580" t="inlineStr"/>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>elistraw</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K580" t="inlineStr"/>
+      <c r="L580" t="inlineStr"/>
+      <c r="M580" t="inlineStr"/>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Tim Elmore</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Growing Leaders</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Gen Z leadership expert</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>GrowingLeaders</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>timelmore</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K581" t="inlineStr"/>
+      <c r="L581" t="inlineStr"/>
+      <c r="M581" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Reed Maltbie</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Coaching the Whole Athlete</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Youth coaching advocate</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr"/>
+      <c r="F582" t="inlineStr"/>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>coachmaltbie</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K582" t="inlineStr"/>
+      <c r="L582" t="inlineStr"/>
+      <c r="M582" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Jeff Janssen</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Janssen Sports Leadership Center</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Sports leadership training</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>JanssenSportsLeadership</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>janssensports</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K583" t="inlineStr"/>
+      <c r="L583" t="inlineStr"/>
+      <c r="M583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Paddy Upton</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Elite Sports Coach</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr"/>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Author, international coach</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr"/>
+      <c r="F584" t="inlineStr"/>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>paddyupton1</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K584" t="inlineStr"/>
+      <c r="L584" t="inlineStr"/>
+      <c r="M584" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Dr. Colleen Hacker</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Mental Skills Coach</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>US Soccer</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Olympic mental coach</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr"/>
+      <c r="F585" t="inlineStr"/>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>colleenhacker</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K585" t="inlineStr"/>
+      <c r="L585" t="inlineStr"/>
+      <c r="M585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Alan Stein Jr.</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Performance Coach</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr"/>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Speaker &amp; author</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>AlanSteinJr</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>alansteinjr</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K586" t="inlineStr"/>
+      <c r="L586" t="inlineStr"/>
+      <c r="M586" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Lindsey Wilson</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Sports Leadership Educator</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr"/>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Coaching content creator</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr"/>
+      <c r="F587" t="inlineStr"/>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>coachwilson_</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K587" t="inlineStr"/>
+      <c r="L587" t="inlineStr"/>
+      <c r="M587" t="inlineStr"/>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Betsy Butterick</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Culture Coach</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>TOC Culture</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Culture consulting</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr"/>
+      <c r="F588" t="inlineStr"/>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>betsybutterick</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K588" t="inlineStr"/>
+      <c r="L588" t="inlineStr"/>
+      <c r="M588" t="inlineStr"/>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Dr. Patrick Cohn</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Mental Performance Coach</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Peak Sports</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Mental game expert</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr"/>
+      <c r="F589" t="inlineStr"/>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr"/>
+      <c r="I589" t="inlineStr"/>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K589" t="inlineStr"/>
+      <c r="L589" t="inlineStr"/>
+      <c r="M589" t="inlineStr"/>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Eric Thomas</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Motivational Speaker</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr"/>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>ET the Hip Hop Preacher</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr"/>
+      <c r="F590" t="inlineStr"/>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr"/>
+      <c r="I590" t="inlineStr"/>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K590" t="inlineStr"/>
+      <c r="L590" t="inlineStr"/>
+      <c r="M590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Coach Pain</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Motivational Coach</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr"/>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Motivational speaker</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr"/>
+      <c r="F591" t="inlineStr"/>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr"/>
+      <c r="I591" t="inlineStr"/>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K591" t="inlineStr"/>
+      <c r="L591" t="inlineStr"/>
+      <c r="M591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Inky Johnson</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Motivational Speaker</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr"/>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Former athlete</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>InkyJohnson</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr"/>
+      <c r="I592" t="inlineStr"/>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K592" t="inlineStr"/>
+      <c r="L592" t="inlineStr"/>
+      <c r="M592" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Ed Mylett</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Peak Performance Coach</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr"/>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>The Ed Mylett Show</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>EdMylett</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr"/>
+      <c r="I593" t="inlineStr"/>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K593" t="inlineStr"/>
+      <c r="L593" t="inlineStr"/>
+      <c r="M593" t="inlineStr"/>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Kwame Brown</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Sports Commentator</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr"/>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Sports culture commentary</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr"/>
+      <c r="F594" t="inlineStr"/>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr"/>
+      <c r="I594" t="inlineStr"/>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K594" t="inlineStr"/>
+      <c r="L594" t="inlineStr"/>
+      <c r="M594" t="inlineStr"/>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Pure Sports Mindset</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Mental Performance Coaching</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr"/>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Mindset coaching org</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr"/>
+      <c r="F595" t="inlineStr"/>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr"/>
+      <c r="I595" t="inlineStr"/>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K595" t="inlineStr"/>
+      <c r="L595" t="inlineStr"/>
+      <c r="M595" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Dr. Jerry Lynch</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Sports Psychologist</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Way of Champions</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Author &amp; coach</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>WayofChampions</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr"/>
+      <c r="I596" t="inlineStr"/>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K596" t="inlineStr"/>
+      <c r="L596" t="inlineStr"/>
+      <c r="M596" t="inlineStr"/>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Michael Lombardi</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>NFL Executive</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>The GM Shuffle</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>NFL leadership insights</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr"/>
+      <c r="F597" t="inlineStr"/>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr"/>
+      <c r="I597" t="inlineStr"/>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K597" t="inlineStr"/>
+      <c r="L597" t="inlineStr"/>
+      <c r="M597" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Joe Daniel</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Football Coach</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Joe Daniel Football</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>YouTube football analysis</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr"/>
+      <c r="F598" t="inlineStr"/>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr"/>
+      <c r="I598" t="inlineStr"/>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K598" t="inlineStr"/>
+      <c r="L598" t="inlineStr"/>
+      <c r="M598" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Bo Hanson</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>4x Olympian</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Athlete Assessments</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>DISC profiling in sport</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>AthleteAssessments</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr"/>
+      <c r="I599" t="inlineStr"/>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K599" t="inlineStr"/>
+      <c r="L599" t="inlineStr"/>
+      <c r="M599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Evan Burk</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Podcast Host</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>The Highest Level</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Sports leadership podcast</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr"/>
+      <c r="F600" t="inlineStr"/>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr"/>
+      <c r="I600" t="inlineStr"/>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K600" t="inlineStr"/>
+      <c r="L600" t="inlineStr"/>
+      <c r="M600" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Dr. Jim Afremow</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Sports Psychologist</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr"/>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Author, mental performance</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr"/>
+      <c r="F601" t="inlineStr"/>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr"/>
+      <c r="I601" t="inlineStr"/>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K601" t="inlineStr"/>
+      <c r="L601" t="inlineStr"/>
+      <c r="M601" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Positive Coaching Alliance</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr"/>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Youth sports leadership</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>PositiveCoachUS</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr"/>
+      <c r="I602" t="inlineStr"/>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K602" t="inlineStr"/>
+      <c r="L602" t="inlineStr"/>
+      <c r="M602" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Proactive Coaching</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr"/>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Character-based teams</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>proactivecoach</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr"/>
+      <c r="I603" t="inlineStr"/>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K603" t="inlineStr"/>
+      <c r="L603" t="inlineStr"/>
+      <c r="M603" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Expert Sport Coaching</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr"/>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Sports coaching community</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>expertsportcoach</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr"/>
+      <c r="I604" t="inlineStr"/>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K604" t="inlineStr"/>
+      <c r="L604" t="inlineStr"/>
+      <c r="M604" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Coaching Culture Podcast</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr"/>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Sports leadership podcast</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>CoachingCulturePod</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr"/>
+      <c r="I605" t="inlineStr"/>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K605" t="inlineStr"/>
+      <c r="L605" t="inlineStr"/>
+      <c r="M605" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Way of Champions</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr"/>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Jerry Lynch &amp; John O'Sullivan</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>WayofChampions</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr"/>
+      <c r="I606" t="inlineStr"/>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="K606" t="inlineStr"/>
+      <c r="L606" t="inlineStr"/>
+      <c r="M606" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
@@ -39019,7 +40021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -39747,6 +40749,26 @@
       <c r="D36" t="inlineStr">
         <is>
           <t>church-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>42</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>sports-leadership-coaching</t>
         </is>
       </c>
     </row>
@@ -39762,7 +40784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G281"/>
+  <dimension ref="A1:G289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -50071,6 +51093,302 @@
         </is>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>69c4b6c57644e8b883c291bf</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>2026-04-05T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>69c4b6e47644e8b883c2927a</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>2026-04-05T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>69c4b77a3f4faec7d431c3ac</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>2026-03-30T03:00:00Z</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>69c4b78c7644e8b883c29886</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>2026-04-05T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>69c4b79e7644e8b883c29954</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>2026-04-05T14:20:00Z</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>69c4b7a93f4faec7d431c583</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>2026-03-28T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>69c4b7b63f4faec7d431c5c2</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>2026-04-05T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Sports Leadership &amp; Coaching</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>69c4b7be7644e8b883c29a8f</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>2026-04-05T11:30:00Z</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Design Thinking in Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1362,7 +1362,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1603,7 +1608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y626"/>
+  <dimension ref="A1:Y643"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40260,6 +40265,380 @@
         </is>
       </c>
     </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Tim Brown</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Co-Chair</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>IDEO</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Popularised design thinking with Change by Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>David Kelley</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Stanford d.school &amp; IDEO</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Built two most influential DT institutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Tom Kelley</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>IDEO</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Creative Confidence co-author</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Jeanne Liedtka</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>UVA Darden</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>THE design thinking academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Jake Knapp</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Design Sprint</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Created Design Sprint at Google Ventures</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Jonathan Courtney</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>AJ&amp;Smart</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>YouTube DT educator, Sprint facilitator</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Chris Pacione</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>LUMA Institute</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>LUMA System of Innovation creator</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Suzanne Gibbs Howard</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Dean</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>IDEO U</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>DT education leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Soren Kaplan</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>USC/InnovationPoint</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Leapfrogging author, Thinkers50</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Lee-Sean Huang</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Foossa</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Social innovation + DT facilitator</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Darin Eich</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>InnovationLearning.org</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>DT in higher education</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Stacy Neier Beran</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Loyola Chicago</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Think by Design 2024 author</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Nicole Dessain</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>DessainCo</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>HR + design thinking specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Mia Blume</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Design Dept</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Design leadership coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Sandy Speicher</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Former CEO</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>IDEO</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Built IDEO U, DT in education</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Eli Woolery</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Stanford d.school</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>DT educator, podcast host</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Jeremy Utley</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Stanford d.school</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Ideaflow author, DT + AI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -40272,7 +40651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -41040,6 +41419,26 @@
       <c r="D38" t="inlineStr">
         <is>
           <t>introverted-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>17</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>design-thinking-leadership</t>
         </is>
       </c>
     </row>
@@ -41055,7 +41454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G297"/>
+  <dimension ref="A1:G305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -51956,6 +52355,270 @@
         </is>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>69c4c104</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>69c4c107</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>69c4c109</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr"/>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>69c4c10a</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>69c4c13b</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>69c4c13d</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>69c4c123</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Design Thinking in Leadership</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>69c4c124</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Facilitation & Workshop Design + Middle Management
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1387,7 +1387,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1407,7 +1412,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1608,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y643"/>
+  <dimension ref="A1:Y660"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40639,6 +40649,1178 @@
         </is>
       </c>
     </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Sam Kaner</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Author &amp; Facilitator</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Community At Work</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Author of 'Facilitator's Guide to Participatory Decision-Making', foundational facilitation text</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr"/>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr"/>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr"/>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>@Samster120</t>
+        </is>
+      </c>
+      <c r="L644" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M644" t="inlineStr"/>
+      <c r="N644" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O644" t="inlineStr"/>
+      <c r="P644" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q644" t="inlineStr"/>
+      <c r="R644" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Keith McCandless</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Co-Creator, Liberating Structures</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Liberating Structures</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Co-created 33 Liberating Structures microstructures for group facilitation</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr"/>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr"/>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr"/>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>@KeithMcCandless</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M645" t="inlineStr"/>
+      <c r="N645" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O645" t="inlineStr"/>
+      <c r="P645" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q645" t="inlineStr"/>
+      <c r="R645" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Henri Lipmanowicz</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Co-Creator, Liberating Structures</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Liberating Structures</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Co-created Liberating Structures with Keith McCandless, former Merck executive</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr"/>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr"/>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr"/>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K646" t="inlineStr"/>
+      <c r="L646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M646" t="inlineStr"/>
+      <c r="N646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O646" t="inlineStr"/>
+      <c r="P646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q646" t="inlineStr"/>
+      <c r="R646" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Leanne Hughes</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Facilitator &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>First Time Facilitator</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Host of First Time Facilitator podcast, Australian facilitation specialist</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr"/>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>@leannehughes</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr"/>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>@leannehughes</t>
+        </is>
+      </c>
+      <c r="L647" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M647" t="inlineStr"/>
+      <c r="N647" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O647" t="inlineStr"/>
+      <c r="P647" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q647" t="inlineStr"/>
+      <c r="R647" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Dr. Myriam Hadnes</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Facilitator &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Workshops Work</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Host of top 5% Workshops Work podcast, facilitation researcher</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr"/>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>@myriamhadnes</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr"/>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>@myriamHadnes</t>
+        </is>
+      </c>
+      <c r="L648" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M648" t="inlineStr"/>
+      <c r="N648" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O648" t="inlineStr"/>
+      <c r="P648" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q648" t="inlineStr"/>
+      <c r="R648" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Michael Wilkinson</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>CEO &amp; Facilitation Expert</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Leadership Strategies</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Author of 'Secrets of Facilitation', certified master facilitator trainer</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr"/>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr"/>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr"/>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>@mwilkinsonmd</t>
+        </is>
+      </c>
+      <c r="L649" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M649" t="inlineStr"/>
+      <c r="N649" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O649" t="inlineStr">
+        <is>
+          <t>@mwilkfacilitator</t>
+        </is>
+      </c>
+      <c r="P649" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Q649" t="inlineStr"/>
+      <c r="R649" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Ingrid Bens</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Author &amp; Facilitator</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Participative Dynamics</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Author of 'Facilitating with Ease', practical facilitation guide</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr"/>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr"/>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr"/>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K650" t="inlineStr"/>
+      <c r="L650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M650" t="inlineStr"/>
+      <c r="N650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O650" t="inlineStr"/>
+      <c r="P650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q650" t="inlineStr"/>
+      <c r="R650" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Roger Schwarz</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Author &amp; Consultant</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Roger Schwarz &amp; Associates</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Author of 'The Skilled Facilitator', mutual learning approach pioneer</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr"/>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr"/>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr"/>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>@LeadSmarter</t>
+        </is>
+      </c>
+      <c r="L651" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M651" t="inlineStr"/>
+      <c r="N651" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O651" t="inlineStr"/>
+      <c r="P651" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q651" t="inlineStr"/>
+      <c r="R651" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Adam Kahane</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Reos Partners</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Author of 'Facilitating Breakthrough', specialises in complex multi-stakeholder facilitation</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr"/>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr"/>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr"/>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>@adamkahane</t>
+        </is>
+      </c>
+      <c r="L652" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M652" t="inlineStr"/>
+      <c r="N652" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O652" t="inlineStr"/>
+      <c r="P652" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q652" t="inlineStr"/>
+      <c r="R652" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Daniel Stillman</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Author &amp; Podcast Host</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>The Conversation Factory</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Author of 'Good Talk', hosts The Conversation Factory podcast on facilitation design</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr"/>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>@dastillman</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr"/>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>@dastillman</t>
+        </is>
+      </c>
+      <c r="L653" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M653" t="inlineStr"/>
+      <c r="N653" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O653" t="inlineStr"/>
+      <c r="P653" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q653" t="inlineStr"/>
+      <c r="R653" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Adriana Girdler</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>CEO &amp; YouTuber</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>CornerStone Dynamics</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>YouTube 200K+ subscribers, workshop design and project management specialist</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>CornerStone Dynamics</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr"/>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr"/>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K654" t="inlineStr"/>
+      <c r="L654" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M654" t="inlineStr"/>
+      <c r="N654" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O654" t="inlineStr">
+        <is>
+          <t>Adriana Girdler</t>
+        </is>
+      </c>
+      <c r="P654" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="Q654" t="inlineStr"/>
+      <c r="R654" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Martin Gilbraith</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Facilitator &amp; Trainer</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Former Chair of International Association of Facilitators (IAF)</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr"/>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr"/>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr"/>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K655" t="inlineStr">
+        <is>
+          <t>@martingilbraith</t>
+        </is>
+      </c>
+      <c r="L655" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M655" t="inlineStr"/>
+      <c r="N655" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O655" t="inlineStr"/>
+      <c r="P655" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q655" t="inlineStr"/>
+      <c r="R655" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Beatrice Briggs</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>IIFAC</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Founded International Institute for Facilitation and Change, Latin America facilitation pioneer</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr"/>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr"/>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr"/>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K656" t="inlineStr"/>
+      <c r="L656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M656" t="inlineStr"/>
+      <c r="N656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O656" t="inlineStr"/>
+      <c r="P656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q656" t="inlineStr"/>
+      <c r="R656" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Nancy White</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Online Facilitation Pioneer</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Full Circle Associates</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Co-author 'Digital Habitats', pioneer of online facilitation and virtual community design</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr"/>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr"/>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr"/>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K657" t="inlineStr">
+        <is>
+          <t>@NancyWhite</t>
+        </is>
+      </c>
+      <c r="L657" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M657" t="inlineStr"/>
+      <c r="N657" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O657" t="inlineStr"/>
+      <c r="P657" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q657" t="inlineStr"/>
+      <c r="R657" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Teresa Brazen</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Head of Content</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>SessionLab</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Leads content at SessionLab, workshop experience design platform</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr"/>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr"/>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>@TeresaBrazen</t>
+        </is>
+      </c>
+      <c r="L658" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M658" t="inlineStr"/>
+      <c r="N658" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O658" t="inlineStr"/>
+      <c r="P658" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q658" t="inlineStr"/>
+      <c r="R658" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Bob Kulhan</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Professor &amp; Author</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Business Improv / Duke University</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Author of 'Getting to Yes And', teaches improvisation-based facilitation at Duke</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr"/>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>@business_improv</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr"/>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>@Kulhan</t>
+        </is>
+      </c>
+      <c r="L659" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M659" t="inlineStr"/>
+      <c r="N659" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O659" t="inlineStr"/>
+      <c r="P659" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q659" t="inlineStr"/>
+      <c r="R659" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Jeff Havens</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Keynote Speaker</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Jeff Havens Companies</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Humour-based facilitation and keynote speaking, unconventional workshop design</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr"/>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>@iamjeffhavens</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr"/>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>@iamjeffhavens</t>
+        </is>
+      </c>
+      <c r="L660" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M660" t="inlineStr"/>
+      <c r="N660" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O660" t="inlineStr"/>
+      <c r="P660" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q660" t="inlineStr"/>
+      <c r="R660" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -40651,7 +41833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -41439,6 +42621,46 @@
       <c r="D39" t="inlineStr">
         <is>
           <t>design-thinking-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Middle Management</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>17</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>middle-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>17</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>facilitation-workshop-design</t>
         </is>
       </c>
     </row>
@@ -41454,7 +42676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G305"/>
+  <dimension ref="A1:G313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -52381,7 +53603,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -52414,7 +53635,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -52447,7 +53667,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -52480,7 +53699,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -52513,7 +53731,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
           <t>customScheduled</t>
@@ -52546,7 +53763,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F303" t="inlineStr"/>
       <c r="G303" t="inlineStr">
         <is>
           <t>customScheduled</t>
@@ -52579,7 +53795,6 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr">
         <is>
           <t>addToQueue</t>
@@ -52612,8 +53827,303 @@
           <t>scheduled</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>69c4ca01ea5839fe524dd729</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>2026-04-06T12:02:00Z</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>69c4ca201acfeeec28fd23b9</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>2026-04-06T12:45:00Z</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>69c4ca031acfeeec28fd230d</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>2026-04-06T03:01:00Z</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>69c4ca041acfeeec28fd2334</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>2026-04-06T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>69c4ca37ea5839fe524dd8b8</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>2026-04-01T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>69c4ca211acfeeec28fd23e0</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>2026-05-12T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>69c4ca061acfeeec28fd2377</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>2026-04-06T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Facilitation &amp; Workshop Design</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>69c4ca05ea5839fe524dd760</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>2026-04-06T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
         <is>
           <t>addToQueue</t>
         </is>

</xml_diff>

<commit_message>
Update handle database — Leadership Podcasters
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1437,7 +1437,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1618,7 +1623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y660"/>
+  <dimension ref="A1:Y677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40670,19 +40675,16 @@
           <t>Author of 'Facilitator's Guide to Participatory Decision-Making', foundational facilitation text</t>
         </is>
       </c>
-      <c r="E644" t="inlineStr"/>
       <c r="F644" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G644" t="inlineStr"/>
       <c r="H644" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I644" t="inlineStr"/>
       <c r="J644" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40698,19 +40700,16 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M644" t="inlineStr"/>
       <c r="N644" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O644" t="inlineStr"/>
       <c r="P644" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q644" t="inlineStr"/>
       <c r="R644" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40738,19 +40737,16 @@
           <t>Co-created 33 Liberating Structures microstructures for group facilitation</t>
         </is>
       </c>
-      <c r="E645" t="inlineStr"/>
       <c r="F645" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G645" t="inlineStr"/>
       <c r="H645" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I645" t="inlineStr"/>
       <c r="J645" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40766,19 +40762,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M645" t="inlineStr"/>
       <c r="N645" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O645" t="inlineStr"/>
       <c r="P645" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q645" t="inlineStr"/>
       <c r="R645" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40806,43 +40799,36 @@
           <t>Co-created Liberating Structures with Keith McCandless, former Merck executive</t>
         </is>
       </c>
-      <c r="E646" t="inlineStr"/>
       <c r="F646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G646" t="inlineStr"/>
       <c r="H646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I646" t="inlineStr"/>
       <c r="J646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K646" t="inlineStr"/>
       <c r="L646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M646" t="inlineStr"/>
       <c r="N646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O646" t="inlineStr"/>
       <c r="P646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q646" t="inlineStr"/>
       <c r="R646" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40870,7 +40856,6 @@
           <t>Host of First Time Facilitator podcast, Australian facilitation specialist</t>
         </is>
       </c>
-      <c r="E647" t="inlineStr"/>
       <c r="F647" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40886,7 +40871,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I647" t="inlineStr"/>
       <c r="J647" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40902,19 +40886,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M647" t="inlineStr"/>
       <c r="N647" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O647" t="inlineStr"/>
       <c r="P647" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q647" t="inlineStr"/>
       <c r="R647" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40942,7 +40923,6 @@
           <t>Host of top 5% Workshops Work podcast, facilitation researcher</t>
         </is>
       </c>
-      <c r="E648" t="inlineStr"/>
       <c r="F648" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40958,7 +40938,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I648" t="inlineStr"/>
       <c r="J648" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -40974,19 +40953,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M648" t="inlineStr"/>
       <c r="N648" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O648" t="inlineStr"/>
       <c r="P648" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q648" t="inlineStr"/>
       <c r="R648" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41014,19 +40990,16 @@
           <t>Author of 'Secrets of Facilitation', certified master facilitator trainer</t>
         </is>
       </c>
-      <c r="E649" t="inlineStr"/>
       <c r="F649" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G649" t="inlineStr"/>
       <c r="H649" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I649" t="inlineStr"/>
       <c r="J649" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41042,7 +41015,6 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M649" t="inlineStr"/>
       <c r="N649" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41058,7 +41030,6 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="Q649" t="inlineStr"/>
       <c r="R649" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41086,43 +41057,36 @@
           <t>Author of 'Facilitating with Ease', practical facilitation guide</t>
         </is>
       </c>
-      <c r="E650" t="inlineStr"/>
       <c r="F650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G650" t="inlineStr"/>
       <c r="H650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I650" t="inlineStr"/>
       <c r="J650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K650" t="inlineStr"/>
       <c r="L650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M650" t="inlineStr"/>
       <c r="N650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O650" t="inlineStr"/>
       <c r="P650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q650" t="inlineStr"/>
       <c r="R650" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41150,19 +41114,16 @@
           <t>Author of 'The Skilled Facilitator', mutual learning approach pioneer</t>
         </is>
       </c>
-      <c r="E651" t="inlineStr"/>
       <c r="F651" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G651" t="inlineStr"/>
       <c r="H651" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I651" t="inlineStr"/>
       <c r="J651" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41178,19 +41139,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M651" t="inlineStr"/>
       <c r="N651" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O651" t="inlineStr"/>
       <c r="P651" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q651" t="inlineStr"/>
       <c r="R651" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41218,19 +41176,16 @@
           <t>Author of 'Facilitating Breakthrough', specialises in complex multi-stakeholder facilitation</t>
         </is>
       </c>
-      <c r="E652" t="inlineStr"/>
       <c r="F652" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G652" t="inlineStr"/>
       <c r="H652" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I652" t="inlineStr"/>
       <c r="J652" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41246,19 +41201,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M652" t="inlineStr"/>
       <c r="N652" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O652" t="inlineStr"/>
       <c r="P652" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q652" t="inlineStr"/>
       <c r="R652" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41286,7 +41238,6 @@
           <t>Author of 'Good Talk', hosts The Conversation Factory podcast on facilitation design</t>
         </is>
       </c>
-      <c r="E653" t="inlineStr"/>
       <c r="F653" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41302,7 +41253,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I653" t="inlineStr"/>
       <c r="J653" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41318,19 +41268,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M653" t="inlineStr"/>
       <c r="N653" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O653" t="inlineStr"/>
       <c r="P653" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q653" t="inlineStr"/>
       <c r="R653" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41368,25 +41315,21 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="G654" t="inlineStr"/>
       <c r="H654" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I654" t="inlineStr"/>
       <c r="J654" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K654" t="inlineStr"/>
       <c r="L654" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M654" t="inlineStr"/>
       <c r="N654" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41402,7 +41345,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="Q654" t="inlineStr"/>
       <c r="R654" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41430,19 +41372,16 @@
           <t>Former Chair of International Association of Facilitators (IAF)</t>
         </is>
       </c>
-      <c r="E655" t="inlineStr"/>
       <c r="F655" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G655" t="inlineStr"/>
       <c r="H655" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I655" t="inlineStr"/>
       <c r="J655" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41458,19 +41397,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M655" t="inlineStr"/>
       <c r="N655" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O655" t="inlineStr"/>
       <c r="P655" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q655" t="inlineStr"/>
       <c r="R655" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41498,43 +41434,36 @@
           <t>Founded International Institute for Facilitation and Change, Latin America facilitation pioneer</t>
         </is>
       </c>
-      <c r="E656" t="inlineStr"/>
       <c r="F656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G656" t="inlineStr"/>
       <c r="H656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I656" t="inlineStr"/>
       <c r="J656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K656" t="inlineStr"/>
       <c r="L656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M656" t="inlineStr"/>
       <c r="N656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O656" t="inlineStr"/>
       <c r="P656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q656" t="inlineStr"/>
       <c r="R656" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41562,19 +41491,16 @@
           <t>Co-author 'Digital Habitats', pioneer of online facilitation and virtual community design</t>
         </is>
       </c>
-      <c r="E657" t="inlineStr"/>
       <c r="F657" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G657" t="inlineStr"/>
       <c r="H657" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I657" t="inlineStr"/>
       <c r="J657" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41590,19 +41516,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M657" t="inlineStr"/>
       <c r="N657" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O657" t="inlineStr"/>
       <c r="P657" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q657" t="inlineStr"/>
       <c r="R657" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41630,19 +41553,16 @@
           <t>Leads content at SessionLab, workshop experience design platform</t>
         </is>
       </c>
-      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G658" t="inlineStr"/>
       <c r="H658" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I658" t="inlineStr"/>
       <c r="J658" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41658,19 +41578,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M658" t="inlineStr"/>
       <c r="N658" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O658" t="inlineStr"/>
       <c r="P658" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q658" t="inlineStr"/>
       <c r="R658" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41698,7 +41615,6 @@
           <t>Author of 'Getting to Yes And', teaches improvisation-based facilitation at Duke</t>
         </is>
       </c>
-      <c r="E659" t="inlineStr"/>
       <c r="F659" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41714,7 +41630,6 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="I659" t="inlineStr"/>
       <c r="J659" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41730,19 +41645,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M659" t="inlineStr"/>
       <c r="N659" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O659" t="inlineStr"/>
       <c r="P659" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q659" t="inlineStr"/>
       <c r="R659" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41770,7 +41682,6 @@
           <t>Humour-based facilitation and keynote speaking, unconventional workshop design</t>
         </is>
       </c>
-      <c r="E660" t="inlineStr"/>
       <c r="F660" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41786,7 +41697,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I660" t="inlineStr"/>
       <c r="J660" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41802,20 +41712,1157 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M660" t="inlineStr"/>
       <c r="N660" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O660" t="inlineStr"/>
       <c r="P660" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q660" t="inlineStr"/>
       <c r="R660" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Ryan Hawk</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Host, The Learning Leader Show</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>The Learning Leader</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>500+ episodes interviewing world-class leaders on habits and mindsets of sustained excellence</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr"/>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>@ryanhawk12</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr"/>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K661" t="inlineStr">
+        <is>
+          <t>@RyanHawk12</t>
+        </is>
+      </c>
+      <c r="L661" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M661" t="inlineStr"/>
+      <c r="N661" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O661" t="inlineStr"/>
+      <c r="P661" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q661" t="inlineStr"/>
+      <c r="R661" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Dave Stachowiak</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Host, Coaching for Leaders</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Coaching for Leaders</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>50M+ downloads since 2011, weekly leadership development podcast, Dale Carnegie trainer</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr"/>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr"/>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr"/>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>@davestachowiak</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M662" t="inlineStr"/>
+      <c r="N662" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O662" t="inlineStr"/>
+      <c r="P662" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q662" t="inlineStr"/>
+      <c r="R662" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Muriel Wilkins</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Host, Coaching Real Leaders (HBR)</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Paravis Partners / HBR</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Takes listeners inside real executive coaching sessions, making leadership coaching accessible</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr"/>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr"/>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr"/>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K663" t="inlineStr"/>
+      <c r="L663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M663" t="inlineStr"/>
+      <c r="N663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O663" t="inlineStr"/>
+      <c r="P663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q663" t="inlineStr"/>
+      <c r="R663" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Anne Morriss</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Co-Host, Fixable (TED)</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>The Leadership Consortium / TED</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>TED podcast offering fast actionable leadership solutions with Frances Frei</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr"/>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>@annemorriss</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr"/>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K664" t="inlineStr"/>
+      <c r="L664" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M664" t="inlineStr"/>
+      <c r="N664" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O664" t="inlineStr"/>
+      <c r="P664" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q664" t="inlineStr"/>
+      <c r="R664" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Jan Rutherford</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Co-Host, The Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Self-Reliant Leadership</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Former Army Special Forces, 420+ episodes interviewing great leaders</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr"/>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr"/>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr"/>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K665" t="inlineStr"/>
+      <c r="L665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M665" t="inlineStr"/>
+      <c r="N665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O665" t="inlineStr"/>
+      <c r="P665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q665" t="inlineStr"/>
+      <c r="R665" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Jim Vaselopulos</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Co-Host, The Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Rafti Advisors</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>C-level business strategist co-hosting with Jan Rutherford</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr"/>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr"/>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr"/>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K666" t="inlineStr"/>
+      <c r="L666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M666" t="inlineStr"/>
+      <c r="N666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O666" t="inlineStr"/>
+      <c r="P666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q666" t="inlineStr"/>
+      <c r="R666" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Ben Fanning</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Host, Lead the Team</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>The Fanning Group</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Gold Stevie Award winner, 600+ CEO interviews, top 2% globally</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr"/>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>@benfanning1</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr"/>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>@BenFanning1</t>
+        </is>
+      </c>
+      <c r="L667" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M667" t="inlineStr"/>
+      <c r="N667" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O667" t="inlineStr"/>
+      <c r="P667" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q667" t="inlineStr"/>
+      <c r="R667" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Gene Hammett</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Host, Growth Think Tank</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Core Elevation</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>1200+ episodes since 2014 with Inc company founders on leadership growth</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr"/>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>@genehammett</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr"/>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr"/>
+      <c r="L668" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M668" t="inlineStr"/>
+      <c r="N668" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O668" t="inlineStr"/>
+      <c r="P668" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q668" t="inlineStr"/>
+      <c r="R668" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Hala Taha</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Host, Young and Profiting</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>YAP Media</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>100M+ listens, 3000+ episodes, built YAP Media empire from podcast</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr"/>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>@yapwithhala</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr"/>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>@yapwithhala</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M669" t="inlineStr">
+        <is>
+          <t>@yapwithhala</t>
+        </is>
+      </c>
+      <c r="N669" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="O669" t="inlineStr"/>
+      <c r="P669" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q669" t="inlineStr"/>
+      <c r="R669" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Martin G. Moore</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Host, No Bullsh!t Leadership</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Your CEO Mentor</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Australian leadership expert, 3M+ downloads, WSJ bestselling author</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr"/>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>@yourceomentor</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr"/>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr"/>
+      <c r="L670" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M670" t="inlineStr"/>
+      <c r="N670" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O670" t="inlineStr"/>
+      <c r="P670" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q670" t="inlineStr"/>
+      <c r="R670" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Guy Raz</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Host, How I Built This (NPR)</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>NPR / TED</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Iconic storytelling podcast exploring how entrepreneurs built famous companies</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr"/>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr"/>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr"/>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K671" t="inlineStr"/>
+      <c r="L671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M671" t="inlineStr"/>
+      <c r="N671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O671" t="inlineStr"/>
+      <c r="P671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q671" t="inlineStr"/>
+      <c r="R671" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Alison Beard</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Co-Host, HBR IdeaCast</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Harvard Business Review</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Executive Editor at HBR hosting one of longest-running business podcasts</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr"/>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr"/>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>@alisonbeard</t>
+        </is>
+      </c>
+      <c r="L672" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M672" t="inlineStr"/>
+      <c r="N672" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O672" t="inlineStr"/>
+      <c r="P672" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q672" t="inlineStr"/>
+      <c r="R672" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Diane Brady</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Co-Host, Leadership Next (Fortune)</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Fortune Magazine</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Fortune podcast featuring CEO interviews on business transformation</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr"/>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr"/>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K673" t="inlineStr"/>
+      <c r="L673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M673" t="inlineStr"/>
+      <c r="N673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O673" t="inlineStr"/>
+      <c r="P673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q673" t="inlineStr"/>
+      <c r="R673" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Karan Ferrell-Rhodes</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Host, Lead at the Top of Your Game</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Shockingly Different Leadership</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Celebrates firebrand leaders with ingenuity in underrepresented communities</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr"/>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr"/>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr"/>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K674" t="inlineStr"/>
+      <c r="L674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M674" t="inlineStr"/>
+      <c r="N674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O674" t="inlineStr"/>
+      <c r="P674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q674" t="inlineStr"/>
+      <c r="R674" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Scott Miller</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Host, On Leadership (FranklinCovey)</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>FranklinCovey</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>23 years at FranklinCovey, reaches 5M+ leaders weekly, Master Mentors author</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr"/>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr"/>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr"/>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K675" t="inlineStr"/>
+      <c r="L675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M675" t="inlineStr"/>
+      <c r="N675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O675" t="inlineStr"/>
+      <c r="P675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q675" t="inlineStr"/>
+      <c r="R675" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>John Lee Dumas</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Host, Entrepreneurs on Fire</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>EOFire</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Daily podcast with 100M+ listens, 3000+ entrepreneur interviews</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr"/>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr"/>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr"/>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K676" t="inlineStr"/>
+      <c r="L676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M676" t="inlineStr"/>
+      <c r="N676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O676" t="inlineStr"/>
+      <c r="P676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q676" t="inlineStr"/>
+      <c r="R676" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Jocko Willink</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Host, Jocko Podcast</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Echelon Front</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Former Navy SEAL commander, discipline-focused leadership, 250K-1M monthly listeners</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr"/>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr"/>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>@jaborraz</t>
+        </is>
+      </c>
+      <c r="L677" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M677" t="inlineStr"/>
+      <c r="N677" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O677" t="inlineStr"/>
+      <c r="P677" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q677" t="inlineStr"/>
+      <c r="R677" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
@@ -41833,7 +42880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -42661,6 +43708,26 @@
       <c r="D41" t="inlineStr">
         <is>
           <t>facilitation-workshop-design</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>17</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>leadership-podcasters</t>
         </is>
       </c>
     </row>
@@ -42676,7 +43743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G313"/>
+  <dimension ref="A1:G321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -54129,6 +55196,302 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>69c4ccb9ea5839fe524df00f</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>2026-04-06T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>69c4ccd81acfeeec28fd3d0e</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>2026-04-06T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>69c4ccbb1acfeeec28fd3c43</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>2026-04-06T10:52:00Z</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>69c4ccbcea5839fe524df062</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>2026-04-06T17:02:00Z</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>69c4ccd91acfeeec28fd3d33</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>2026-04-02T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>69c4ccdbea5839fe524df0db</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>2026-05-13T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>69c4ccbeea5839fe524df088</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>2026-04-06T22:02:00Z</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Leadership Podcasters</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>69c4ccbd1acfeeec28fd3c7b</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>2026-04-06T14:01:00Z</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — Military to Civilian Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1462,7 +1462,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1623,7 +1628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y677"/>
+  <dimension ref="A1:Y694"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41749,7 +41754,6 @@
           <t>500+ episodes interviewing world-class leaders on habits and mindsets of sustained excellence</t>
         </is>
       </c>
-      <c r="E661" t="inlineStr"/>
       <c r="F661" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41765,7 +41769,6 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="I661" t="inlineStr"/>
       <c r="J661" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41781,19 +41784,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M661" t="inlineStr"/>
       <c r="N661" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O661" t="inlineStr"/>
       <c r="P661" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q661" t="inlineStr"/>
       <c r="R661" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41821,19 +41821,16 @@
           <t>50M+ downloads since 2011, weekly leadership development podcast, Dale Carnegie trainer</t>
         </is>
       </c>
-      <c r="E662" t="inlineStr"/>
       <c r="F662" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G662" t="inlineStr"/>
       <c r="H662" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I662" t="inlineStr"/>
       <c r="J662" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41849,19 +41846,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M662" t="inlineStr"/>
       <c r="N662" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O662" t="inlineStr"/>
       <c r="P662" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q662" t="inlineStr"/>
       <c r="R662" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41889,43 +41883,36 @@
           <t>Takes listeners inside real executive coaching sessions, making leadership coaching accessible</t>
         </is>
       </c>
-      <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G663" t="inlineStr"/>
       <c r="H663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I663" t="inlineStr"/>
       <c r="J663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K663" t="inlineStr"/>
       <c r="L663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M663" t="inlineStr"/>
       <c r="N663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O663" t="inlineStr"/>
       <c r="P663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q663" t="inlineStr"/>
       <c r="R663" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41953,7 +41940,6 @@
           <t>TED podcast offering fast actionable leadership solutions with Frances Frei</t>
         </is>
       </c>
-      <c r="E664" t="inlineStr"/>
       <c r="F664" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -41969,31 +41955,26 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I664" t="inlineStr"/>
       <c r="J664" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K664" t="inlineStr"/>
       <c r="L664" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M664" t="inlineStr"/>
       <c r="N664" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O664" t="inlineStr"/>
       <c r="P664" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q664" t="inlineStr"/>
       <c r="R664" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42021,43 +42002,36 @@
           <t>Former Army Special Forces, 420+ episodes interviewing great leaders</t>
         </is>
       </c>
-      <c r="E665" t="inlineStr"/>
       <c r="F665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G665" t="inlineStr"/>
       <c r="H665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I665" t="inlineStr"/>
       <c r="J665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K665" t="inlineStr"/>
       <c r="L665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M665" t="inlineStr"/>
       <c r="N665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O665" t="inlineStr"/>
       <c r="P665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q665" t="inlineStr"/>
       <c r="R665" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42085,43 +42059,36 @@
           <t>C-level business strategist co-hosting with Jan Rutherford</t>
         </is>
       </c>
-      <c r="E666" t="inlineStr"/>
       <c r="F666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G666" t="inlineStr"/>
       <c r="H666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I666" t="inlineStr"/>
       <c r="J666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K666" t="inlineStr"/>
       <c r="L666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M666" t="inlineStr"/>
       <c r="N666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O666" t="inlineStr"/>
       <c r="P666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q666" t="inlineStr"/>
       <c r="R666" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42149,7 +42116,6 @@
           <t>Gold Stevie Award winner, 600+ CEO interviews, top 2% globally</t>
         </is>
       </c>
-      <c r="E667" t="inlineStr"/>
       <c r="F667" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42165,7 +42131,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I667" t="inlineStr"/>
       <c r="J667" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42181,19 +42146,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M667" t="inlineStr"/>
       <c r="N667" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O667" t="inlineStr"/>
       <c r="P667" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q667" t="inlineStr"/>
       <c r="R667" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42221,7 +42183,6 @@
           <t>1200+ episodes since 2014 with Inc company founders on leadership growth</t>
         </is>
       </c>
-      <c r="E668" t="inlineStr"/>
       <c r="F668" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42237,31 +42198,26 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I668" t="inlineStr"/>
       <c r="J668" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K668" t="inlineStr"/>
       <c r="L668" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M668" t="inlineStr"/>
       <c r="N668" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O668" t="inlineStr"/>
       <c r="P668" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q668" t="inlineStr"/>
       <c r="R668" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42289,7 +42245,6 @@
           <t>100M+ listens, 3000+ episodes, built YAP Media empire from podcast</t>
         </is>
       </c>
-      <c r="E669" t="inlineStr"/>
       <c r="F669" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42305,7 +42260,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I669" t="inlineStr"/>
       <c r="J669" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42331,13 +42285,11 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="O669" t="inlineStr"/>
       <c r="P669" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q669" t="inlineStr"/>
       <c r="R669" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42365,7 +42317,6 @@
           <t>Australian leadership expert, 3M+ downloads, WSJ bestselling author</t>
         </is>
       </c>
-      <c r="E670" t="inlineStr"/>
       <c r="F670" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42381,31 +42332,26 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I670" t="inlineStr"/>
       <c r="J670" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K670" t="inlineStr"/>
       <c r="L670" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M670" t="inlineStr"/>
       <c r="N670" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O670" t="inlineStr"/>
       <c r="P670" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q670" t="inlineStr"/>
       <c r="R670" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42433,43 +42379,36 @@
           <t>Iconic storytelling podcast exploring how entrepreneurs built famous companies</t>
         </is>
       </c>
-      <c r="E671" t="inlineStr"/>
       <c r="F671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G671" t="inlineStr"/>
       <c r="H671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I671" t="inlineStr"/>
       <c r="J671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K671" t="inlineStr"/>
       <c r="L671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M671" t="inlineStr"/>
       <c r="N671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O671" t="inlineStr"/>
       <c r="P671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q671" t="inlineStr"/>
       <c r="R671" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42497,19 +42436,16 @@
           <t>Executive Editor at HBR hosting one of longest-running business podcasts</t>
         </is>
       </c>
-      <c r="E672" t="inlineStr"/>
       <c r="F672" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G672" t="inlineStr"/>
       <c r="H672" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I672" t="inlineStr"/>
       <c r="J672" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42525,19 +42461,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M672" t="inlineStr"/>
       <c r="N672" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O672" t="inlineStr"/>
       <c r="P672" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q672" t="inlineStr"/>
       <c r="R672" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42565,43 +42498,36 @@
           <t>Fortune podcast featuring CEO interviews on business transformation</t>
         </is>
       </c>
-      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G673" t="inlineStr"/>
       <c r="H673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I673" t="inlineStr"/>
       <c r="J673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K673" t="inlineStr"/>
       <c r="L673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M673" t="inlineStr"/>
       <c r="N673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O673" t="inlineStr"/>
       <c r="P673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q673" t="inlineStr"/>
       <c r="R673" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42629,43 +42555,36 @@
           <t>Celebrates firebrand leaders with ingenuity in underrepresented communities</t>
         </is>
       </c>
-      <c r="E674" t="inlineStr"/>
       <c r="F674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G674" t="inlineStr"/>
       <c r="H674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I674" t="inlineStr"/>
       <c r="J674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K674" t="inlineStr"/>
       <c r="L674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M674" t="inlineStr"/>
       <c r="N674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O674" t="inlineStr"/>
       <c r="P674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q674" t="inlineStr"/>
       <c r="R674" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42693,43 +42612,36 @@
           <t>23 years at FranklinCovey, reaches 5M+ leaders weekly, Master Mentors author</t>
         </is>
       </c>
-      <c r="E675" t="inlineStr"/>
       <c r="F675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G675" t="inlineStr"/>
       <c r="H675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I675" t="inlineStr"/>
       <c r="J675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K675" t="inlineStr"/>
       <c r="L675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M675" t="inlineStr"/>
       <c r="N675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O675" t="inlineStr"/>
       <c r="P675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q675" t="inlineStr"/>
       <c r="R675" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42757,43 +42669,36 @@
           <t>Daily podcast with 100M+ listens, 3000+ entrepreneur interviews</t>
         </is>
       </c>
-      <c r="E676" t="inlineStr"/>
       <c r="F676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G676" t="inlineStr"/>
       <c r="H676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I676" t="inlineStr"/>
       <c r="J676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K676" t="inlineStr"/>
       <c r="L676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M676" t="inlineStr"/>
       <c r="N676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O676" t="inlineStr"/>
       <c r="P676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q676" t="inlineStr"/>
       <c r="R676" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42821,19 +42726,16 @@
           <t>Former Navy SEAL commander, discipline-focused leadership, 250K-1M monthly listeners</t>
         </is>
       </c>
-      <c r="E677" t="inlineStr"/>
       <c r="F677" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G677" t="inlineStr"/>
       <c r="H677" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I677" t="inlineStr"/>
       <c r="J677" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42849,20 +42751,1225 @@
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="M677" t="inlineStr"/>
       <c r="N677" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O677" t="inlineStr"/>
       <c r="P677" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q677" t="inlineStr"/>
       <c r="R677" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Mike Erwin</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Founder &amp; Executive Director</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Team Red White &amp; Blue</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>West Point grad, 3x combat veteran, author of Lead Yourself First and Leadership is a Relationship</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>TeamRWB</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>@teamrwb</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr"/>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>@teamrwb</t>
+        </is>
+      </c>
+      <c r="L678" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M678" t="inlineStr"/>
+      <c r="N678" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O678" t="inlineStr">
+        <is>
+          <t>Team Red White &amp; Blue</t>
+        </is>
+      </c>
+      <c r="P678" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="Q678" t="inlineStr"/>
+      <c r="R678" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Stan McChrystal</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>McChrystal Group</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Retired 4-star general, author of Team of Teams and On Character</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>@stanmcchrystal</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr"/>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>@StanMcChrystal</t>
+        </is>
+      </c>
+      <c r="L679" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M679" t="inlineStr"/>
+      <c r="N679" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O679" t="inlineStr"/>
+      <c r="P679" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q679" t="inlineStr"/>
+      <c r="R679" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Mike Abrashoff</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Former USS Benfold commander, author of It's Your Ship (1M+ copies sold)</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr"/>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr"/>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr"/>
+      <c r="L680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M680" t="inlineStr"/>
+      <c r="N680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O680" t="inlineStr"/>
+      <c r="P680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q680" t="inlineStr"/>
+      <c r="R680" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Tom Kolditz</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Doerr Institute, Rice University</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Retired Brigadier General, built world's largest university-based leader development program</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr"/>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr"/>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K681" t="inlineStr"/>
+      <c r="L681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M681" t="inlineStr"/>
+      <c r="N681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O681" t="inlineStr"/>
+      <c r="P681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q681" t="inlineStr"/>
+      <c r="R681" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Nicole Malachowski</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Advocate</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Nicole Malachowski &amp; Associates</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>First female Thunderbird pilot, National Women's Hall of Fame, combat veteran</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>NicoleMalachowskiLLC</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>@realmalachowski</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr"/>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K682" t="inlineStr">
+        <is>
+          <t>@RealMalachowski</t>
+        </is>
+      </c>
+      <c r="L682" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M682" t="inlineStr"/>
+      <c r="N682" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O682" t="inlineStr"/>
+      <c r="P682" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q682" t="inlineStr"/>
+      <c r="R682" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Carey Lohrenz</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Author</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>First female F-14 Tomcat pilot, author of Fearless Leadership</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>@careylohrenz</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr"/>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K683" t="inlineStr">
+        <is>
+          <t>@CareyLohrenz</t>
+        </is>
+      </c>
+      <c r="L683" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M683" t="inlineStr"/>
+      <c r="N683" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O683" t="inlineStr"/>
+      <c r="P683" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q683" t="inlineStr"/>
+      <c r="R683" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Rorke Denver</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Ever Onward</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Navy SEAL Commander, NYT bestselling author of Damn Few, starred in Act of Valor</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>@rorkedenverauthor</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>@rorketdenver</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr"/>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K684" t="inlineStr"/>
+      <c r="L684" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M684" t="inlineStr"/>
+      <c r="N684" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O684" t="inlineStr"/>
+      <c r="P684" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q684" t="inlineStr"/>
+      <c r="R684" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Jason Redman</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Coach</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Retired Navy SEAL shot 8 times in combat, author of Overcome and The Trident</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>@jasonredmanww</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr"/>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K685" t="inlineStr">
+        <is>
+          <t>@JasonRedmanWW</t>
+        </is>
+      </c>
+      <c r="L685" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M685" t="inlineStr">
+        <is>
+          <t>@jasonredmanww</t>
+        </is>
+      </c>
+      <c r="N685" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="O685" t="inlineStr"/>
+      <c r="P685" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q685" t="inlineStr"/>
+      <c r="R685" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Jeff Boss</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Adaptability Consultant</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Former DEVGRU operator, Forbes/Entrepreneur contributor, author of Navigating Chaos</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr"/>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr"/>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K686" t="inlineStr"/>
+      <c r="L686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M686" t="inlineStr"/>
+      <c r="N686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O686" t="inlineStr"/>
+      <c r="P686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q686" t="inlineStr"/>
+      <c r="R686" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Chad Storlie</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Author &amp; Adjunct Professor</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Retired Green Beret, author of Combat Leader to Corporate Leader, 80+ publications in HBR/Forbes</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr"/>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr"/>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K687" t="inlineStr"/>
+      <c r="L687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M687" t="inlineStr"/>
+      <c r="N687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O687" t="inlineStr"/>
+      <c r="P687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q687" t="inlineStr"/>
+      <c r="R687" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Larry Broughton</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Broughton Hotels / Yoogozi</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Former Green Beret, award-winning hotelier, mentor, keynote speaker on veteran entrepreneurship</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>larrybroughton</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>@larrybroughton</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr"/>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K688" t="inlineStr">
+        <is>
+          <t>@larrybroughton</t>
+        </is>
+      </c>
+      <c r="L688" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M688" t="inlineStr"/>
+      <c r="N688" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O688" t="inlineStr"/>
+      <c r="P688" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q688" t="inlineStr"/>
+      <c r="R688" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Shawn Ryan</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Podcast Host</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>The Shawn Ryan Show / Vigilance Elite</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Former Navy SEAL &amp; CIA contractor, top-10 Spotify podcast host</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>ShawnRyanShow</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>@shawnryan762</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr"/>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K689" t="inlineStr">
+        <is>
+          <t>@ShawnRyanShow</t>
+        </is>
+      </c>
+      <c r="L689" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M689" t="inlineStr">
+        <is>
+          <t>@shawnryanshow</t>
+        </is>
+      </c>
+      <c r="N689" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="O689" t="inlineStr">
+        <is>
+          <t>Shawn Ryan Show</t>
+        </is>
+      </c>
+      <c r="P689" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="Q689" t="inlineStr"/>
+      <c r="R689" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Andy Stumpf</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Podcast Host</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Cleared Hot Podcast</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Former DEVGRU operator, world record holder, leadership podcaster</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr"/>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>@andystumpf212</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr"/>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K690" t="inlineStr">
+        <is>
+          <t>@AndyStumpf77</t>
+        </is>
+      </c>
+      <c r="L690" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M690" t="inlineStr"/>
+      <c r="N690" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O690" t="inlineStr"/>
+      <c r="P690" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q690" t="inlineStr"/>
+      <c r="R690" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Wes Moore</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Governor</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>State of Maryland</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>82nd Airborne combat veteran, bestselling author of The Other Wes Moore</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>@iamwesmoore</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr"/>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr"/>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K691" t="inlineStr">
+        <is>
+          <t>@iamwesmoore</t>
+        </is>
+      </c>
+      <c r="L691" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M691" t="inlineStr"/>
+      <c r="N691" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O691" t="inlineStr"/>
+      <c r="P691" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q691" t="inlineStr"/>
+      <c r="R691" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Nick Lavery</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Active Duty Green Beret</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>U.S. Army Special Forces</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Only amputee in Special Forces history still serving on active duty after 30+ surgeries</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>@nick.machine.lavery</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr"/>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K692" t="inlineStr"/>
+      <c r="L692" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M692" t="inlineStr"/>
+      <c r="N692" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O692" t="inlineStr"/>
+      <c r="P692" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q692" t="inlineStr"/>
+      <c r="R692" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Curtez Riggs</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Founder &amp; President</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Military Influencer Conference</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Army veteran who built the premier annual gathering for military entrepreneurs &amp; creators</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>@curtezriggs</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr"/>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K693" t="inlineStr"/>
+      <c r="L693" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M693" t="inlineStr"/>
+      <c r="N693" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O693" t="inlineStr"/>
+      <c r="P693" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q693" t="inlineStr"/>
+      <c r="R693" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Lavar Matthews</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Speaker &amp; Strategist</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Decorated Army veteran, Columbia-trained human capital strategist on inclusive leadership</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr"/>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr"/>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr"/>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K694" t="inlineStr"/>
+      <c r="L694" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M694" t="inlineStr"/>
+      <c r="N694" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O694" t="inlineStr"/>
+      <c r="P694" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Q694" t="inlineStr"/>
+      <c r="R694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
@@ -42880,7 +43987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -43728,6 +44835,26 @@
       <c r="D42" t="inlineStr">
         <is>
           <t>leadership-podcasters</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>17</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>military-to-civilian-leadership</t>
         </is>
       </c>
     </row>
@@ -43743,7 +44870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G321"/>
+  <dimension ref="A1:G329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -55492,6 +56619,302 @@
         </is>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>60370296a73c5c70fa70c977</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>69c4d89bea5839fe524e1240</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>2026-04-06T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>69bb7e247be9f8b1716f91c7</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>69c4d89d1acfeeec28fd5eee</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>2026-04-06T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>69bb7ee47be9f8b1716f9388</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>69c4d8a0ea5839fe524e1266</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>2026-04-06T11:01:00Z</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>69bb7e7b7be9f8b1716f927a</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>69c4d8cc1acfeeec28fd5faf</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>2026-03-31T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>69bb7fdc7be9f8b1716f9570</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>69c4d8b51acfeeec28fd5f1c</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>2026-04-06T18:01:00Z</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>69bb7eff7be9f8b1716f93c9</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>69c4d8d6ea5839fe524e1364</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>2026-04-12T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>69bb7f1d7be9f8b1716f9409</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>69c4d8b6ea5839fe524e12a9</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>2026-04-06T23:01:00Z</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Military to Civilian Leadership</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>69c4d8b71acfeeec28fd5f42</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>2026-04-06T15:02:00Z</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database — EdTech Leadership
</commit_message>
<xml_diff>
--- a/data/handle-database.xlsx
+++ b/data/handle-database.xlsx
@@ -1487,7 +1487,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1628,7 +1633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y694"/>
+  <dimension ref="A1:Y727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -42808,7 +42813,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I678" t="inlineStr"/>
       <c r="J678" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42824,7 +42828,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M678" t="inlineStr"/>
       <c r="N678" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42840,7 +42843,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="Q678" t="inlineStr"/>
       <c r="R678" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42868,7 +42870,6 @@
           <t>Retired 4-star general, author of Team of Teams and On Character</t>
         </is>
       </c>
-      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42884,7 +42885,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I679" t="inlineStr"/>
       <c r="J679" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42900,19 +42900,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M679" t="inlineStr"/>
       <c r="N679" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O679" t="inlineStr"/>
       <c r="P679" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q679" t="inlineStr"/>
       <c r="R679" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -42940,43 +42937,36 @@
           <t>Former USS Benfold commander, author of It's Your Ship (1M+ copies sold)</t>
         </is>
       </c>
-      <c r="E680" t="inlineStr"/>
       <c r="F680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G680" t="inlineStr"/>
       <c r="H680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I680" t="inlineStr"/>
       <c r="J680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K680" t="inlineStr"/>
       <c r="L680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M680" t="inlineStr"/>
       <c r="N680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O680" t="inlineStr"/>
       <c r="P680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q680" t="inlineStr"/>
       <c r="R680" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43004,43 +42994,36 @@
           <t>Retired Brigadier General, built world's largest university-based leader development program</t>
         </is>
       </c>
-      <c r="E681" t="inlineStr"/>
       <c r="F681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G681" t="inlineStr"/>
       <c r="H681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I681" t="inlineStr"/>
       <c r="J681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K681" t="inlineStr"/>
       <c r="L681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M681" t="inlineStr"/>
       <c r="N681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O681" t="inlineStr"/>
       <c r="P681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q681" t="inlineStr"/>
       <c r="R681" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43088,7 +43071,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I682" t="inlineStr"/>
       <c r="J682" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43104,19 +43086,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M682" t="inlineStr"/>
       <c r="N682" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O682" t="inlineStr"/>
       <c r="P682" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q682" t="inlineStr"/>
       <c r="R682" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43144,7 +43123,6 @@
           <t>First female F-14 Tomcat pilot, author of Fearless Leadership</t>
         </is>
       </c>
-      <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43160,7 +43138,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I683" t="inlineStr"/>
       <c r="J683" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43176,19 +43153,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M683" t="inlineStr"/>
       <c r="N683" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O683" t="inlineStr"/>
       <c r="P683" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q683" t="inlineStr"/>
       <c r="R683" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43236,31 +43210,26 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I684" t="inlineStr"/>
       <c r="J684" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K684" t="inlineStr"/>
       <c r="L684" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M684" t="inlineStr"/>
       <c r="N684" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O684" t="inlineStr"/>
       <c r="P684" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q684" t="inlineStr"/>
       <c r="R684" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43288,7 +43257,6 @@
           <t>Retired Navy SEAL shot 8 times in combat, author of Overcome and The Trident</t>
         </is>
       </c>
-      <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43304,7 +43272,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I685" t="inlineStr"/>
       <c r="J685" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43330,13 +43297,11 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="O685" t="inlineStr"/>
       <c r="P685" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q685" t="inlineStr"/>
       <c r="R685" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43364,43 +43329,36 @@
           <t>Former DEVGRU operator, Forbes/Entrepreneur contributor, author of Navigating Chaos</t>
         </is>
       </c>
-      <c r="E686" t="inlineStr"/>
       <c r="F686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G686" t="inlineStr"/>
       <c r="H686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I686" t="inlineStr"/>
       <c r="J686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K686" t="inlineStr"/>
       <c r="L686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M686" t="inlineStr"/>
       <c r="N686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O686" t="inlineStr"/>
       <c r="P686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q686" t="inlineStr"/>
       <c r="R686" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43428,43 +43386,36 @@
           <t>Retired Green Beret, author of Combat Leader to Corporate Leader, 80+ publications in HBR/Forbes</t>
         </is>
       </c>
-      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G687" t="inlineStr"/>
       <c r="H687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I687" t="inlineStr"/>
       <c r="J687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K687" t="inlineStr"/>
       <c r="L687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M687" t="inlineStr"/>
       <c r="N687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O687" t="inlineStr"/>
       <c r="P687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q687" t="inlineStr"/>
       <c r="R687" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43512,7 +43463,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I688" t="inlineStr"/>
       <c r="J688" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43528,19 +43478,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M688" t="inlineStr"/>
       <c r="N688" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O688" t="inlineStr"/>
       <c r="P688" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q688" t="inlineStr"/>
       <c r="R688" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43588,7 +43535,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I689" t="inlineStr"/>
       <c r="J689" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43624,7 +43570,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="Q689" t="inlineStr"/>
       <c r="R689" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43652,7 +43597,6 @@
           <t>Former DEVGRU operator, world record holder, leadership podcaster</t>
         </is>
       </c>
-      <c r="E690" t="inlineStr"/>
       <c r="F690" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43668,7 +43612,6 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I690" t="inlineStr"/>
       <c r="J690" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43684,19 +43627,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M690" t="inlineStr"/>
       <c r="N690" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O690" t="inlineStr"/>
       <c r="P690" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q690" t="inlineStr"/>
       <c r="R690" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43734,13 +43674,11 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="G691" t="inlineStr"/>
       <c r="H691" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I691" t="inlineStr"/>
       <c r="J691" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43756,19 +43694,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="M691" t="inlineStr"/>
       <c r="N691" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O691" t="inlineStr"/>
       <c r="P691" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q691" t="inlineStr"/>
       <c r="R691" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43796,7 +43731,6 @@
           <t>Only amputee in Special Forces history still serving on active duty after 30+ surgeries</t>
         </is>
       </c>
-      <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43812,31 +43746,26 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I692" t="inlineStr"/>
       <c r="J692" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K692" t="inlineStr"/>
       <c r="L692" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M692" t="inlineStr"/>
       <c r="N692" t="inlineStr">
         <is>
           <t>LIKELY</t>
         </is>
       </c>
-      <c r="O692" t="inlineStr"/>
       <c r="P692" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q692" t="inlineStr"/>
       <c r="R692" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43864,7 +43793,6 @@
           <t>Army veteran who built the premier annual gathering for military entrepreneurs &amp; creators</t>
         </is>
       </c>
-      <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43880,31 +43808,26 @@
           <t>VERIFIED</t>
         </is>
       </c>
-      <c r="I693" t="inlineStr"/>
       <c r="J693" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K693" t="inlineStr"/>
       <c r="L693" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M693" t="inlineStr"/>
       <c r="N693" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O693" t="inlineStr"/>
       <c r="P693" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q693" t="inlineStr"/>
       <c r="R693" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
@@ -43932,48 +43855,2832 @@
           <t>Decorated Army veteran, Columbia-trained human capital strategist on inclusive leadership</t>
         </is>
       </c>
-      <c r="E694" t="inlineStr"/>
       <c r="F694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="G694" t="inlineStr"/>
       <c r="H694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="I694" t="inlineStr"/>
       <c r="J694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="K694" t="inlineStr"/>
       <c r="L694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M694" t="inlineStr"/>
       <c r="N694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="O694" t="inlineStr"/>
       <c r="P694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Q694" t="inlineStr"/>
       <c r="R694" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Monica Burns</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>EdTech Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Class Tech Tips</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Apple Distinguished Educator, Easy EdTech Podcast</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>classtechtips</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>classtechtips</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K695" t="inlineStr">
+        <is>
+          <t>classtechtips</t>
+        </is>
+      </c>
+      <c r="L695" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M695" t="inlineStr"/>
+      <c r="N695" t="inlineStr">
+        <is>
+          <t>ClassTechTips</t>
+        </is>
+      </c>
+      <c r="O695" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P695" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q695" t="inlineStr">
+        <is>
+          <t>classtechtips</t>
+        </is>
+      </c>
+      <c r="R695" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S695" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="T695" t="inlineStr">
+        <is>
+          <t>ClassTechTips</t>
+        </is>
+      </c>
+      <c r="U695" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V695" t="inlineStr"/>
+      <c r="W695" t="inlineStr"/>
+      <c r="X695" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y695" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Vicki Davis</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Instructional Technology Director</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Cool Cat Teacher</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>10-Minute Teacher Podcast, 162K+ followers</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>coolcatteacher</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr"/>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>coolcatteacher</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K696" t="inlineStr">
+        <is>
+          <t>coolcatteacher</t>
+        </is>
+      </c>
+      <c r="L696" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M696" t="inlineStr"/>
+      <c r="N696" t="inlineStr">
+        <is>
+          <t>coolcatteacher</t>
+        </is>
+      </c>
+      <c r="O696" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P696" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q696" t="inlineStr">
+        <is>
+          <t>coolcatteacher</t>
+        </is>
+      </c>
+      <c r="R696" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S696" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="T696" t="inlineStr">
+        <is>
+          <t>coolcatteacher</t>
+        </is>
+      </c>
+      <c r="U696" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V696" t="inlineStr"/>
+      <c r="W696" t="inlineStr">
+        <is>
+          <t>coolcatteacher.com</t>
+        </is>
+      </c>
+      <c r="X696" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y696" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Richard Culatta</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>ISTE+ASCD</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Author of Digital for Good, former FCC advisor</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>richardculatta</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>rculatta</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K697" t="inlineStr"/>
+      <c r="L697" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M697" t="inlineStr"/>
+      <c r="N697" t="inlineStr">
+        <is>
+          <t>rec54</t>
+        </is>
+      </c>
+      <c r="O697" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P697" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q697" t="inlineStr"/>
+      <c r="R697" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S697" t="inlineStr"/>
+      <c r="T697" t="inlineStr"/>
+      <c r="U697" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V697" t="inlineStr"/>
+      <c r="W697" t="inlineStr"/>
+      <c r="X697" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y697" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Matt Miller</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Ditch That Textbook</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Top 10 edtech influencer worldwide</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>ditchthattextbook</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>facebook.com</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>ditchthattextbook</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K698" t="inlineStr">
+        <is>
+          <t>ditchthattextbook</t>
+        </is>
+      </c>
+      <c r="L698" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M698" t="inlineStr"/>
+      <c r="N698" t="inlineStr">
+        <is>
+          <t>jmattmiller</t>
+        </is>
+      </c>
+      <c r="O698" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P698" t="inlineStr">
+        <is>
+          <t>x.com</t>
+        </is>
+      </c>
+      <c r="Q698" t="inlineStr">
+        <is>
+          <t>ditchthattextbook</t>
+        </is>
+      </c>
+      <c r="R698" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="S698" t="inlineStr">
+        <is>
+          <t>tiktok.com</t>
+        </is>
+      </c>
+      <c r="T698" t="inlineStr">
+        <is>
+          <t>DitchThatTextbook</t>
+        </is>
+      </c>
+      <c r="U698" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V698" t="inlineStr"/>
+      <c r="W698" t="inlineStr">
+        <is>
+          <t>ditchthattextbook.com</t>
+        </is>
+      </c>
+      <c r="X698" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="Y698" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Kasey Bell</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Digital Learning Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Shake Up Learning</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Google Certified Innovator, podcast host</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>shakeuplearning</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr"/>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>shakeuplearning</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>instagram.com</t>
+        </is>
+      </c>
+      <c r="K699" t="inlineStr">
+        <is>
+          <t>shakeuplearning</t>
+        </is>
+      </c>
+      <c r="L699" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M699" t="inlineStr">
+        <is>
+          <t>threads.net</t>
+        </is>
+      </c>
+      <c r="N699" t="inlineStr"/>
+      <c r="O699" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P699" t="inlineStr"/>
+      <c r="Q699" t="inlineStr"/>
+      <c r="R699" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S699" t="inlineStr"/>
+      <c r="T699" t="inlineStr">
+        <is>
+          <t>ShakeUpLearning</t>
+        </is>
+      </c>
+      <c r="U699" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="V699" t="inlineStr"/>
+      <c r="W699" t="inlineStr"/>
+      <c r="X699" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y699" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Alfonso Mendoza</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Digital Learning Coordinator</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Sharyland ISD</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>My EdTech Life podcast host</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>MyEdTechLife</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr"/>
+      <c r="H700" t="inlineStr"/>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J700" t="inlineStr"/>
+      <c r="K700" t="inlineStr"/>
+      <c r="L700" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M700" t="inlineStr"/>
+      <c r="N700" t="inlineStr">
+        <is>
+          <t>MyEdTechLife</t>
+        </is>
+      </c>
+      <c r="O700" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P700" t="inlineStr"/>
+      <c r="Q700" t="inlineStr"/>
+      <c r="R700" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="S700" t="inlineStr"/>
+      <c r="T700" t="inlineStr"/>
+      <c r="U700" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="V700" t="inlineStr"/>
+      <c r="W700" t="inlineStr"/>
+      <c r="X700" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="Y700" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Jean-Claude Brizard</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Digital Promise</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Former Chicago Public Schools CEO</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>BrizardJC</t>
+     